<commit_message>
Update tracker via web editor (1 edits)
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2080" uniqueCount="827">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2080" uniqueCount="826">
   <si>
     <t>Hana Aliyah Mufidah</t>
   </si>
@@ -1546,7 +1546,7 @@
     <t>YES — rewrite all drafts in own voice before pasting</t>
   </si>
   <si>
-    <t>Submitted</t>
+    <t>Not submitted</t>
   </si>
   <si>
     <t>Score 4.5/5 — see career-ops/reports/001-tether-2026-05-06.md</t>
@@ -1577,9 +1577,6 @@
   </si>
   <si>
     <t>60–90s; open with one specific Bitfinex KYC pain point I have observed; one sentence on why frontend specifically (React/Redux + KYC); one Nespay proof (Sumsub + Kredibel on React/Next); one question on KYC roadmap. Bullets only.</t>
-  </si>
-  <si>
-    <t>Not submitted</t>
   </si>
   <si>
     <t>Score 4.2/5 — see career-ops/reports/002-tether-2026-05-06.md. Gaps: Redux + SASS not on CV; brush up Redux Toolkit before interview.</t>
@@ -10533,10 +10530,10 @@
         <v>508</v>
       </c>
       <c r="R3" s="21" t="s">
+        <v>509</v>
+      </c>
+      <c r="S3" s="21" t="s">
         <v>520</v>
-      </c>
-      <c r="S3" s="21" t="s">
-        <v>521</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
@@ -10544,46 +10541,46 @@
         <f>ROW()-1</f>
       </c>
       <c r="B4" s="21" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="C4" s="21" t="s">
         <v>78</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E4" s="21" t="s">
         <v>88</v>
       </c>
       <c r="F4" s="21" t="s">
+        <v>523</v>
+      </c>
+      <c r="G4" s="21" t="s">
         <v>524</v>
       </c>
-      <c r="G4" s="21" t="s">
+      <c r="H4" s="21" t="s">
         <v>525</v>
       </c>
-      <c r="H4" s="21" t="s">
+      <c r="I4" s="21" t="s">
+        <v>525</v>
+      </c>
+      <c r="J4" s="21" t="s">
+        <v>525</v>
+      </c>
+      <c r="K4" s="21" t="s">
+        <v>525</v>
+      </c>
+      <c r="L4" s="21" t="s">
+        <v>525</v>
+      </c>
+      <c r="M4" s="21" t="s">
         <v>526</v>
       </c>
-      <c r="I4" s="21" t="s">
-        <v>526</v>
-      </c>
-      <c r="J4" s="21" t="s">
-        <v>526</v>
-      </c>
-      <c r="K4" s="21" t="s">
-        <v>526</v>
-      </c>
-      <c r="L4" s="21" t="s">
-        <v>526</v>
-      </c>
-      <c r="M4" s="21" t="s">
+      <c r="N4" s="21" t="s">
         <v>527</v>
       </c>
-      <c r="N4" s="21" t="s">
+      <c r="O4" s="21" t="s">
         <v>528</v>
-      </c>
-      <c r="O4" s="21" t="s">
-        <v>529</v>
       </c>
       <c r="P4" s="21" t="s">
         <v>507</v>
@@ -10592,10 +10589,10 @@
         <v>508</v>
       </c>
       <c r="R4" s="21" t="s">
-        <v>520</v>
+        <v>509</v>
       </c>
       <c r="S4" s="21" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
     </row>
   </sheetData>
@@ -10688,7 +10685,7 @@
         <v>61</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>14</v>
@@ -10697,10 +10694,10 @@
         <v>13</v>
       </c>
       <c r="E1" s="7" t="s">
+        <v>531</v>
+      </c>
+      <c r="F1" s="7" t="s">
         <v>532</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>533</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>63</v>
@@ -10709,28 +10706,28 @@
         <v>44</v>
       </c>
       <c r="I1" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="J1" s="7" t="s">
         <v>534</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="K1" s="7" t="s">
         <v>535</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="L1" s="7" t="s">
         <v>536</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="M1" s="7" t="s">
         <v>537</v>
       </c>
-      <c r="M1" s="7" t="s">
+      <c r="N1" s="7" t="s">
         <v>538</v>
       </c>
-      <c r="N1" s="7" t="s">
+      <c r="O1" s="7" t="s">
         <v>539</v>
       </c>
-      <c r="O1" s="7" t="s">
+      <c r="P1" s="7" t="s">
         <v>540</v>
-      </c>
-      <c r="P1" s="7" t="s">
-        <v>541</v>
       </c>
       <c r="Q1" s="7" t="s">
         <v>69</v>
@@ -10741,7 +10738,7 @@
         <f>ROW()-1</f>
       </c>
       <c r="B2" s="1" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>78</v>
@@ -10758,7 +10755,7 @@
         <v>51</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>497</v>
@@ -10770,7 +10767,7 @@
       <c r="O2" s="1"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
@@ -15012,7 +15009,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -15028,16 +15025,16 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
+        <v>543</v>
+      </c>
+      <c r="D2" s="7" t="s">
         <v>544</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>545</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>69</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -15045,13 +15042,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="10" t="s">
+        <v>546</v>
+      </c>
+      <c r="C3" s="22" t="s">
         <v>547</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="D3" s="10" t="s">
         <v>548</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>549</v>
       </c>
       <c r="E3" s="10"/>
       <c r="F3" s="10"/>
@@ -15061,13 +15058,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="10" t="s">
+        <v>549</v>
+      </c>
+      <c r="C4" s="22" t="s">
         <v>550</v>
       </c>
-      <c r="C4" s="22" t="s">
-        <v>551</v>
-      </c>
       <c r="D4" s="10" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="E4" s="10"/>
       <c r="F4" s="10"/>
@@ -15077,16 +15074,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="10" t="s">
+        <v>551</v>
+      </c>
+      <c r="C5" s="22" t="s">
         <v>552</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="D5" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E5" s="10" t="s">
         <v>553</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>554</v>
       </c>
       <c r="F5" s="10"/>
     </row>
@@ -15098,13 +15095,13 @@
         <v>360</v>
       </c>
       <c r="C6" s="22" t="s">
+        <v>554</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E6" s="10" t="s">
         <v>555</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>556</v>
       </c>
       <c r="F6" s="10"/>
     </row>
@@ -15116,13 +15113,13 @@
         <v>287</v>
       </c>
       <c r="C7" s="22" t="s">
+        <v>556</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E7" s="10" t="s">
         <v>557</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>558</v>
       </c>
       <c r="F7" s="10"/>
     </row>
@@ -15131,16 +15128,16 @@
         <v>6</v>
       </c>
       <c r="B8" s="10" t="s">
+        <v>558</v>
+      </c>
+      <c r="C8" s="22" t="s">
         <v>559</v>
       </c>
-      <c r="C8" s="22" t="s">
+      <c r="D8" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E8" s="10" t="s">
         <v>560</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>561</v>
       </c>
       <c r="F8" s="10"/>
     </row>
@@ -15149,16 +15146,16 @@
         <v>7</v>
       </c>
       <c r="B9" s="10" t="s">
+        <v>561</v>
+      </c>
+      <c r="C9" s="22" t="s">
         <v>562</v>
       </c>
-      <c r="C9" s="22" t="s">
+      <c r="D9" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E9" s="10" t="s">
         <v>563</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>564</v>
       </c>
       <c r="F9" s="10"/>
     </row>
@@ -15170,13 +15167,13 @@
         <v>148</v>
       </c>
       <c r="C10" s="22" t="s">
+        <v>564</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E10" s="10" t="s">
         <v>565</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>566</v>
       </c>
       <c r="F10" s="10"/>
     </row>
@@ -15185,16 +15182,16 @@
         <v>9</v>
       </c>
       <c r="B11" s="10" t="s">
+        <v>566</v>
+      </c>
+      <c r="C11" s="22" t="s">
         <v>567</v>
       </c>
-      <c r="C11" s="22" t="s">
+      <c r="D11" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E11" s="10" t="s">
         <v>568</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>569</v>
       </c>
       <c r="F11" s="10"/>
     </row>
@@ -15203,16 +15200,16 @@
         <v>10</v>
       </c>
       <c r="B12" s="10" t="s">
+        <v>569</v>
+      </c>
+      <c r="C12" s="22" t="s">
         <v>570</v>
       </c>
-      <c r="C12" s="22" t="s">
+      <c r="D12" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E12" s="10" t="s">
         <v>571</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>572</v>
       </c>
       <c r="F12" s="10"/>
     </row>
@@ -15221,16 +15218,16 @@
         <v>11</v>
       </c>
       <c r="B13" s="10" t="s">
+        <v>572</v>
+      </c>
+      <c r="C13" s="22" t="s">
         <v>573</v>
       </c>
-      <c r="C13" s="22" t="s">
+      <c r="D13" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E13" s="10" t="s">
         <v>574</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>575</v>
       </c>
       <c r="F13" s="10"/>
     </row>
@@ -15239,16 +15236,16 @@
         <v>12</v>
       </c>
       <c r="B14" s="10" t="s">
+        <v>575</v>
+      </c>
+      <c r="C14" s="22" t="s">
         <v>576</v>
       </c>
-      <c r="C14" s="22" t="s">
+      <c r="D14" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E14" s="10" t="s">
         <v>577</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>578</v>
       </c>
       <c r="F14" s="10"/>
     </row>
@@ -15257,16 +15254,16 @@
         <v>13</v>
       </c>
       <c r="B15" s="10" t="s">
+        <v>578</v>
+      </c>
+      <c r="C15" s="22" t="s">
         <v>579</v>
       </c>
-      <c r="C15" s="22" t="s">
+      <c r="D15" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E15" s="10" t="s">
         <v>580</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>581</v>
       </c>
       <c r="F15" s="10"/>
     </row>
@@ -15275,16 +15272,16 @@
         <v>14</v>
       </c>
       <c r="B16" s="10" t="s">
+        <v>581</v>
+      </c>
+      <c r="C16" s="22" t="s">
         <v>582</v>
       </c>
-      <c r="C16" s="22" t="s">
+      <c r="D16" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E16" s="10" t="s">
         <v>583</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>584</v>
       </c>
       <c r="F16" s="10"/>
     </row>
@@ -15293,16 +15290,16 @@
         <v>15</v>
       </c>
       <c r="B17" s="10" t="s">
+        <v>584</v>
+      </c>
+      <c r="C17" s="22" t="s">
         <v>585</v>
       </c>
-      <c r="C17" s="22" t="s">
+      <c r="D17" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E17" s="10" t="s">
         <v>586</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>587</v>
       </c>
       <c r="F17" s="10"/>
     </row>
@@ -15311,16 +15308,16 @@
         <v>16</v>
       </c>
       <c r="B18" s="10" t="s">
+        <v>587</v>
+      </c>
+      <c r="C18" s="22" t="s">
         <v>588</v>
       </c>
-      <c r="C18" s="22" t="s">
+      <c r="D18" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E18" s="10" t="s">
         <v>589</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E18" s="10" t="s">
-        <v>590</v>
       </c>
       <c r="F18" s="10"/>
     </row>
@@ -15332,13 +15329,13 @@
         <v>185</v>
       </c>
       <c r="C19" s="22" t="s">
+        <v>590</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E19" s="10" t="s">
         <v>591</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E19" s="10" t="s">
-        <v>592</v>
       </c>
       <c r="F19" s="10"/>
     </row>
@@ -15347,16 +15344,16 @@
         <v>18</v>
       </c>
       <c r="B20" s="10" t="s">
+        <v>592</v>
+      </c>
+      <c r="C20" s="22" t="s">
         <v>593</v>
       </c>
-      <c r="C20" s="22" t="s">
+      <c r="D20" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E20" s="10" t="s">
         <v>594</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E20" s="10" t="s">
-        <v>595</v>
       </c>
       <c r="F20" s="10"/>
     </row>
@@ -15365,16 +15362,16 @@
         <v>19</v>
       </c>
       <c r="B21" s="10" t="s">
+        <v>595</v>
+      </c>
+      <c r="C21" s="22" t="s">
         <v>596</v>
       </c>
-      <c r="C21" s="22" t="s">
+      <c r="D21" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E21" s="10" t="s">
         <v>597</v>
-      </c>
-      <c r="D21" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E21" s="10" t="s">
-        <v>598</v>
       </c>
       <c r="F21" s="10"/>
     </row>
@@ -15383,16 +15380,16 @@
         <v>20</v>
       </c>
       <c r="B22" s="10" t="s">
+        <v>598</v>
+      </c>
+      <c r="C22" s="22" t="s">
         <v>599</v>
       </c>
-      <c r="C22" s="22" t="s">
+      <c r="D22" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E22" s="10" t="s">
         <v>600</v>
-      </c>
-      <c r="D22" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>601</v>
       </c>
       <c r="F22" s="10"/>
     </row>
@@ -15401,16 +15398,16 @@
         <v>21</v>
       </c>
       <c r="B23" s="10" t="s">
+        <v>601</v>
+      </c>
+      <c r="C23" s="22" t="s">
         <v>602</v>
       </c>
-      <c r="C23" s="22" t="s">
+      <c r="D23" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E23" s="10" t="s">
         <v>603</v>
-      </c>
-      <c r="D23" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E23" s="10" t="s">
-        <v>604</v>
       </c>
       <c r="F23" s="10"/>
     </row>
@@ -15419,16 +15416,16 @@
         <v>22</v>
       </c>
       <c r="B24" s="10" t="s">
+        <v>604</v>
+      </c>
+      <c r="C24" s="22" t="s">
         <v>605</v>
       </c>
-      <c r="C24" s="22" t="s">
+      <c r="D24" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E24" s="10" t="s">
         <v>606</v>
-      </c>
-      <c r="D24" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E24" s="10" t="s">
-        <v>607</v>
       </c>
       <c r="F24" s="10"/>
     </row>
@@ -15437,16 +15434,16 @@
         <v>23</v>
       </c>
       <c r="B25" s="10" t="s">
+        <v>607</v>
+      </c>
+      <c r="C25" s="22" t="s">
         <v>608</v>
       </c>
-      <c r="C25" s="22" t="s">
+      <c r="D25" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E25" s="10" t="s">
         <v>609</v>
-      </c>
-      <c r="D25" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E25" s="10" t="s">
-        <v>610</v>
       </c>
       <c r="F25" s="10"/>
     </row>
@@ -15455,16 +15452,16 @@
         <v>24</v>
       </c>
       <c r="B26" s="10" t="s">
+        <v>610</v>
+      </c>
+      <c r="C26" s="22" t="s">
         <v>611</v>
       </c>
-      <c r="C26" s="22" t="s">
+      <c r="D26" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E26" s="10" t="s">
         <v>612</v>
-      </c>
-      <c r="D26" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E26" s="10" t="s">
-        <v>613</v>
       </c>
       <c r="F26" s="10"/>
     </row>
@@ -15473,16 +15470,16 @@
         <v>25</v>
       </c>
       <c r="B27" s="10" t="s">
+        <v>613</v>
+      </c>
+      <c r="C27" s="22" t="s">
         <v>614</v>
       </c>
-      <c r="C27" s="22" t="s">
+      <c r="D27" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E27" s="10" t="s">
         <v>615</v>
-      </c>
-      <c r="D27" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E27" s="10" t="s">
-        <v>616</v>
       </c>
       <c r="F27" s="10"/>
     </row>
@@ -15491,16 +15488,16 @@
         <v>26</v>
       </c>
       <c r="B28" s="10" t="s">
+        <v>616</v>
+      </c>
+      <c r="C28" s="22" t="s">
         <v>617</v>
       </c>
-      <c r="C28" s="22" t="s">
+      <c r="D28" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E28" s="10" t="s">
         <v>618</v>
-      </c>
-      <c r="D28" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E28" s="10" t="s">
-        <v>619</v>
       </c>
       <c r="F28" s="10"/>
     </row>
@@ -15509,16 +15506,16 @@
         <v>27</v>
       </c>
       <c r="B29" s="10" t="s">
+        <v>619</v>
+      </c>
+      <c r="C29" s="22" t="s">
         <v>620</v>
       </c>
-      <c r="C29" s="22" t="s">
+      <c r="D29" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E29" s="10" t="s">
         <v>621</v>
-      </c>
-      <c r="D29" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E29" s="10" t="s">
-        <v>622</v>
       </c>
       <c r="F29" s="10"/>
     </row>
@@ -15527,16 +15524,16 @@
         <v>28</v>
       </c>
       <c r="B30" s="10" t="s">
+        <v>622</v>
+      </c>
+      <c r="C30" s="22" t="s">
         <v>623</v>
       </c>
-      <c r="C30" s="22" t="s">
+      <c r="D30" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E30" s="10" t="s">
         <v>624</v>
-      </c>
-      <c r="D30" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E30" s="10" t="s">
-        <v>625</v>
       </c>
       <c r="F30" s="10"/>
     </row>
@@ -15545,16 +15542,16 @@
         <v>29</v>
       </c>
       <c r="B31" s="10" t="s">
+        <v>625</v>
+      </c>
+      <c r="C31" s="22" t="s">
         <v>626</v>
       </c>
-      <c r="C31" s="22" t="s">
+      <c r="D31" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E31" s="10" t="s">
         <v>627</v>
-      </c>
-      <c r="D31" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E31" s="10" t="s">
-        <v>628</v>
       </c>
       <c r="F31" s="10"/>
     </row>
@@ -15563,16 +15560,16 @@
         <v>30</v>
       </c>
       <c r="B32" s="10" t="s">
+        <v>628</v>
+      </c>
+      <c r="C32" s="22" t="s">
         <v>629</v>
       </c>
-      <c r="C32" s="22" t="s">
+      <c r="D32" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E32" s="10" t="s">
         <v>630</v>
-      </c>
-      <c r="D32" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E32" s="10" t="s">
-        <v>631</v>
       </c>
       <c r="F32" s="10"/>
     </row>
@@ -15581,16 +15578,16 @@
         <v>31</v>
       </c>
       <c r="B33" s="10" t="s">
+        <v>631</v>
+      </c>
+      <c r="C33" s="22" t="s">
         <v>632</v>
       </c>
-      <c r="C33" s="22" t="s">
+      <c r="D33" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E33" s="10" t="s">
         <v>633</v>
-      </c>
-      <c r="D33" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E33" s="10" t="s">
-        <v>634</v>
       </c>
       <c r="F33" s="10"/>
     </row>
@@ -15602,13 +15599,13 @@
         <v>109</v>
       </c>
       <c r="C34" s="22" t="s">
+        <v>634</v>
+      </c>
+      <c r="D34" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E34" s="10" t="s">
         <v>635</v>
-      </c>
-      <c r="D34" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E34" s="10" t="s">
-        <v>636</v>
       </c>
       <c r="F34" s="10"/>
     </row>
@@ -15620,13 +15617,13 @@
         <v>430</v>
       </c>
       <c r="C35" s="22" t="s">
+        <v>636</v>
+      </c>
+      <c r="D35" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E35" s="10" t="s">
         <v>637</v>
-      </c>
-      <c r="D35" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E35" s="10" t="s">
-        <v>638</v>
       </c>
       <c r="F35" s="10"/>
     </row>
@@ -15635,16 +15632,16 @@
         <v>34</v>
       </c>
       <c r="B36" s="10" t="s">
+        <v>638</v>
+      </c>
+      <c r="C36" s="22" t="s">
         <v>639</v>
       </c>
-      <c r="C36" s="22" t="s">
+      <c r="D36" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E36" s="10" t="s">
         <v>640</v>
-      </c>
-      <c r="D36" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E36" s="10" t="s">
-        <v>641</v>
       </c>
       <c r="F36" s="10"/>
     </row>
@@ -15656,13 +15653,13 @@
         <v>122</v>
       </c>
       <c r="C37" s="22" t="s">
+        <v>641</v>
+      </c>
+      <c r="D37" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E37" s="10" t="s">
         <v>642</v>
-      </c>
-      <c r="D37" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E37" s="10" t="s">
-        <v>643</v>
       </c>
       <c r="F37" s="10"/>
     </row>
@@ -15671,16 +15668,16 @@
         <v>36</v>
       </c>
       <c r="B38" s="10" t="s">
+        <v>643</v>
+      </c>
+      <c r="C38" s="22" t="s">
         <v>644</v>
       </c>
-      <c r="C38" s="22" t="s">
+      <c r="D38" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E38" s="10" t="s">
         <v>645</v>
-      </c>
-      <c r="D38" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E38" s="10" t="s">
-        <v>646</v>
       </c>
       <c r="F38" s="10"/>
     </row>
@@ -15689,16 +15686,16 @@
         <v>37</v>
       </c>
       <c r="B39" s="10" t="s">
+        <v>646</v>
+      </c>
+      <c r="C39" s="22" t="s">
         <v>647</v>
       </c>
-      <c r="C39" s="22" t="s">
+      <c r="D39" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E39" s="10" t="s">
         <v>648</v>
-      </c>
-      <c r="D39" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E39" s="10" t="s">
-        <v>649</v>
       </c>
       <c r="F39" s="10"/>
     </row>
@@ -15707,16 +15704,16 @@
         <v>38</v>
       </c>
       <c r="B40" s="10" t="s">
+        <v>649</v>
+      </c>
+      <c r="C40" s="22" t="s">
         <v>650</v>
       </c>
-      <c r="C40" s="22" t="s">
+      <c r="D40" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E40" s="10" t="s">
         <v>651</v>
-      </c>
-      <c r="D40" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E40" s="10" t="s">
-        <v>652</v>
       </c>
       <c r="F40" s="10"/>
     </row>
@@ -15728,13 +15725,13 @@
         <v>323</v>
       </c>
       <c r="C41" s="22" t="s">
+        <v>652</v>
+      </c>
+      <c r="D41" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E41" s="10" t="s">
         <v>653</v>
-      </c>
-      <c r="D41" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E41" s="10" t="s">
-        <v>654</v>
       </c>
       <c r="F41" s="10"/>
     </row>
@@ -15743,16 +15740,16 @@
         <v>40</v>
       </c>
       <c r="B42" s="10" t="s">
+        <v>654</v>
+      </c>
+      <c r="C42" s="22" t="s">
         <v>655</v>
       </c>
-      <c r="C42" s="22" t="s">
+      <c r="D42" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E42" s="10" t="s">
         <v>656</v>
-      </c>
-      <c r="D42" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E42" s="10" t="s">
-        <v>657</v>
       </c>
       <c r="F42" s="10"/>
     </row>
@@ -15761,16 +15758,16 @@
         <v>41</v>
       </c>
       <c r="B43" s="10" t="s">
+        <v>657</v>
+      </c>
+      <c r="C43" s="22" t="s">
         <v>658</v>
       </c>
-      <c r="C43" s="22" t="s">
+      <c r="D43" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E43" s="10" t="s">
         <v>659</v>
-      </c>
-      <c r="D43" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E43" s="10" t="s">
-        <v>660</v>
       </c>
       <c r="F43" s="10"/>
     </row>
@@ -15779,16 +15776,16 @@
         <v>42</v>
       </c>
       <c r="B44" s="10" t="s">
+        <v>660</v>
+      </c>
+      <c r="C44" s="22" t="s">
         <v>661</v>
       </c>
-      <c r="C44" s="22" t="s">
+      <c r="D44" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E44" s="10" t="s">
         <v>662</v>
-      </c>
-      <c r="D44" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E44" s="10" t="s">
-        <v>663</v>
       </c>
       <c r="F44" s="10"/>
     </row>
@@ -15797,16 +15794,16 @@
         <v>43</v>
       </c>
       <c r="B45" s="10" t="s">
+        <v>663</v>
+      </c>
+      <c r="C45" s="22" t="s">
         <v>664</v>
       </c>
-      <c r="C45" s="22" t="s">
+      <c r="D45" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E45" s="10" t="s">
         <v>665</v>
-      </c>
-      <c r="D45" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E45" s="10" t="s">
-        <v>666</v>
       </c>
       <c r="F45" s="10"/>
     </row>
@@ -15818,13 +15815,13 @@
         <v>278</v>
       </c>
       <c r="C46" s="22" t="s">
+        <v>666</v>
+      </c>
+      <c r="D46" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E46" s="10" t="s">
         <v>667</v>
-      </c>
-      <c r="D46" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E46" s="10" t="s">
-        <v>668</v>
       </c>
       <c r="F46" s="10"/>
     </row>
@@ -15833,16 +15830,16 @@
         <v>45</v>
       </c>
       <c r="B47" s="10" t="s">
+        <v>668</v>
+      </c>
+      <c r="C47" s="22" t="s">
         <v>669</v>
       </c>
-      <c r="C47" s="22" t="s">
+      <c r="D47" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E47" s="10" t="s">
         <v>670</v>
-      </c>
-      <c r="D47" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E47" s="10" t="s">
-        <v>671</v>
       </c>
       <c r="F47" s="10"/>
     </row>
@@ -15854,13 +15851,13 @@
         <v>180</v>
       </c>
       <c r="C48" s="22" t="s">
+        <v>671</v>
+      </c>
+      <c r="D48" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E48" s="10" t="s">
         <v>672</v>
-      </c>
-      <c r="D48" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E48" s="10" t="s">
-        <v>673</v>
       </c>
       <c r="F48" s="10"/>
     </row>
@@ -15869,16 +15866,16 @@
         <v>47</v>
       </c>
       <c r="B49" s="10" t="s">
+        <v>673</v>
+      </c>
+      <c r="C49" s="22" t="s">
         <v>674</v>
       </c>
-      <c r="C49" s="22" t="s">
+      <c r="D49" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E49" s="10" t="s">
         <v>675</v>
-      </c>
-      <c r="D49" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E49" s="10" t="s">
-        <v>676</v>
       </c>
       <c r="F49" s="10"/>
     </row>
@@ -15887,16 +15884,16 @@
         <v>48</v>
       </c>
       <c r="B50" s="10" t="s">
+        <v>676</v>
+      </c>
+      <c r="C50" s="22" t="s">
         <v>677</v>
       </c>
-      <c r="C50" s="22" t="s">
+      <c r="D50" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E50" s="10" t="s">
         <v>678</v>
-      </c>
-      <c r="D50" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E50" s="10" t="s">
-        <v>679</v>
       </c>
       <c r="F50" s="10"/>
     </row>
@@ -15905,16 +15902,16 @@
         <v>49</v>
       </c>
       <c r="B51" s="10" t="s">
+        <v>679</v>
+      </c>
+      <c r="C51" s="22" t="s">
         <v>680</v>
       </c>
-      <c r="C51" s="22" t="s">
+      <c r="D51" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E51" s="10" t="s">
         <v>681</v>
-      </c>
-      <c r="D51" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E51" s="10" t="s">
-        <v>682</v>
       </c>
       <c r="F51" s="10"/>
     </row>
@@ -15923,16 +15920,16 @@
         <v>50</v>
       </c>
       <c r="B52" s="10" t="s">
+        <v>682</v>
+      </c>
+      <c r="C52" s="22" t="s">
         <v>683</v>
       </c>
-      <c r="C52" s="22" t="s">
+      <c r="D52" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E52" s="10" t="s">
         <v>684</v>
-      </c>
-      <c r="D52" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E52" s="10" t="s">
-        <v>685</v>
       </c>
       <c r="F52" s="10"/>
     </row>
@@ -15941,16 +15938,16 @@
         <v>51</v>
       </c>
       <c r="B53" s="10" t="s">
+        <v>685</v>
+      </c>
+      <c r="C53" s="22" t="s">
         <v>686</v>
       </c>
-      <c r="C53" s="22" t="s">
+      <c r="D53" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E53" s="10" t="s">
         <v>687</v>
-      </c>
-      <c r="D53" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E53" s="10" t="s">
-        <v>688</v>
       </c>
       <c r="F53" s="10"/>
     </row>
@@ -15959,16 +15956,16 @@
         <v>52</v>
       </c>
       <c r="B54" s="10" t="s">
+        <v>688</v>
+      </c>
+      <c r="C54" s="22" t="s">
         <v>689</v>
       </c>
-      <c r="C54" s="22" t="s">
+      <c r="D54" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E54" s="10" t="s">
         <v>690</v>
-      </c>
-      <c r="D54" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E54" s="10" t="s">
-        <v>691</v>
       </c>
       <c r="F54" s="10"/>
     </row>
@@ -15977,16 +15974,16 @@
         <v>53</v>
       </c>
       <c r="B55" s="10" t="s">
+        <v>691</v>
+      </c>
+      <c r="C55" s="22" t="s">
         <v>692</v>
       </c>
-      <c r="C55" s="22" t="s">
+      <c r="D55" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E55" s="10" t="s">
         <v>693</v>
-      </c>
-      <c r="D55" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E55" s="10" t="s">
-        <v>694</v>
       </c>
       <c r="F55" s="10"/>
     </row>
@@ -15998,13 +15995,13 @@
         <v>117</v>
       </c>
       <c r="C56" s="22" t="s">
+        <v>694</v>
+      </c>
+      <c r="D56" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E56" s="10" t="s">
         <v>695</v>
-      </c>
-      <c r="D56" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E56" s="10" t="s">
-        <v>696</v>
       </c>
       <c r="F56" s="10"/>
     </row>
@@ -16013,16 +16010,16 @@
         <v>55</v>
       </c>
       <c r="B57" s="10" t="s">
+        <v>696</v>
+      </c>
+      <c r="C57" s="22" t="s">
         <v>697</v>
       </c>
-      <c r="C57" s="22" t="s">
+      <c r="D57" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E57" s="10" t="s">
         <v>698</v>
-      </c>
-      <c r="D57" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E57" s="10" t="s">
-        <v>699</v>
       </c>
       <c r="F57" s="10"/>
     </row>
@@ -16031,16 +16028,16 @@
         <v>56</v>
       </c>
       <c r="B58" s="10" t="s">
+        <v>699</v>
+      </c>
+      <c r="C58" s="22" t="s">
         <v>700</v>
       </c>
-      <c r="C58" s="22" t="s">
+      <c r="D58" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E58" s="10" t="s">
         <v>701</v>
-      </c>
-      <c r="D58" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E58" s="10" t="s">
-        <v>702</v>
       </c>
       <c r="F58" s="10"/>
     </row>
@@ -16052,13 +16049,13 @@
         <v>259</v>
       </c>
       <c r="C59" s="22" t="s">
+        <v>702</v>
+      </c>
+      <c r="D59" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E59" s="10" t="s">
         <v>703</v>
-      </c>
-      <c r="D59" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E59" s="10" t="s">
-        <v>704</v>
       </c>
       <c r="F59" s="10"/>
     </row>
@@ -16070,13 +16067,13 @@
         <v>127</v>
       </c>
       <c r="C60" s="22" t="s">
+        <v>704</v>
+      </c>
+      <c r="D60" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E60" s="10" t="s">
         <v>705</v>
-      </c>
-      <c r="D60" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E60" s="10" t="s">
-        <v>706</v>
       </c>
       <c r="F60" s="10"/>
     </row>
@@ -16088,13 +16085,13 @@
         <v>136</v>
       </c>
       <c r="C61" s="22" t="s">
+        <v>706</v>
+      </c>
+      <c r="D61" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E61" s="10" t="s">
         <v>707</v>
-      </c>
-      <c r="D61" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E61" s="10" t="s">
-        <v>708</v>
       </c>
       <c r="F61" s="10"/>
     </row>
@@ -16106,13 +16103,13 @@
         <v>161</v>
       </c>
       <c r="C62" s="22" t="s">
+        <v>708</v>
+      </c>
+      <c r="D62" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E62" s="10" t="s">
         <v>709</v>
-      </c>
-      <c r="D62" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E62" s="10" t="s">
-        <v>710</v>
       </c>
       <c r="F62" s="10"/>
     </row>
@@ -16124,13 +16121,13 @@
         <v>218</v>
       </c>
       <c r="C63" s="22" t="s">
+        <v>710</v>
+      </c>
+      <c r="D63" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E63" s="10" t="s">
         <v>711</v>
-      </c>
-      <c r="D63" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E63" s="10" t="s">
-        <v>712</v>
       </c>
       <c r="F63" s="10"/>
     </row>
@@ -16142,13 +16139,13 @@
         <v>350</v>
       </c>
       <c r="C64" s="22" t="s">
+        <v>712</v>
+      </c>
+      <c r="D64" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E64" s="10" t="s">
         <v>713</v>
-      </c>
-      <c r="D64" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E64" s="10" t="s">
-        <v>714</v>
       </c>
       <c r="F64" s="10"/>
     </row>
@@ -16160,13 +16157,13 @@
         <v>402</v>
       </c>
       <c r="C65" s="22" t="s">
+        <v>714</v>
+      </c>
+      <c r="D65" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E65" s="10" t="s">
         <v>715</v>
-      </c>
-      <c r="D65" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E65" s="10" t="s">
-        <v>716</v>
       </c>
       <c r="F65" s="10"/>
     </row>
@@ -16178,13 +16175,13 @@
         <v>390</v>
       </c>
       <c r="C66" s="22" t="s">
+        <v>716</v>
+      </c>
+      <c r="D66" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E66" s="10" t="s">
         <v>717</v>
-      </c>
-      <c r="D66" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E66" s="10" t="s">
-        <v>718</v>
       </c>
       <c r="F66" s="10"/>
     </row>
@@ -16196,13 +16193,13 @@
         <v>383</v>
       </c>
       <c r="C67" s="22" t="s">
+        <v>718</v>
+      </c>
+      <c r="D67" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E67" s="10" t="s">
         <v>719</v>
-      </c>
-      <c r="D67" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E67" s="10" t="s">
-        <v>720</v>
       </c>
       <c r="F67" s="10"/>
     </row>
@@ -16211,16 +16208,16 @@
         <v>66</v>
       </c>
       <c r="B68" s="10" t="s">
+        <v>720</v>
+      </c>
+      <c r="C68" s="22" t="s">
         <v>721</v>
       </c>
-      <c r="C68" s="22" t="s">
+      <c r="D68" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E68" s="10" t="s">
         <v>722</v>
-      </c>
-      <c r="D68" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E68" s="10" t="s">
-        <v>723</v>
       </c>
       <c r="F68" s="10"/>
     </row>
@@ -16229,16 +16226,16 @@
         <v>67</v>
       </c>
       <c r="B69" s="10" t="s">
+        <v>723</v>
+      </c>
+      <c r="C69" s="22" t="s">
         <v>724</v>
       </c>
-      <c r="C69" s="22" t="s">
+      <c r="D69" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E69" s="10" t="s">
         <v>725</v>
-      </c>
-      <c r="D69" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E69" s="10" t="s">
-        <v>726</v>
       </c>
       <c r="F69" s="10"/>
     </row>
@@ -16247,16 +16244,16 @@
         <v>68</v>
       </c>
       <c r="B70" s="10" t="s">
+        <v>726</v>
+      </c>
+      <c r="C70" s="22" t="s">
         <v>727</v>
       </c>
-      <c r="C70" s="22" t="s">
+      <c r="D70" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E70" s="10" t="s">
         <v>728</v>
-      </c>
-      <c r="D70" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E70" s="10" t="s">
-        <v>729</v>
       </c>
       <c r="F70" s="10"/>
     </row>
@@ -16268,13 +16265,13 @@
         <v>145</v>
       </c>
       <c r="C71" s="22" t="s">
+        <v>729</v>
+      </c>
+      <c r="D71" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E71" s="10" t="s">
         <v>730</v>
-      </c>
-      <c r="D71" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E71" s="10" t="s">
-        <v>731</v>
       </c>
       <c r="F71" s="10"/>
     </row>
@@ -16283,16 +16280,16 @@
         <v>70</v>
       </c>
       <c r="B72" s="10" t="s">
+        <v>731</v>
+      </c>
+      <c r="C72" s="22" t="s">
         <v>732</v>
       </c>
-      <c r="C72" s="22" t="s">
+      <c r="D72" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E72" s="10" t="s">
         <v>733</v>
-      </c>
-      <c r="D72" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E72" s="10" t="s">
-        <v>734</v>
       </c>
       <c r="F72" s="10"/>
     </row>
@@ -16304,13 +16301,13 @@
         <v>363</v>
       </c>
       <c r="C73" s="22" t="s">
+        <v>734</v>
+      </c>
+      <c r="D73" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E73" s="10" t="s">
         <v>735</v>
-      </c>
-      <c r="D73" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E73" s="10" t="s">
-        <v>736</v>
       </c>
       <c r="F73" s="10"/>
     </row>
@@ -16322,13 +16319,13 @@
         <v>366</v>
       </c>
       <c r="C74" s="22" t="s">
+        <v>736</v>
+      </c>
+      <c r="D74" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E74" s="10" t="s">
         <v>737</v>
-      </c>
-      <c r="D74" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E74" s="10" t="s">
-        <v>738</v>
       </c>
       <c r="F74" s="10"/>
     </row>
@@ -16340,13 +16337,13 @@
         <v>413</v>
       </c>
       <c r="C75" s="22" t="s">
+        <v>738</v>
+      </c>
+      <c r="D75" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E75" s="10" t="s">
         <v>739</v>
-      </c>
-      <c r="D75" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E75" s="10" t="s">
-        <v>740</v>
       </c>
       <c r="F75" s="10"/>
     </row>
@@ -16355,16 +16352,16 @@
         <v>74</v>
       </c>
       <c r="B76" s="10" t="s">
+        <v>740</v>
+      </c>
+      <c r="C76" s="22" t="s">
         <v>741</v>
       </c>
-      <c r="C76" s="22" t="s">
+      <c r="D76" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E76" s="10" t="s">
         <v>742</v>
-      </c>
-      <c r="D76" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E76" s="10" t="s">
-        <v>743</v>
       </c>
       <c r="F76" s="10"/>
     </row>
@@ -16373,16 +16370,16 @@
         <v>75</v>
       </c>
       <c r="B77" s="10" t="s">
+        <v>743</v>
+      </c>
+      <c r="C77" s="22" t="s">
         <v>744</v>
       </c>
-      <c r="C77" s="22" t="s">
+      <c r="D77" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E77" s="10" t="s">
         <v>745</v>
-      </c>
-      <c r="D77" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E77" s="10" t="s">
-        <v>746</v>
       </c>
       <c r="F77" s="10"/>
     </row>
@@ -16391,16 +16388,16 @@
         <v>76</v>
       </c>
       <c r="B78" s="10" t="s">
+        <v>746</v>
+      </c>
+      <c r="C78" s="22" t="s">
         <v>747</v>
       </c>
-      <c r="C78" s="22" t="s">
+      <c r="D78" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E78" s="10" t="s">
         <v>748</v>
-      </c>
-      <c r="D78" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E78" s="10" t="s">
-        <v>749</v>
       </c>
       <c r="F78" s="10"/>
     </row>
@@ -16412,13 +16409,13 @@
         <v>393</v>
       </c>
       <c r="C79" s="22" t="s">
+        <v>749</v>
+      </c>
+      <c r="D79" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E79" s="10" t="s">
         <v>750</v>
-      </c>
-      <c r="D79" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E79" s="10" t="s">
-        <v>751</v>
       </c>
       <c r="F79" s="10"/>
     </row>
@@ -16427,16 +16424,16 @@
         <v>78</v>
       </c>
       <c r="B80" s="10" t="s">
+        <v>751</v>
+      </c>
+      <c r="C80" s="22" t="s">
         <v>752</v>
       </c>
-      <c r="C80" s="22" t="s">
+      <c r="D80" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E80" s="10" t="s">
         <v>753</v>
-      </c>
-      <c r="D80" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E80" s="10" t="s">
-        <v>754</v>
       </c>
       <c r="F80" s="10"/>
     </row>
@@ -16445,16 +16442,16 @@
         <v>79</v>
       </c>
       <c r="B81" s="10" t="s">
+        <v>754</v>
+      </c>
+      <c r="C81" s="22" t="s">
         <v>755</v>
       </c>
-      <c r="C81" s="22" t="s">
+      <c r="D81" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E81" s="10" t="s">
         <v>756</v>
-      </c>
-      <c r="D81" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E81" s="10" t="s">
-        <v>757</v>
       </c>
       <c r="F81" s="10"/>
     </row>
@@ -16466,13 +16463,13 @@
         <v>309</v>
       </c>
       <c r="C82" s="22" t="s">
+        <v>757</v>
+      </c>
+      <c r="D82" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E82" s="10" t="s">
         <v>758</v>
-      </c>
-      <c r="D82" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E82" s="10" t="s">
-        <v>759</v>
       </c>
       <c r="F82" s="10"/>
     </row>
@@ -16484,13 +16481,13 @@
         <v>296</v>
       </c>
       <c r="C83" s="22" t="s">
+        <v>759</v>
+      </c>
+      <c r="D83" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E83" s="10" t="s">
         <v>760</v>
-      </c>
-      <c r="D83" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E83" s="10" t="s">
-        <v>761</v>
       </c>
       <c r="F83" s="10"/>
     </row>
@@ -16499,16 +16496,16 @@
         <v>82</v>
       </c>
       <c r="B84" s="10" t="s">
+        <v>761</v>
+      </c>
+      <c r="C84" s="22" t="s">
         <v>762</v>
       </c>
-      <c r="C84" s="22" t="s">
+      <c r="D84" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E84" s="10" t="s">
         <v>763</v>
-      </c>
-      <c r="D84" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E84" s="10" t="s">
-        <v>764</v>
       </c>
       <c r="F84" s="10"/>
     </row>
@@ -16517,16 +16514,16 @@
         <v>83</v>
       </c>
       <c r="B85" s="10" t="s">
+        <v>764</v>
+      </c>
+      <c r="C85" s="22" t="s">
         <v>765</v>
       </c>
-      <c r="C85" s="22" t="s">
+      <c r="D85" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E85" s="10" t="s">
         <v>766</v>
-      </c>
-      <c r="D85" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E85" s="10" t="s">
-        <v>767</v>
       </c>
       <c r="F85" s="10"/>
     </row>
@@ -16535,16 +16532,16 @@
         <v>84</v>
       </c>
       <c r="B86" s="10" t="s">
+        <v>767</v>
+      </c>
+      <c r="C86" s="22" t="s">
         <v>768</v>
       </c>
-      <c r="C86" s="22" t="s">
+      <c r="D86" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E86" s="10" t="s">
         <v>769</v>
-      </c>
-      <c r="D86" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E86" s="10" t="s">
-        <v>770</v>
       </c>
       <c r="F86" s="10"/>
     </row>
@@ -16553,16 +16550,16 @@
         <v>85</v>
       </c>
       <c r="B87" s="10" t="s">
+        <v>770</v>
+      </c>
+      <c r="C87" s="22" t="s">
         <v>771</v>
       </c>
-      <c r="C87" s="22" t="s">
+      <c r="D87" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E87" s="10" t="s">
         <v>772</v>
-      </c>
-      <c r="D87" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E87" s="10" t="s">
-        <v>773</v>
       </c>
       <c r="F87" s="10"/>
     </row>
@@ -16571,16 +16568,16 @@
         <v>86</v>
       </c>
       <c r="B88" s="10" t="s">
+        <v>773</v>
+      </c>
+      <c r="C88" s="22" t="s">
         <v>774</v>
       </c>
-      <c r="C88" s="22" t="s">
+      <c r="D88" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E88" s="10" t="s">
         <v>775</v>
-      </c>
-      <c r="D88" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E88" s="10" t="s">
-        <v>776</v>
       </c>
       <c r="F88" s="10"/>
     </row>
@@ -16589,16 +16586,16 @@
         <v>87</v>
       </c>
       <c r="B89" s="10" t="s">
+        <v>776</v>
+      </c>
+      <c r="C89" s="22" t="s">
         <v>777</v>
       </c>
-      <c r="C89" s="22" t="s">
+      <c r="D89" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E89" s="10" t="s">
         <v>778</v>
-      </c>
-      <c r="D89" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E89" s="10" t="s">
-        <v>779</v>
       </c>
       <c r="F89" s="10"/>
     </row>
@@ -16607,16 +16604,16 @@
         <v>88</v>
       </c>
       <c r="B90" s="10" t="s">
+        <v>779</v>
+      </c>
+      <c r="C90" s="22" t="s">
         <v>780</v>
       </c>
-      <c r="C90" s="22" t="s">
+      <c r="D90" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E90" s="10" t="s">
         <v>781</v>
-      </c>
-      <c r="D90" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E90" s="10" t="s">
-        <v>782</v>
       </c>
       <c r="F90" s="10"/>
     </row>
@@ -16625,16 +16622,16 @@
         <v>89</v>
       </c>
       <c r="B91" s="10" t="s">
+        <v>782</v>
+      </c>
+      <c r="C91" s="22" t="s">
         <v>783</v>
       </c>
-      <c r="C91" s="22" t="s">
+      <c r="D91" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E91" s="10" t="s">
         <v>784</v>
-      </c>
-      <c r="D91" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E91" s="10" t="s">
-        <v>785</v>
       </c>
       <c r="F91" s="10"/>
     </row>
@@ -16646,13 +16643,13 @@
         <v>100</v>
       </c>
       <c r="C92" s="22" t="s">
+        <v>785</v>
+      </c>
+      <c r="D92" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E92" s="10" t="s">
         <v>786</v>
-      </c>
-      <c r="D92" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E92" s="10" t="s">
-        <v>787</v>
       </c>
       <c r="F92" s="10"/>
     </row>
@@ -16661,16 +16658,16 @@
         <v>91</v>
       </c>
       <c r="B93" s="10" t="s">
+        <v>787</v>
+      </c>
+      <c r="C93" s="22" t="s">
         <v>788</v>
       </c>
-      <c r="C93" s="22" t="s">
+      <c r="D93" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E93" s="10" t="s">
         <v>789</v>
-      </c>
-      <c r="D93" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E93" s="10" t="s">
-        <v>790</v>
       </c>
       <c r="F93" s="10"/>
     </row>
@@ -16679,16 +16676,16 @@
         <v>92</v>
       </c>
       <c r="B94" s="10" t="s">
+        <v>790</v>
+      </c>
+      <c r="C94" s="22" t="s">
         <v>791</v>
       </c>
-      <c r="C94" s="22" t="s">
+      <c r="D94" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E94" s="10" t="s">
         <v>792</v>
-      </c>
-      <c r="D94" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E94" s="10" t="s">
-        <v>793</v>
       </c>
       <c r="F94" s="10"/>
     </row>
@@ -16697,16 +16694,16 @@
         <v>93</v>
       </c>
       <c r="B95" s="10" t="s">
+        <v>793</v>
+      </c>
+      <c r="C95" s="22" t="s">
         <v>794</v>
       </c>
-      <c r="C95" s="22" t="s">
+      <c r="D95" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E95" s="10" t="s">
         <v>795</v>
-      </c>
-      <c r="D95" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E95" s="10" t="s">
-        <v>796</v>
       </c>
       <c r="F95" s="10"/>
     </row>
@@ -16715,16 +16712,16 @@
         <v>94</v>
       </c>
       <c r="B96" s="10" t="s">
+        <v>796</v>
+      </c>
+      <c r="C96" s="22" t="s">
         <v>797</v>
       </c>
-      <c r="C96" s="22" t="s">
+      <c r="D96" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E96" s="10" t="s">
         <v>798</v>
-      </c>
-      <c r="D96" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E96" s="10" t="s">
-        <v>799</v>
       </c>
       <c r="F96" s="10"/>
     </row>
@@ -16733,16 +16730,16 @@
         <v>95</v>
       </c>
       <c r="B97" s="10" t="s">
+        <v>799</v>
+      </c>
+      <c r="C97" s="22" t="s">
         <v>800</v>
       </c>
-      <c r="C97" s="22" t="s">
+      <c r="D97" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E97" s="10" t="s">
         <v>801</v>
-      </c>
-      <c r="D97" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E97" s="10" t="s">
-        <v>802</v>
       </c>
       <c r="F97" s="10"/>
     </row>
@@ -16751,16 +16748,16 @@
         <v>96</v>
       </c>
       <c r="B98" s="10" t="s">
+        <v>802</v>
+      </c>
+      <c r="C98" s="22" t="s">
         <v>803</v>
       </c>
-      <c r="C98" s="22" t="s">
+      <c r="D98" s="10" t="s">
+        <v>548</v>
+      </c>
+      <c r="E98" s="10" t="s">
         <v>804</v>
-      </c>
-      <c r="D98" s="10" t="s">
-        <v>549</v>
-      </c>
-      <c r="E98" s="10" t="s">
-        <v>805</v>
       </c>
       <c r="F98" s="10"/>
     </row>
@@ -16893,7 +16890,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -16903,10 +16900,10 @@
         <v>44</v>
       </c>
       <c r="B2" s="7" t="s">
+        <v>806</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>807</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -16914,10 +16911,10 @@
         <v>47</v>
       </c>
       <c r="B3" s="8" t="s">
+        <v>808</v>
+      </c>
+      <c r="C3" s="8" t="s">
         <v>809</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>810</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -16925,10 +16922,10 @@
         <v>49</v>
       </c>
       <c r="B4" s="8" t="s">
+        <v>810</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>811</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>812</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -16936,10 +16933,10 @@
         <v>51</v>
       </c>
       <c r="B5" s="8" t="s">
+        <v>812</v>
+      </c>
+      <c r="C5" s="8" t="s">
         <v>813</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>814</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -16947,10 +16944,10 @@
         <v>53</v>
       </c>
       <c r="B6" s="8" t="s">
+        <v>814</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>815</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>816</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -16958,10 +16955,10 @@
         <v>55</v>
       </c>
       <c r="B7" s="8" t="s">
+        <v>816</v>
+      </c>
+      <c r="C7" s="8" t="s">
         <v>817</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>818</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -16969,10 +16966,10 @@
         <v>56</v>
       </c>
       <c r="B8" s="8" t="s">
+        <v>818</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>819</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>820</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -16980,10 +16977,10 @@
         <v>57</v>
       </c>
       <c r="B9" s="8" t="s">
+        <v>820</v>
+      </c>
+      <c r="C9" s="8" t="s">
         <v>821</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>822</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -16991,10 +16988,10 @@
         <v>58</v>
       </c>
       <c r="B10" s="8" t="s">
+        <v>822</v>
+      </c>
+      <c r="C10" s="8" t="s">
         <v>823</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>824</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -17002,10 +16999,10 @@
         <v>59</v>
       </c>
       <c r="B11" s="8" t="s">
+        <v>824</v>
+      </c>
+      <c r="C11" s="8" t="s">
         <v>825</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>826</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clear test-promoted Applications row (Tether Wallets)
Row 2 was created during a click-test of the Submitted -> Applications
auto-promote flow, but no actual application was submitted. Clear the
row's data fields (preserving the =ROW()-1 formula in column A) and
reset the matching Preparations row's Submission status to "Not
submitted" so the two sheets agree.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -1158,7 +1158,6 @@
     <mergeCell ref="A27:D27"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A32:D32"/>
     <mergeCell ref="A20:D20"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="A26:D26"/>
@@ -1170,6 +1169,7 @@
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A28:D28"/>
     <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A32:D32"/>
     <mergeCell ref="B7:D7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11723,54 +11723,22 @@
         <f>ROW()-1</f>
         <v/>
       </c>
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>Tether</t>
-        </is>
-      </c>
-      <c r="D2" s="1" t="inlineStr">
-        <is>
-          <t>Backend Engineer (Wallets) — 100% Remote</t>
-        </is>
-      </c>
+      <c r="B2" s="1" t="n"/>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
       <c r="E2" s="1" t="n"/>
       <c r="F2" s="1" t="n"/>
-      <c r="G2" s="1" t="inlineStr">
-        <is>
-          <t>https://careers.tether.io/o/backend-engineer-wallets-100-remote-29</t>
-        </is>
-      </c>
-      <c r="H2" s="1" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-      <c r="I2" s="1" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="J2" s="1" t="inlineStr">
-        <is>
-          <t>career-ops/output/cv-hana-aliyah-mufidah-tether-2026-05-06.pdf</t>
-        </is>
-      </c>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
       <c r="K2" s="1" t="n"/>
       <c r="L2" s="1" t="n"/>
       <c r="M2" s="1" t="n"/>
       <c r="N2" s="1" t="n"/>
       <c r="O2" s="1" t="n"/>
       <c r="P2" s="1" t="n"/>
-      <c r="Q2" s="1" t="inlineStr">
-        <is>
-          <t>Promoted from Preparations row 2</t>
-        </is>
-      </c>
+      <c r="Q2" s="1" t="n"/>
     </row>
     <row r="3">
       <c r="A3">

</xml_diff>

<commit_message>
Trim Applications Status dropdown: remove Wishlist and SKIP
The lifecycle in the Applications sheet starts after the Preparations
hand-off, so Wishlist is redundant (that state lives on the Wishlist
sheet via Decision). SKIP duplicates Discarded — pick one. Dropdown is
now: Evaluated / Applied / Responded / Interview / Offer / Rejected /
Discarded. Web editor's DROPDOWN_COLORS map updated to match.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -16148,12 +16148,9 @@
       <formula>"SKIP"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation sqref="H10:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Wishlist,Evaluated,Applied,Responded,Interview,Offer,Rejected,Discarded,SKIP"</formula1>
-    </dataValidation>
+  <dataValidations count="1">
     <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Wishlist,Evaluated,Applied,Responded,Interview,Offer,Rejected,Discarded,SKIP"</formula1>
+      <formula1>"Evaluated,Applied,Responded,Interview,Offer,Rejected,Discarded"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Flag SumUp as office-first across Companies + Wishlist
SumUp's JD boilerplate explicitly states they're an office-first
company; "regularly working together in the same physical space" is
a stated requirement. Locations are Berlin/Cologne/Copenhagen/London/
São Paulo etc., and flexible work is case-by-case via the first
interview only.

- Companies sheet (row 66): note now reads "OFFICE-FIRST — not remote"
- Wishlist: 26 SumUp rows now have "Office-first (not remote)"
  prepended to Notes

User is open to relocation, so this is informational rather than a
skip reason — but the flag prevents misreading future SumUp listings
as remote.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -131,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -174,6 +174,9 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1161,7 +1164,6 @@
     <mergeCell ref="A27:D27"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A32:D32"/>
     <mergeCell ref="A20:D20"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="A26:D26"/>
@@ -1173,6 +1175,7 @@
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A28:D28"/>
     <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A32:D32"/>
     <mergeCell ref="B7:D7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8438,9 +8441,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L140" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unclear</t>
+      <c r="L140" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unclear</t>
         </is>
       </c>
     </row>
@@ -9488,9 +9491,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L161" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L161" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -9538,9 +9541,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L162" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L162" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -9588,9 +9591,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L163" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L163" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -9638,9 +9641,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L164" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L164" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -9688,9 +9691,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L165" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L165" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -9738,9 +9741,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L166" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L166" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -9788,9 +9791,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L167" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L167" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -9838,9 +9841,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L168" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L168" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -9888,9 +9891,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L169" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L169" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -9938,9 +9941,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L170" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L170" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -9988,9 +9991,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L171" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L171" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -10038,9 +10041,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L172" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L172" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -10088,9 +10091,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L173" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L173" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -10138,9 +10141,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L174" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L174" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -10188,9 +10191,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L175" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L175" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -10238,9 +10241,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L176" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L176" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -10288,9 +10291,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L177" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L177" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -10338,9 +10341,9 @@
           <t>Apply</t>
         </is>
       </c>
-      <c r="L178" s="18" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L178" s="21" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -10388,9 +10391,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L179" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L179" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -10438,9 +10441,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L180" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L180" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -10488,9 +10491,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L181" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L181" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -10538,9 +10541,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L182" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L182" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -10588,9 +10591,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L183" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unknown</t>
+      <c r="L183" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -11033,7 +11036,11 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L192" s="23" t="inlineStr"/>
+      <c r="L192" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote)</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="23">
@@ -11082,7 +11089,11 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L193" s="23" t="inlineStr"/>
+      <c r="L193" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote)</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="23">
@@ -18299,9 +18310,9 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="E66" s="10" t="inlineStr">
-        <is>
-          <t>Berlin / London. Payments fintech, EU + LATAM hiring.</t>
+      <c r="E66" s="24" t="inlineStr">
+        <is>
+          <t>Berlin / London. Payments fintech, EU + LATAM hiring. OFFICE-FIRST — not remote. Flexible work case-by-case via interview.</t>
         </is>
       </c>
       <c r="F66" s="10" t="n"/>

</xml_diff>

<commit_message>
Exclude Wayve (stack mismatch) and SumUp (office-first) from scans
Wayve roles center on embedded/automotive/AV stack (C/C++, Linux BSP,
Yocto, QNX, AUTOSAR, SoC bring-up, CAN/PCIe/I2C, ISO 26262). Hard
mismatch with the user's web/backend profile.

SumUp is office-first (per their JD boilerplate) and produces many
duplicate listings per scan; relocation friction plus dup noise
makes it not worth recurring scans. Existing SumUp Wishlist rows
are kept (still flagged office-first); user can prune via Skip when
ready.

Wayve cleanup:
- 10 Wayve rows removed from Wishlist
- portals.yml: enabled: false, notes updated (gitignored, local-only)
- data/pipeline.md: 16 Wayve lines removed (gitignored)
- data/scan-history.tsv: 16 Wayve entries flipped to 'excluded'

Companies sheet:
- Wayve (r75): Enabled=No, Status=Excluded, stack-mismatch note
- SumUp (r66): Enabled=No, Status=Excluded, office-first + dup note

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -1419,7 +1419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L199"/>
+  <dimension ref="A1:L189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="1" min="1" max="1"/>
@@ -8909,17 +8909,17 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Wayve</t>
+          <t>Zapier</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Application Software Engineer</t>
-        </is>
-      </c>
-      <c r="E150" s="13" t="inlineStr">
-        <is>
-          <t>https://wayve.firststage.co/jobs?gh_jid=8455160002</t>
+          <t>Software Engineer — Release Engineering</t>
+        </is>
+      </c>
+      <c r="E150" s="19" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/zapier/6948a0e6-a580-4e9d-b109-20652d9a1507</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -8959,17 +8959,17 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Wayve</t>
+          <t>Zapier</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Application Software Engineer - Relocation to Tokyo</t>
+          <t>Sr. Engineer, Backend - Enterprise</t>
         </is>
       </c>
       <c r="E151" s="19" t="inlineStr">
         <is>
-          <t>https://wayve.firststage.co/jobs?gh_jid=8460441002</t>
+          <t>https://jobs.ashbyhq.com/zapier/423d1bb7-1c08-458e-8a17-29a63cf23d92</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -9009,17 +9009,17 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Wayve</t>
+          <t>Zapier</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer - 3D Rendering</t>
+          <t>Sr. Fullstack Engineer, Identity Platform</t>
         </is>
       </c>
       <c r="E152" s="19" t="inlineStr">
         <is>
-          <t>https://wayve.firststage.co/jobs?gh_jid=8482674002</t>
+          <t>https://jobs.ashbyhq.com/zapier/3b141014-1d0f-426e-94e5-997b2cfd6ae8</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -9059,17 +9059,17 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Wayve</t>
+          <t>SumUp</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer - Data Enrichment</t>
-        </is>
-      </c>
-      <c r="E153" s="19" t="inlineStr">
-        <is>
-          <t>https://wayve.firststage.co/jobs?gh_jid=8482664002</t>
+          <t>(Senior) Backend Engineer (Golang) - Global Bank</t>
+        </is>
+      </c>
+      <c r="E153" s="13" t="inlineStr">
+        <is>
+          <t>https://sumup.com/careers/positions/8207386002?gh_jid=8207386002</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -9091,9 +9091,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L153" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unclear</t>
+      <c r="L153" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -9109,17 +9109,17 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Wayve</t>
+          <t>SumUp</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Software Engineer - OS &amp; Kernel, Robot Software</t>
-        </is>
-      </c>
-      <c r="E154" s="19" t="inlineStr">
-        <is>
-          <t>https://wayve.firststage.co/jobs?gh_jid=8423176002</t>
+          <t>(Senior) Backend Engineer - Global Bank</t>
+        </is>
+      </c>
+      <c r="E154" s="13" t="inlineStr">
+        <is>
+          <t>https://sumup.com/careers/positions/8207403002?gh_jid=8207403002</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
@@ -9141,9 +9141,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L154" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unclear</t>
+      <c r="L154" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -9159,17 +9159,17 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Wayve</t>
+          <t>SumUp</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Software Engineer - Sensor Systems, Robot Software</t>
-        </is>
-      </c>
-      <c r="E155" s="19" t="inlineStr">
-        <is>
-          <t>https://wayve.firststage.co/jobs?gh_jid=8423839002</t>
+          <t>(Senior/Mid) Software Engineer, Golang - Payments Platform</t>
+        </is>
+      </c>
+      <c r="E155" s="13" t="inlineStr">
+        <is>
+          <t>https://sumup.com/careers/positions/8520784002?gh_jid=8520784002</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
@@ -9191,9 +9191,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L155" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unclear</t>
+      <c r="L155" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -9209,17 +9209,17 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Wayve</t>
+          <t>SumUp</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Software Engineer - System Performance, Robot Software</t>
-        </is>
-      </c>
-      <c r="E156" s="19" t="inlineStr">
-        <is>
-          <t>https://wayve.firststage.co/jobs?gh_jid=8482117002</t>
+          <t>Backend Engineer - POS</t>
+        </is>
+      </c>
+      <c r="E156" s="13" t="inlineStr">
+        <is>
+          <t>https://sumup.com/careers/positions/8427119002?gh_jid=8427119002</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -9241,9 +9241,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L156" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unclear</t>
+      <c r="L156" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -9259,17 +9259,17 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Wayve</t>
+          <t>SumUp</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Software Engineer -System Performance, Robot Software</t>
-        </is>
-      </c>
-      <c r="E157" s="19" t="inlineStr">
-        <is>
-          <t>https://wayve.firststage.co/jobs?gh_jid=8389765002</t>
+          <t>Backend Engineer - Transfers</t>
+        </is>
+      </c>
+      <c r="E157" s="13" t="inlineStr">
+        <is>
+          <t>https://sumup.com/careers/positions/8388972002?gh_jid=8388972002</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
@@ -9291,9 +9291,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L157" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unclear</t>
+      <c r="L157" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -9309,17 +9309,17 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Zapier</t>
+          <t>SumUp</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Software Engineer — Release Engineering</t>
-        </is>
-      </c>
-      <c r="E158" s="19" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/zapier/6948a0e6-a580-4e9d-b109-20652d9a1507</t>
+          <t>Backend engineer (Go)-  Payments Experience</t>
+        </is>
+      </c>
+      <c r="E158" s="13" t="inlineStr">
+        <is>
+          <t>https://sumup.com/careers/positions/8497866002?gh_jid=8497866002</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -9341,9 +9341,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L158" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unclear</t>
+      <c r="L158" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -9359,17 +9359,17 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Zapier</t>
+          <t>SumUp</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Sr. Engineer, Backend - Enterprise</t>
-        </is>
-      </c>
-      <c r="E159" s="19" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/zapier/423d1bb7-1c08-458e-8a17-29a63cf23d92</t>
+          <t>Fullstack Engineer (NodeJs)</t>
+        </is>
+      </c>
+      <c r="E159" s="13" t="inlineStr">
+        <is>
+          <t>https://sumup.com/careers/positions/8482959002?gh_jid=8482959002</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -9391,9 +9391,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L159" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unclear</t>
+      <c r="L159" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -9409,17 +9409,17 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Zapier</t>
+          <t>SumUp</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Sr. Fullstack Engineer, Identity Platform</t>
-        </is>
-      </c>
-      <c r="E160" s="19" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/zapier/3b141014-1d0f-426e-94e5-997b2cfd6ae8</t>
+          <t>Junior Backend Engineer (Golang) -  Payments Tribe</t>
+        </is>
+      </c>
+      <c r="E160" s="13" t="inlineStr">
+        <is>
+          <t>https://sumup.com/careers/positions/8520406002?gh_jid=8520406002</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -9441,9 +9441,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L160" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unclear</t>
+      <c r="L160" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
       </c>
     </row>
@@ -9464,12 +9464,12 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>(Senior) Backend Engineer (Golang) - Global Bank</t>
+          <t>Senior AI Backend Engineer</t>
         </is>
       </c>
       <c r="E161" s="13" t="inlineStr">
         <is>
-          <t>https://sumup.com/careers/positions/8207386002?gh_jid=8207386002</t>
+          <t>https://sumup.com/careers/positions/8468006002?gh_jid=8468006002</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
@@ -9514,12 +9514,12 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>(Senior) Backend Engineer - Global Bank</t>
+          <t>Senior Backend Engineer</t>
         </is>
       </c>
       <c r="E162" s="13" t="inlineStr">
         <is>
-          <t>https://sumup.com/careers/positions/8207403002?gh_jid=8207403002</t>
+          <t>https://sumup.com/careers/positions/7480776002?gh_jid=7480776002</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -9564,12 +9564,12 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>(Senior/Mid) Software Engineer, Golang - Payments Platform</t>
+          <t>Senior Backend Engineer (Golang) - Bank</t>
         </is>
       </c>
       <c r="E163" s="13" t="inlineStr">
         <is>
-          <t>https://sumup.com/careers/positions/8520784002?gh_jid=8520784002</t>
+          <t>https://sumup.com/careers/positions/8454657002?gh_jid=8454657002</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
@@ -9614,12 +9614,12 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Backend Engineer - POS</t>
+          <t>Senior Backend Engineer - Accounts</t>
         </is>
       </c>
       <c r="E164" s="13" t="inlineStr">
         <is>
-          <t>https://sumup.com/careers/positions/8427119002?gh_jid=8427119002</t>
+          <t>https://sumup.com/careers/positions/8418287002?gh_jid=8418287002</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
@@ -9664,12 +9664,12 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Backend Engineer - Transfers</t>
+          <t>Senior Backend Engineer - Fiscalization</t>
         </is>
       </c>
       <c r="E165" s="13" t="inlineStr">
         <is>
-          <t>https://sumup.com/careers/positions/8388972002?gh_jid=8388972002</t>
+          <t>https://sumup.com/careers/positions/8222274002?gh_jid=8222274002</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
@@ -9714,12 +9714,12 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Backend engineer (Go)-  Payments Experience</t>
+          <t>Senior Backend Engineer - Golang</t>
         </is>
       </c>
       <c r="E166" s="13" t="inlineStr">
         <is>
-          <t>https://sumup.com/careers/positions/8497866002?gh_jid=8497866002</t>
+          <t>https://sumup.com/careers/positions/8429621002?gh_jid=8429621002</t>
         </is>
       </c>
       <c r="F166" t="inlineStr">
@@ -9764,12 +9764,12 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Fullstack Engineer (NodeJs)</t>
+          <t>Senior Backend Engineer - Transfers</t>
         </is>
       </c>
       <c r="E167" s="13" t="inlineStr">
         <is>
-          <t>https://sumup.com/careers/positions/8482959002?gh_jid=8482959002</t>
+          <t>https://sumup.com/careers/positions/8383464002?gh_jid=8383464002</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
@@ -9814,12 +9814,12 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Junior Backend Engineer (Golang) -  Payments Tribe</t>
+          <t>Senior Backend Engineer Go - Payments Reporting</t>
         </is>
       </c>
       <c r="E168" s="13" t="inlineStr">
         <is>
-          <t>https://sumup.com/careers/positions/8520406002?gh_jid=8520406002</t>
+          <t>https://sumup.com/careers/positions/8494767002?gh_jid=8494767002</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -9864,12 +9864,12 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Senior AI Backend Engineer</t>
+          <t>Senior Backend Engineer- Global Bank</t>
         </is>
       </c>
       <c r="E169" s="13" t="inlineStr">
         <is>
-          <t>https://sumup.com/careers/positions/8468006002?gh_jid=8468006002</t>
+          <t>https://sumup.com/careers/positions/6651430002?gh_jid=6651430002</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
@@ -9898,50 +9898,50 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B170" t="inlineStr">
+      <c r="A170" s="18">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B170" s="18" t="inlineStr">
         <is>
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="C170" t="inlineStr">
+      <c r="C170" s="18" t="inlineStr">
         <is>
           <t>SumUp</t>
         </is>
       </c>
-      <c r="D170" t="inlineStr">
-        <is>
-          <t>Senior Backend Engineer</t>
+      <c r="D170" s="18" t="inlineStr">
+        <is>
+          <t>Senior Fullstack Engineer (NodeJs)</t>
         </is>
       </c>
       <c r="E170" s="13" t="inlineStr">
         <is>
-          <t>https://sumup.com/careers/positions/7480776002?gh_jid=7480776002</t>
-        </is>
-      </c>
-      <c r="F170" t="inlineStr">
+          <t>https://sumup.com/careers/positions/8537166002?gh_jid=8537166002</t>
+        </is>
+      </c>
+      <c r="F170" s="18" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="H170" t="inlineStr">
+      <c r="H170" s="18" t="inlineStr">
         <is>
           <t>Tier A</t>
         </is>
       </c>
-      <c r="I170" t="n">
-        <v>3</v>
+      <c r="I170" s="18" t="n">
+        <v>5</v>
       </c>
       <c r="J170" s="1" t="n"/>
-      <c r="K170" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L170" s="23" t="inlineStr">
+      <c r="K170" s="18" t="inlineStr">
+        <is>
+          <t>Apply</t>
+        </is>
+      </c>
+      <c r="L170" s="21" t="inlineStr">
         <is>
           <t>Office-first (not remote). Loc:  | verify: unknown</t>
         </is>
@@ -9964,12 +9964,12 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Senior Backend Engineer (Golang) - Bank</t>
+          <t>Senior Software Engineer</t>
         </is>
       </c>
       <c r="E171" s="13" t="inlineStr">
         <is>
-          <t>https://sumup.com/careers/positions/8454657002?gh_jid=8454657002</t>
+          <t>https://sumup.com/careers/positions/8468000002?gh_jid=8468000002</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
@@ -10014,12 +10014,12 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Senior Backend Engineer - Accounts</t>
+          <t>Software Engineer</t>
         </is>
       </c>
       <c r="E172" s="13" t="inlineStr">
         <is>
-          <t>https://sumup.com/careers/positions/8418287002?gh_jid=8418287002</t>
+          <t>https://sumup.com/careers/positions/8448678002?gh_jid=8448678002</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
@@ -10064,12 +10064,12 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Senior Backend Engineer - Fiscalization</t>
+          <t>Software Engineer (Golang) - Online Payments</t>
         </is>
       </c>
       <c r="E173" s="13" t="inlineStr">
         <is>
-          <t>https://sumup.com/careers/positions/8222274002?gh_jid=8222274002</t>
+          <t>https://sumup.com/careers/positions/8520790002?gh_jid=8520790002</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
@@ -10114,12 +10114,12 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Senior Backend Engineer - Golang</t>
+          <t>Software Engineer II</t>
         </is>
       </c>
       <c r="E174" s="13" t="inlineStr">
         <is>
-          <t>https://sumup.com/careers/positions/8429621002?gh_jid=8429621002</t>
+          <t>https://sumup.com/careers/positions/8468005002?gh_jid=8468005002</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
@@ -10164,12 +10164,12 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Senior Backend Engineer - Transfers</t>
+          <t>Software Engineering Manager</t>
         </is>
       </c>
       <c r="E175" s="13" t="inlineStr">
         <is>
-          <t>https://sumup.com/careers/positions/8383464002?gh_jid=8383464002</t>
+          <t>https://sumup.com/careers/positions/8420811002?gh_jid=8420811002</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
@@ -10198,404 +10198,396 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C176" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D176" t="inlineStr">
-        <is>
-          <t>Senior Backend Engineer Go - Payments Reporting</t>
-        </is>
-      </c>
-      <c r="E176" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8494767002?gh_jid=8494767002</t>
-        </is>
-      </c>
-      <c r="F176" t="inlineStr">
+      <c r="A176" s="23">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B176" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C176" s="23" t="inlineStr">
+        <is>
+          <t>Glean</t>
+        </is>
+      </c>
+      <c r="D176" s="23" t="inlineStr">
+        <is>
+          <t>Software Engineer, Backend</t>
+        </is>
+      </c>
+      <c r="E176" s="23" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4581643005</t>
+        </is>
+      </c>
+      <c r="F176" s="23" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="H176" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I176" t="n">
-        <v>3</v>
-      </c>
-      <c r="J176" s="1" t="n"/>
-      <c r="K176" t="inlineStr">
+      <c r="G176" s="23" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H176" s="23" t="inlineStr">
+        <is>
+          <t>Loc: San Francisco Bay Area</t>
+        </is>
+      </c>
+      <c r="I176" s="23" t="n"/>
+      <c r="J176" s="23" t="n"/>
+      <c r="K176" s="23" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L176" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
+      <c r="L176" s="23" t="inlineStr"/>
     </row>
     <row r="177">
-      <c r="A177">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C177" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D177" t="inlineStr">
-        <is>
-          <t>Senior Backend Engineer- Global Bank</t>
-        </is>
-      </c>
-      <c r="E177" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/6651430002?gh_jid=6651430002</t>
-        </is>
-      </c>
-      <c r="F177" t="inlineStr">
+      <c r="A177" s="23">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B177" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C177" s="23" t="inlineStr">
+        <is>
+          <t>Intercom</t>
+        </is>
+      </c>
+      <c r="D177" s="23" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer - Team Web</t>
+        </is>
+      </c>
+      <c r="E177" s="23" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/intercom/jobs/7276257</t>
+        </is>
+      </c>
+      <c r="F177" s="23" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="H177" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I177" t="n">
-        <v>3</v>
-      </c>
-      <c r="J177" s="1" t="n"/>
-      <c r="K177" t="inlineStr">
+      <c r="G177" s="23" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H177" s="23" t="inlineStr">
+        <is>
+          <t>Loc: London, England</t>
+        </is>
+      </c>
+      <c r="I177" s="23" t="n"/>
+      <c r="J177" s="23" t="n"/>
+      <c r="K177" s="23" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L177" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
+      <c r="L177" s="23" t="inlineStr"/>
     </row>
     <row r="178">
-      <c r="A178" s="18">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B178" s="18" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C178" s="18" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D178" s="18" t="inlineStr">
-        <is>
-          <t>Senior Fullstack Engineer (NodeJs)</t>
-        </is>
-      </c>
-      <c r="E178" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8537166002?gh_jid=8537166002</t>
-        </is>
-      </c>
-      <c r="F178" s="18" t="inlineStr">
+      <c r="A178" s="23">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B178" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C178" s="23" t="inlineStr">
+        <is>
+          <t>Contentful</t>
+        </is>
+      </c>
+      <c r="D178" s="23" t="inlineStr">
+        <is>
+          <t>Fullstack Software Engineer (f/m/d)</t>
+        </is>
+      </c>
+      <c r="E178" s="23" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/contentful/jobs/7553930</t>
+        </is>
+      </c>
+      <c r="F178" s="23" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="H178" s="18" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I178" s="18" t="n">
-        <v>5</v>
-      </c>
-      <c r="J178" s="1" t="n"/>
-      <c r="K178" s="18" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="L178" s="21" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
+      <c r="G178" s="23" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H178" s="23" t="inlineStr">
+        <is>
+          <t>Loc: London, England</t>
+        </is>
+      </c>
+      <c r="I178" s="23" t="n"/>
+      <c r="J178" s="23" t="n"/>
+      <c r="K178" s="23" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L178" s="23" t="inlineStr"/>
     </row>
     <row r="179">
-      <c r="A179">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B179" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C179" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D179" t="inlineStr">
-        <is>
-          <t>Senior Software Engineer</t>
-        </is>
-      </c>
-      <c r="E179" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8468000002?gh_jid=8468000002</t>
-        </is>
-      </c>
-      <c r="F179" t="inlineStr">
+      <c r="A179" s="23">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B179" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C179" s="23" t="inlineStr">
+        <is>
+          <t>Contentful</t>
+        </is>
+      </c>
+      <c r="D179" s="23" t="inlineStr">
+        <is>
+          <t>Senior Backend Engineer - AI Platform (f/m/d)</t>
+        </is>
+      </c>
+      <c r="E179" s="23" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/contentful/jobs/7776562</t>
+        </is>
+      </c>
+      <c r="F179" s="23" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="H179" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I179" t="n">
-        <v>3</v>
-      </c>
-      <c r="J179" s="1" t="n"/>
-      <c r="K179" t="inlineStr">
+      <c r="G179" s="23" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H179" s="23" t="inlineStr">
+        <is>
+          <t>Loc: London, England</t>
+        </is>
+      </c>
+      <c r="I179" s="23" t="n"/>
+      <c r="J179" s="23" t="n"/>
+      <c r="K179" s="23" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L179" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
+      <c r="L179" s="23" t="inlineStr"/>
     </row>
     <row r="180">
-      <c r="A180">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C180" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D180" t="inlineStr">
-        <is>
-          <t>Software Engineer</t>
-        </is>
-      </c>
-      <c r="E180" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8448678002?gh_jid=8448678002</t>
-        </is>
-      </c>
-      <c r="F180" t="inlineStr">
+      <c r="A180" s="23">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B180" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C180" s="23" t="inlineStr">
+        <is>
+          <t>Contentful</t>
+        </is>
+      </c>
+      <c r="D180" s="23" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer - Backend &amp; Infrastructure (f/m/d)</t>
+        </is>
+      </c>
+      <c r="E180" s="23" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/contentful/jobs/7760966</t>
+        </is>
+      </c>
+      <c r="F180" s="23" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="H180" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I180" t="n">
-        <v>3</v>
-      </c>
-      <c r="J180" s="1" t="n"/>
-      <c r="K180" t="inlineStr">
+      <c r="G180" s="23" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H180" s="23" t="inlineStr">
+        <is>
+          <t>Loc: Berlin, Germany</t>
+        </is>
+      </c>
+      <c r="I180" s="23" t="n"/>
+      <c r="J180" s="23" t="n"/>
+      <c r="K180" s="23" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L180" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
+      <c r="L180" s="23" t="inlineStr"/>
     </row>
     <row r="181">
-      <c r="A181">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C181" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D181" t="inlineStr">
-        <is>
-          <t>Software Engineer (Golang) - Online Payments</t>
-        </is>
-      </c>
-      <c r="E181" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8520790002?gh_jid=8520790002</t>
-        </is>
-      </c>
-      <c r="F181" t="inlineStr">
+      <c r="A181" s="23">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B181" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C181" s="23" t="inlineStr">
+        <is>
+          <t>N26</t>
+        </is>
+      </c>
+      <c r="D181" s="23" t="inlineStr">
+        <is>
+          <t>Backend Engineer - Acquire</t>
+        </is>
+      </c>
+      <c r="E181" s="23" t="inlineStr">
+        <is>
+          <t>https://n26.com/en-eu/careers/positions/7742395?gh_jid=7742395</t>
+        </is>
+      </c>
+      <c r="F181" s="23" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="H181" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I181" t="n">
-        <v>3</v>
-      </c>
-      <c r="J181" s="1" t="n"/>
-      <c r="K181" t="inlineStr">
+      <c r="G181" s="23" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H181" s="23" t="inlineStr">
+        <is>
+          <t>Loc: Berlin</t>
+        </is>
+      </c>
+      <c r="I181" s="23" t="n"/>
+      <c r="J181" s="23" t="n"/>
+      <c r="K181" s="23" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L181" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
+      <c r="L181" s="23" t="inlineStr"/>
     </row>
     <row r="182">
-      <c r="A182">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C182" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D182" t="inlineStr">
-        <is>
-          <t>Software Engineer II</t>
-        </is>
-      </c>
-      <c r="E182" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8468005002?gh_jid=8468005002</t>
-        </is>
-      </c>
-      <c r="F182" t="inlineStr">
+      <c r="A182" s="23">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B182" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C182" s="23" t="inlineStr">
+        <is>
+          <t>N26</t>
+        </is>
+      </c>
+      <c r="D182" s="23" t="inlineStr">
+        <is>
+          <t>Backend Engineer - Engagement</t>
+        </is>
+      </c>
+      <c r="E182" s="23" t="inlineStr">
+        <is>
+          <t>https://n26.com/en-eu/careers/positions/7640893?gh_jid=7640893</t>
+        </is>
+      </c>
+      <c r="F182" s="23" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="H182" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I182" t="n">
-        <v>3</v>
-      </c>
-      <c r="J182" s="1" t="n"/>
-      <c r="K182" t="inlineStr">
+      <c r="G182" s="23" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H182" s="23" t="inlineStr">
+        <is>
+          <t>Loc: Berlin / Barcelona</t>
+        </is>
+      </c>
+      <c r="I182" s="23" t="n"/>
+      <c r="J182" s="23" t="n"/>
+      <c r="K182" s="23" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L182" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
+      <c r="L182" s="23" t="inlineStr"/>
     </row>
     <row r="183">
-      <c r="A183">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C183" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D183" t="inlineStr">
-        <is>
-          <t>Software Engineering Manager</t>
-        </is>
-      </c>
-      <c r="E183" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8420811002?gh_jid=8420811002</t>
-        </is>
-      </c>
-      <c r="F183" t="inlineStr">
+      <c r="A183" s="23">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B183" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C183" s="23" t="inlineStr">
+        <is>
+          <t>N26</t>
+        </is>
+      </c>
+      <c r="D183" s="23" t="inlineStr">
+        <is>
+          <t>Senior Full-Stack Security Automation Engineer</t>
+        </is>
+      </c>
+      <c r="E183" s="23" t="inlineStr">
+        <is>
+          <t>https://n26.com/en-eu/careers/positions/7597686?gh_jid=7597686</t>
+        </is>
+      </c>
+      <c r="F183" s="23" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="H183" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I183" t="n">
-        <v>3</v>
-      </c>
-      <c r="J183" s="1" t="n"/>
-      <c r="K183" t="inlineStr">
+      <c r="G183" s="23" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H183" s="23" t="inlineStr">
+        <is>
+          <t>Loc: Barcelona</t>
+        </is>
+      </c>
+      <c r="I183" s="23" t="n"/>
+      <c r="J183" s="23" t="n"/>
+      <c r="K183" s="23" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L183" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
+      <c r="L183" s="23" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="23">
@@ -10609,17 +10601,17 @@
       </c>
       <c r="C184" s="23" t="inlineStr">
         <is>
-          <t>Glean</t>
+          <t>SumUp</t>
         </is>
       </c>
       <c r="D184" s="23" t="inlineStr">
         <is>
-          <t>Software Engineer, Backend</t>
+          <t>Senior Backend Engineer - Accounts</t>
         </is>
       </c>
       <c r="E184" s="23" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4581643005</t>
+          <t>https://sumup.com/careers/positions/8418083002?gh_jid=8418083002</t>
         </is>
       </c>
       <c r="F184" s="23" t="inlineStr">
@@ -10634,7 +10626,7 @@
       </c>
       <c r="H184" s="23" t="inlineStr">
         <is>
-          <t>Loc: San Francisco Bay Area</t>
+          <t>Loc: Berlin, Germany</t>
         </is>
       </c>
       <c r="I184" s="23" t="n"/>
@@ -10644,7 +10636,11 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L184" s="23" t="inlineStr"/>
+      <c r="L184" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote)</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="23">
@@ -10658,17 +10654,17 @@
       </c>
       <c r="C185" s="23" t="inlineStr">
         <is>
-          <t>Intercom</t>
+          <t>SumUp</t>
         </is>
       </c>
       <c r="D185" s="23" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - Team Web</t>
+          <t>Senior Backend Engineer - Fiscalization</t>
         </is>
       </c>
       <c r="E185" s="23" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/intercom/jobs/7276257</t>
+          <t>https://sumup.com/careers/positions/8321240002?gh_jid=8321240002</t>
         </is>
       </c>
       <c r="F185" s="23" t="inlineStr">
@@ -10683,7 +10679,7 @@
       </c>
       <c r="H185" s="23" t="inlineStr">
         <is>
-          <t>Loc: London, England</t>
+          <t>Loc: Berlin, Germany</t>
         </is>
       </c>
       <c r="I185" s="23" t="n"/>
@@ -10693,7 +10689,11 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L185" s="23" t="inlineStr"/>
+      <c r="L185" s="23" t="inlineStr">
+        <is>
+          <t>Office-first (not remote)</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="23">
@@ -10707,17 +10707,17 @@
       </c>
       <c r="C186" s="23" t="inlineStr">
         <is>
-          <t>Contentful</t>
+          <t>Legora</t>
         </is>
       </c>
       <c r="D186" s="23" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer (f/m/d)</t>
+          <t>Senior Backend Engineer</t>
         </is>
       </c>
       <c r="E186" s="23" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/contentful/jobs/7553930</t>
+          <t>https://jobs.ashbyhq.com/legora/b0dcbd44-38c5-46fc-aa9a-610fe881fc1c</t>
         </is>
       </c>
       <c r="F186" s="23" t="inlineStr">
@@ -10732,7 +10732,7 @@
       </c>
       <c r="H186" s="23" t="inlineStr">
         <is>
-          <t>Loc: London, England</t>
+          <t>Loc: Malmö</t>
         </is>
       </c>
       <c r="I186" s="23" t="n"/>
@@ -10756,17 +10756,17 @@
       </c>
       <c r="C187" s="23" t="inlineStr">
         <is>
-          <t>Contentful</t>
+          <t>Legora</t>
         </is>
       </c>
       <c r="D187" s="23" t="inlineStr">
         <is>
-          <t>Senior Backend Engineer - AI Platform (f/m/d)</t>
+          <t>Senior Software Engineer</t>
         </is>
       </c>
       <c r="E187" s="23" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/contentful/jobs/7776562</t>
+          <t>https://jobs.ashbyhq.com/legora/2ec4729a-82e2-4e7b-90d9-c9afb8e941bb</t>
         </is>
       </c>
       <c r="F187" s="23" t="inlineStr">
@@ -10781,7 +10781,7 @@
       </c>
       <c r="H187" s="23" t="inlineStr">
         <is>
-          <t>Loc: London, England</t>
+          <t>Loc: Stockholm HQ</t>
         </is>
       </c>
       <c r="I187" s="23" t="n"/>
@@ -10805,17 +10805,17 @@
       </c>
       <c r="C188" s="23" t="inlineStr">
         <is>
-          <t>Contentful</t>
+          <t>HelloFresh</t>
         </is>
       </c>
       <c r="D188" s="23" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Backend &amp; Infrastructure (f/m/d)</t>
+          <t>React Native Developer, Growth</t>
         </is>
       </c>
       <c r="E188" s="23" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/contentful/jobs/7760966</t>
+          <t>https://careers.hellofresh.com/global/en/job/7862406?gh_jid=7862406</t>
         </is>
       </c>
       <c r="F188" s="23" t="inlineStr">
@@ -10830,7 +10830,7 @@
       </c>
       <c r="H188" s="23" t="inlineStr">
         <is>
-          <t>Loc: Berlin, Germany</t>
+          <t>Loc: Toronto, Ontario, Canada</t>
         </is>
       </c>
       <c r="I188" s="23" t="n"/>
@@ -10854,17 +10854,17 @@
       </c>
       <c r="C189" s="23" t="inlineStr">
         <is>
-          <t>N26</t>
+          <t>Pigment</t>
         </is>
       </c>
       <c r="D189" s="23" t="inlineStr">
         <is>
-          <t>Backend Engineer - Acquire</t>
+          <t>Senior Backend Software Engineer</t>
         </is>
       </c>
       <c r="E189" s="23" t="inlineStr">
         <is>
-          <t>https://n26.com/en-eu/careers/positions/7742395?gh_jid=7742395</t>
+          <t>https://jobs.lever.co/pigment/bf7cacad-0f52-4db4-88d4-ad7b22bd852e</t>
         </is>
       </c>
       <c r="F189" s="23" t="inlineStr">
@@ -10879,7 +10879,7 @@
       </c>
       <c r="H189" s="23" t="inlineStr">
         <is>
-          <t>Loc: Berlin</t>
+          <t>Loc: France</t>
         </is>
       </c>
       <c r="I189" s="23" t="n"/>
@@ -10890,504 +10890,6 @@
         </is>
       </c>
       <c r="L189" s="23" t="inlineStr"/>
-    </row>
-    <row r="190">
-      <c r="A190" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B190" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C190" s="23" t="inlineStr">
-        <is>
-          <t>N26</t>
-        </is>
-      </c>
-      <c r="D190" s="23" t="inlineStr">
-        <is>
-          <t>Backend Engineer - Engagement</t>
-        </is>
-      </c>
-      <c r="E190" s="23" t="inlineStr">
-        <is>
-          <t>https://n26.com/en-eu/careers/positions/7640893?gh_jid=7640893</t>
-        </is>
-      </c>
-      <c r="F190" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G190" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H190" s="23" t="inlineStr">
-        <is>
-          <t>Loc: Berlin / Barcelona</t>
-        </is>
-      </c>
-      <c r="I190" s="23" t="n"/>
-      <c r="J190" s="23" t="n"/>
-      <c r="K190" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L190" s="23" t="inlineStr"/>
-    </row>
-    <row r="191">
-      <c r="A191" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B191" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C191" s="23" t="inlineStr">
-        <is>
-          <t>N26</t>
-        </is>
-      </c>
-      <c r="D191" s="23" t="inlineStr">
-        <is>
-          <t>Senior Full-Stack Security Automation Engineer</t>
-        </is>
-      </c>
-      <c r="E191" s="23" t="inlineStr">
-        <is>
-          <t>https://n26.com/en-eu/careers/positions/7597686?gh_jid=7597686</t>
-        </is>
-      </c>
-      <c r="F191" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G191" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H191" s="23" t="inlineStr">
-        <is>
-          <t>Loc: Barcelona</t>
-        </is>
-      </c>
-      <c r="I191" s="23" t="n"/>
-      <c r="J191" s="23" t="n"/>
-      <c r="K191" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L191" s="23" t="inlineStr"/>
-    </row>
-    <row r="192">
-      <c r="A192" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B192" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C192" s="23" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D192" s="23" t="inlineStr">
-        <is>
-          <t>Senior Backend Engineer - Accounts</t>
-        </is>
-      </c>
-      <c r="E192" s="23" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8418083002?gh_jid=8418083002</t>
-        </is>
-      </c>
-      <c r="F192" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G192" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H192" s="23" t="inlineStr">
-        <is>
-          <t>Loc: Berlin, Germany</t>
-        </is>
-      </c>
-      <c r="I192" s="23" t="n"/>
-      <c r="J192" s="23" t="n"/>
-      <c r="K192" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L192" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote)</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B193" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C193" s="23" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D193" s="23" t="inlineStr">
-        <is>
-          <t>Senior Backend Engineer - Fiscalization</t>
-        </is>
-      </c>
-      <c r="E193" s="23" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8321240002?gh_jid=8321240002</t>
-        </is>
-      </c>
-      <c r="F193" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G193" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H193" s="23" t="inlineStr">
-        <is>
-          <t>Loc: Berlin, Germany</t>
-        </is>
-      </c>
-      <c r="I193" s="23" t="n"/>
-      <c r="J193" s="23" t="n"/>
-      <c r="K193" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L193" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote)</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B194" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C194" s="23" t="inlineStr">
-        <is>
-          <t>Legora</t>
-        </is>
-      </c>
-      <c r="D194" s="23" t="inlineStr">
-        <is>
-          <t>Senior Backend Engineer</t>
-        </is>
-      </c>
-      <c r="E194" s="23" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/legora/b0dcbd44-38c5-46fc-aa9a-610fe881fc1c</t>
-        </is>
-      </c>
-      <c r="F194" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G194" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H194" s="23" t="inlineStr">
-        <is>
-          <t>Loc: Malmö</t>
-        </is>
-      </c>
-      <c r="I194" s="23" t="n"/>
-      <c r="J194" s="23" t="n"/>
-      <c r="K194" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L194" s="23" t="inlineStr"/>
-    </row>
-    <row r="195">
-      <c r="A195" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B195" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C195" s="23" t="inlineStr">
-        <is>
-          <t>Legora</t>
-        </is>
-      </c>
-      <c r="D195" s="23" t="inlineStr">
-        <is>
-          <t>Senior Software Engineer</t>
-        </is>
-      </c>
-      <c r="E195" s="23" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/legora/2ec4729a-82e2-4e7b-90d9-c9afb8e941bb</t>
-        </is>
-      </c>
-      <c r="F195" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G195" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H195" s="23" t="inlineStr">
-        <is>
-          <t>Loc: Stockholm HQ</t>
-        </is>
-      </c>
-      <c r="I195" s="23" t="n"/>
-      <c r="J195" s="23" t="n"/>
-      <c r="K195" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L195" s="23" t="inlineStr"/>
-    </row>
-    <row r="196">
-      <c r="A196" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B196" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C196" s="23" t="inlineStr">
-        <is>
-          <t>HelloFresh</t>
-        </is>
-      </c>
-      <c r="D196" s="23" t="inlineStr">
-        <is>
-          <t>React Native Developer, Growth</t>
-        </is>
-      </c>
-      <c r="E196" s="23" t="inlineStr">
-        <is>
-          <t>https://careers.hellofresh.com/global/en/job/7862406?gh_jid=7862406</t>
-        </is>
-      </c>
-      <c r="F196" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G196" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H196" s="23" t="inlineStr">
-        <is>
-          <t>Loc: Toronto, Ontario, Canada</t>
-        </is>
-      </c>
-      <c r="I196" s="23" t="n"/>
-      <c r="J196" s="23" t="n"/>
-      <c r="K196" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L196" s="23" t="inlineStr"/>
-    </row>
-    <row r="197">
-      <c r="A197" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B197" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C197" s="23" t="inlineStr">
-        <is>
-          <t>Wayve</t>
-        </is>
-      </c>
-      <c r="D197" s="23" t="inlineStr">
-        <is>
-          <t>Application Software Engineer</t>
-        </is>
-      </c>
-      <c r="E197" s="23" t="inlineStr">
-        <is>
-          <t>https://wayve.firststage.co/jobs?gh_jid=8431122002</t>
-        </is>
-      </c>
-      <c r="F197" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G197" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H197" s="23" t="inlineStr">
-        <is>
-          <t>Loc: Germany</t>
-        </is>
-      </c>
-      <c r="I197" s="23" t="n"/>
-      <c r="J197" s="23" t="n"/>
-      <c r="K197" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L197" s="23" t="inlineStr"/>
-    </row>
-    <row r="198">
-      <c r="A198" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B198" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C198" s="23" t="inlineStr">
-        <is>
-          <t>Wayve</t>
-        </is>
-      </c>
-      <c r="D198" s="23" t="inlineStr">
-        <is>
-          <t>Application Software Engineer - Relocation to Tokyo</t>
-        </is>
-      </c>
-      <c r="E198" s="23" t="inlineStr">
-        <is>
-          <t>https://wayve.firststage.co/jobs?gh_jid=8460447002</t>
-        </is>
-      </c>
-      <c r="F198" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G198" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H198" s="23" t="inlineStr">
-        <is>
-          <t>Loc: London (relocates to Tokyo)</t>
-        </is>
-      </c>
-      <c r="I198" s="23" t="n"/>
-      <c r="J198" s="23" t="n"/>
-      <c r="K198" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L198" s="23" t="inlineStr"/>
-    </row>
-    <row r="199">
-      <c r="A199" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B199" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C199" s="23" t="inlineStr">
-        <is>
-          <t>Pigment</t>
-        </is>
-      </c>
-      <c r="D199" s="23" t="inlineStr">
-        <is>
-          <t>Senior Backend Software Engineer</t>
-        </is>
-      </c>
-      <c r="E199" s="23" t="inlineStr">
-        <is>
-          <t>https://jobs.lever.co/pigment/bf7cacad-0f52-4db4-88d4-ad7b22bd852e</t>
-        </is>
-      </c>
-      <c r="F199" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G199" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H199" s="23" t="inlineStr">
-        <is>
-          <t>Loc: France</t>
-        </is>
-      </c>
-      <c r="I199" s="23" t="n"/>
-      <c r="J199" s="23" t="n"/>
-      <c r="K199" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L199" s="23" t="inlineStr"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="J2:J1000">
@@ -11539,41 +11041,33 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E147" r:id="rId107"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E148" r:id="rId108"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E149" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E150" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E151" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E152" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E153" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E154" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E155" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E156" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E157" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E158" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E159" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E160" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E161" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E162" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E163" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E164" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E165" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E166" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E167" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E168" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E169" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E170" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E171" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E172" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E173" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E174" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E175" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E176" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E177" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E178" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E179" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E180" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E181" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E182" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E183" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E184" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E158" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E159" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E160" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E161" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E162" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E163" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E164" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E165" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E166" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E167" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E168" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E169" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E170" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E171" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E172" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E173" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E174" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E175" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E176" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E177" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E178" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E179" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E180" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E181" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E182" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E183" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E184" r:id="rId136"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -18307,15 +17801,19 @@
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E66" s="24" t="inlineStr">
         <is>
-          <t>Berlin / London. Payments fintech, EU + LATAM hiring. OFFICE-FIRST — not remote. Flexible work case-by-case via interview.</t>
-        </is>
-      </c>
-      <c r="F66" s="10" t="n"/>
+          <t>Berlin / London. Payments fintech, EU + LATAM hiring. OFFICE-FIRST — not remote. Flexible work case-by-case via interview. Excluded from scans (relocation friction + many duplicates).</t>
+        </is>
+      </c>
+      <c r="F66" s="10" t="inlineStr">
+        <is>
+          <t>Excluded</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="10" t="n">
@@ -18541,15 +18039,19 @@
       </c>
       <c r="D75" s="10" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E75" s="10" t="inlineStr">
-        <is>
-          <t>London UK. Embodied AI for self-driving, ML &amp; robotics roles.</t>
-        </is>
-      </c>
-      <c r="F75" s="10" t="n"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E75" s="24" t="inlineStr">
+        <is>
+          <t>London UK / Tokyo. Self-driving AV — hardware/automotive/embedded stack (C/C++, Linux BSP, Yocto, QNX, AUTOSAR, SoC bring-up). NOT relevant to user's web/backend profile. Excluded from scans.</t>
+        </is>
+      </c>
+      <c r="F75" s="10" t="inlineStr">
+        <is>
+          <t>Excluded</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="10" t="n">

</xml_diff>

<commit_message>
Remove all 26 SumUp opportunities from Wishlist
Following the company-level exclusion (office-first + dup-heavy),
prune existing SumUp rows from Wishlist for a clean break. Also
removed 24 SumUp lines from data/pipeline.md and flipped 24 entries
in data/scan-history.tsv to 'excluded' so future scans won't re-add.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -1419,7 +1419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L189"/>
+  <dimension ref="A1:L163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="1" min="1" max="1"/>
@@ -8409,17 +8409,17 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>SumUp</t>
+          <t>Synthesia</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Backend Engineer (Global Bank Tribe)</t>
+          <t>Software Engineer, Back End Leaning (Tech Lead Level)</t>
         </is>
       </c>
       <c r="E140" s="13" t="inlineStr">
         <is>
-          <t>https://sumup.com/careers/positions/8420739002?gh_jid=8420739002</t>
+          <t>https://jobs.ashbyhq.com/synthesia/bf515974-3bab-46cb-85fd-5bacafcc1a91</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -8441,9 +8441,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="L140" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unclear</t>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>Loc:  | verify: unclear</t>
         </is>
       </c>
     </row>
@@ -8464,12 +8464,12 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Software Engineer, Back End Leaning (Tech Lead Level)</t>
+          <t>Software Engineer, Front End Leaning (Accessibility)</t>
         </is>
       </c>
       <c r="E141" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/synthesia/bf515974-3bab-46cb-85fd-5bacafcc1a91</t>
+          <t>https://jobs.ashbyhq.com/synthesia/e1fedec8-ea12-4e7f-95e1-475b95dbd517</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -8514,12 +8514,12 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Software Engineer, Front End Leaning (Accessibility)</t>
+          <t>Software Engineer, Front End Leaning (Tech Lead level)</t>
         </is>
       </c>
       <c r="E142" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/synthesia/e1fedec8-ea12-4e7f-95e1-475b95dbd517</t>
+          <t>https://jobs.ashbyhq.com/synthesia/22a00ec6-ac40-4b87-97bc-a0f7bf724be7</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -8564,12 +8564,12 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Software Engineer, Front End Leaning (Tech Lead level)</t>
+          <t>Webflow Developer / Front-End Engineer</t>
         </is>
       </c>
       <c r="E143" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/synthesia/22a00ec6-ac40-4b87-97bc-a0f7bf724be7</t>
+          <t>https://jobs.ashbyhq.com/synthesia/dcc970b0-9043-4fc6-b628-3b8dad021c84</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -8609,17 +8609,17 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Synthesia</t>
+          <t>Trade Republic</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Webflow Developer / Front-End Engineer</t>
+          <t>Backend Engineer (Berlin)</t>
         </is>
       </c>
       <c r="E144" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/synthesia/dcc970b0-9043-4fc6-b628-3b8dad021c84</t>
+          <t>https://traderepublic.com/en-de/about?jobId=6539149003&amp;gh_jid=6539149003</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -8664,12 +8664,12 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Backend Engineer (Berlin)</t>
+          <t>Backend Engineer (Haskell)</t>
         </is>
       </c>
       <c r="E145" s="13" t="inlineStr">
         <is>
-          <t>https://traderepublic.com/en-de/about?jobId=6539149003&amp;gh_jid=6539149003</t>
+          <t>https://traderepublic.com/en-de/about?jobId=7718242003&amp;gh_jid=7718242003</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
@@ -8714,12 +8714,12 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Backend Engineer (Haskell)</t>
+          <t>Backend Engineer (London)</t>
         </is>
       </c>
       <c r="E146" s="13" t="inlineStr">
         <is>
-          <t>https://traderepublic.com/en-de/about?jobId=7718242003&amp;gh_jid=7718242003</t>
+          <t>https://traderepublic.com/en-de/about?jobId=6327292003&amp;gh_jid=6327292003</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -8764,12 +8764,12 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Backend Engineer (London)</t>
+          <t>Backend Engineer (Paris)</t>
         </is>
       </c>
       <c r="E147" s="13" t="inlineStr">
         <is>
-          <t>https://traderepublic.com/en-de/about?jobId=6327292003&amp;gh_jid=6327292003</t>
+          <t>https://traderepublic.com/en-de/about?jobId=6539038003&amp;gh_jid=6539038003</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -8814,12 +8814,12 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Backend Engineer (Paris)</t>
+          <t>Graduate Backend Engineering Programme - Paris</t>
         </is>
       </c>
       <c r="E148" s="13" t="inlineStr">
         <is>
-          <t>https://traderepublic.com/en-de/about?jobId=6539038003&amp;gh_jid=6539038003</t>
+          <t>https://traderepublic.com/en-de/about?jobId=7714721003&amp;gh_jid=7714721003</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -8859,17 +8859,17 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Trade Republic</t>
+          <t>Zapier</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Graduate Backend Engineering Programme - Paris</t>
-        </is>
-      </c>
-      <c r="E149" s="13" t="inlineStr">
-        <is>
-          <t>https://traderepublic.com/en-de/about?jobId=7714721003&amp;gh_jid=7714721003</t>
+          <t>Software Engineer — Release Engineering</t>
+        </is>
+      </c>
+      <c r="E149" s="19" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/zapier/6948a0e6-a580-4e9d-b109-20652d9a1507</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -8914,12 +8914,12 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Software Engineer — Release Engineering</t>
+          <t>Sr. Engineer, Backend - Enterprise</t>
         </is>
       </c>
       <c r="E150" s="19" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/zapier/6948a0e6-a580-4e9d-b109-20652d9a1507</t>
+          <t>https://jobs.ashbyhq.com/zapier/423d1bb7-1c08-458e-8a17-29a63cf23d92</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -8964,12 +8964,12 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Sr. Engineer, Backend - Enterprise</t>
+          <t>Sr. Fullstack Engineer, Identity Platform</t>
         </is>
       </c>
       <c r="E151" s="19" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/zapier/423d1bb7-1c08-458e-8a17-29a63cf23d92</t>
+          <t>https://jobs.ashbyhq.com/zapier/3b141014-1d0f-426e-94e5-997b2cfd6ae8</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -8998,1898 +8998,592 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>Zapier</t>
-        </is>
-      </c>
-      <c r="D152" t="inlineStr">
-        <is>
-          <t>Sr. Fullstack Engineer, Identity Platform</t>
-        </is>
-      </c>
-      <c r="E152" s="19" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/zapier/3b141014-1d0f-426e-94e5-997b2cfd6ae8</t>
-        </is>
-      </c>
-      <c r="F152" t="inlineStr">
+      <c r="A152" s="23">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B152" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C152" s="23" t="inlineStr">
+        <is>
+          <t>Glean</t>
+        </is>
+      </c>
+      <c r="D152" s="23" t="inlineStr">
+        <is>
+          <t>Software Engineer, Backend</t>
+        </is>
+      </c>
+      <c r="E152" s="23" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4581643005</t>
+        </is>
+      </c>
+      <c r="F152" s="23" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="H152" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I152" t="n">
-        <v>3</v>
-      </c>
-      <c r="J152" s="1" t="n"/>
-      <c r="K152" t="inlineStr">
+      <c r="G152" s="23" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H152" s="23" t="inlineStr">
+        <is>
+          <t>Loc: San Francisco Bay Area</t>
+        </is>
+      </c>
+      <c r="I152" s="23" t="n"/>
+      <c r="J152" s="23" t="n"/>
+      <c r="K152" s="23" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L152" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unclear</t>
-        </is>
-      </c>
+      <c r="L152" s="23" t="inlineStr"/>
     </row>
     <row r="153">
-      <c r="A153">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>(Senior) Backend Engineer (Golang) - Global Bank</t>
-        </is>
-      </c>
-      <c r="E153" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8207386002?gh_jid=8207386002</t>
-        </is>
-      </c>
-      <c r="F153" t="inlineStr">
+      <c r="A153" s="23">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B153" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C153" s="23" t="inlineStr">
+        <is>
+          <t>Intercom</t>
+        </is>
+      </c>
+      <c r="D153" s="23" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer - Team Web</t>
+        </is>
+      </c>
+      <c r="E153" s="23" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/intercom/jobs/7276257</t>
+        </is>
+      </c>
+      <c r="F153" s="23" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="H153" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I153" t="n">
-        <v>3</v>
-      </c>
-      <c r="J153" s="1" t="n"/>
-      <c r="K153" t="inlineStr">
+      <c r="G153" s="23" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H153" s="23" t="inlineStr">
+        <is>
+          <t>Loc: London, England</t>
+        </is>
+      </c>
+      <c r="I153" s="23" t="n"/>
+      <c r="J153" s="23" t="n"/>
+      <c r="K153" s="23" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L153" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
+      <c r="L153" s="23" t="inlineStr"/>
     </row>
     <row r="154">
-      <c r="A154">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D154" t="inlineStr">
-        <is>
-          <t>(Senior) Backend Engineer - Global Bank</t>
-        </is>
-      </c>
-      <c r="E154" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8207403002?gh_jid=8207403002</t>
-        </is>
-      </c>
-      <c r="F154" t="inlineStr">
+      <c r="A154" s="23">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B154" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C154" s="23" t="inlineStr">
+        <is>
+          <t>Contentful</t>
+        </is>
+      </c>
+      <c r="D154" s="23" t="inlineStr">
+        <is>
+          <t>Fullstack Software Engineer (f/m/d)</t>
+        </is>
+      </c>
+      <c r="E154" s="23" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/contentful/jobs/7553930</t>
+        </is>
+      </c>
+      <c r="F154" s="23" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="H154" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I154" t="n">
-        <v>3</v>
-      </c>
-      <c r="J154" s="1" t="n"/>
-      <c r="K154" t="inlineStr">
+      <c r="G154" s="23" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H154" s="23" t="inlineStr">
+        <is>
+          <t>Loc: London, England</t>
+        </is>
+      </c>
+      <c r="I154" s="23" t="n"/>
+      <c r="J154" s="23" t="n"/>
+      <c r="K154" s="23" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L154" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
+      <c r="L154" s="23" t="inlineStr"/>
     </row>
     <row r="155">
-      <c r="A155">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D155" t="inlineStr">
-        <is>
-          <t>(Senior/Mid) Software Engineer, Golang - Payments Platform</t>
-        </is>
-      </c>
-      <c r="E155" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8520784002?gh_jid=8520784002</t>
-        </is>
-      </c>
-      <c r="F155" t="inlineStr">
+      <c r="A155" s="23">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B155" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C155" s="23" t="inlineStr">
+        <is>
+          <t>Contentful</t>
+        </is>
+      </c>
+      <c r="D155" s="23" t="inlineStr">
+        <is>
+          <t>Senior Backend Engineer - AI Platform (f/m/d)</t>
+        </is>
+      </c>
+      <c r="E155" s="23" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/contentful/jobs/7776562</t>
+        </is>
+      </c>
+      <c r="F155" s="23" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="H155" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I155" t="n">
-        <v>3</v>
-      </c>
-      <c r="J155" s="1" t="n"/>
-      <c r="K155" t="inlineStr">
+      <c r="G155" s="23" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H155" s="23" t="inlineStr">
+        <is>
+          <t>Loc: London, England</t>
+        </is>
+      </c>
+      <c r="I155" s="23" t="n"/>
+      <c r="J155" s="23" t="n"/>
+      <c r="K155" s="23" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L155" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
+      <c r="L155" s="23" t="inlineStr"/>
     </row>
     <row r="156">
-      <c r="A156">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D156" t="inlineStr">
-        <is>
-          <t>Backend Engineer - POS</t>
-        </is>
-      </c>
-      <c r="E156" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8427119002?gh_jid=8427119002</t>
-        </is>
-      </c>
-      <c r="F156" t="inlineStr">
+      <c r="A156" s="23">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B156" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C156" s="23" t="inlineStr">
+        <is>
+          <t>Contentful</t>
+        </is>
+      </c>
+      <c r="D156" s="23" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer - Backend &amp; Infrastructure (f/m/d)</t>
+        </is>
+      </c>
+      <c r="E156" s="23" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/contentful/jobs/7760966</t>
+        </is>
+      </c>
+      <c r="F156" s="23" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="H156" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I156" t="n">
-        <v>3</v>
-      </c>
-      <c r="J156" s="1" t="n"/>
-      <c r="K156" t="inlineStr">
+      <c r="G156" s="23" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H156" s="23" t="inlineStr">
+        <is>
+          <t>Loc: Berlin, Germany</t>
+        </is>
+      </c>
+      <c r="I156" s="23" t="n"/>
+      <c r="J156" s="23" t="n"/>
+      <c r="K156" s="23" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L156" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
+      <c r="L156" s="23" t="inlineStr"/>
     </row>
     <row r="157">
-      <c r="A157">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D157" t="inlineStr">
-        <is>
-          <t>Backend Engineer - Transfers</t>
-        </is>
-      </c>
-      <c r="E157" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8388972002?gh_jid=8388972002</t>
-        </is>
-      </c>
-      <c r="F157" t="inlineStr">
+      <c r="A157" s="23">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B157" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C157" s="23" t="inlineStr">
+        <is>
+          <t>N26</t>
+        </is>
+      </c>
+      <c r="D157" s="23" t="inlineStr">
+        <is>
+          <t>Backend Engineer - Acquire</t>
+        </is>
+      </c>
+      <c r="E157" s="23" t="inlineStr">
+        <is>
+          <t>https://n26.com/en-eu/careers/positions/7742395?gh_jid=7742395</t>
+        </is>
+      </c>
+      <c r="F157" s="23" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="H157" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I157" t="n">
-        <v>3</v>
-      </c>
-      <c r="J157" s="1" t="n"/>
-      <c r="K157" t="inlineStr">
+      <c r="G157" s="23" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H157" s="23" t="inlineStr">
+        <is>
+          <t>Loc: Berlin</t>
+        </is>
+      </c>
+      <c r="I157" s="23" t="n"/>
+      <c r="J157" s="23" t="n"/>
+      <c r="K157" s="23" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L157" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
+      <c r="L157" s="23" t="inlineStr"/>
     </row>
     <row r="158">
-      <c r="A158">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D158" t="inlineStr">
-        <is>
-          <t>Backend engineer (Go)-  Payments Experience</t>
-        </is>
-      </c>
-      <c r="E158" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8497866002?gh_jid=8497866002</t>
-        </is>
-      </c>
-      <c r="F158" t="inlineStr">
+      <c r="A158" s="23">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B158" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C158" s="23" t="inlineStr">
+        <is>
+          <t>N26</t>
+        </is>
+      </c>
+      <c r="D158" s="23" t="inlineStr">
+        <is>
+          <t>Backend Engineer - Engagement</t>
+        </is>
+      </c>
+      <c r="E158" s="23" t="inlineStr">
+        <is>
+          <t>https://n26.com/en-eu/careers/positions/7640893?gh_jid=7640893</t>
+        </is>
+      </c>
+      <c r="F158" s="23" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="H158" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I158" t="n">
-        <v>3</v>
-      </c>
-      <c r="J158" s="1" t="n"/>
-      <c r="K158" t="inlineStr">
+      <c r="G158" s="23" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H158" s="23" t="inlineStr">
+        <is>
+          <t>Loc: Berlin / Barcelona</t>
+        </is>
+      </c>
+      <c r="I158" s="23" t="n"/>
+      <c r="J158" s="23" t="n"/>
+      <c r="K158" s="23" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L158" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
+      <c r="L158" s="23" t="inlineStr"/>
     </row>
     <row r="159">
-      <c r="A159">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D159" t="inlineStr">
-        <is>
-          <t>Fullstack Engineer (NodeJs)</t>
-        </is>
-      </c>
-      <c r="E159" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8482959002?gh_jid=8482959002</t>
-        </is>
-      </c>
-      <c r="F159" t="inlineStr">
+      <c r="A159" s="23">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B159" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C159" s="23" t="inlineStr">
+        <is>
+          <t>N26</t>
+        </is>
+      </c>
+      <c r="D159" s="23" t="inlineStr">
+        <is>
+          <t>Senior Full-Stack Security Automation Engineer</t>
+        </is>
+      </c>
+      <c r="E159" s="23" t="inlineStr">
+        <is>
+          <t>https://n26.com/en-eu/careers/positions/7597686?gh_jid=7597686</t>
+        </is>
+      </c>
+      <c r="F159" s="23" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="H159" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I159" t="n">
-        <v>3</v>
-      </c>
-      <c r="J159" s="1" t="n"/>
-      <c r="K159" t="inlineStr">
+      <c r="G159" s="23" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H159" s="23" t="inlineStr">
+        <is>
+          <t>Loc: Barcelona</t>
+        </is>
+      </c>
+      <c r="I159" s="23" t="n"/>
+      <c r="J159" s="23" t="n"/>
+      <c r="K159" s="23" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L159" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
+      <c r="L159" s="23" t="inlineStr"/>
     </row>
     <row r="160">
-      <c r="A160">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D160" t="inlineStr">
-        <is>
-          <t>Junior Backend Engineer (Golang) -  Payments Tribe</t>
-        </is>
-      </c>
-      <c r="E160" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8520406002?gh_jid=8520406002</t>
-        </is>
-      </c>
-      <c r="F160" t="inlineStr">
+      <c r="A160" s="23">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B160" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C160" s="23" t="inlineStr">
+        <is>
+          <t>Legora</t>
+        </is>
+      </c>
+      <c r="D160" s="23" t="inlineStr">
+        <is>
+          <t>Senior Backend Engineer</t>
+        </is>
+      </c>
+      <c r="E160" s="23" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/legora/b0dcbd44-38c5-46fc-aa9a-610fe881fc1c</t>
+        </is>
+      </c>
+      <c r="F160" s="23" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="H160" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I160" t="n">
-        <v>3</v>
-      </c>
-      <c r="J160" s="1" t="n"/>
-      <c r="K160" t="inlineStr">
+      <c r="G160" s="23" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H160" s="23" t="inlineStr">
+        <is>
+          <t>Loc: Malmö</t>
+        </is>
+      </c>
+      <c r="I160" s="23" t="n"/>
+      <c r="J160" s="23" t="n"/>
+      <c r="K160" s="23" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L160" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
+      <c r="L160" s="23" t="inlineStr"/>
     </row>
     <row r="161">
-      <c r="A161">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D161" t="inlineStr">
-        <is>
-          <t>Senior AI Backend Engineer</t>
-        </is>
-      </c>
-      <c r="E161" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8468006002?gh_jid=8468006002</t>
-        </is>
-      </c>
-      <c r="F161" t="inlineStr">
+      <c r="A161" s="23">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B161" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C161" s="23" t="inlineStr">
+        <is>
+          <t>Legora</t>
+        </is>
+      </c>
+      <c r="D161" s="23" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer</t>
+        </is>
+      </c>
+      <c r="E161" s="23" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/legora/2ec4729a-82e2-4e7b-90d9-c9afb8e941bb</t>
+        </is>
+      </c>
+      <c r="F161" s="23" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="H161" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I161" t="n">
-        <v>3</v>
-      </c>
-      <c r="J161" s="1" t="n"/>
-      <c r="K161" t="inlineStr">
+      <c r="G161" s="23" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H161" s="23" t="inlineStr">
+        <is>
+          <t>Loc: Stockholm HQ</t>
+        </is>
+      </c>
+      <c r="I161" s="23" t="n"/>
+      <c r="J161" s="23" t="n"/>
+      <c r="K161" s="23" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L161" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
+      <c r="L161" s="23" t="inlineStr"/>
     </row>
     <row r="162">
-      <c r="A162">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C162" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D162" t="inlineStr">
-        <is>
-          <t>Senior Backend Engineer</t>
-        </is>
-      </c>
-      <c r="E162" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/7480776002?gh_jid=7480776002</t>
-        </is>
-      </c>
-      <c r="F162" t="inlineStr">
+      <c r="A162" s="23">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B162" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C162" s="23" t="inlineStr">
+        <is>
+          <t>HelloFresh</t>
+        </is>
+      </c>
+      <c r="D162" s="23" t="inlineStr">
+        <is>
+          <t>React Native Developer, Growth</t>
+        </is>
+      </c>
+      <c r="E162" s="23" t="inlineStr">
+        <is>
+          <t>https://careers.hellofresh.com/global/en/job/7862406?gh_jid=7862406</t>
+        </is>
+      </c>
+      <c r="F162" s="23" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="H162" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I162" t="n">
-        <v>3</v>
-      </c>
-      <c r="J162" s="1" t="n"/>
-      <c r="K162" t="inlineStr">
+      <c r="G162" s="23" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H162" s="23" t="inlineStr">
+        <is>
+          <t>Loc: Toronto, Ontario, Canada</t>
+        </is>
+      </c>
+      <c r="I162" s="23" t="n"/>
+      <c r="J162" s="23" t="n"/>
+      <c r="K162" s="23" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L162" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
+      <c r="L162" s="23" t="inlineStr"/>
     </row>
     <row r="163">
-      <c r="A163">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B163" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C163" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D163" t="inlineStr">
-        <is>
-          <t>Senior Backend Engineer (Golang) - Bank</t>
-        </is>
-      </c>
-      <c r="E163" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8454657002?gh_jid=8454657002</t>
-        </is>
-      </c>
-      <c r="F163" t="inlineStr">
+      <c r="A163" s="23">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B163" s="23" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C163" s="23" t="inlineStr">
+        <is>
+          <t>Pigment</t>
+        </is>
+      </c>
+      <c r="D163" s="23" t="inlineStr">
+        <is>
+          <t>Senior Backend Software Engineer</t>
+        </is>
+      </c>
+      <c r="E163" s="23" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/pigment/bf7cacad-0f52-4db4-88d4-ad7b22bd852e</t>
+        </is>
+      </c>
+      <c r="F163" s="23" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="H163" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I163" t="n">
-        <v>3</v>
-      </c>
-      <c r="J163" s="1" t="n"/>
-      <c r="K163" t="inlineStr">
+      <c r="G163" s="23" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H163" s="23" t="inlineStr">
+        <is>
+          <t>Loc: France</t>
+        </is>
+      </c>
+      <c r="I163" s="23" t="n"/>
+      <c r="J163" s="23" t="n"/>
+      <c r="K163" s="23" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="L163" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C164" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D164" t="inlineStr">
-        <is>
-          <t>Senior Backend Engineer - Accounts</t>
-        </is>
-      </c>
-      <c r="E164" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8418287002?gh_jid=8418287002</t>
-        </is>
-      </c>
-      <c r="F164" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="H164" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I164" t="n">
-        <v>3</v>
-      </c>
-      <c r="J164" s="1" t="n"/>
-      <c r="K164" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L164" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C165" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D165" t="inlineStr">
-        <is>
-          <t>Senior Backend Engineer - Fiscalization</t>
-        </is>
-      </c>
-      <c r="E165" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8222274002?gh_jid=8222274002</t>
-        </is>
-      </c>
-      <c r="F165" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="H165" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I165" t="n">
-        <v>3</v>
-      </c>
-      <c r="J165" s="1" t="n"/>
-      <c r="K165" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L165" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C166" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D166" t="inlineStr">
-        <is>
-          <t>Senior Backend Engineer - Golang</t>
-        </is>
-      </c>
-      <c r="E166" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8429621002?gh_jid=8429621002</t>
-        </is>
-      </c>
-      <c r="F166" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="H166" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I166" t="n">
-        <v>3</v>
-      </c>
-      <c r="J166" s="1" t="n"/>
-      <c r="K166" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L166" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C167" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D167" t="inlineStr">
-        <is>
-          <t>Senior Backend Engineer - Transfers</t>
-        </is>
-      </c>
-      <c r="E167" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8383464002?gh_jid=8383464002</t>
-        </is>
-      </c>
-      <c r="F167" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="H167" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I167" t="n">
-        <v>3</v>
-      </c>
-      <c r="J167" s="1" t="n"/>
-      <c r="K167" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L167" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C168" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D168" t="inlineStr">
-        <is>
-          <t>Senior Backend Engineer Go - Payments Reporting</t>
-        </is>
-      </c>
-      <c r="E168" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8494767002?gh_jid=8494767002</t>
-        </is>
-      </c>
-      <c r="F168" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="H168" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I168" t="n">
-        <v>3</v>
-      </c>
-      <c r="J168" s="1" t="n"/>
-      <c r="K168" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L168" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B169" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C169" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D169" t="inlineStr">
-        <is>
-          <t>Senior Backend Engineer- Global Bank</t>
-        </is>
-      </c>
-      <c r="E169" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/6651430002?gh_jid=6651430002</t>
-        </is>
-      </c>
-      <c r="F169" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="H169" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I169" t="n">
-        <v>3</v>
-      </c>
-      <c r="J169" s="1" t="n"/>
-      <c r="K169" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L169" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" s="18">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B170" s="18" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C170" s="18" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D170" s="18" t="inlineStr">
-        <is>
-          <t>Senior Fullstack Engineer (NodeJs)</t>
-        </is>
-      </c>
-      <c r="E170" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8537166002?gh_jid=8537166002</t>
-        </is>
-      </c>
-      <c r="F170" s="18" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="H170" s="18" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I170" s="18" t="n">
-        <v>5</v>
-      </c>
-      <c r="J170" s="1" t="n"/>
-      <c r="K170" s="18" t="inlineStr">
-        <is>
-          <t>Apply</t>
-        </is>
-      </c>
-      <c r="L170" s="21" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B171" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C171" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D171" t="inlineStr">
-        <is>
-          <t>Senior Software Engineer</t>
-        </is>
-      </c>
-      <c r="E171" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8468000002?gh_jid=8468000002</t>
-        </is>
-      </c>
-      <c r="F171" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="H171" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I171" t="n">
-        <v>3</v>
-      </c>
-      <c r="J171" s="1" t="n"/>
-      <c r="K171" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L171" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B172" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C172" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D172" t="inlineStr">
-        <is>
-          <t>Software Engineer</t>
-        </is>
-      </c>
-      <c r="E172" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8448678002?gh_jid=8448678002</t>
-        </is>
-      </c>
-      <c r="F172" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="H172" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I172" t="n">
-        <v>3</v>
-      </c>
-      <c r="J172" s="1" t="n"/>
-      <c r="K172" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L172" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D173" t="inlineStr">
-        <is>
-          <t>Software Engineer (Golang) - Online Payments</t>
-        </is>
-      </c>
-      <c r="E173" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8520790002?gh_jid=8520790002</t>
-        </is>
-      </c>
-      <c r="F173" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="H173" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I173" t="n">
-        <v>3</v>
-      </c>
-      <c r="J173" s="1" t="n"/>
-      <c r="K173" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L173" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D174" t="inlineStr">
-        <is>
-          <t>Software Engineer II</t>
-        </is>
-      </c>
-      <c r="E174" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8468005002?gh_jid=8468005002</t>
-        </is>
-      </c>
-      <c r="F174" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="H174" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I174" t="n">
-        <v>3</v>
-      </c>
-      <c r="J174" s="1" t="n"/>
-      <c r="K174" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L174" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D175" t="inlineStr">
-        <is>
-          <t>Software Engineering Manager</t>
-        </is>
-      </c>
-      <c r="E175" s="13" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8420811002?gh_jid=8420811002</t>
-        </is>
-      </c>
-      <c r="F175" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="H175" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I175" t="n">
-        <v>3</v>
-      </c>
-      <c r="J175" s="1" t="n"/>
-      <c r="K175" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L175" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote). Loc:  | verify: unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B176" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C176" s="23" t="inlineStr">
-        <is>
-          <t>Glean</t>
-        </is>
-      </c>
-      <c r="D176" s="23" t="inlineStr">
-        <is>
-          <t>Software Engineer, Backend</t>
-        </is>
-      </c>
-      <c r="E176" s="23" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4581643005</t>
-        </is>
-      </c>
-      <c r="F176" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G176" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H176" s="23" t="inlineStr">
-        <is>
-          <t>Loc: San Francisco Bay Area</t>
-        </is>
-      </c>
-      <c r="I176" s="23" t="n"/>
-      <c r="J176" s="23" t="n"/>
-      <c r="K176" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L176" s="23" t="inlineStr"/>
-    </row>
-    <row r="177">
-      <c r="A177" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B177" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C177" s="23" t="inlineStr">
-        <is>
-          <t>Intercom</t>
-        </is>
-      </c>
-      <c r="D177" s="23" t="inlineStr">
-        <is>
-          <t>Senior Full Stack Engineer - Team Web</t>
-        </is>
-      </c>
-      <c r="E177" s="23" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/intercom/jobs/7276257</t>
-        </is>
-      </c>
-      <c r="F177" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G177" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H177" s="23" t="inlineStr">
-        <is>
-          <t>Loc: London, England</t>
-        </is>
-      </c>
-      <c r="I177" s="23" t="n"/>
-      <c r="J177" s="23" t="n"/>
-      <c r="K177" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L177" s="23" t="inlineStr"/>
-    </row>
-    <row r="178">
-      <c r="A178" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B178" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C178" s="23" t="inlineStr">
-        <is>
-          <t>Contentful</t>
-        </is>
-      </c>
-      <c r="D178" s="23" t="inlineStr">
-        <is>
-          <t>Fullstack Software Engineer (f/m/d)</t>
-        </is>
-      </c>
-      <c r="E178" s="23" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/contentful/jobs/7553930</t>
-        </is>
-      </c>
-      <c r="F178" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G178" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H178" s="23" t="inlineStr">
-        <is>
-          <t>Loc: London, England</t>
-        </is>
-      </c>
-      <c r="I178" s="23" t="n"/>
-      <c r="J178" s="23" t="n"/>
-      <c r="K178" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L178" s="23" t="inlineStr"/>
-    </row>
-    <row r="179">
-      <c r="A179" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B179" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C179" s="23" t="inlineStr">
-        <is>
-          <t>Contentful</t>
-        </is>
-      </c>
-      <c r="D179" s="23" t="inlineStr">
-        <is>
-          <t>Senior Backend Engineer - AI Platform (f/m/d)</t>
-        </is>
-      </c>
-      <c r="E179" s="23" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/contentful/jobs/7776562</t>
-        </is>
-      </c>
-      <c r="F179" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G179" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H179" s="23" t="inlineStr">
-        <is>
-          <t>Loc: London, England</t>
-        </is>
-      </c>
-      <c r="I179" s="23" t="n"/>
-      <c r="J179" s="23" t="n"/>
-      <c r="K179" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L179" s="23" t="inlineStr"/>
-    </row>
-    <row r="180">
-      <c r="A180" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B180" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C180" s="23" t="inlineStr">
-        <is>
-          <t>Contentful</t>
-        </is>
-      </c>
-      <c r="D180" s="23" t="inlineStr">
-        <is>
-          <t>Senior Software Engineer - Backend &amp; Infrastructure (f/m/d)</t>
-        </is>
-      </c>
-      <c r="E180" s="23" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/contentful/jobs/7760966</t>
-        </is>
-      </c>
-      <c r="F180" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G180" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H180" s="23" t="inlineStr">
-        <is>
-          <t>Loc: Berlin, Germany</t>
-        </is>
-      </c>
-      <c r="I180" s="23" t="n"/>
-      <c r="J180" s="23" t="n"/>
-      <c r="K180" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L180" s="23" t="inlineStr"/>
-    </row>
-    <row r="181">
-      <c r="A181" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B181" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C181" s="23" t="inlineStr">
-        <is>
-          <t>N26</t>
-        </is>
-      </c>
-      <c r="D181" s="23" t="inlineStr">
-        <is>
-          <t>Backend Engineer - Acquire</t>
-        </is>
-      </c>
-      <c r="E181" s="23" t="inlineStr">
-        <is>
-          <t>https://n26.com/en-eu/careers/positions/7742395?gh_jid=7742395</t>
-        </is>
-      </c>
-      <c r="F181" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G181" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H181" s="23" t="inlineStr">
-        <is>
-          <t>Loc: Berlin</t>
-        </is>
-      </c>
-      <c r="I181" s="23" t="n"/>
-      <c r="J181" s="23" t="n"/>
-      <c r="K181" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L181" s="23" t="inlineStr"/>
-    </row>
-    <row r="182">
-      <c r="A182" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B182" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C182" s="23" t="inlineStr">
-        <is>
-          <t>N26</t>
-        </is>
-      </c>
-      <c r="D182" s="23" t="inlineStr">
-        <is>
-          <t>Backend Engineer - Engagement</t>
-        </is>
-      </c>
-      <c r="E182" s="23" t="inlineStr">
-        <is>
-          <t>https://n26.com/en-eu/careers/positions/7640893?gh_jid=7640893</t>
-        </is>
-      </c>
-      <c r="F182" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G182" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H182" s="23" t="inlineStr">
-        <is>
-          <t>Loc: Berlin / Barcelona</t>
-        </is>
-      </c>
-      <c r="I182" s="23" t="n"/>
-      <c r="J182" s="23" t="n"/>
-      <c r="K182" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L182" s="23" t="inlineStr"/>
-    </row>
-    <row r="183">
-      <c r="A183" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B183" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C183" s="23" t="inlineStr">
-        <is>
-          <t>N26</t>
-        </is>
-      </c>
-      <c r="D183" s="23" t="inlineStr">
-        <is>
-          <t>Senior Full-Stack Security Automation Engineer</t>
-        </is>
-      </c>
-      <c r="E183" s="23" t="inlineStr">
-        <is>
-          <t>https://n26.com/en-eu/careers/positions/7597686?gh_jid=7597686</t>
-        </is>
-      </c>
-      <c r="F183" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G183" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H183" s="23" t="inlineStr">
-        <is>
-          <t>Loc: Barcelona</t>
-        </is>
-      </c>
-      <c r="I183" s="23" t="n"/>
-      <c r="J183" s="23" t="n"/>
-      <c r="K183" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L183" s="23" t="inlineStr"/>
-    </row>
-    <row r="184">
-      <c r="A184" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B184" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C184" s="23" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D184" s="23" t="inlineStr">
-        <is>
-          <t>Senior Backend Engineer - Accounts</t>
-        </is>
-      </c>
-      <c r="E184" s="23" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8418083002?gh_jid=8418083002</t>
-        </is>
-      </c>
-      <c r="F184" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G184" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H184" s="23" t="inlineStr">
-        <is>
-          <t>Loc: Berlin, Germany</t>
-        </is>
-      </c>
-      <c r="I184" s="23" t="n"/>
-      <c r="J184" s="23" t="n"/>
-      <c r="K184" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L184" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote)</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B185" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C185" s="23" t="inlineStr">
-        <is>
-          <t>SumUp</t>
-        </is>
-      </c>
-      <c r="D185" s="23" t="inlineStr">
-        <is>
-          <t>Senior Backend Engineer - Fiscalization</t>
-        </is>
-      </c>
-      <c r="E185" s="23" t="inlineStr">
-        <is>
-          <t>https://sumup.com/careers/positions/8321240002?gh_jid=8321240002</t>
-        </is>
-      </c>
-      <c r="F185" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G185" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H185" s="23" t="inlineStr">
-        <is>
-          <t>Loc: Berlin, Germany</t>
-        </is>
-      </c>
-      <c r="I185" s="23" t="n"/>
-      <c r="J185" s="23" t="n"/>
-      <c r="K185" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L185" s="23" t="inlineStr">
-        <is>
-          <t>Office-first (not remote)</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B186" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C186" s="23" t="inlineStr">
-        <is>
-          <t>Legora</t>
-        </is>
-      </c>
-      <c r="D186" s="23" t="inlineStr">
-        <is>
-          <t>Senior Backend Engineer</t>
-        </is>
-      </c>
-      <c r="E186" s="23" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/legora/b0dcbd44-38c5-46fc-aa9a-610fe881fc1c</t>
-        </is>
-      </c>
-      <c r="F186" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G186" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H186" s="23" t="inlineStr">
-        <is>
-          <t>Loc: Malmö</t>
-        </is>
-      </c>
-      <c r="I186" s="23" t="n"/>
-      <c r="J186" s="23" t="n"/>
-      <c r="K186" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L186" s="23" t="inlineStr"/>
-    </row>
-    <row r="187">
-      <c r="A187" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B187" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C187" s="23" t="inlineStr">
-        <is>
-          <t>Legora</t>
-        </is>
-      </c>
-      <c r="D187" s="23" t="inlineStr">
-        <is>
-          <t>Senior Software Engineer</t>
-        </is>
-      </c>
-      <c r="E187" s="23" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/legora/2ec4729a-82e2-4e7b-90d9-c9afb8e941bb</t>
-        </is>
-      </c>
-      <c r="F187" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G187" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H187" s="23" t="inlineStr">
-        <is>
-          <t>Loc: Stockholm HQ</t>
-        </is>
-      </c>
-      <c r="I187" s="23" t="n"/>
-      <c r="J187" s="23" t="n"/>
-      <c r="K187" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L187" s="23" t="inlineStr"/>
-    </row>
-    <row r="188">
-      <c r="A188" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B188" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C188" s="23" t="inlineStr">
-        <is>
-          <t>HelloFresh</t>
-        </is>
-      </c>
-      <c r="D188" s="23" t="inlineStr">
-        <is>
-          <t>React Native Developer, Growth</t>
-        </is>
-      </c>
-      <c r="E188" s="23" t="inlineStr">
-        <is>
-          <t>https://careers.hellofresh.com/global/en/job/7862406?gh_jid=7862406</t>
-        </is>
-      </c>
-      <c r="F188" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G188" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H188" s="23" t="inlineStr">
-        <is>
-          <t>Loc: Toronto, Ontario, Canada</t>
-        </is>
-      </c>
-      <c r="I188" s="23" t="n"/>
-      <c r="J188" s="23" t="n"/>
-      <c r="K188" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L188" s="23" t="inlineStr"/>
-    </row>
-    <row r="189">
-      <c r="A189" s="23">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B189" s="23" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C189" s="23" t="inlineStr">
-        <is>
-          <t>Pigment</t>
-        </is>
-      </c>
-      <c r="D189" s="23" t="inlineStr">
-        <is>
-          <t>Senior Backend Software Engineer</t>
-        </is>
-      </c>
-      <c r="E189" s="23" t="inlineStr">
-        <is>
-          <t>https://jobs.lever.co/pigment/bf7cacad-0f52-4db4-88d4-ad7b22bd852e</t>
-        </is>
-      </c>
-      <c r="F189" s="23" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G189" s="23" t="inlineStr">
-        <is>
-          <t>Visa sponsorship needed</t>
-        </is>
-      </c>
-      <c r="H189" s="23" t="inlineStr">
-        <is>
-          <t>Loc: France</t>
-        </is>
-      </c>
-      <c r="I189" s="23" t="n"/>
-      <c r="J189" s="23" t="n"/>
-      <c r="K189" s="23" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="L189" s="23" t="inlineStr"/>
+      <c r="L163" s="23" t="inlineStr"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="J2:J1000">
@@ -11031,43 +9725,23 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E137" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E138" r:id="rId98"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E139" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E140" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E141" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E142" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E143" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E144" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E145" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E146" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E147" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E148" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E149" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E158" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E159" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E160" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E161" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E162" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E163" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E164" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E165" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E166" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E167" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E168" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E169" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E170" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E171" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E172" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E173" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E174" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E175" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E176" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E177" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E178" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E179" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E180" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E181" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E182" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E183" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E184" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E141" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E142" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E143" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E144" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E145" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E146" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E147" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E148" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E149" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E176" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E177" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E178" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E179" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E180" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E181" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E182" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E183" r:id="rId116"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Recommended status to Wishlist Decision dropdown
New non-destructive flag the agent uses to surface strong candidates
("look at this first") after a scan. Distinct from Apply (committed),
Saved (bookmarked), and Skip (auto-deletes). Gold color #ffe082 in
the web editor.

Marked as Recommended after the gittap/remote3/cryptocurrencyjobs
scan: GitTap Senior Fullstack (r155), Penguin Finance (r157), Grove
Labs (r161).

Decision dropdown now: Pending, Recommended, Apply, Skip, Saved.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -1167,7 +1167,6 @@
     <mergeCell ref="A27:D27"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A32:D32"/>
     <mergeCell ref="A20:D20"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="A26:D26"/>
@@ -1179,6 +1178,7 @@
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A28:D28"/>
     <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A32:D32"/>
     <mergeCell ref="B7:D7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8597,7 +8597,7 @@
       <c r="J155" s="25" t="n"/>
       <c r="K155" s="25" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Recommended</t>
         </is>
       </c>
       <c r="L155" s="25" t="inlineStr"/>
@@ -8695,7 +8695,7 @@
       <c r="J157" s="25" t="n"/>
       <c r="K157" s="25" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Recommended</t>
         </is>
       </c>
       <c r="L157" s="25" t="inlineStr"/>
@@ -8891,7 +8891,7 @@
       <c r="J161" s="25" t="n"/>
       <c r="K161" s="25" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Recommended</t>
         </is>
       </c>
       <c r="L161" s="25" t="inlineStr"/>
@@ -9075,18 +9075,12 @@
       <formula>5</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
-    <dataValidation sqref="I10:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"1,2,3,4,5"</formula1>
-    </dataValidation>
+  <dataValidations count="2">
     <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
-    <dataValidation sqref="K10:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Pending,Apply,Skip,Saved"</formula1>
-    </dataValidation>
     <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Pending,Apply,Skip,Saved"</formula1>
+      <formula1>"Pending,Recommended,Apply,Skip,Saved"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>

</xml_diff>

<commit_message>
Prefix Wishlist Decision values with priority numbers
Sorting Decision alphabetically previously gave Apply→Pending→
Recommended→Saved→Skip — not the natural priority order. Renaming
to "1. Apply", "2. Recommended", "3. Saved", "4. Pending", "5. Skip"
so alphabetical sort = priority sort and the user can lean on the
column-sort feature directly.

- xlsx data validation list updated
- 143 existing Decision cells rewritten to prefixed form
- DROPDOWN_COLORS in docs/app.js keyed by new strings
- WISHLIST_DELETE_ON_SAVE updated to "5. Skip"

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -1542,7 +1542,7 @@
       <c r="J2" s="11" t="n"/>
       <c r="K2" s="11" t="inlineStr">
         <is>
-          <t>Apply</t>
+          <t>1. Apply</t>
         </is>
       </c>
       <c r="L2" s="11" t="inlineStr">
@@ -1593,7 +1593,7 @@
       <c r="J3" s="1" t="n"/>
       <c r="K3" s="1" t="inlineStr">
         <is>
-          <t>Apply</t>
+          <t>1. Apply</t>
         </is>
       </c>
       <c r="L3" s="1" t="inlineStr">
@@ -1644,7 +1644,7 @@
       <c r="J4" s="1" t="n"/>
       <c r="K4" s="1" t="inlineStr">
         <is>
-          <t>Apply</t>
+          <t>1. Apply</t>
         </is>
       </c>
       <c r="L4" s="1" t="inlineStr">
@@ -1695,7 +1695,7 @@
       <c r="J5" s="1" t="n"/>
       <c r="K5" s="1" t="inlineStr">
         <is>
-          <t>Apply</t>
+          <t>1. Apply</t>
         </is>
       </c>
       <c r="L5" s="1" t="inlineStr">
@@ -1746,7 +1746,7 @@
       <c r="J6" s="1" t="n"/>
       <c r="K6" s="1" t="inlineStr">
         <is>
-          <t>Saved</t>
+          <t>3. Saved</t>
         </is>
       </c>
       <c r="L6" s="1" t="inlineStr">
@@ -1797,7 +1797,7 @@
       <c r="J7" s="1" t="n"/>
       <c r="K7" s="1" t="inlineStr">
         <is>
-          <t>Saved</t>
+          <t>3. Saved</t>
         </is>
       </c>
       <c r="L7" s="1" t="inlineStr">
@@ -1848,7 +1848,7 @@
       <c r="J8" s="1" t="n"/>
       <c r="K8" s="1" t="inlineStr">
         <is>
-          <t>Saved</t>
+          <t>3. Saved</t>
         </is>
       </c>
       <c r="L8" s="1" t="inlineStr">
@@ -1899,7 +1899,7 @@
       <c r="J9" s="11" t="n"/>
       <c r="K9" s="14" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L9" s="14" t="inlineStr">
@@ -1950,7 +1950,7 @@
       <c r="J10" s="17" t="n"/>
       <c r="K10" s="15" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L10" s="15" t="inlineStr">
@@ -2001,7 +2001,7 @@
       <c r="J11" s="17" t="n"/>
       <c r="K11" s="15" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L11" s="15" t="inlineStr">
@@ -2052,7 +2052,7 @@
       <c r="J12" s="1" t="n"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -2103,7 +2103,7 @@
       <c r="J13" s="1" t="n"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -2154,7 +2154,7 @@
       <c r="J14" s="1" t="n"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -2205,7 +2205,7 @@
       <c r="J15" s="1" t="n"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -2256,7 +2256,7 @@
       <c r="J16" s="1" t="n"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -2307,7 +2307,7 @@
       <c r="J17" s="1" t="n"/>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -2358,7 +2358,7 @@
       <c r="J18" s="1" t="n"/>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -2409,7 +2409,7 @@
       <c r="J19" s="1" t="n"/>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -2460,7 +2460,7 @@
       <c r="J20" s="1" t="n"/>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2511,7 +2511,7 @@
       <c r="J21" s="1" t="n"/>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2562,7 +2562,7 @@
       <c r="J22" s="1" t="n"/>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -2613,7 +2613,7 @@
       <c r="J23" s="1" t="n"/>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
@@ -2664,7 +2664,7 @@
       <c r="J24" s="1" t="n"/>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -2715,7 +2715,7 @@
       <c r="J25" s="1" t="n"/>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -2766,7 +2766,7 @@
       <c r="J26" s="1" t="n"/>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -2817,7 +2817,7 @@
       <c r="J27" s="1" t="n"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -2868,7 +2868,7 @@
       <c r="J28" s="1" t="n"/>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -2919,7 +2919,7 @@
       <c r="J29" s="1" t="n"/>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -2970,7 +2970,7 @@
       <c r="J30" s="1" t="n"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -3021,7 +3021,7 @@
       <c r="J31" s="1" t="n"/>
       <c r="K31" s="18" t="inlineStr">
         <is>
-          <t>Apply</t>
+          <t>1. Apply</t>
         </is>
       </c>
       <c r="L31" s="18" t="inlineStr">
@@ -3072,7 +3072,7 @@
       <c r="J32" s="1" t="n"/>
       <c r="K32" s="18" t="inlineStr">
         <is>
-          <t>Apply</t>
+          <t>1. Apply</t>
         </is>
       </c>
       <c r="L32" s="18" t="inlineStr">
@@ -3123,7 +3123,7 @@
       <c r="J33" s="1" t="n"/>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -3174,7 +3174,7 @@
       <c r="J34" s="1" t="n"/>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -3225,7 +3225,7 @@
       <c r="J35" s="1" t="n"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -3276,7 +3276,7 @@
       <c r="J36" s="1" t="n"/>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -3327,7 +3327,7 @@
       <c r="J37" s="1" t="n"/>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -3378,7 +3378,7 @@
       <c r="J38" s="1" t="n"/>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -3429,7 +3429,7 @@
       <c r="J39" s="1" t="n"/>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -3480,7 +3480,7 @@
       <c r="J40" s="1" t="n"/>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -3531,7 +3531,7 @@
       <c r="J41" s="1" t="n"/>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -3582,7 +3582,7 @@
       <c r="J42" s="1" t="n"/>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -3633,7 +3633,7 @@
       <c r="J43" s="1" t="n"/>
       <c r="K43" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
@@ -3684,7 +3684,7 @@
       <c r="J44" s="1" t="n"/>
       <c r="K44" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -3735,7 +3735,7 @@
       <c r="J45" s="1" t="n"/>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
@@ -3786,7 +3786,7 @@
       <c r="J46" s="1" t="n"/>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -3837,7 +3837,7 @@
       <c r="J47" s="1" t="n"/>
       <c r="K47" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -3888,7 +3888,7 @@
       <c r="J48" s="1" t="n"/>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
@@ -3939,7 +3939,7 @@
       <c r="J49" s="1" t="n"/>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -3990,7 +3990,7 @@
       <c r="J50" s="1" t="n"/>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -4041,7 +4041,7 @@
       <c r="J51" s="1" t="n"/>
       <c r="K51" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
@@ -4092,7 +4092,7 @@
       <c r="J52" s="1" t="n"/>
       <c r="K52" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -4143,7 +4143,7 @@
       <c r="J53" s="1" t="n"/>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
@@ -4194,7 +4194,7 @@
       <c r="J54" s="1" t="n"/>
       <c r="K54" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
@@ -4245,7 +4245,7 @@
       <c r="J55" s="1" t="n"/>
       <c r="K55" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
@@ -4296,7 +4296,7 @@
       <c r="J56" s="1" t="n"/>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
@@ -4347,7 +4347,7 @@
       <c r="J57" s="1" t="n"/>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
@@ -4398,7 +4398,7 @@
       <c r="J58" s="1" t="n"/>
       <c r="K58" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
@@ -4449,7 +4449,7 @@
       <c r="J59" s="1" t="n"/>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
@@ -4500,7 +4500,7 @@
       <c r="J60" s="1" t="n"/>
       <c r="K60" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
@@ -4551,7 +4551,7 @@
       <c r="J61" s="1" t="n"/>
       <c r="K61" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
@@ -4602,7 +4602,7 @@
       <c r="J62" s="1" t="n"/>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
@@ -4653,7 +4653,7 @@
       <c r="J63" s="1" t="n"/>
       <c r="K63" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
@@ -4704,7 +4704,7 @@
       <c r="J64" s="1" t="n"/>
       <c r="K64" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
@@ -4755,7 +4755,7 @@
       <c r="J65" s="1" t="n"/>
       <c r="K65" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
@@ -4806,7 +4806,7 @@
       <c r="J66" s="1" t="n"/>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
@@ -4857,7 +4857,7 @@
       <c r="J67" s="1" t="n"/>
       <c r="K67" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
@@ -4908,7 +4908,7 @@
       <c r="J68" s="1" t="n"/>
       <c r="K68" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
@@ -4959,7 +4959,7 @@
       <c r="J69" s="1" t="n"/>
       <c r="K69" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
@@ -5010,7 +5010,7 @@
       <c r="J70" s="1" t="n"/>
       <c r="K70" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
@@ -5061,7 +5061,7 @@
       <c r="J71" s="1" t="n"/>
       <c r="K71" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
@@ -5112,7 +5112,7 @@
       <c r="J72" s="1" t="n"/>
       <c r="K72" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
@@ -5163,7 +5163,7 @@
       <c r="J73" s="1" t="n"/>
       <c r="K73" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
@@ -5214,7 +5214,7 @@
       <c r="J74" s="1" t="n"/>
       <c r="K74" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
@@ -5265,7 +5265,7 @@
       <c r="J75" s="1" t="n"/>
       <c r="K75" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
@@ -5316,7 +5316,7 @@
       <c r="J76" s="1" t="n"/>
       <c r="K76" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
@@ -5367,7 +5367,7 @@
       <c r="J77" s="1" t="n"/>
       <c r="K77" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
@@ -5418,7 +5418,7 @@
       <c r="J78" s="1" t="n"/>
       <c r="K78" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
@@ -5469,7 +5469,7 @@
       <c r="J79" s="1" t="n"/>
       <c r="K79" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
@@ -5520,7 +5520,7 @@
       <c r="J80" s="1" t="n"/>
       <c r="K80" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
@@ -5571,7 +5571,7 @@
       <c r="J81" s="1" t="n"/>
       <c r="K81" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
@@ -5622,7 +5622,7 @@
       <c r="J82" s="1" t="n"/>
       <c r="K82" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
@@ -5673,7 +5673,7 @@
       <c r="J83" s="1" t="n"/>
       <c r="K83" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
@@ -5724,7 +5724,7 @@
       <c r="J84" s="1" t="n"/>
       <c r="K84" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
@@ -5775,7 +5775,7 @@
       <c r="J85" s="1" t="n"/>
       <c r="K85" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
@@ -5826,7 +5826,7 @@
       <c r="J86" s="1" t="n"/>
       <c r="K86" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
@@ -5877,7 +5877,7 @@
       <c r="J87" s="1" t="n"/>
       <c r="K87" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
@@ -5928,7 +5928,7 @@
       <c r="J88" s="1" t="n"/>
       <c r="K88" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
@@ -5979,7 +5979,7 @@
       <c r="J89" s="1" t="n"/>
       <c r="K89" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
@@ -6030,7 +6030,7 @@
       <c r="J90" s="1" t="n"/>
       <c r="K90" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
@@ -6081,7 +6081,7 @@
       <c r="J91" s="1" t="n"/>
       <c r="K91" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
@@ -6132,7 +6132,7 @@
       <c r="J92" s="1" t="n"/>
       <c r="K92" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
@@ -6183,7 +6183,7 @@
       <c r="J93" s="1" t="n"/>
       <c r="K93" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
@@ -6234,7 +6234,7 @@
       <c r="J94" s="1" t="n"/>
       <c r="K94" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
@@ -6285,7 +6285,7 @@
       <c r="J95" s="1" t="n"/>
       <c r="K95" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
@@ -6336,7 +6336,7 @@
       <c r="J96" s="1" t="n"/>
       <c r="K96" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L96" t="inlineStr">
@@ -6387,7 +6387,7 @@
       <c r="J97" s="1" t="n"/>
       <c r="K97" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
@@ -6438,7 +6438,7 @@
       <c r="J98" s="1" t="n"/>
       <c r="K98" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -6489,7 +6489,7 @@
       <c r="J99" s="1" t="n"/>
       <c r="K99" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -6540,7 +6540,7 @@
       <c r="J100" s="1" t="n"/>
       <c r="K100" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
@@ -6591,7 +6591,7 @@
       <c r="J101" s="1" t="n"/>
       <c r="K101" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
@@ -6642,7 +6642,7 @@
       <c r="J102" s="1" t="n"/>
       <c r="K102" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
@@ -6693,7 +6693,7 @@
       <c r="J103" s="1" t="n"/>
       <c r="K103" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -6744,7 +6744,7 @@
       <c r="J104" s="1" t="n"/>
       <c r="K104" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
@@ -6795,7 +6795,7 @@
       <c r="J105" s="1" t="n"/>
       <c r="K105" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
@@ -6846,7 +6846,7 @@
       <c r="J106" s="1" t="n"/>
       <c r="K106" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L106" t="inlineStr">
@@ -6897,7 +6897,7 @@
       <c r="J107" s="1" t="n"/>
       <c r="K107" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -6948,7 +6948,7 @@
       <c r="J108" s="1" t="n"/>
       <c r="K108" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
@@ -6999,7 +6999,7 @@
       <c r="J109" s="1" t="n"/>
       <c r="K109" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -7050,7 +7050,7 @@
       <c r="J110" s="1" t="n"/>
       <c r="K110" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L110" t="inlineStr">
@@ -7101,7 +7101,7 @@
       <c r="J111" s="1" t="n"/>
       <c r="K111" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
@@ -7152,7 +7152,7 @@
       <c r="J112" s="1" t="n"/>
       <c r="K112" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
@@ -7203,7 +7203,7 @@
       <c r="J113" s="1" t="n"/>
       <c r="K113" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L113" t="inlineStr">
@@ -7254,7 +7254,7 @@
       <c r="J114" s="1" t="n"/>
       <c r="K114" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
@@ -7305,7 +7305,7 @@
       <c r="J115" s="1" t="n"/>
       <c r="K115" s="18" t="inlineStr">
         <is>
-          <t>Apply</t>
+          <t>1. Apply</t>
         </is>
       </c>
       <c r="L115" s="18" t="inlineStr">
@@ -7356,7 +7356,7 @@
       <c r="J116" s="1" t="n"/>
       <c r="K116" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L116" t="inlineStr">
@@ -7407,7 +7407,7 @@
       <c r="J117" s="1" t="n"/>
       <c r="K117" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L117" t="inlineStr">
@@ -7458,7 +7458,7 @@
       <c r="J118" s="1" t="n"/>
       <c r="K118" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L118" t="inlineStr">
@@ -7509,7 +7509,7 @@
       <c r="J119" s="1" t="n"/>
       <c r="K119" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L119" t="inlineStr">
@@ -7560,7 +7560,7 @@
       <c r="J120" s="1" t="n"/>
       <c r="K120" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L120" t="inlineStr">
@@ -7611,7 +7611,7 @@
       <c r="J121" s="1" t="n"/>
       <c r="K121" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
@@ -7662,7 +7662,7 @@
       <c r="J122" s="1" t="n"/>
       <c r="K122" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L122" t="inlineStr">
@@ -7713,7 +7713,7 @@
       <c r="J123" s="1" t="n"/>
       <c r="K123" t="inlineStr">
         <is>
-          <t>Apply</t>
+          <t>1. Apply</t>
         </is>
       </c>
       <c r="L123" t="inlineStr">
@@ -7766,7 +7766,7 @@
       <c r="J124" s="20" t="n"/>
       <c r="K124" s="20" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L124" s="20" t="n"/>
@@ -7815,7 +7815,7 @@
       <c r="J125" s="20" t="n"/>
       <c r="K125" s="20" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L125" s="20" t="n"/>
@@ -7864,7 +7864,7 @@
       <c r="J126" s="20" t="n"/>
       <c r="K126" s="20" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L126" s="20" t="n"/>
@@ -7913,7 +7913,7 @@
       <c r="J127" s="20" t="n"/>
       <c r="K127" s="20" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L127" s="20" t="n"/>
@@ -7962,7 +7962,7 @@
       <c r="J128" s="20" t="n"/>
       <c r="K128" s="20" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L128" s="20" t="n"/>
@@ -8011,7 +8011,7 @@
       <c r="J129" s="20" t="n"/>
       <c r="K129" s="20" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L129" s="20" t="n"/>
@@ -8060,7 +8060,7 @@
       <c r="J130" s="20" t="n"/>
       <c r="K130" s="20" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L130" s="20" t="n"/>
@@ -8109,7 +8109,7 @@
       <c r="J131" s="20" t="n"/>
       <c r="K131" s="20" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L131" s="20" t="n"/>
@@ -8158,7 +8158,7 @@
       <c r="J132" s="20" t="n"/>
       <c r="K132" s="20" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L132" s="20" t="n"/>
@@ -8207,7 +8207,7 @@
       <c r="J133" s="20" t="n"/>
       <c r="K133" s="20" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L133" s="20" t="n"/>
@@ -8256,7 +8256,7 @@
       <c r="J134" s="20" t="n"/>
       <c r="K134" s="20" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L134" s="20" t="n"/>
@@ -8597,7 +8597,7 @@
       <c r="J155" s="25" t="n"/>
       <c r="K155" s="25" t="inlineStr">
         <is>
-          <t>Recommended</t>
+          <t>2. Recommended</t>
         </is>
       </c>
       <c r="L155" s="25" t="inlineStr"/>
@@ -8646,7 +8646,7 @@
       <c r="J156" s="25" t="n"/>
       <c r="K156" s="25" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L156" s="25" t="inlineStr"/>
@@ -8695,7 +8695,7 @@
       <c r="J157" s="25" t="n"/>
       <c r="K157" s="25" t="inlineStr">
         <is>
-          <t>Recommended</t>
+          <t>2. Recommended</t>
         </is>
       </c>
       <c r="L157" s="25" t="inlineStr"/>
@@ -8744,7 +8744,7 @@
       <c r="J158" s="25" t="n"/>
       <c r="K158" s="25" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L158" s="25" t="inlineStr"/>
@@ -8793,7 +8793,7 @@
       <c r="J159" s="25" t="n"/>
       <c r="K159" s="25" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L159" s="25" t="inlineStr"/>
@@ -8842,7 +8842,7 @@
       <c r="J160" s="25" t="n"/>
       <c r="K160" s="25" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L160" s="25" t="inlineStr"/>
@@ -8891,7 +8891,7 @@
       <c r="J161" s="25" t="n"/>
       <c r="K161" s="25" t="inlineStr">
         <is>
-          <t>Recommended</t>
+          <t>2. Recommended</t>
         </is>
       </c>
       <c r="L161" s="25" t="inlineStr"/>
@@ -8940,7 +8940,7 @@
       <c r="J162" s="25" t="n"/>
       <c r="K162" s="25" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L162" s="25" t="inlineStr"/>
@@ -8989,7 +8989,7 @@
       <c r="J163" s="25" t="n"/>
       <c r="K163" s="25" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L163" s="25" t="inlineStr"/>
@@ -9038,7 +9038,7 @@
       <c r="J164" s="25" t="n"/>
       <c r="K164" s="25" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>4. Pending</t>
         </is>
       </c>
       <c r="L164" s="25" t="inlineStr"/>
@@ -9080,7 +9080,7 @@
       <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
     <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Pending,Recommended,Apply,Skip,Saved"</formula1>
+      <formula1>"1. Apply,2. Recommended,3. Saved,4. Pending,5. Skip"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>

</xml_diff>

<commit_message>
Drop stale remote3 + cryptocurrencyjobs rows; fix GitTap employer names
Sampled the 8 rows added in 587c2b7 against the live JD pages:

- remote3.co (4 rows, all removed): listings dated 2021-2023; the
  aggregator never expires closed posts. Penguin Finance Nov 2021,
  prePO Nov 2021, Upside Mar 2022, Scroll Jan 2023.
- cryptocurrencyjobs.co (4 rows, all removed): all 4 returned
  "Looks like this career opportunity is no longer available" on
  the JD page despite still ranking in search.
- gittap.jp (2 rows kept): appear current with active Apply
  controls. Updated Company column from the placeholder
  "GitTap (Japan)" to the real employers — Shippio (r155) and
  ReNK CHANNEL (r156) — pulled from the JD pages.

Both stale aggregators set to enabled: false in portals.yml
(gitignored). Memory rule added: sample posting dates before
mass-adding from any new source.

Wishlist down to 156 rows.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -1422,7 +1422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L164"/>
+  <dimension ref="A1:L156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="1" min="1" max="1"/>
@@ -8565,7 +8565,7 @@
       </c>
       <c r="C155" s="25" t="inlineStr">
         <is>
-          <t>GitTap (Japan)</t>
+          <t>Shippio</t>
         </is>
       </c>
       <c r="D155" s="25" t="inlineStr">
@@ -8600,7 +8600,11 @@
           <t>2. Recommended</t>
         </is>
       </c>
-      <c r="L155" s="25" t="inlineStr"/>
+      <c r="L155" s="25" t="inlineStr">
+        <is>
+          <t>(via GitTap)</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="25">
@@ -8614,7 +8618,7 @@
       </c>
       <c r="C156" s="25" t="inlineStr">
         <is>
-          <t>GitTap (Japan)</t>
+          <t>ReNK CHANNEL</t>
         </is>
       </c>
       <c r="D156" s="25" t="inlineStr">
@@ -8649,399 +8653,11 @@
           <t>4. Pending</t>
         </is>
       </c>
-      <c r="L156" s="25" t="inlineStr"/>
-    </row>
-    <row r="157">
-      <c r="A157" s="25">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B157" s="25" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C157" s="25" t="inlineStr">
-        <is>
-          <t>Penguin Finance</t>
-        </is>
-      </c>
-      <c r="D157" s="25" t="inlineStr">
-        <is>
-          <t>Senior Full Stack Developer</t>
-        </is>
-      </c>
-      <c r="E157" s="25" t="inlineStr">
-        <is>
-          <t>https://www.remote3.co/remote-jobs/senior-full-stack-developer</t>
-        </is>
-      </c>
-      <c r="F157" s="25" t="inlineStr">
-        <is>
-          <t>career-ops scan / remote3.co</t>
-        </is>
-      </c>
-      <c r="G157" s="25" t="inlineStr">
-        <is>
-          <t>Remote — worldwide</t>
-        </is>
-      </c>
-      <c r="H157" s="25" t="inlineStr">
-        <is>
-          <t>React + Solidity + Web3.js — strong stack overlap</t>
-        </is>
-      </c>
-      <c r="I157" s="25" t="n"/>
-      <c r="J157" s="25" t="n"/>
-      <c r="K157" s="25" t="inlineStr">
-        <is>
-          <t>2. Recommended</t>
-        </is>
-      </c>
-      <c r="L157" s="25" t="inlineStr"/>
-    </row>
-    <row r="158">
-      <c r="A158" s="25">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B158" s="25" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C158" s="25" t="inlineStr">
-        <is>
-          <t>prePO</t>
-        </is>
-      </c>
-      <c r="D158" s="25" t="inlineStr">
-        <is>
-          <t>Senior Solidity Smart Contract Engineer</t>
-        </is>
-      </c>
-      <c r="E158" s="25" t="inlineStr">
-        <is>
-          <t>https://www.remote3.co/remote-jobs/senior-solidity-smart-contract-engineer</t>
-        </is>
-      </c>
-      <c r="F158" s="25" t="inlineStr">
-        <is>
-          <t>career-ops scan / remote3.co</t>
-        </is>
-      </c>
-      <c r="G158" s="25" t="inlineStr">
-        <is>
-          <t>Remote — worldwide</t>
-        </is>
-      </c>
-      <c r="H158" s="25" t="inlineStr">
-        <is>
-          <t>Solidity-heavy SC engineering</t>
-        </is>
-      </c>
-      <c r="I158" s="25" t="n"/>
-      <c r="J158" s="25" t="n"/>
-      <c r="K158" s="25" t="inlineStr">
-        <is>
-          <t>4. Pending</t>
-        </is>
-      </c>
-      <c r="L158" s="25" t="inlineStr"/>
-    </row>
-    <row r="159">
-      <c r="A159" s="25">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B159" s="25" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C159" s="25" t="inlineStr">
-        <is>
-          <t>Upside</t>
-        </is>
-      </c>
-      <c r="D159" s="25" t="inlineStr">
-        <is>
-          <t>Senior Solidity Developer</t>
-        </is>
-      </c>
-      <c r="E159" s="25" t="inlineStr">
-        <is>
-          <t>https://www.remote3.co/remote-jobs/senior-solidity-developer-upside</t>
-        </is>
-      </c>
-      <c r="F159" s="25" t="inlineStr">
-        <is>
-          <t>career-ops scan / remote3.co</t>
-        </is>
-      </c>
-      <c r="G159" s="25" t="inlineStr">
-        <is>
-          <t>Remote — worldwide</t>
-        </is>
-      </c>
-      <c r="H159" s="25" t="inlineStr">
-        <is>
-          <t>Multi-chain (ETH/SOL/AVAX/Polygon) protocol dev</t>
-        </is>
-      </c>
-      <c r="I159" s="25" t="n"/>
-      <c r="J159" s="25" t="n"/>
-      <c r="K159" s="25" t="inlineStr">
-        <is>
-          <t>4. Pending</t>
-        </is>
-      </c>
-      <c r="L159" s="25" t="inlineStr"/>
-    </row>
-    <row r="160">
-      <c r="A160" s="25">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B160" s="25" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C160" s="25" t="inlineStr">
-        <is>
-          <t>Scroll</t>
-        </is>
-      </c>
-      <c r="D160" s="25" t="inlineStr">
-        <is>
-          <t>Senior Smart Contract Engineer</t>
-        </is>
-      </c>
-      <c r="E160" s="25" t="inlineStr">
-        <is>
-          <t>https://www.remote3.co/remote-jobs/senior-smart-contract-engineer-scroll</t>
-        </is>
-      </c>
-      <c r="F160" s="25" t="inlineStr">
-        <is>
-          <t>career-ops scan / remote3.co</t>
-        </is>
-      </c>
-      <c r="G160" s="25" t="inlineStr">
-        <is>
-          <t>Remote — worldwide</t>
-        </is>
-      </c>
-      <c r="H160" s="25" t="inlineStr">
-        <is>
-          <t>zkRollup L2 — well-funded, Solidity</t>
-        </is>
-      </c>
-      <c r="I160" s="25" t="n"/>
-      <c r="J160" s="25" t="n"/>
-      <c r="K160" s="25" t="inlineStr">
-        <is>
-          <t>4. Pending</t>
-        </is>
-      </c>
-      <c r="L160" s="25" t="inlineStr"/>
-    </row>
-    <row r="161">
-      <c r="A161" s="25">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B161" s="25" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C161" s="25" t="inlineStr">
-        <is>
-          <t>Grove Labs</t>
-        </is>
-      </c>
-      <c r="D161" s="25" t="inlineStr">
-        <is>
-          <t>Senior Full Stack Engineer</t>
-        </is>
-      </c>
-      <c r="E161" s="25" t="inlineStr">
-        <is>
-          <t>https://cryptocurrencyjobs.co/engineering/grove-labs-senior-full-stack-engineer/</t>
-        </is>
-      </c>
-      <c r="F161" s="25" t="inlineStr">
-        <is>
-          <t>career-ops scan / cryptocurrencyjobs.co</t>
-        </is>
-      </c>
-      <c r="G161" s="25" t="inlineStr">
-        <is>
-          <t>Remote — worldwide</t>
-        </is>
-      </c>
-      <c r="H161" s="25" t="inlineStr">
-        <is>
-          <t>Node.js/Python backend; Go is "or similar", not required</t>
-        </is>
-      </c>
-      <c r="I161" s="25" t="n"/>
-      <c r="J161" s="25" t="n"/>
-      <c r="K161" s="25" t="inlineStr">
-        <is>
-          <t>2. Recommended</t>
-        </is>
-      </c>
-      <c r="L161" s="25" t="inlineStr"/>
-    </row>
-    <row r="162">
-      <c r="A162" s="25">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B162" s="25" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C162" s="25" t="inlineStr">
-        <is>
-          <t>Silent Protocol</t>
-        </is>
-      </c>
-      <c r="D162" s="25" t="inlineStr">
-        <is>
-          <t>Full Stack Engineer - Backend Focused (Smart Contract)</t>
-        </is>
-      </c>
-      <c r="E162" s="25" t="inlineStr">
-        <is>
-          <t>https://cryptocurrencyjobs.co/engineering/silent-protocol-full-stack-engineer-backend-focused-smart-contract/</t>
-        </is>
-      </c>
-      <c r="F162" s="25" t="inlineStr">
-        <is>
-          <t>career-ops scan / cryptocurrencyjobs.co</t>
-        </is>
-      </c>
-      <c r="G162" s="25" t="inlineStr">
-        <is>
-          <t>Remote — worldwide</t>
-        </is>
-      </c>
-      <c r="H162" s="25" t="inlineStr">
-        <is>
-          <t>Backend + zk-snarks + Solidity protocol design</t>
-        </is>
-      </c>
-      <c r="I162" s="25" t="n"/>
-      <c r="J162" s="25" t="n"/>
-      <c r="K162" s="25" t="inlineStr">
-        <is>
-          <t>4. Pending</t>
-        </is>
-      </c>
-      <c r="L162" s="25" t="inlineStr"/>
-    </row>
-    <row r="163">
-      <c r="A163" s="25">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B163" s="25" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C163" s="25" t="inlineStr">
-        <is>
-          <t>PayBolt</t>
-        </is>
-      </c>
-      <c r="D163" s="25" t="inlineStr">
-        <is>
-          <t>Fullstack Blockchain Developer (Solidity)</t>
-        </is>
-      </c>
-      <c r="E163" s="25" t="inlineStr">
-        <is>
-          <t>https://cryptocurrencyjobs.co/engineering/paybolt-fullstack-blockchain-developer-solidity/</t>
-        </is>
-      </c>
-      <c r="F163" s="25" t="inlineStr">
-        <is>
-          <t>career-ops scan / cryptocurrencyjobs.co</t>
-        </is>
-      </c>
-      <c r="G163" s="25" t="inlineStr">
-        <is>
-          <t>Remote — worldwide</t>
-        </is>
-      </c>
-      <c r="H163" s="25" t="inlineStr">
-        <is>
-          <t>Payment plugins + ecommerce angle, Solidity</t>
-        </is>
-      </c>
-      <c r="I163" s="25" t="n"/>
-      <c r="J163" s="25" t="n"/>
-      <c r="K163" s="25" t="inlineStr">
-        <is>
-          <t>4. Pending</t>
-        </is>
-      </c>
-      <c r="L163" s="25" t="inlineStr"/>
-    </row>
-    <row r="164">
-      <c r="A164" s="25">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B164" s="25" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C164" s="25" t="inlineStr">
-        <is>
-          <t>Solidity Labs</t>
-        </is>
-      </c>
-      <c r="D164" s="25" t="inlineStr">
-        <is>
-          <t>Senior Smart Contract Engineer</t>
-        </is>
-      </c>
-      <c r="E164" s="25" t="inlineStr">
-        <is>
-          <t>https://cryptocurrencyjobs.co/engineering/solidity-labs-senior-smart-contract-engineer/</t>
-        </is>
-      </c>
-      <c r="F164" s="25" t="inlineStr">
-        <is>
-          <t>career-ops scan / cryptocurrencyjobs.co</t>
-        </is>
-      </c>
-      <c r="G164" s="25" t="inlineStr">
-        <is>
-          <t>Remote — worldwide</t>
-        </is>
-      </c>
-      <c r="H164" s="25" t="inlineStr">
-        <is>
-          <t>5+ yr Solidity, dedicated SC shop</t>
-        </is>
-      </c>
-      <c r="I164" s="25" t="n"/>
-      <c r="J164" s="25" t="n"/>
-      <c r="K164" s="25" t="inlineStr">
-        <is>
-          <t>4. Pending</t>
-        </is>
-      </c>
-      <c r="L164" s="25" t="inlineStr"/>
+      <c r="L156" s="25" t="inlineStr">
+        <is>
+          <t>(via GitTap)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="J2:J1000">

</xml_diff>

<commit_message>
Add stakefish Web3/Fullstack as ideal-fit anchor
User flagged this LinkedIn role as the shape of role they want:
React + TypeScript + Python + web3.js/ethers.js + AWS/Docker,
mid-senior IC, Singapore HQ (GMT+8) with distributed/remote
culture, $140-180K USD base.

- Wishlist row added (r157) with Decision = "2. Recommended",
  Fit Score 5
- Memory: project_ideal_role_shape.md captures the 6 fit signals
  (stack, domain, title, geo, culture, comp) so future scans
  prioritize roles that match this shape

Companies to mine for similar: Figment, Chorus One, Kiln, P2P,
Phantom, Rabby, Zerion, Alchemy, QuickNode etc. — Web3 infra hiring
fullstack/backend (not just Solidity specialists).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -1422,7 +1422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L156"/>
+  <dimension ref="A1:L157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="1" min="1" max="1"/>
@@ -8656,6 +8656,61 @@
       <c r="L156" s="25" t="inlineStr">
         <is>
           <t>(via GitTap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="25">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B157" s="25" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C157" s="25" t="inlineStr">
+        <is>
+          <t>stakefish</t>
+        </is>
+      </c>
+      <c r="D157" s="25" t="inlineStr">
+        <is>
+          <t>Web3 / Full-stack Software Engineer</t>
+        </is>
+      </c>
+      <c r="E157" s="25" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4354681451/</t>
+        </is>
+      </c>
+      <c r="F157" s="25" t="inlineStr">
+        <is>
+          <t>user-submitted (LinkedIn)</t>
+        </is>
+      </c>
+      <c r="G157" s="25" t="inlineStr">
+        <is>
+          <t>Remote — worldwide (Singapore HQ, GMT+8)</t>
+        </is>
+      </c>
+      <c r="H157" s="25" t="inlineStr">
+        <is>
+          <t>React+TS+Python+web3.js, mid-senior IC, distributed culture, $140-180K</t>
+        </is>
+      </c>
+      <c r="I157" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="J157" s="25" t="n"/>
+      <c r="K157" s="25" t="inlineStr">
+        <is>
+          <t>2. Recommended</t>
+        </is>
+      </c>
+      <c r="L157" s="25" t="inlineStr">
+        <is>
+          <t>User-flagged as ideal fit shape (2026-05-07)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark stakefish Web3/Fullstack as 1. Apply (LinkedIn Easy Apply)
Decision changed from "2. Recommended" to "1. Apply" — user is
submitting via LinkedIn Easy Apply with the JD-mirrored summary
generated in this session. Notes record the application date.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -8705,12 +8705,12 @@
       <c r="J157" s="25" t="n"/>
       <c r="K157" s="25" t="inlineStr">
         <is>
-          <t>2. Recommended</t>
+          <t>1. Apply</t>
         </is>
       </c>
       <c r="L157" s="25" t="inlineStr">
         <is>
-          <t>User-flagged as ideal fit shape (2026-05-07)</t>
+          <t>Applied via LinkedIn Easy Apply 2026-05-07. User-flagged as ideal fit shape (2026-05-07)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add stakefish to Applications + commit cv-default.pdf
Wishlist Decision = "1. Apply" doesn't currently auto-add to the
Applications tab — that auto-promote only fires from Preparations
when Submission status flips to Submitted, and Easy Apply skips
Preparations entirely. Filling Applications r2 manually:

- Date Applied: 2026-05-07
- Status: Applied
- CV Used: cv-default.pdf (committed in this commit, copied from
  ~/Documents/personal/Resume-CV/Hana_Aliyah_Mufidah.pdf)
- Source: LinkedIn Easy Apply
- Salary: $140-180K USD
- Follow-up: 2026-05-21 (2 weeks)

Default CV now lives in-repo so any future Easy-Apply / fast-lane
record can reference cv-default.pdf without leaking the user's
filesystem path.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -9423,22 +9423,78 @@
         <f>ROW()-1</f>
         <v/>
       </c>
-      <c r="B2" s="1" t="n"/>
-      <c r="C2" s="1" t="n"/>
-      <c r="D2" s="1" t="n"/>
-      <c r="E2" s="1" t="n"/>
-      <c r="F2" s="1" t="n"/>
-      <c r="G2" s="1" t="n"/>
-      <c r="H2" s="1" t="n"/>
-      <c r="I2" s="1" t="n"/>
-      <c r="J2" s="1" t="n"/>
-      <c r="K2" s="1" t="n"/>
+      <c r="B2" s="22" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C2" s="22" t="inlineStr">
+        <is>
+          <t>stakefish</t>
+        </is>
+      </c>
+      <c r="D2" s="22" t="inlineStr">
+        <is>
+          <t>Web3 / Full-stack Software Engineer</t>
+        </is>
+      </c>
+      <c r="E2" s="22" t="inlineStr">
+        <is>
+          <t>Singapore (remote-friendly)</t>
+        </is>
+      </c>
+      <c r="F2" s="22" t="inlineStr">
+        <is>
+          <t>LinkedIn Easy Apply</t>
+        </is>
+      </c>
+      <c r="G2" s="22" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/jobs/view/4354681451/</t>
+        </is>
+      </c>
+      <c r="H2" s="22" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I2" s="22" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="J2" s="22" t="inlineStr">
+        <is>
+          <t>cv-default.pdf</t>
+        </is>
+      </c>
+      <c r="K2" s="22" t="inlineStr">
+        <is>
+          <t>JD-mirrored summary (LinkedIn Easy Apply)</t>
+        </is>
+      </c>
       <c r="L2" s="1" t="n"/>
-      <c r="M2" s="1" t="n"/>
+      <c r="M2" s="22" t="inlineStr">
+        <is>
+          <t>$140K-$180K USD base</t>
+        </is>
+      </c>
       <c r="N2" s="1" t="n"/>
-      <c r="O2" s="1" t="n"/>
-      <c r="P2" s="1" t="n"/>
-      <c r="Q2" s="1" t="n"/>
+      <c r="O2" s="22" t="inlineStr">
+        <is>
+          <t>Wait for recruiter response</t>
+        </is>
+      </c>
+      <c r="P2" s="22" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="Q2" s="22" t="inlineStr">
+        <is>
+          <t>Web3 staking infra; user-flagged as ideal-fit shape (project_ideal_role_shape.md)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3">

</xml_diff>

<commit_message>
Update tracker via web editor (4 edits)
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -514,6 +514,9 @@
     <t>https://getyourguide.careers/jobs/7526177?gh_jid=7526177</t>
   </si>
   <si>
+    <t>3. Recommended</t>
+  </si>
+  <si>
     <t>Senior Software Engineer (Backend focused) - Supply</t>
   </si>
   <si>
@@ -1166,9 +1169,6 @@
   </si>
   <si>
     <t>Vue/React/JS, 7.5M+ JPY, Japan relocation</t>
-  </si>
-  <si>
-    <t>3. Recommended</t>
   </si>
   <si>
     <t>(via GitTap)</t>
@@ -4607,7 +4607,7 @@
       </c>
       <c r="J31" s="1"/>
       <c r="K31" s="18" t="s">
-        <v>84</v>
+        <v>165</v>
       </c>
       <c r="L31" s="18" t="s">
         <v>120</v>
@@ -4624,10 +4624,10 @@
         <v>160</v>
       </c>
       <c r="D32" s="18" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F32" s="18" t="s">
         <v>104</v>
@@ -4641,7 +4641,7 @@
       </c>
       <c r="J32" s="1"/>
       <c r="K32" s="18" t="s">
-        <v>84</v>
+        <v>165</v>
       </c>
       <c r="L32" s="18" t="s">
         <v>120</v>
@@ -4658,10 +4658,10 @@
         <v>160</v>
       </c>
       <c r="D33" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F33" t="s">
         <v>104</v>
@@ -4692,10 +4692,10 @@
         <v>160</v>
       </c>
       <c r="D34" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F34" t="s">
         <v>104</v>
@@ -4726,10 +4726,10 @@
         <v>160</v>
       </c>
       <c r="D35" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F35" t="s">
         <v>104</v>
@@ -4760,10 +4760,10 @@
         <v>160</v>
       </c>
       <c r="D36" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F36" t="s">
         <v>104</v>
@@ -4794,10 +4794,10 @@
         <v>160</v>
       </c>
       <c r="D37" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F37" t="s">
         <v>104</v>
@@ -4828,10 +4828,10 @@
         <v>160</v>
       </c>
       <c r="D38" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F38" t="s">
         <v>104</v>
@@ -4859,13 +4859,13 @@
         <v>71</v>
       </c>
       <c r="C39" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D39" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E39" s="13" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F39" t="s">
         <v>104</v>
@@ -4893,13 +4893,13 @@
         <v>71</v>
       </c>
       <c r="C40" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D40" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F40" t="s">
         <v>104</v>
@@ -4927,13 +4927,13 @@
         <v>71</v>
       </c>
       <c r="C41" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D41" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E41" s="13" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F41" t="s">
         <v>104</v>
@@ -4961,13 +4961,13 @@
         <v>71</v>
       </c>
       <c r="C42" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D42" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F42" t="s">
         <v>104</v>
@@ -4995,13 +4995,13 @@
         <v>71</v>
       </c>
       <c r="C43" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D43" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E43" s="13" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F43" t="s">
         <v>104</v>
@@ -5029,13 +5029,13 @@
         <v>71</v>
       </c>
       <c r="C44" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D44" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F44" t="s">
         <v>104</v>
@@ -5063,13 +5063,13 @@
         <v>71</v>
       </c>
       <c r="C45" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D45" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E45" s="13" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F45" t="s">
         <v>104</v>
@@ -5097,13 +5097,13 @@
         <v>71</v>
       </c>
       <c r="C46" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D46" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E46" s="13" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F46" t="s">
         <v>104</v>
@@ -5131,13 +5131,13 @@
         <v>71</v>
       </c>
       <c r="C47" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D47" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E47" s="13" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F47" t="s">
         <v>104</v>
@@ -5165,13 +5165,13 @@
         <v>71</v>
       </c>
       <c r="C48" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D48" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F48" t="s">
         <v>104</v>
@@ -5199,13 +5199,13 @@
         <v>71</v>
       </c>
       <c r="C49" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D49" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E49" s="13" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F49" t="s">
         <v>104</v>
@@ -5233,13 +5233,13 @@
         <v>71</v>
       </c>
       <c r="C50" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D50" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E50" s="13" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F50" t="s">
         <v>104</v>
@@ -5267,13 +5267,13 @@
         <v>71</v>
       </c>
       <c r="C51" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D51" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E51" s="13" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F51" t="s">
         <v>104</v>
@@ -5301,13 +5301,13 @@
         <v>71</v>
       </c>
       <c r="C52" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D52" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E52" s="13" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F52" t="s">
         <v>104</v>
@@ -5335,13 +5335,13 @@
         <v>71</v>
       </c>
       <c r="C53" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D53" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E53" s="13" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F53" t="s">
         <v>104</v>
@@ -5369,13 +5369,13 @@
         <v>71</v>
       </c>
       <c r="C54" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D54" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E54" s="13" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F54" t="s">
         <v>104</v>
@@ -5403,13 +5403,13 @@
         <v>71</v>
       </c>
       <c r="C55" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D55" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E55" s="13" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F55" t="s">
         <v>104</v>
@@ -5437,13 +5437,13 @@
         <v>71</v>
       </c>
       <c r="C56" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D56" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E56" s="13" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F56" t="s">
         <v>104</v>
@@ -5471,13 +5471,13 @@
         <v>71</v>
       </c>
       <c r="C57" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D57" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E57" s="13" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F57" t="s">
         <v>104</v>
@@ -5505,13 +5505,13 @@
         <v>71</v>
       </c>
       <c r="C58" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D58" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E58" s="13" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F58" t="s">
         <v>104</v>
@@ -5539,13 +5539,13 @@
         <v>71</v>
       </c>
       <c r="C59" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D59" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E59" s="13" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F59" t="s">
         <v>104</v>
@@ -5573,13 +5573,13 @@
         <v>71</v>
       </c>
       <c r="C60" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D60" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E60" s="13" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F60" t="s">
         <v>104</v>
@@ -5607,13 +5607,13 @@
         <v>71</v>
       </c>
       <c r="C61" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D61" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E61" s="13" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F61" t="s">
         <v>104</v>
@@ -5641,13 +5641,13 @@
         <v>71</v>
       </c>
       <c r="C62" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D62" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E62" s="13" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F62" t="s">
         <v>104</v>
@@ -5675,13 +5675,13 @@
         <v>71</v>
       </c>
       <c r="C63" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D63" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E63" s="13" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F63" t="s">
         <v>104</v>
@@ -5709,13 +5709,13 @@
         <v>71</v>
       </c>
       <c r="C64" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D64" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E64" s="13" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F64" t="s">
         <v>104</v>
@@ -5743,13 +5743,13 @@
         <v>71</v>
       </c>
       <c r="C65" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D65" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E65" s="13" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F65" t="s">
         <v>104</v>
@@ -5777,13 +5777,13 @@
         <v>71</v>
       </c>
       <c r="C66" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D66" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E66" s="13" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="F66" t="s">
         <v>104</v>
@@ -5811,13 +5811,13 @@
         <v>71</v>
       </c>
       <c r="C67" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D67" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E67" s="13" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F67" t="s">
         <v>104</v>
@@ -5845,13 +5845,13 @@
         <v>71</v>
       </c>
       <c r="C68" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D68" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E68" s="13" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F68" t="s">
         <v>104</v>
@@ -5879,13 +5879,13 @@
         <v>71</v>
       </c>
       <c r="C69" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D69" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E69" s="13" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F69" t="s">
         <v>104</v>
@@ -5913,13 +5913,13 @@
         <v>71</v>
       </c>
       <c r="C70" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D70" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E70" s="13" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F70" t="s">
         <v>104</v>
@@ -5947,13 +5947,13 @@
         <v>71</v>
       </c>
       <c r="C71" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D71" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E71" s="13" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F71" t="s">
         <v>104</v>
@@ -5981,13 +5981,13 @@
         <v>71</v>
       </c>
       <c r="C72" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D72" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E72" s="13" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F72" t="s">
         <v>104</v>
@@ -6015,13 +6015,13 @@
         <v>71</v>
       </c>
       <c r="C73" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D73" t="s">
         <v>122</v>
       </c>
       <c r="E73" s="13" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F73" t="s">
         <v>104</v>
@@ -6049,13 +6049,13 @@
         <v>71</v>
       </c>
       <c r="C74" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D74" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E74" s="13" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F74" t="s">
         <v>104</v>
@@ -6083,13 +6083,13 @@
         <v>71</v>
       </c>
       <c r="C75" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D75" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E75" s="13" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F75" t="s">
         <v>104</v>
@@ -6117,13 +6117,13 @@
         <v>71</v>
       </c>
       <c r="C76" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D76" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E76" s="13" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="F76" t="s">
         <v>104</v>
@@ -6151,13 +6151,13 @@
         <v>71</v>
       </c>
       <c r="C77" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D77" t="s">
         <v>122</v>
       </c>
       <c r="E77" s="13" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F77" t="s">
         <v>104</v>
@@ -6185,13 +6185,13 @@
         <v>71</v>
       </c>
       <c r="C78" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D78" t="s">
         <v>122</v>
       </c>
       <c r="E78" s="13" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F78" t="s">
         <v>104</v>
@@ -6219,13 +6219,13 @@
         <v>71</v>
       </c>
       <c r="C79" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D79" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E79" s="13" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F79" t="s">
         <v>104</v>
@@ -6253,13 +6253,13 @@
         <v>71</v>
       </c>
       <c r="C80" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D80" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E80" s="13" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F80" t="s">
         <v>104</v>
@@ -6287,13 +6287,13 @@
         <v>71</v>
       </c>
       <c r="C81" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D81" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E81" s="13" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F81" t="s">
         <v>104</v>
@@ -6321,13 +6321,13 @@
         <v>71</v>
       </c>
       <c r="C82" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D82" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E82" s="13" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F82" t="s">
         <v>104</v>
@@ -6355,13 +6355,13 @@
         <v>71</v>
       </c>
       <c r="C83" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D83" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E83" s="13" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F83" t="s">
         <v>104</v>
@@ -6389,13 +6389,13 @@
         <v>71</v>
       </c>
       <c r="C84" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D84" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E84" s="13" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F84" t="s">
         <v>104</v>
@@ -6423,13 +6423,13 @@
         <v>71</v>
       </c>
       <c r="C85" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D85" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E85" s="13" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F85" t="s">
         <v>104</v>
@@ -6457,13 +6457,13 @@
         <v>71</v>
       </c>
       <c r="C86" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D86" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E86" s="13" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F86" t="s">
         <v>104</v>
@@ -6491,13 +6491,13 @@
         <v>71</v>
       </c>
       <c r="C87" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D87" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E87" s="13" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F87" t="s">
         <v>104</v>
@@ -6525,13 +6525,13 @@
         <v>71</v>
       </c>
       <c r="C88" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D88" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E88" s="13" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F88" t="s">
         <v>104</v>
@@ -6559,13 +6559,13 @@
         <v>71</v>
       </c>
       <c r="C89" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D89" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E89" s="13" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F89" t="s">
         <v>104</v>
@@ -6593,13 +6593,13 @@
         <v>71</v>
       </c>
       <c r="C90" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D90" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E90" s="13" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F90" t="s">
         <v>104</v>
@@ -6627,13 +6627,13 @@
         <v>71</v>
       </c>
       <c r="C91" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D91" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E91" s="13" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F91" t="s">
         <v>104</v>
@@ -6661,13 +6661,13 @@
         <v>71</v>
       </c>
       <c r="C92" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D92" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E92" s="13" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F92" t="s">
         <v>104</v>
@@ -6695,13 +6695,13 @@
         <v>71</v>
       </c>
       <c r="C93" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D93" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E93" s="13" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="F93" t="s">
         <v>104</v>
@@ -6729,13 +6729,13 @@
         <v>71</v>
       </c>
       <c r="C94" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D94" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E94" s="13" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F94" t="s">
         <v>104</v>
@@ -6763,13 +6763,13 @@
         <v>71</v>
       </c>
       <c r="C95" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D95" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E95" s="13" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F95" t="s">
         <v>104</v>
@@ -6797,13 +6797,13 @@
         <v>71</v>
       </c>
       <c r="C96" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D96" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E96" s="13" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F96" t="s">
         <v>104</v>
@@ -6831,13 +6831,13 @@
         <v>71</v>
       </c>
       <c r="C97" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D97" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E97" s="13" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F97" t="s">
         <v>104</v>
@@ -6865,13 +6865,13 @@
         <v>71</v>
       </c>
       <c r="C98" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D98" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E98" s="13" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F98" t="s">
         <v>104</v>
@@ -6899,13 +6899,13 @@
         <v>71</v>
       </c>
       <c r="C99" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D99" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E99" s="13" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="F99" t="s">
         <v>104</v>
@@ -6933,13 +6933,13 @@
         <v>71</v>
       </c>
       <c r="C100" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D100" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E100" s="13" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="F100" t="s">
         <v>104</v>
@@ -6967,13 +6967,13 @@
         <v>71</v>
       </c>
       <c r="C101" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D101" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E101" s="13" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="F101" t="s">
         <v>104</v>
@@ -7001,13 +7001,13 @@
         <v>71</v>
       </c>
       <c r="C102" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D102" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E102" s="13" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="F102" t="s">
         <v>104</v>
@@ -7035,13 +7035,13 @@
         <v>71</v>
       </c>
       <c r="C103" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D103" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E103" s="13" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="F103" t="s">
         <v>104</v>
@@ -7069,13 +7069,13 @@
         <v>71</v>
       </c>
       <c r="C104" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D104" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E104" s="13" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F104" t="s">
         <v>104</v>
@@ -7103,13 +7103,13 @@
         <v>71</v>
       </c>
       <c r="C105" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D105" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E105" s="13" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="F105" t="s">
         <v>104</v>
@@ -7137,13 +7137,13 @@
         <v>71</v>
       </c>
       <c r="C106" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D106" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E106" s="13" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F106" t="s">
         <v>104</v>
@@ -7174,10 +7174,10 @@
         <v>108</v>
       </c>
       <c r="D107" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E107" s="13" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F107" t="s">
         <v>104</v>
@@ -7205,13 +7205,13 @@
         <v>71</v>
       </c>
       <c r="C108" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D108" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E108" s="13" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="F108" t="s">
         <v>104</v>
@@ -7239,13 +7239,13 @@
         <v>71</v>
       </c>
       <c r="C109" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D109" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E109" s="13" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F109" t="s">
         <v>104</v>
@@ -7273,13 +7273,13 @@
         <v>71</v>
       </c>
       <c r="C110" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D110" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E110" s="13" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F110" t="s">
         <v>104</v>
@@ -7307,13 +7307,13 @@
         <v>71</v>
       </c>
       <c r="C111" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D111" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E111" s="13" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F111" t="s">
         <v>104</v>
@@ -7341,13 +7341,13 @@
         <v>71</v>
       </c>
       <c r="C112" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D112" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="E112" s="13" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="F112" t="s">
         <v>104</v>
@@ -7375,13 +7375,13 @@
         <v>71</v>
       </c>
       <c r="C113" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D113" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="E113" s="13" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F113" t="s">
         <v>104</v>
@@ -7409,13 +7409,13 @@
         <v>71</v>
       </c>
       <c r="C114" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D114" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E114" s="13" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="F114" t="s">
         <v>104</v>
@@ -7443,13 +7443,13 @@
         <v>71</v>
       </c>
       <c r="C115" s="18" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D115" s="18" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E115" s="13" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F115" s="18" t="s">
         <v>104</v>
@@ -7463,7 +7463,7 @@
       </c>
       <c r="J115" s="1"/>
       <c r="K115" s="18" t="s">
-        <v>84</v>
+        <v>165</v>
       </c>
       <c r="L115" s="18" t="s">
         <v>120</v>
@@ -7477,13 +7477,13 @@
         <v>71</v>
       </c>
       <c r="C116" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D116" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E116" s="13" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F116" t="s">
         <v>104</v>
@@ -7511,13 +7511,13 @@
         <v>71</v>
       </c>
       <c r="C117" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D117" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E117" s="13" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="F117" t="s">
         <v>104</v>
@@ -7545,13 +7545,13 @@
         <v>71</v>
       </c>
       <c r="C118" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D118" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="E118" s="13" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F118" t="s">
         <v>104</v>
@@ -7579,13 +7579,13 @@
         <v>71</v>
       </c>
       <c r="C119" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D119" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E119" s="13" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="F119" t="s">
         <v>104</v>
@@ -7613,13 +7613,13 @@
         <v>71</v>
       </c>
       <c r="C120" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D120" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E120" s="13" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F120" t="s">
         <v>104</v>
@@ -7647,13 +7647,13 @@
         <v>71</v>
       </c>
       <c r="C121" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D121" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E121" s="13" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F121" t="s">
         <v>104</v>
@@ -7681,13 +7681,13 @@
         <v>71</v>
       </c>
       <c r="C122" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D122" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E122" s="13" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="F122" t="s">
         <v>104</v>
@@ -7715,13 +7715,13 @@
         <v>71</v>
       </c>
       <c r="C123" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D123" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E123" s="19" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F123" t="s">
         <v>104</v>
@@ -7735,7 +7735,7 @@
       </c>
       <c r="J123" s="1"/>
       <c r="K123" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="L123" t="s">
         <v>120</v>
@@ -7746,25 +7746,25 @@
         <f>ROW()-1</f>
       </c>
       <c r="B124" s="20" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C124" s="20" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D124" s="20" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E124" s="20" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F124" s="20" t="s">
         <v>104</v>
       </c>
       <c r="G124" s="20" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="H124" s="20" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="I124" s="20"/>
       <c r="J124" s="20"/>
@@ -7778,25 +7778,25 @@
         <f>ROW()-1</f>
       </c>
       <c r="B125" s="20" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C125" s="20" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D125" s="20" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E125" s="20" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F125" s="20" t="s">
         <v>104</v>
       </c>
       <c r="G125" s="20" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="H125" s="20" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="I125" s="20"/>
       <c r="J125" s="20"/>
@@ -7810,7 +7810,7 @@
         <f>ROW()-1</f>
       </c>
       <c r="B126" s="20" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C126" s="20" t="s">
         <v>135</v>
@@ -7819,16 +7819,16 @@
         <v>138</v>
       </c>
       <c r="E126" s="20" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="F126" s="20" t="s">
         <v>104</v>
       </c>
       <c r="G126" s="20" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="H126" s="20" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="I126" s="20"/>
       <c r="J126" s="20"/>
@@ -7842,7 +7842,7 @@
         <f>ROW()-1</f>
       </c>
       <c r="B127" s="20" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C127" s="20" t="s">
         <v>135</v>
@@ -7851,16 +7851,16 @@
         <v>140</v>
       </c>
       <c r="E127" s="20" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F127" s="20" t="s">
         <v>104</v>
       </c>
       <c r="G127" s="20" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="H127" s="20" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="I127" s="20"/>
       <c r="J127" s="20"/>
@@ -7874,7 +7874,7 @@
         <f>ROW()-1</f>
       </c>
       <c r="B128" s="20" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C128" s="20" t="s">
         <v>135</v>
@@ -7883,16 +7883,16 @@
         <v>142</v>
       </c>
       <c r="E128" s="20" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F128" s="20" t="s">
         <v>104</v>
       </c>
       <c r="G128" s="20" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="H128" s="20" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="I128" s="20"/>
       <c r="J128" s="20"/>
@@ -7906,25 +7906,25 @@
         <f>ROW()-1</f>
       </c>
       <c r="B129" s="20" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C129" s="20" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D129" s="20" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E129" s="20" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F129" s="20" t="s">
         <v>104</v>
       </c>
       <c r="G129" s="20" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="H129" s="20" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="I129" s="20"/>
       <c r="J129" s="20"/>
@@ -7938,25 +7938,25 @@
         <f>ROW()-1</f>
       </c>
       <c r="B130" s="20" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C130" s="20" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D130" s="20" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E130" s="20" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="F130" s="20" t="s">
         <v>104</v>
       </c>
       <c r="G130" s="20" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="H130" s="20" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="I130" s="20"/>
       <c r="J130" s="20"/>
@@ -7970,25 +7970,25 @@
         <f>ROW()-1</f>
       </c>
       <c r="B131" s="20" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C131" s="20" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D131" s="20" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E131" s="20" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F131" s="20" t="s">
         <v>104</v>
       </c>
       <c r="G131" s="20" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="H131" s="20" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="I131" s="20"/>
       <c r="J131" s="20"/>
@@ -8002,25 +8002,25 @@
         <f>ROW()-1</f>
       </c>
       <c r="B132" s="20" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C132" s="20" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D132" s="20" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E132" s="20" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F132" s="20" t="s">
         <v>104</v>
       </c>
       <c r="G132" s="20" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="H132" s="20" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="I132" s="20"/>
       <c r="J132" s="20"/>
@@ -8034,25 +8034,25 @@
         <f>ROW()-1</f>
       </c>
       <c r="B133" s="20" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C133" s="20" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D133" s="20" t="s">
         <v>122</v>
       </c>
       <c r="E133" s="20" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="F133" s="20" t="s">
         <v>104</v>
       </c>
       <c r="G133" s="20" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="H133" s="20" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="I133" s="20"/>
       <c r="J133" s="20"/>
@@ -8066,25 +8066,25 @@
         <f>ROW()-1</f>
       </c>
       <c r="B134" s="20" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C134" s="20" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D134" s="20" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E134" s="20" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F134" s="20" t="s">
         <v>104</v>
       </c>
       <c r="G134" s="20" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="H134" s="20" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="I134" s="20"/>
       <c r="J134" s="20"/>
@@ -8098,30 +8098,30 @@
         <f>ROW()-1</f>
       </c>
       <c r="B135" s="20" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C135" s="20" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D135" s="20" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E135" s="20" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F135" s="20" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="G135" s="20" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="H135" s="20" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="I135" s="20"/>
       <c r="J135" s="20"/>
       <c r="K135" s="20" t="s">
-        <v>383</v>
+        <v>165</v>
       </c>
       <c r="L135" s="20" t="s">
         <v>384</v>
@@ -8132,7 +8132,7 @@
         <f>ROW()-1</f>
       </c>
       <c r="B136" s="20" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C136" s="20" t="s">
         <v>385</v>
@@ -8144,10 +8144,10 @@
         <v>387</v>
       </c>
       <c r="F136" s="20" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="G136" s="20" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="H136" s="20" t="s">
         <v>388</v>
@@ -8166,7 +8166,7 @@
         <f>ROW()-1</f>
       </c>
       <c r="B137" s="20" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C137" s="20" t="s">
         <v>389</v>
@@ -8529,7 +8529,7 @@
         <f>ROW()-1</f>
       </c>
       <c r="B4" s="22" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C4" s="22" t="s">
         <v>79</v>
@@ -8726,7 +8726,7 @@
         <f>ROW()-1</f>
       </c>
       <c r="B2" s="22" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C2" s="22" t="s">
         <v>389</v>
@@ -8747,7 +8747,7 @@
         <v>51</v>
       </c>
       <c r="I2" s="22" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="J2" s="22" t="s">
         <v>457</v>
@@ -13110,7 +13110,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C7" s="23" t="s">
         <v>478</v>
@@ -13326,7 +13326,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C19" s="23" t="s">
         <v>512</v>
@@ -13614,7 +13614,7 @@
         <v>33</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C35" s="23" t="s">
         <v>558</v>
@@ -13722,7 +13722,7 @@
         <v>39</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C41" s="23" t="s">
         <v>574</v>
@@ -13812,7 +13812,7 @@
         <v>44</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C46" s="23" t="s">
         <v>588</v>
@@ -13848,7 +13848,7 @@
         <v>46</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C48" s="23" t="s">
         <v>593</v>
@@ -14046,7 +14046,7 @@
         <v>57</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C59" s="23" t="s">
         <v>624</v>
@@ -14136,7 +14136,7 @@
         <v>62</v>
       </c>
       <c r="B64" s="10" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C64" s="23" t="s">
         <v>635</v>
@@ -14192,7 +14192,7 @@
         <v>65</v>
       </c>
       <c r="B67" s="10" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C67" s="23" t="s">
         <v>645</v>
@@ -14318,7 +14318,7 @@
         <v>72</v>
       </c>
       <c r="B74" s="10" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C74" s="23" t="s">
         <v>664</v>
@@ -14410,7 +14410,7 @@
         <v>77</v>
       </c>
       <c r="B79" s="10" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C79" s="23" t="s">
         <v>678</v>
@@ -14464,7 +14464,7 @@
         <v>80</v>
       </c>
       <c r="B82" s="10" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C82" s="23" t="s">
         <v>686</v>
@@ -14482,7 +14482,7 @@
         <v>81</v>
       </c>
       <c r="B83" s="10" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C83" s="23" t="s">
         <v>688</v>

</xml_diff>

<commit_message>
Update tracker via web editor (12 edits, 2 Apply/Easy-Apply propagated)
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1691" uniqueCount="755">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1701" uniqueCount="756">
   <si>
     <t>Hana Aliyah Mufidah</t>
   </si>
@@ -250,60 +250,60 @@
     <t>WEB3 • USER PICK • Rust-preferred (C++/Haskell ok)</t>
   </si>
   <si>
+    <t>1. Apply</t>
+  </si>
+  <si>
+    <t>Loc: Remote (global) | Rust preferred (not required)</t>
+  </si>
+  <si>
+    <t>Tether</t>
+  </si>
+  <si>
+    <t>Backend Engineer - Wallets (100% Remote)</t>
+  </si>
+  <si>
+    <t>https://careers.tether.io/o/backend-engineer-wallets-100-remote-29</t>
+  </si>
+  <si>
+    <t>User-added (Tether careers)</t>
+  </si>
+  <si>
+    <t>WEB3 • USDT issuer • SAME-TZ ⭐</t>
+  </si>
+  <si>
+    <t>Loc: VN | verify: GLOBAL_OK (JSON-LD)</t>
+  </si>
+  <si>
+    <t>Senior Frontend Developer (100% Remote Worldwide)</t>
+  </si>
+  <si>
+    <t>https://careers.tether.io/o/senior-frontend-developer-kyc-worldwide</t>
+  </si>
+  <si>
+    <t>Loc: AE,CZ,EG,ES,HR,IN,IT,MY,NL,VN | verify: GLOBAL_OK (JSON-LD)</t>
+  </si>
+  <si>
+    <t>Senior Fullstack Developer (100% remote Worldwide)</t>
+  </si>
+  <si>
+    <t>https://careers.tether.io/o/senior-fullstack-developer-100-remote-worldwide</t>
+  </si>
+  <si>
+    <t>WEB3 • USDT issuer</t>
+  </si>
+  <si>
+    <t>Loc: AE,CH,ES,GR,IN,IT,NG,NL | verify: GLOBAL_OK (JSON-LD)</t>
+  </si>
+  <si>
+    <t>Senior Backend Developer</t>
+  </si>
+  <si>
+    <t>https://careers.tether.io/o/senior-backend-developer-norway</t>
+  </si>
+  <si>
     <t>4. Saved</t>
   </si>
   <si>
-    <t>Loc: Remote (global) | Rust preferred (not required)</t>
-  </si>
-  <si>
-    <t>Tether</t>
-  </si>
-  <si>
-    <t>Backend Engineer - Wallets (100% Remote)</t>
-  </si>
-  <si>
-    <t>https://careers.tether.io/o/backend-engineer-wallets-100-remote-29</t>
-  </si>
-  <si>
-    <t>User-added (Tether careers)</t>
-  </si>
-  <si>
-    <t>WEB3 • USDT issuer • SAME-TZ ⭐</t>
-  </si>
-  <si>
-    <t>1. Apply</t>
-  </si>
-  <si>
-    <t>Loc: VN | verify: GLOBAL_OK (JSON-LD)</t>
-  </si>
-  <si>
-    <t>Senior Frontend Developer (100% Remote Worldwide)</t>
-  </si>
-  <si>
-    <t>https://careers.tether.io/o/senior-frontend-developer-kyc-worldwide</t>
-  </si>
-  <si>
-    <t>Loc: AE,CZ,EG,ES,HR,IN,IT,MY,NL,VN | verify: GLOBAL_OK (JSON-LD)</t>
-  </si>
-  <si>
-    <t>Senior Fullstack Developer (100% remote Worldwide)</t>
-  </si>
-  <si>
-    <t>https://careers.tether.io/o/senior-fullstack-developer-100-remote-worldwide</t>
-  </si>
-  <si>
-    <t>WEB3 • USDT issuer</t>
-  </si>
-  <si>
-    <t>Loc: AE,CH,ES,GR,IN,IT,NG,NL | verify: GLOBAL_OK (JSON-LD)</t>
-  </si>
-  <si>
-    <t>Senior Backend Developer</t>
-  </si>
-  <si>
-    <t>https://careers.tether.io/o/senior-backend-developer-norway</t>
-  </si>
-  <si>
     <t>Loc: NO | verify: GLOBAL_OK (JSON-LD)</t>
   </si>
   <si>
@@ -1349,6 +1349,9 @@
   </si>
   <si>
     <t>Score 4.0/5 — see career-ops/reports/003-tether-fs-2026-05-07.md. Gaps (all preferred only): Kubernetes, Holepunch p2p, AI/ML infra.</t>
+  </si>
+  <si>
+    <t>[object Object]</t>
   </si>
   <si>
     <t>Date Applied</t>
@@ -3655,10 +3658,10 @@
       </c>
       <c r="J3" s="1"/>
       <c r="K3" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="L3" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -3672,10 +3675,10 @@
         <v>79</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E4" s="13" t="s">
         <v>86</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>87</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>82</v>
@@ -3689,10 +3692,10 @@
       </c>
       <c r="J4" s="1"/>
       <c r="K4" s="1" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -3706,27 +3709,27 @@
         <v>79</v>
       </c>
       <c r="D5" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="E5" s="13" t="s">
         <v>89</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>90</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>82</v>
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I5" s="1">
         <v>5</v>
       </c>
       <c r="J5" s="1"/>
       <c r="K5" s="1" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -3740,24 +3743,24 @@
         <v>79</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E6" s="13" t="s">
         <v>93</v>
-      </c>
-      <c r="E6" s="13" t="s">
-        <v>94</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>82</v>
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I6" s="1">
         <v>5</v>
       </c>
       <c r="J6" s="1"/>
       <c r="K6" s="1" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="L6" s="1" t="s">
         <v>95</v>
@@ -3774,7 +3777,7 @@
         <v>79</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E7" s="13" t="s">
         <v>96</v>
@@ -3784,14 +3787,14 @@
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I7" s="1">
         <v>5</v>
       </c>
       <c r="J7" s="1"/>
       <c r="K7" s="1" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="L7" s="1" t="s">
         <v>97</v>
@@ -3818,14 +3821,14 @@
       </c>
       <c r="G8" s="1"/>
       <c r="H8" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I8" s="1">
         <v>5</v>
       </c>
       <c r="J8" s="1"/>
       <c r="K8" s="1" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
       <c r="L8" s="1" t="s">
         <v>100</v>
@@ -8327,7 +8330,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:S4"/>
+  <dimension ref="A1:S6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="5" style="1" customWidth="1"/>
@@ -8479,7 +8482,7 @@
         <v>426</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F3" s="22" t="s">
         <v>427</v>
@@ -8538,7 +8541,7 @@
         <v>436</v>
       </c>
       <c r="E4" s="22" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F4" s="22" t="s">
         <v>437</v>
@@ -8581,6 +8584,40 @@
       </c>
       <c r="S4" s="22" t="s">
         <v>443</v>
+      </c>
+    </row>
+    <row r="5" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="R5" s="1" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="6" spans="2:18" x14ac:dyDescent="0.25">
+      <c r="B6" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="R6" s="1" t="s">
+        <v>424</v>
       </c>
     </row>
   </sheetData>
@@ -8673,7 +8710,7 @@
         <v>61</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>14</v>
@@ -8682,10 +8719,10 @@
         <v>13</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>63</v>
@@ -8694,28 +8731,28 @@
         <v>44</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="O1" s="7" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="P1" s="7" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="Q1" s="7" t="s">
         <v>70</v>
@@ -8735,10 +8772,10 @@
         <v>390</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="F2" s="22" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="G2" s="22" t="s">
         <v>391</v>
@@ -8750,24 +8787,24 @@
         <v>355</v>
       </c>
       <c r="J2" s="22" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="K2" s="22" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="L2" s="1"/>
       <c r="M2" s="22" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="N2" s="1"/>
       <c r="O2" s="22" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="P2" s="22" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="Q2" s="22" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
@@ -13009,7 +13046,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -13025,16 +13062,16 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>70</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -13042,13 +13079,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E3" s="10"/>
       <c r="F3" s="10"/>
@@ -13058,13 +13095,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="10" t="s">
+        <v>471</v>
+      </c>
+      <c r="C4" s="23" t="s">
+        <v>472</v>
+      </c>
+      <c r="D4" s="10" t="s">
         <v>470</v>
-      </c>
-      <c r="C4" s="23" t="s">
-        <v>471</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>469</v>
       </c>
       <c r="E4" s="10"/>
       <c r="F4" s="10"/>
@@ -13074,16 +13111,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="F5" s="10"/>
     </row>
@@ -13092,16 +13129,16 @@
         <v>4</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="F6" s="10"/>
     </row>
@@ -13113,13 +13150,13 @@
         <v>246</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="F7" s="10"/>
     </row>
@@ -13128,16 +13165,16 @@
         <v>6</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="F8" s="10"/>
     </row>
@@ -13146,16 +13183,16 @@
         <v>7</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="F9" s="10"/>
     </row>
@@ -13167,13 +13204,13 @@
         <v>147</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="F10" s="10"/>
     </row>
@@ -13182,16 +13219,16 @@
         <v>9</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="F11" s="10"/>
     </row>
@@ -13200,16 +13237,16 @@
         <v>10</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F12" s="10"/>
     </row>
@@ -13218,16 +13255,16 @@
         <v>11</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="F13" s="10"/>
     </row>
@@ -13236,16 +13273,16 @@
         <v>12</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="F14" s="10"/>
     </row>
@@ -13254,16 +13291,16 @@
         <v>13</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F15" s="10"/>
     </row>
@@ -13272,16 +13309,16 @@
         <v>14</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="F16" s="10"/>
     </row>
@@ -13290,16 +13327,16 @@
         <v>15</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="F17" s="10"/>
     </row>
@@ -13308,16 +13345,16 @@
         <v>16</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="F18" s="10"/>
     </row>
@@ -13329,13 +13366,13 @@
         <v>185</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F19" s="10"/>
     </row>
@@ -13344,16 +13381,16 @@
         <v>18</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="F20" s="10"/>
     </row>
@@ -13362,16 +13399,16 @@
         <v>19</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="F21" s="10"/>
     </row>
@@ -13380,16 +13417,16 @@
         <v>20</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="F22" s="10"/>
     </row>
@@ -13398,16 +13435,16 @@
         <v>21</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="C23" s="23" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="F23" s="10"/>
     </row>
@@ -13416,16 +13453,16 @@
         <v>22</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="F24" s="10"/>
     </row>
@@ -13434,16 +13471,16 @@
         <v>23</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="C25" s="23" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="F25" s="10"/>
     </row>
@@ -13452,16 +13489,16 @@
         <v>24</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="F26" s="10"/>
     </row>
@@ -13470,16 +13507,16 @@
         <v>25</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="C27" s="23" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="F27" s="10"/>
     </row>
@@ -13488,16 +13525,16 @@
         <v>26</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F28" s="10"/>
     </row>
@@ -13506,16 +13543,16 @@
         <v>27</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="C29" s="23" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F29" s="10"/>
     </row>
@@ -13524,16 +13561,16 @@
         <v>28</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="C30" s="23" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="F30" s="10"/>
     </row>
@@ -13542,16 +13579,16 @@
         <v>29</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="C31" s="23" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="F31" s="10"/>
     </row>
@@ -13560,16 +13597,16 @@
         <v>30</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="C32" s="23" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="F32" s="10"/>
     </row>
@@ -13578,16 +13615,16 @@
         <v>31</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="C33" s="23" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="F33" s="10"/>
     </row>
@@ -13599,13 +13636,13 @@
         <v>108</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="F34" s="10"/>
     </row>
@@ -13617,13 +13654,13 @@
         <v>352</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="F35" s="10"/>
     </row>
@@ -13632,16 +13669,16 @@
         <v>34</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="C36" s="23" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="F36" s="10"/>
     </row>
@@ -13653,13 +13690,13 @@
         <v>121</v>
       </c>
       <c r="C37" s="23" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="F37" s="10"/>
     </row>
@@ -13668,16 +13705,16 @@
         <v>36</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="C38" s="23" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="D38" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="F38" s="10"/>
     </row>
@@ -13686,16 +13723,16 @@
         <v>37</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C39" s="23" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="F39" s="10"/>
     </row>
@@ -13704,16 +13741,16 @@
         <v>38</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="F40" s="10"/>
     </row>
@@ -13725,13 +13762,13 @@
         <v>282</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="F41" s="10"/>
     </row>
@@ -13740,16 +13777,16 @@
         <v>40</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="F42" s="10"/>
     </row>
@@ -13758,16 +13795,16 @@
         <v>41</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="F43" s="10"/>
     </row>
@@ -13776,16 +13813,16 @@
         <v>42</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="C44" s="23" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="D44" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="F44" s="10"/>
     </row>
@@ -13794,16 +13831,16 @@
         <v>43</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="C45" s="23" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="F45" s="10"/>
     </row>
@@ -13815,13 +13852,13 @@
         <v>237</v>
       </c>
       <c r="C46" s="23" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="F46" s="10"/>
     </row>
@@ -13830,16 +13867,16 @@
         <v>45</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="C47" s="23" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="F47" s="10"/>
     </row>
@@ -13851,13 +13888,13 @@
         <v>180</v>
       </c>
       <c r="C48" s="23" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D48" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="F48" s="10"/>
     </row>
@@ -13866,16 +13903,16 @@
         <v>47</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="C49" s="23" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="D49" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E49" s="10" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="F49" s="10"/>
     </row>
@@ -13884,16 +13921,16 @@
         <v>48</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="C50" s="23" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="D50" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="F50" s="10"/>
     </row>
@@ -13902,16 +13939,16 @@
         <v>49</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="D51" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="F51" s="10"/>
     </row>
@@ -13920,16 +13957,16 @@
         <v>50</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="C52" s="23" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="D52" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="F52" s="10"/>
     </row>
@@ -13938,16 +13975,16 @@
         <v>51</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="C53" s="23" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="D53" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="F53" s="10"/>
     </row>
@@ -13956,16 +13993,16 @@
         <v>52</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="C54" s="23" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="D54" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="F54" s="10"/>
     </row>
@@ -13974,16 +14011,16 @@
         <v>53</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="C55" s="23" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="D55" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="F55" s="10"/>
     </row>
@@ -13995,13 +14032,13 @@
         <v>116</v>
       </c>
       <c r="C56" s="23" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="D56" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E56" s="10" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="F56" s="10"/>
     </row>
@@ -14010,16 +14047,16 @@
         <v>55</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="C57" s="23" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="D57" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="F57" s="10"/>
     </row>
@@ -14028,16 +14065,16 @@
         <v>56</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="C58" s="23" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="D58" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E58" s="10" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="F58" s="10"/>
     </row>
@@ -14049,13 +14086,13 @@
         <v>218</v>
       </c>
       <c r="C59" s="23" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="D59" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="F59" s="10"/>
     </row>
@@ -14067,13 +14104,13 @@
         <v>126</v>
       </c>
       <c r="C60" s="23" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="D60" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E60" s="10" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="F60" s="10"/>
     </row>
@@ -14085,13 +14122,13 @@
         <v>135</v>
       </c>
       <c r="C61" s="23" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="D61" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E61" s="10" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="F61" s="10"/>
     </row>
@@ -14103,13 +14140,13 @@
         <v>160</v>
       </c>
       <c r="C62" s="23" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="D62" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E62" s="10" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="F62" s="10"/>
     </row>
@@ -14118,16 +14155,16 @@
         <v>61</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="C63" s="23" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="D63" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E63" s="10" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="F63" s="10"/>
     </row>
@@ -14139,13 +14176,13 @@
         <v>309</v>
       </c>
       <c r="C64" s="23" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="D64" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E64" s="10" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="F64" s="10"/>
     </row>
@@ -14154,16 +14191,16 @@
         <v>63</v>
       </c>
       <c r="B65" s="10" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="C65" s="23" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="D65" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E65" s="10" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="F65" s="10"/>
     </row>
@@ -14172,19 +14209,19 @@
         <v>64</v>
       </c>
       <c r="B66" s="10" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="C66" s="23" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="D66" s="10" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="E66" s="24" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="F66" s="10" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
@@ -14195,13 +14232,13 @@
         <v>336</v>
       </c>
       <c r="C67" s="23" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="D67" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="F67" s="10"/>
     </row>
@@ -14210,16 +14247,16 @@
         <v>66</v>
       </c>
       <c r="B68" s="10" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="C68" s="23" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="D68" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E68" s="10" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="F68" s="10"/>
     </row>
@@ -14228,16 +14265,16 @@
         <v>67</v>
       </c>
       <c r="B69" s="10" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="C69" s="23" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="D69" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E69" s="10" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="F69" s="10"/>
     </row>
@@ -14246,16 +14283,16 @@
         <v>68</v>
       </c>
       <c r="B70" s="10" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="C70" s="23" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="D70" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E70" s="10" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="F70" s="10"/>
     </row>
@@ -14267,13 +14304,13 @@
         <v>144</v>
       </c>
       <c r="C71" s="23" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="D71" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E71" s="10" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="F71" s="10"/>
     </row>
@@ -14282,16 +14319,16 @@
         <v>70</v>
       </c>
       <c r="B72" s="10" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="C72" s="23" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="D72" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E72" s="10" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="F72" s="10"/>
     </row>
@@ -14300,16 +14337,16 @@
         <v>71</v>
       </c>
       <c r="B73" s="10" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="C73" s="23" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="D73" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E73" s="10" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="F73" s="10"/>
     </row>
@@ -14321,13 +14358,13 @@
         <v>319</v>
       </c>
       <c r="C74" s="23" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="D74" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E74" s="10" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="F74" s="10"/>
     </row>
@@ -14336,19 +14373,19 @@
         <v>73</v>
       </c>
       <c r="B75" s="10" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="C75" s="23" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="D75" s="10" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="E75" s="24" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="F75" s="10" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
@@ -14356,16 +14393,16 @@
         <v>74</v>
       </c>
       <c r="B76" s="10" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="C76" s="23" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="D76" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E76" s="10" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="F76" s="10"/>
     </row>
@@ -14374,16 +14411,16 @@
         <v>75</v>
       </c>
       <c r="B77" s="10" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="C77" s="23" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="D77" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="F77" s="10"/>
     </row>
@@ -14392,16 +14429,16 @@
         <v>76</v>
       </c>
       <c r="B78" s="10" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="C78" s="23" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="D78" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E78" s="10" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="F78" s="10"/>
     </row>
@@ -14413,13 +14450,13 @@
         <v>343</v>
       </c>
       <c r="C79" s="23" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="D79" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E79" s="10" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="F79" s="10"/>
     </row>
@@ -14428,16 +14465,16 @@
         <v>78</v>
       </c>
       <c r="B80" s="10" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="C80" s="23" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="D80" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E80" s="10" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="F80" s="10"/>
     </row>
@@ -14446,16 +14483,16 @@
         <v>79</v>
       </c>
       <c r="B81" s="10" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="C81" s="23" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="D81" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="F81" s="10"/>
     </row>
@@ -14467,13 +14504,13 @@
         <v>268</v>
       </c>
       <c r="C82" s="23" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="D82" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E82" s="10" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="F82" s="10"/>
     </row>
@@ -14485,13 +14522,13 @@
         <v>255</v>
       </c>
       <c r="C83" s="23" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="D83" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="F83" s="10"/>
     </row>
@@ -14500,16 +14537,16 @@
         <v>82</v>
       </c>
       <c r="B84" s="10" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="C84" s="23" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="D84" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E84" s="10" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="F84" s="10"/>
     </row>
@@ -14518,16 +14555,16 @@
         <v>83</v>
       </c>
       <c r="B85" s="10" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="C85" s="23" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="D85" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E85" s="10" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="F85" s="10"/>
     </row>
@@ -14536,16 +14573,16 @@
         <v>84</v>
       </c>
       <c r="B86" s="10" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="C86" s="23" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="D86" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E86" s="10" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="F86" s="10"/>
     </row>
@@ -14554,16 +14591,16 @@
         <v>85</v>
       </c>
       <c r="B87" s="10" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="C87" s="23" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="D87" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E87" s="10" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="F87" s="10"/>
     </row>
@@ -14572,16 +14609,16 @@
         <v>86</v>
       </c>
       <c r="B88" s="10" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="C88" s="23" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="D88" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E88" s="10" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="F88" s="10"/>
     </row>
@@ -14590,16 +14627,16 @@
         <v>87</v>
       </c>
       <c r="B89" s="10" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="C89" s="23" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="D89" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E89" s="10" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="F89" s="10"/>
     </row>
@@ -14608,16 +14645,16 @@
         <v>88</v>
       </c>
       <c r="B90" s="10" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="C90" s="23" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="D90" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E90" s="10" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="F90" s="10"/>
     </row>
@@ -14626,16 +14663,16 @@
         <v>89</v>
       </c>
       <c r="B91" s="10" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="C91" s="23" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="D91" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E91" s="10" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="F91" s="10"/>
     </row>
@@ -14647,13 +14684,13 @@
         <v>101</v>
       </c>
       <c r="C92" s="23" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="D92" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E92" s="10" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="F92" s="10"/>
     </row>
@@ -14662,16 +14699,16 @@
         <v>91</v>
       </c>
       <c r="B93" s="10" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="C93" s="23" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="D93" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E93" s="10" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="F93" s="10"/>
     </row>
@@ -14680,16 +14717,16 @@
         <v>92</v>
       </c>
       <c r="B94" s="10" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="C94" s="23" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="D94" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E94" s="10" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="F94" s="10"/>
     </row>
@@ -14698,16 +14735,16 @@
         <v>93</v>
       </c>
       <c r="B95" s="10" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="C95" s="23" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="D95" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E95" s="10" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="F95" s="10"/>
     </row>
@@ -14716,16 +14753,16 @@
         <v>94</v>
       </c>
       <c r="B96" s="10" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="C96" s="23" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="D96" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E96" s="10" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="F96" s="10"/>
     </row>
@@ -14734,16 +14771,16 @@
         <v>95</v>
       </c>
       <c r="B97" s="10" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="C97" s="23" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="D97" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E97" s="10" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="F97" s="10"/>
     </row>
@@ -14752,16 +14789,16 @@
         <v>96</v>
       </c>
       <c r="B98" s="10" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="C98" s="23" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="D98" s="10" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E98" s="10" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="F98" s="10"/>
     </row>
@@ -14894,7 +14931,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -14904,10 +14941,10 @@
         <v>44</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -14915,10 +14952,10 @@
         <v>47</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -14926,10 +14963,10 @@
         <v>49</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -14937,10 +14974,10 @@
         <v>51</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -14948,10 +14985,10 @@
         <v>53</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -14959,10 +14996,10 @@
         <v>55</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -14970,10 +15007,10 @@
         <v>56</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -14981,10 +15018,10 @@
         <v>57</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -14992,10 +15029,10 @@
         <v>58</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -15003,10 +15040,10 @@
         <v>59</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Espresso Systems: revert Decision to Saved, remove Preparations row
User confirmed the Espresso Systems application is a simple CV-drop —
no need for the full Preparations workflow (tailored CV, form
question drafts, video plan, etc.).

- Wishlist r2 Decision: "1. Apply" -> "4. Saved", note flagged as
  "Simple application (CV drop only) — no prep needed"
- Preparations row removed (was r5 with skeleton-only data)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -1164,7 +1164,6 @@
     <mergeCell ref="A27:D27"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A32:D32"/>
     <mergeCell ref="A20:D20"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="A26:D26"/>
@@ -1176,6 +1175,7 @@
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A28:D28"/>
     <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A32:D32"/>
     <mergeCell ref="B7:D7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1539,12 +1539,12 @@
       <c r="J2" s="11" t="n"/>
       <c r="K2" s="11" t="inlineStr">
         <is>
-          <t>1. Apply</t>
+          <t>4. Saved</t>
         </is>
       </c>
       <c r="L2" s="11" t="inlineStr">
         <is>
-          <t>Loc: Remote (global) | Rust preferred (not required)</t>
+          <t>Simple application (CV drop only) — no prep needed. Loc: Remote (global) | Rust preferred (not required)</t>
         </is>
       </c>
     </row>
@@ -8550,7 +8550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S6"/>
+  <dimension ref="A1:S5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="1" min="1" max="1"/>
@@ -8967,51 +8967,20 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>Espresso Systems</t>
+          <t>Zapier</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>Software Engineer, Infrastructure</t>
+          <t>Software Engineer — Release Engineering</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/Espresso/bf359a02-5579-4d8b-a254-23c989f67af5</t>
+          <t>https://jobs.ashbyhq.com/zapier/6948a0e6-a580-4e9d-b109-20652d9a1507</t>
         </is>
       </c>
       <c r="R5" s="1" t="inlineStr">
-        <is>
-          <t>Not submitted</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B6" s="1" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C6" s="1" t="inlineStr">
-        <is>
-          <t>Zapier</t>
-        </is>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
-        <is>
-          <t>Software Engineer — Release Engineering</t>
-        </is>
-      </c>
-      <c r="E6" s="1" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/zapier/6948a0e6-a580-4e9d-b109-20652d9a1507</t>
-        </is>
-      </c>
-      <c r="R6" s="1" t="inlineStr">
         <is>
           <t>Not submitted</t>
         </is>

</xml_diff>

<commit_message>
StraitsX Mid SE Blockchain: switch to Easy Apply path
User opted out of full prep flow — default CV, no tailored essays,
direct submission via Greenhouse form.

- Wishlist r138: Decision "1. Apply" -> "2. Easy Apply"
- Preparations r6 removed (Easy Apply skips prep)
- Applications r3 added (Status=Applied, today's date,
  cv-default.pdf, follow-up 2026-05-21)

Cover letter draft kept in prep/straitsx-mid-software-engineer-
blockchain-2026-05-07.md for optional attachment given the Go gap.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -8468,7 +8468,7 @@
       <c r="J138" s="25" t="n"/>
       <c r="K138" s="25" t="inlineStr">
         <is>
-          <t>1. Apply</t>
+          <t>2. Easy Apply</t>
         </is>
       </c>
       <c r="L138" s="25" t="inlineStr">
@@ -8608,7 +8608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="1" min="1" max="1"/>
@@ -8967,61 +8967,6 @@
         </is>
       </c>
       <c r="N5" s="1" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="25">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B6" s="25" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C6" s="25" t="inlineStr">
-        <is>
-          <t>StraitsX</t>
-        </is>
-      </c>
-      <c r="D6" s="25" t="inlineStr">
-        <is>
-          <t>Mid Software Engineer - Blockchain</t>
-        </is>
-      </c>
-      <c r="E6" s="25" t="inlineStr">
-        <is>
-          <t>https://job-boards.eu.greenhouse.io/straitsx/jobs/4839243101</t>
-        </is>
-      </c>
-      <c r="F6" s="25" t="inlineStr">
-        <is>
-          <t>cv-default.pdf</t>
-        </is>
-      </c>
-      <c r="G6" s="25" t="inlineStr">
-        <is>
-          <t>Default CV (replace if tailoring)</t>
-        </is>
-      </c>
-      <c r="H6" s="25" t="inlineStr">
-        <is>
-          <t>prep/straitsx-mid-software-engineer-blockchain-2026-05-07.md</t>
-        </is>
-      </c>
-      <c r="I6" s="25" t="n"/>
-      <c r="J6" s="25" t="n"/>
-      <c r="K6" s="25" t="n"/>
-      <c r="L6" s="25" t="n"/>
-      <c r="M6" s="25" t="inlineStr">
-        <is>
-          <t>Not submitted</t>
-        </is>
-      </c>
-      <c r="N6" s="25" t="inlineStr">
-        <is>
-          <t>Light form: standard fields + salary + notice + English + PDPA. No essay questions.</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="P2:P1000">
@@ -9279,22 +9224,74 @@
         <f>ROW()-1</f>
         <v/>
       </c>
-      <c r="B3" s="1" t="n"/>
-      <c r="C3" s="1" t="n"/>
-      <c r="D3" s="1" t="n"/>
-      <c r="E3" s="1" t="n"/>
-      <c r="F3" s="1" t="n"/>
-      <c r="G3" s="1" t="n"/>
-      <c r="H3" s="1" t="n"/>
-      <c r="I3" s="1" t="n"/>
-      <c r="J3" s="1" t="n"/>
-      <c r="K3" s="1" t="n"/>
+      <c r="B3" s="22" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C3" s="22" t="inlineStr">
+        <is>
+          <t>StraitsX</t>
+        </is>
+      </c>
+      <c r="D3" s="22" t="inlineStr">
+        <is>
+          <t>Mid Software Engineer - Blockchain</t>
+        </is>
+      </c>
+      <c r="E3" s="22" t="inlineStr">
+        <is>
+          <t>Jakarta, Indonesia (home)</t>
+        </is>
+      </c>
+      <c r="F3" s="22" t="inlineStr">
+        <is>
+          <t>Greenhouse (LinkedIn redirect)</t>
+        </is>
+      </c>
+      <c r="G3" s="22" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/straitsx/jobs/4839243101</t>
+        </is>
+      </c>
+      <c r="H3" s="22" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I3" s="22" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="J3" s="22" t="inlineStr">
+        <is>
+          <t>cv-default.pdf</t>
+        </is>
+      </c>
+      <c r="K3" s="22" t="inlineStr">
+        <is>
+          <t>Optional draft in prep/straitsx-mid-software-engineer-blockchain-2026-05-07.md</t>
+        </is>
+      </c>
       <c r="L3" s="1" t="n"/>
       <c r="M3" s="1" t="n"/>
       <c r="N3" s="1" t="n"/>
-      <c r="O3" s="1" t="n"/>
-      <c r="P3" s="1" t="n"/>
-      <c r="Q3" s="1" t="n"/>
+      <c r="O3" s="22" t="inlineStr">
+        <is>
+          <t>Wait for recruiter response</t>
+        </is>
+      </c>
+      <c r="P3" s="22" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="Q3" s="22" t="inlineStr">
+        <is>
+          <t>Easy Apply path; user opted out of full prep flow. Go gap noted.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4">

</xml_diff>

<commit_message>
Update tracker via web editor (3 edits)
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1638" uniqueCount="748">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1639" uniqueCount="747">
   <si>
     <t>Hana Aliyah Mufidah</t>
   </si>
@@ -1379,9 +1379,6 @@
   </si>
   <si>
     <t>Promoted from Preparations row 2</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>Promoted from Preparations row 3</t>
@@ -8493,10 +8490,10 @@
         <v>405</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>454</v>
+        <v>447</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>454</v>
+        <v>448</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>88</v>
@@ -8510,7 +8507,9 @@
       <c r="J5" s="1" t="s">
         <v>406</v>
       </c>
-      <c r="K5" s="1"/>
+      <c r="K5" s="1" t="s">
+        <v>449</v>
+      </c>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
@@ -8521,7 +8520,7 @@
         <v>452</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
@@ -12700,7 +12699,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -12716,16 +12715,16 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
+        <v>456</v>
+      </c>
+      <c r="D2" s="7" t="s">
         <v>457</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>458</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>71</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -12733,13 +12732,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="10" t="s">
+        <v>459</v>
+      </c>
+      <c r="C3" s="23" t="s">
         <v>460</v>
       </c>
-      <c r="C3" s="23" t="s">
+      <c r="D3" s="10" t="s">
         <v>461</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>462</v>
       </c>
       <c r="E3" s="10"/>
       <c r="F3" s="10"/>
@@ -12749,13 +12748,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="10" t="s">
+        <v>462</v>
+      </c>
+      <c r="C4" s="23" t="s">
         <v>463</v>
       </c>
-      <c r="C4" s="23" t="s">
-        <v>464</v>
-      </c>
       <c r="D4" s="10" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="E4" s="10"/>
       <c r="F4" s="10"/>
@@ -12765,16 +12764,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="10" t="s">
+        <v>464</v>
+      </c>
+      <c r="C5" s="23" t="s">
         <v>465</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="D5" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E5" s="10" t="s">
         <v>466</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>467</v>
       </c>
       <c r="F5" s="10"/>
     </row>
@@ -12783,16 +12782,16 @@
         <v>4</v>
       </c>
       <c r="B6" s="10" t="s">
+        <v>467</v>
+      </c>
+      <c r="C6" s="23" t="s">
         <v>468</v>
       </c>
-      <c r="C6" s="23" t="s">
+      <c r="D6" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E6" s="10" t="s">
         <v>469</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>470</v>
       </c>
       <c r="F6" s="10"/>
     </row>
@@ -12804,13 +12803,13 @@
         <v>246</v>
       </c>
       <c r="C7" s="23" t="s">
+        <v>470</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E7" s="10" t="s">
         <v>471</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>472</v>
       </c>
       <c r="F7" s="10"/>
     </row>
@@ -12819,16 +12818,16 @@
         <v>6</v>
       </c>
       <c r="B8" s="10" t="s">
+        <v>472</v>
+      </c>
+      <c r="C8" s="23" t="s">
         <v>473</v>
       </c>
-      <c r="C8" s="23" t="s">
+      <c r="D8" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E8" s="10" t="s">
         <v>474</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>475</v>
       </c>
       <c r="F8" s="10"/>
     </row>
@@ -12837,16 +12836,16 @@
         <v>7</v>
       </c>
       <c r="B9" s="10" t="s">
+        <v>475</v>
+      </c>
+      <c r="C9" s="23" t="s">
         <v>476</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="D9" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E9" s="10" t="s">
         <v>477</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>478</v>
       </c>
       <c r="F9" s="10"/>
     </row>
@@ -12858,13 +12857,13 @@
         <v>147</v>
       </c>
       <c r="C10" s="23" t="s">
+        <v>478</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E10" s="10" t="s">
         <v>479</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>480</v>
       </c>
       <c r="F10" s="10"/>
     </row>
@@ -12873,16 +12872,16 @@
         <v>9</v>
       </c>
       <c r="B11" s="10" t="s">
+        <v>480</v>
+      </c>
+      <c r="C11" s="23" t="s">
         <v>481</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="D11" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E11" s="10" t="s">
         <v>482</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>483</v>
       </c>
       <c r="F11" s="10"/>
     </row>
@@ -12891,16 +12890,16 @@
         <v>10</v>
       </c>
       <c r="B12" s="10" t="s">
+        <v>483</v>
+      </c>
+      <c r="C12" s="23" t="s">
         <v>484</v>
       </c>
-      <c r="C12" s="23" t="s">
+      <c r="D12" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E12" s="10" t="s">
         <v>485</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>486</v>
       </c>
       <c r="F12" s="10"/>
     </row>
@@ -12909,16 +12908,16 @@
         <v>11</v>
       </c>
       <c r="B13" s="10" t="s">
+        <v>486</v>
+      </c>
+      <c r="C13" s="23" t="s">
         <v>487</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="D13" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E13" s="10" t="s">
         <v>488</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>489</v>
       </c>
       <c r="F13" s="10"/>
     </row>
@@ -12927,16 +12926,16 @@
         <v>12</v>
       </c>
       <c r="B14" s="10" t="s">
+        <v>489</v>
+      </c>
+      <c r="C14" s="23" t="s">
         <v>490</v>
       </c>
-      <c r="C14" s="23" t="s">
+      <c r="D14" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E14" s="10" t="s">
         <v>491</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>492</v>
       </c>
       <c r="F14" s="10"/>
     </row>
@@ -12945,16 +12944,16 @@
         <v>13</v>
       </c>
       <c r="B15" s="10" t="s">
+        <v>492</v>
+      </c>
+      <c r="C15" s="23" t="s">
         <v>493</v>
       </c>
-      <c r="C15" s="23" t="s">
+      <c r="D15" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E15" s="10" t="s">
         <v>494</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>495</v>
       </c>
       <c r="F15" s="10"/>
     </row>
@@ -12963,16 +12962,16 @@
         <v>14</v>
       </c>
       <c r="B16" s="10" t="s">
+        <v>495</v>
+      </c>
+      <c r="C16" s="23" t="s">
         <v>496</v>
       </c>
-      <c r="C16" s="23" t="s">
+      <c r="D16" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E16" s="10" t="s">
         <v>497</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>498</v>
       </c>
       <c r="F16" s="10"/>
     </row>
@@ -12981,16 +12980,16 @@
         <v>15</v>
       </c>
       <c r="B17" s="10" t="s">
+        <v>498</v>
+      </c>
+      <c r="C17" s="23" t="s">
         <v>499</v>
       </c>
-      <c r="C17" s="23" t="s">
+      <c r="D17" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E17" s="10" t="s">
         <v>500</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>501</v>
       </c>
       <c r="F17" s="10"/>
     </row>
@@ -12999,16 +12998,16 @@
         <v>16</v>
       </c>
       <c r="B18" s="10" t="s">
+        <v>501</v>
+      </c>
+      <c r="C18" s="23" t="s">
         <v>502</v>
       </c>
-      <c r="C18" s="23" t="s">
+      <c r="D18" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E18" s="10" t="s">
         <v>503</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E18" s="10" t="s">
-        <v>504</v>
       </c>
       <c r="F18" s="10"/>
     </row>
@@ -13020,13 +13019,13 @@
         <v>185</v>
       </c>
       <c r="C19" s="23" t="s">
+        <v>504</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E19" s="10" t="s">
         <v>505</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E19" s="10" t="s">
-        <v>506</v>
       </c>
       <c r="F19" s="10"/>
     </row>
@@ -13035,16 +13034,16 @@
         <v>18</v>
       </c>
       <c r="B20" s="10" t="s">
+        <v>506</v>
+      </c>
+      <c r="C20" s="23" t="s">
         <v>507</v>
       </c>
-      <c r="C20" s="23" t="s">
+      <c r="D20" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E20" s="10" t="s">
         <v>508</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E20" s="10" t="s">
-        <v>509</v>
       </c>
       <c r="F20" s="10"/>
     </row>
@@ -13053,16 +13052,16 @@
         <v>19</v>
       </c>
       <c r="B21" s="10" t="s">
+        <v>509</v>
+      </c>
+      <c r="C21" s="23" t="s">
         <v>510</v>
       </c>
-      <c r="C21" s="23" t="s">
+      <c r="D21" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E21" s="10" t="s">
         <v>511</v>
-      </c>
-      <c r="D21" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E21" s="10" t="s">
-        <v>512</v>
       </c>
       <c r="F21" s="10"/>
     </row>
@@ -13071,16 +13070,16 @@
         <v>20</v>
       </c>
       <c r="B22" s="10" t="s">
+        <v>512</v>
+      </c>
+      <c r="C22" s="23" t="s">
         <v>513</v>
       </c>
-      <c r="C22" s="23" t="s">
+      <c r="D22" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E22" s="10" t="s">
         <v>514</v>
-      </c>
-      <c r="D22" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>515</v>
       </c>
       <c r="F22" s="10"/>
     </row>
@@ -13089,16 +13088,16 @@
         <v>21</v>
       </c>
       <c r="B23" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="C23" s="23" t="s">
         <v>516</v>
       </c>
-      <c r="C23" s="23" t="s">
+      <c r="D23" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E23" s="10" t="s">
         <v>517</v>
-      </c>
-      <c r="D23" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E23" s="10" t="s">
-        <v>518</v>
       </c>
       <c r="F23" s="10"/>
     </row>
@@ -13107,16 +13106,16 @@
         <v>22</v>
       </c>
       <c r="B24" s="10" t="s">
+        <v>518</v>
+      </c>
+      <c r="C24" s="23" t="s">
         <v>519</v>
       </c>
-      <c r="C24" s="23" t="s">
+      <c r="D24" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E24" s="10" t="s">
         <v>520</v>
-      </c>
-      <c r="D24" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E24" s="10" t="s">
-        <v>521</v>
       </c>
       <c r="F24" s="10"/>
     </row>
@@ -13125,16 +13124,16 @@
         <v>23</v>
       </c>
       <c r="B25" s="10" t="s">
+        <v>521</v>
+      </c>
+      <c r="C25" s="23" t="s">
         <v>522</v>
       </c>
-      <c r="C25" s="23" t="s">
+      <c r="D25" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E25" s="10" t="s">
         <v>523</v>
-      </c>
-      <c r="D25" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E25" s="10" t="s">
-        <v>524</v>
       </c>
       <c r="F25" s="10"/>
     </row>
@@ -13143,16 +13142,16 @@
         <v>24</v>
       </c>
       <c r="B26" s="10" t="s">
+        <v>524</v>
+      </c>
+      <c r="C26" s="23" t="s">
         <v>525</v>
       </c>
-      <c r="C26" s="23" t="s">
+      <c r="D26" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E26" s="10" t="s">
         <v>526</v>
-      </c>
-      <c r="D26" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E26" s="10" t="s">
-        <v>527</v>
       </c>
       <c r="F26" s="10"/>
     </row>
@@ -13161,16 +13160,16 @@
         <v>25</v>
       </c>
       <c r="B27" s="10" t="s">
+        <v>527</v>
+      </c>
+      <c r="C27" s="23" t="s">
         <v>528</v>
       </c>
-      <c r="C27" s="23" t="s">
+      <c r="D27" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E27" s="10" t="s">
         <v>529</v>
-      </c>
-      <c r="D27" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E27" s="10" t="s">
-        <v>530</v>
       </c>
       <c r="F27" s="10"/>
     </row>
@@ -13179,16 +13178,16 @@
         <v>26</v>
       </c>
       <c r="B28" s="10" t="s">
+        <v>530</v>
+      </c>
+      <c r="C28" s="23" t="s">
         <v>531</v>
       </c>
-      <c r="C28" s="23" t="s">
+      <c r="D28" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E28" s="10" t="s">
         <v>532</v>
-      </c>
-      <c r="D28" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E28" s="10" t="s">
-        <v>533</v>
       </c>
       <c r="F28" s="10"/>
     </row>
@@ -13197,16 +13196,16 @@
         <v>27</v>
       </c>
       <c r="B29" s="10" t="s">
+        <v>533</v>
+      </c>
+      <c r="C29" s="23" t="s">
         <v>534</v>
       </c>
-      <c r="C29" s="23" t="s">
+      <c r="D29" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E29" s="10" t="s">
         <v>535</v>
-      </c>
-      <c r="D29" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E29" s="10" t="s">
-        <v>536</v>
       </c>
       <c r="F29" s="10"/>
     </row>
@@ -13215,16 +13214,16 @@
         <v>28</v>
       </c>
       <c r="B30" s="10" t="s">
+        <v>536</v>
+      </c>
+      <c r="C30" s="23" t="s">
         <v>537</v>
       </c>
-      <c r="C30" s="23" t="s">
+      <c r="D30" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E30" s="10" t="s">
         <v>538</v>
-      </c>
-      <c r="D30" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E30" s="10" t="s">
-        <v>539</v>
       </c>
       <c r="F30" s="10"/>
     </row>
@@ -13233,16 +13232,16 @@
         <v>29</v>
       </c>
       <c r="B31" s="10" t="s">
+        <v>539</v>
+      </c>
+      <c r="C31" s="23" t="s">
         <v>540</v>
       </c>
-      <c r="C31" s="23" t="s">
+      <c r="D31" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E31" s="10" t="s">
         <v>541</v>
-      </c>
-      <c r="D31" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E31" s="10" t="s">
-        <v>542</v>
       </c>
       <c r="F31" s="10"/>
     </row>
@@ -13251,16 +13250,16 @@
         <v>30</v>
       </c>
       <c r="B32" s="10" t="s">
+        <v>542</v>
+      </c>
+      <c r="C32" s="23" t="s">
         <v>543</v>
       </c>
-      <c r="C32" s="23" t="s">
+      <c r="D32" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E32" s="10" t="s">
         <v>544</v>
-      </c>
-      <c r="D32" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E32" s="10" t="s">
-        <v>545</v>
       </c>
       <c r="F32" s="10"/>
     </row>
@@ -13269,16 +13268,16 @@
         <v>31</v>
       </c>
       <c r="B33" s="10" t="s">
+        <v>545</v>
+      </c>
+      <c r="C33" s="23" t="s">
         <v>546</v>
       </c>
-      <c r="C33" s="23" t="s">
+      <c r="D33" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E33" s="10" t="s">
         <v>547</v>
-      </c>
-      <c r="D33" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E33" s="10" t="s">
-        <v>548</v>
       </c>
       <c r="F33" s="10"/>
     </row>
@@ -13290,13 +13289,13 @@
         <v>108</v>
       </c>
       <c r="C34" s="23" t="s">
+        <v>548</v>
+      </c>
+      <c r="D34" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E34" s="10" t="s">
         <v>549</v>
-      </c>
-      <c r="D34" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E34" s="10" t="s">
-        <v>550</v>
       </c>
       <c r="F34" s="10"/>
     </row>
@@ -13308,13 +13307,13 @@
         <v>350</v>
       </c>
       <c r="C35" s="23" t="s">
+        <v>550</v>
+      </c>
+      <c r="D35" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E35" s="10" t="s">
         <v>551</v>
-      </c>
-      <c r="D35" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E35" s="10" t="s">
-        <v>552</v>
       </c>
       <c r="F35" s="10"/>
     </row>
@@ -13323,16 +13322,16 @@
         <v>34</v>
       </c>
       <c r="B36" s="10" t="s">
+        <v>552</v>
+      </c>
+      <c r="C36" s="23" t="s">
         <v>553</v>
       </c>
-      <c r="C36" s="23" t="s">
+      <c r="D36" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E36" s="10" t="s">
         <v>554</v>
-      </c>
-      <c r="D36" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E36" s="10" t="s">
-        <v>555</v>
       </c>
       <c r="F36" s="10"/>
     </row>
@@ -13344,13 +13343,13 @@
         <v>121</v>
       </c>
       <c r="C37" s="23" t="s">
+        <v>555</v>
+      </c>
+      <c r="D37" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E37" s="10" t="s">
         <v>556</v>
-      </c>
-      <c r="D37" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E37" s="10" t="s">
-        <v>557</v>
       </c>
       <c r="F37" s="10"/>
     </row>
@@ -13359,16 +13358,16 @@
         <v>36</v>
       </c>
       <c r="B38" s="10" t="s">
+        <v>557</v>
+      </c>
+      <c r="C38" s="23" t="s">
         <v>558</v>
       </c>
-      <c r="C38" s="23" t="s">
+      <c r="D38" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E38" s="10" t="s">
         <v>559</v>
-      </c>
-      <c r="D38" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E38" s="10" t="s">
-        <v>560</v>
       </c>
       <c r="F38" s="10"/>
     </row>
@@ -13377,16 +13376,16 @@
         <v>37</v>
       </c>
       <c r="B39" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="C39" s="23" t="s">
         <v>561</v>
       </c>
-      <c r="C39" s="23" t="s">
+      <c r="D39" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E39" s="10" t="s">
         <v>562</v>
-      </c>
-      <c r="D39" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E39" s="10" t="s">
-        <v>563</v>
       </c>
       <c r="F39" s="10"/>
     </row>
@@ -13395,16 +13394,16 @@
         <v>38</v>
       </c>
       <c r="B40" s="10" t="s">
+        <v>563</v>
+      </c>
+      <c r="C40" s="23" t="s">
         <v>564</v>
       </c>
-      <c r="C40" s="23" t="s">
+      <c r="D40" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E40" s="10" t="s">
         <v>565</v>
-      </c>
-      <c r="D40" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E40" s="10" t="s">
-        <v>566</v>
       </c>
       <c r="F40" s="10"/>
     </row>
@@ -13416,13 +13415,13 @@
         <v>280</v>
       </c>
       <c r="C41" s="23" t="s">
+        <v>566</v>
+      </c>
+      <c r="D41" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E41" s="10" t="s">
         <v>567</v>
-      </c>
-      <c r="D41" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E41" s="10" t="s">
-        <v>568</v>
       </c>
       <c r="F41" s="10"/>
     </row>
@@ -13431,16 +13430,16 @@
         <v>40</v>
       </c>
       <c r="B42" s="10" t="s">
+        <v>568</v>
+      </c>
+      <c r="C42" s="23" t="s">
         <v>569</v>
       </c>
-      <c r="C42" s="23" t="s">
+      <c r="D42" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E42" s="10" t="s">
         <v>570</v>
-      </c>
-      <c r="D42" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E42" s="10" t="s">
-        <v>571</v>
       </c>
       <c r="F42" s="10"/>
     </row>
@@ -13449,16 +13448,16 @@
         <v>41</v>
       </c>
       <c r="B43" s="10" t="s">
+        <v>571</v>
+      </c>
+      <c r="C43" s="23" t="s">
         <v>572</v>
       </c>
-      <c r="C43" s="23" t="s">
+      <c r="D43" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E43" s="10" t="s">
         <v>573</v>
-      </c>
-      <c r="D43" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E43" s="10" t="s">
-        <v>574</v>
       </c>
       <c r="F43" s="10"/>
     </row>
@@ -13467,16 +13466,16 @@
         <v>42</v>
       </c>
       <c r="B44" s="10" t="s">
+        <v>574</v>
+      </c>
+      <c r="C44" s="23" t="s">
         <v>575</v>
       </c>
-      <c r="C44" s="23" t="s">
+      <c r="D44" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E44" s="10" t="s">
         <v>576</v>
-      </c>
-      <c r="D44" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E44" s="10" t="s">
-        <v>577</v>
       </c>
       <c r="F44" s="10"/>
     </row>
@@ -13485,16 +13484,16 @@
         <v>43</v>
       </c>
       <c r="B45" s="10" t="s">
+        <v>577</v>
+      </c>
+      <c r="C45" s="23" t="s">
         <v>578</v>
       </c>
-      <c r="C45" s="23" t="s">
+      <c r="D45" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E45" s="10" t="s">
         <v>579</v>
-      </c>
-      <c r="D45" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E45" s="10" t="s">
-        <v>580</v>
       </c>
       <c r="F45" s="10"/>
     </row>
@@ -13506,13 +13505,13 @@
         <v>237</v>
       </c>
       <c r="C46" s="23" t="s">
+        <v>580</v>
+      </c>
+      <c r="D46" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E46" s="10" t="s">
         <v>581</v>
-      </c>
-      <c r="D46" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E46" s="10" t="s">
-        <v>582</v>
       </c>
       <c r="F46" s="10"/>
     </row>
@@ -13521,16 +13520,16 @@
         <v>45</v>
       </c>
       <c r="B47" s="10" t="s">
+        <v>582</v>
+      </c>
+      <c r="C47" s="23" t="s">
         <v>583</v>
       </c>
-      <c r="C47" s="23" t="s">
+      <c r="D47" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E47" s="10" t="s">
         <v>584</v>
-      </c>
-      <c r="D47" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E47" s="10" t="s">
-        <v>585</v>
       </c>
       <c r="F47" s="10"/>
     </row>
@@ -13542,13 +13541,13 @@
         <v>180</v>
       </c>
       <c r="C48" s="23" t="s">
+        <v>585</v>
+      </c>
+      <c r="D48" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E48" s="10" t="s">
         <v>586</v>
-      </c>
-      <c r="D48" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E48" s="10" t="s">
-        <v>587</v>
       </c>
       <c r="F48" s="10"/>
     </row>
@@ -13557,16 +13556,16 @@
         <v>47</v>
       </c>
       <c r="B49" s="10" t="s">
+        <v>587</v>
+      </c>
+      <c r="C49" s="23" t="s">
         <v>588</v>
       </c>
-      <c r="C49" s="23" t="s">
+      <c r="D49" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E49" s="10" t="s">
         <v>589</v>
-      </c>
-      <c r="D49" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E49" s="10" t="s">
-        <v>590</v>
       </c>
       <c r="F49" s="10"/>
     </row>
@@ -13575,16 +13574,16 @@
         <v>48</v>
       </c>
       <c r="B50" s="10" t="s">
+        <v>590</v>
+      </c>
+      <c r="C50" s="23" t="s">
         <v>591</v>
       </c>
-      <c r="C50" s="23" t="s">
+      <c r="D50" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E50" s="10" t="s">
         <v>592</v>
-      </c>
-      <c r="D50" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E50" s="10" t="s">
-        <v>593</v>
       </c>
       <c r="F50" s="10"/>
     </row>
@@ -13593,16 +13592,16 @@
         <v>49</v>
       </c>
       <c r="B51" s="10" t="s">
+        <v>593</v>
+      </c>
+      <c r="C51" s="23" t="s">
         <v>594</v>
       </c>
-      <c r="C51" s="23" t="s">
+      <c r="D51" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E51" s="10" t="s">
         <v>595</v>
-      </c>
-      <c r="D51" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E51" s="10" t="s">
-        <v>596</v>
       </c>
       <c r="F51" s="10"/>
     </row>
@@ -13611,16 +13610,16 @@
         <v>50</v>
       </c>
       <c r="B52" s="10" t="s">
+        <v>596</v>
+      </c>
+      <c r="C52" s="23" t="s">
         <v>597</v>
       </c>
-      <c r="C52" s="23" t="s">
+      <c r="D52" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E52" s="10" t="s">
         <v>598</v>
-      </c>
-      <c r="D52" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E52" s="10" t="s">
-        <v>599</v>
       </c>
       <c r="F52" s="10"/>
     </row>
@@ -13629,16 +13628,16 @@
         <v>51</v>
       </c>
       <c r="B53" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="C53" s="23" t="s">
         <v>600</v>
       </c>
-      <c r="C53" s="23" t="s">
+      <c r="D53" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E53" s="10" t="s">
         <v>601</v>
-      </c>
-      <c r="D53" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E53" s="10" t="s">
-        <v>602</v>
       </c>
       <c r="F53" s="10"/>
     </row>
@@ -13647,16 +13646,16 @@
         <v>52</v>
       </c>
       <c r="B54" s="10" t="s">
+        <v>602</v>
+      </c>
+      <c r="C54" s="23" t="s">
         <v>603</v>
       </c>
-      <c r="C54" s="23" t="s">
+      <c r="D54" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E54" s="10" t="s">
         <v>604</v>
-      </c>
-      <c r="D54" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E54" s="10" t="s">
-        <v>605</v>
       </c>
       <c r="F54" s="10"/>
     </row>
@@ -13665,16 +13664,16 @@
         <v>53</v>
       </c>
       <c r="B55" s="10" t="s">
+        <v>605</v>
+      </c>
+      <c r="C55" s="23" t="s">
         <v>606</v>
       </c>
-      <c r="C55" s="23" t="s">
+      <c r="D55" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E55" s="10" t="s">
         <v>607</v>
-      </c>
-      <c r="D55" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E55" s="10" t="s">
-        <v>608</v>
       </c>
       <c r="F55" s="10"/>
     </row>
@@ -13686,13 +13685,13 @@
         <v>116</v>
       </c>
       <c r="C56" s="23" t="s">
+        <v>608</v>
+      </c>
+      <c r="D56" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E56" s="10" t="s">
         <v>609</v>
-      </c>
-      <c r="D56" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E56" s="10" t="s">
-        <v>610</v>
       </c>
       <c r="F56" s="10"/>
     </row>
@@ -13701,16 +13700,16 @@
         <v>55</v>
       </c>
       <c r="B57" s="10" t="s">
+        <v>610</v>
+      </c>
+      <c r="C57" s="23" t="s">
         <v>611</v>
       </c>
-      <c r="C57" s="23" t="s">
+      <c r="D57" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E57" s="10" t="s">
         <v>612</v>
-      </c>
-      <c r="D57" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E57" s="10" t="s">
-        <v>613</v>
       </c>
       <c r="F57" s="10"/>
     </row>
@@ -13719,16 +13718,16 @@
         <v>56</v>
       </c>
       <c r="B58" s="10" t="s">
+        <v>613</v>
+      </c>
+      <c r="C58" s="23" t="s">
         <v>614</v>
       </c>
-      <c r="C58" s="23" t="s">
+      <c r="D58" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E58" s="10" t="s">
         <v>615</v>
-      </c>
-      <c r="D58" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E58" s="10" t="s">
-        <v>616</v>
       </c>
       <c r="F58" s="10"/>
     </row>
@@ -13740,13 +13739,13 @@
         <v>218</v>
       </c>
       <c r="C59" s="23" t="s">
+        <v>616</v>
+      </c>
+      <c r="D59" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E59" s="10" t="s">
         <v>617</v>
-      </c>
-      <c r="D59" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E59" s="10" t="s">
-        <v>618</v>
       </c>
       <c r="F59" s="10"/>
     </row>
@@ -13758,13 +13757,13 @@
         <v>126</v>
       </c>
       <c r="C60" s="23" t="s">
+        <v>618</v>
+      </c>
+      <c r="D60" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E60" s="10" t="s">
         <v>619</v>
-      </c>
-      <c r="D60" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E60" s="10" t="s">
-        <v>620</v>
       </c>
       <c r="F60" s="10"/>
     </row>
@@ -13776,13 +13775,13 @@
         <v>135</v>
       </c>
       <c r="C61" s="23" t="s">
+        <v>620</v>
+      </c>
+      <c r="D61" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E61" s="10" t="s">
         <v>621</v>
-      </c>
-      <c r="D61" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E61" s="10" t="s">
-        <v>622</v>
       </c>
       <c r="F61" s="10"/>
     </row>
@@ -13794,13 +13793,13 @@
         <v>160</v>
       </c>
       <c r="C62" s="23" t="s">
+        <v>622</v>
+      </c>
+      <c r="D62" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E62" s="10" t="s">
         <v>623</v>
-      </c>
-      <c r="D62" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E62" s="10" t="s">
-        <v>624</v>
       </c>
       <c r="F62" s="10"/>
     </row>
@@ -13809,16 +13808,16 @@
         <v>61</v>
       </c>
       <c r="B63" s="10" t="s">
+        <v>624</v>
+      </c>
+      <c r="C63" s="23" t="s">
         <v>625</v>
       </c>
-      <c r="C63" s="23" t="s">
+      <c r="D63" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E63" s="10" t="s">
         <v>626</v>
-      </c>
-      <c r="D63" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E63" s="10" t="s">
-        <v>627</v>
       </c>
       <c r="F63" s="10"/>
     </row>
@@ -13830,13 +13829,13 @@
         <v>307</v>
       </c>
       <c r="C64" s="23" t="s">
+        <v>627</v>
+      </c>
+      <c r="D64" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E64" s="10" t="s">
         <v>628</v>
-      </c>
-      <c r="D64" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E64" s="10" t="s">
-        <v>629</v>
       </c>
       <c r="F64" s="10"/>
     </row>
@@ -13845,16 +13844,16 @@
         <v>63</v>
       </c>
       <c r="B65" s="10" t="s">
+        <v>629</v>
+      </c>
+      <c r="C65" s="23" t="s">
         <v>630</v>
       </c>
-      <c r="C65" s="23" t="s">
+      <c r="D65" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E65" s="10" t="s">
         <v>631</v>
-      </c>
-      <c r="D65" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E65" s="10" t="s">
-        <v>632</v>
       </c>
       <c r="F65" s="10"/>
     </row>
@@ -13863,19 +13862,19 @@
         <v>64</v>
       </c>
       <c r="B66" s="10" t="s">
+        <v>632</v>
+      </c>
+      <c r="C66" s="23" t="s">
         <v>633</v>
       </c>
-      <c r="C66" s="23" t="s">
+      <c r="D66" s="10" t="s">
         <v>634</v>
       </c>
-      <c r="D66" s="10" t="s">
+      <c r="E66" s="24" t="s">
         <v>635</v>
       </c>
-      <c r="E66" s="24" t="s">
+      <c r="F66" s="10" t="s">
         <v>636</v>
-      </c>
-      <c r="F66" s="10" t="s">
-        <v>637</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
@@ -13886,13 +13885,13 @@
         <v>334</v>
       </c>
       <c r="C67" s="23" t="s">
+        <v>637</v>
+      </c>
+      <c r="D67" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E67" s="10" t="s">
         <v>638</v>
-      </c>
-      <c r="D67" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E67" s="10" t="s">
-        <v>639</v>
       </c>
       <c r="F67" s="10"/>
     </row>
@@ -13901,16 +13900,16 @@
         <v>66</v>
       </c>
       <c r="B68" s="10" t="s">
+        <v>639</v>
+      </c>
+      <c r="C68" s="23" t="s">
         <v>640</v>
       </c>
-      <c r="C68" s="23" t="s">
+      <c r="D68" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E68" s="10" t="s">
         <v>641</v>
-      </c>
-      <c r="D68" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E68" s="10" t="s">
-        <v>642</v>
       </c>
       <c r="F68" s="10"/>
     </row>
@@ -13919,16 +13918,16 @@
         <v>67</v>
       </c>
       <c r="B69" s="10" t="s">
+        <v>642</v>
+      </c>
+      <c r="C69" s="23" t="s">
         <v>643</v>
       </c>
-      <c r="C69" s="23" t="s">
+      <c r="D69" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E69" s="10" t="s">
         <v>644</v>
-      </c>
-      <c r="D69" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E69" s="10" t="s">
-        <v>645</v>
       </c>
       <c r="F69" s="10"/>
     </row>
@@ -13937,16 +13936,16 @@
         <v>68</v>
       </c>
       <c r="B70" s="10" t="s">
+        <v>645</v>
+      </c>
+      <c r="C70" s="23" t="s">
         <v>646</v>
       </c>
-      <c r="C70" s="23" t="s">
+      <c r="D70" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E70" s="10" t="s">
         <v>647</v>
-      </c>
-      <c r="D70" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E70" s="10" t="s">
-        <v>648</v>
       </c>
       <c r="F70" s="10"/>
     </row>
@@ -13958,13 +13957,13 @@
         <v>144</v>
       </c>
       <c r="C71" s="23" t="s">
+        <v>648</v>
+      </c>
+      <c r="D71" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E71" s="10" t="s">
         <v>649</v>
-      </c>
-      <c r="D71" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E71" s="10" t="s">
-        <v>650</v>
       </c>
       <c r="F71" s="10"/>
     </row>
@@ -13973,16 +13972,16 @@
         <v>70</v>
       </c>
       <c r="B72" s="10" t="s">
+        <v>650</v>
+      </c>
+      <c r="C72" s="23" t="s">
         <v>651</v>
       </c>
-      <c r="C72" s="23" t="s">
+      <c r="D72" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E72" s="10" t="s">
         <v>652</v>
-      </c>
-      <c r="D72" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E72" s="10" t="s">
-        <v>653</v>
       </c>
       <c r="F72" s="10"/>
     </row>
@@ -13991,16 +13990,16 @@
         <v>71</v>
       </c>
       <c r="B73" s="10" t="s">
+        <v>653</v>
+      </c>
+      <c r="C73" s="23" t="s">
         <v>654</v>
       </c>
-      <c r="C73" s="23" t="s">
+      <c r="D73" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E73" s="10" t="s">
         <v>655</v>
-      </c>
-      <c r="D73" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E73" s="10" t="s">
-        <v>656</v>
       </c>
       <c r="F73" s="10"/>
     </row>
@@ -14012,13 +14011,13 @@
         <v>317</v>
       </c>
       <c r="C74" s="23" t="s">
+        <v>656</v>
+      </c>
+      <c r="D74" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E74" s="10" t="s">
         <v>657</v>
-      </c>
-      <c r="D74" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E74" s="10" t="s">
-        <v>658</v>
       </c>
       <c r="F74" s="10"/>
     </row>
@@ -14027,19 +14026,19 @@
         <v>73</v>
       </c>
       <c r="B75" s="10" t="s">
+        <v>658</v>
+      </c>
+      <c r="C75" s="23" t="s">
         <v>659</v>
       </c>
-      <c r="C75" s="23" t="s">
+      <c r="D75" s="10" t="s">
+        <v>634</v>
+      </c>
+      <c r="E75" s="24" t="s">
         <v>660</v>
       </c>
-      <c r="D75" s="10" t="s">
-        <v>635</v>
-      </c>
-      <c r="E75" s="24" t="s">
-        <v>661</v>
-      </c>
       <c r="F75" s="10" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
@@ -14047,16 +14046,16 @@
         <v>74</v>
       </c>
       <c r="B76" s="10" t="s">
+        <v>661</v>
+      </c>
+      <c r="C76" s="23" t="s">
         <v>662</v>
       </c>
-      <c r="C76" s="23" t="s">
+      <c r="D76" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E76" s="10" t="s">
         <v>663</v>
-      </c>
-      <c r="D76" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E76" s="10" t="s">
-        <v>664</v>
       </c>
       <c r="F76" s="10"/>
     </row>
@@ -14065,16 +14064,16 @@
         <v>75</v>
       </c>
       <c r="B77" s="10" t="s">
+        <v>664</v>
+      </c>
+      <c r="C77" s="23" t="s">
         <v>665</v>
       </c>
-      <c r="C77" s="23" t="s">
+      <c r="D77" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E77" s="10" t="s">
         <v>666</v>
-      </c>
-      <c r="D77" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E77" s="10" t="s">
-        <v>667</v>
       </c>
       <c r="F77" s="10"/>
     </row>
@@ -14083,16 +14082,16 @@
         <v>76</v>
       </c>
       <c r="B78" s="10" t="s">
+        <v>667</v>
+      </c>
+      <c r="C78" s="23" t="s">
         <v>668</v>
       </c>
-      <c r="C78" s="23" t="s">
+      <c r="D78" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E78" s="10" t="s">
         <v>669</v>
-      </c>
-      <c r="D78" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E78" s="10" t="s">
-        <v>670</v>
       </c>
       <c r="F78" s="10"/>
     </row>
@@ -14104,13 +14103,13 @@
         <v>341</v>
       </c>
       <c r="C79" s="23" t="s">
+        <v>670</v>
+      </c>
+      <c r="D79" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E79" s="10" t="s">
         <v>671</v>
-      </c>
-      <c r="D79" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E79" s="10" t="s">
-        <v>672</v>
       </c>
       <c r="F79" s="10"/>
     </row>
@@ -14119,16 +14118,16 @@
         <v>78</v>
       </c>
       <c r="B80" s="10" t="s">
+        <v>672</v>
+      </c>
+      <c r="C80" s="23" t="s">
         <v>673</v>
       </c>
-      <c r="C80" s="23" t="s">
+      <c r="D80" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E80" s="10" t="s">
         <v>674</v>
-      </c>
-      <c r="D80" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E80" s="10" t="s">
-        <v>675</v>
       </c>
       <c r="F80" s="10"/>
     </row>
@@ -14137,16 +14136,16 @@
         <v>79</v>
       </c>
       <c r="B81" s="10" t="s">
+        <v>675</v>
+      </c>
+      <c r="C81" s="23" t="s">
         <v>676</v>
       </c>
-      <c r="C81" s="23" t="s">
+      <c r="D81" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E81" s="10" t="s">
         <v>677</v>
-      </c>
-      <c r="D81" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E81" s="10" t="s">
-        <v>678</v>
       </c>
       <c r="F81" s="10"/>
     </row>
@@ -14158,13 +14157,13 @@
         <v>266</v>
       </c>
       <c r="C82" s="23" t="s">
+        <v>678</v>
+      </c>
+      <c r="D82" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E82" s="10" t="s">
         <v>679</v>
-      </c>
-      <c r="D82" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E82" s="10" t="s">
-        <v>680</v>
       </c>
       <c r="F82" s="10"/>
     </row>
@@ -14176,13 +14175,13 @@
         <v>255</v>
       </c>
       <c r="C83" s="23" t="s">
+        <v>680</v>
+      </c>
+      <c r="D83" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E83" s="10" t="s">
         <v>681</v>
-      </c>
-      <c r="D83" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E83" s="10" t="s">
-        <v>682</v>
       </c>
       <c r="F83" s="10"/>
     </row>
@@ -14191,16 +14190,16 @@
         <v>82</v>
       </c>
       <c r="B84" s="10" t="s">
+        <v>682</v>
+      </c>
+      <c r="C84" s="23" t="s">
         <v>683</v>
       </c>
-      <c r="C84" s="23" t="s">
+      <c r="D84" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E84" s="10" t="s">
         <v>684</v>
-      </c>
-      <c r="D84" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E84" s="10" t="s">
-        <v>685</v>
       </c>
       <c r="F84" s="10"/>
     </row>
@@ -14209,16 +14208,16 @@
         <v>83</v>
       </c>
       <c r="B85" s="10" t="s">
+        <v>685</v>
+      </c>
+      <c r="C85" s="23" t="s">
         <v>686</v>
       </c>
-      <c r="C85" s="23" t="s">
+      <c r="D85" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E85" s="10" t="s">
         <v>687</v>
-      </c>
-      <c r="D85" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E85" s="10" t="s">
-        <v>688</v>
       </c>
       <c r="F85" s="10"/>
     </row>
@@ -14227,16 +14226,16 @@
         <v>84</v>
       </c>
       <c r="B86" s="10" t="s">
+        <v>688</v>
+      </c>
+      <c r="C86" s="23" t="s">
         <v>689</v>
       </c>
-      <c r="C86" s="23" t="s">
+      <c r="D86" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E86" s="10" t="s">
         <v>690</v>
-      </c>
-      <c r="D86" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E86" s="10" t="s">
-        <v>691</v>
       </c>
       <c r="F86" s="10"/>
     </row>
@@ -14245,16 +14244,16 @@
         <v>85</v>
       </c>
       <c r="B87" s="10" t="s">
+        <v>691</v>
+      </c>
+      <c r="C87" s="23" t="s">
         <v>692</v>
       </c>
-      <c r="C87" s="23" t="s">
+      <c r="D87" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E87" s="10" t="s">
         <v>693</v>
-      </c>
-      <c r="D87" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E87" s="10" t="s">
-        <v>694</v>
       </c>
       <c r="F87" s="10"/>
     </row>
@@ -14263,16 +14262,16 @@
         <v>86</v>
       </c>
       <c r="B88" s="10" t="s">
+        <v>694</v>
+      </c>
+      <c r="C88" s="23" t="s">
         <v>695</v>
       </c>
-      <c r="C88" s="23" t="s">
+      <c r="D88" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E88" s="10" t="s">
         <v>696</v>
-      </c>
-      <c r="D88" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E88" s="10" t="s">
-        <v>697</v>
       </c>
       <c r="F88" s="10"/>
     </row>
@@ -14281,16 +14280,16 @@
         <v>87</v>
       </c>
       <c r="B89" s="10" t="s">
+        <v>697</v>
+      </c>
+      <c r="C89" s="23" t="s">
         <v>698</v>
       </c>
-      <c r="C89" s="23" t="s">
+      <c r="D89" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E89" s="10" t="s">
         <v>699</v>
-      </c>
-      <c r="D89" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E89" s="10" t="s">
-        <v>700</v>
       </c>
       <c r="F89" s="10"/>
     </row>
@@ -14299,16 +14298,16 @@
         <v>88</v>
       </c>
       <c r="B90" s="10" t="s">
+        <v>700</v>
+      </c>
+      <c r="C90" s="23" t="s">
         <v>701</v>
       </c>
-      <c r="C90" s="23" t="s">
+      <c r="D90" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E90" s="10" t="s">
         <v>702</v>
-      </c>
-      <c r="D90" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E90" s="10" t="s">
-        <v>703</v>
       </c>
       <c r="F90" s="10"/>
     </row>
@@ -14317,16 +14316,16 @@
         <v>89</v>
       </c>
       <c r="B91" s="10" t="s">
+        <v>703</v>
+      </c>
+      <c r="C91" s="23" t="s">
         <v>704</v>
       </c>
-      <c r="C91" s="23" t="s">
+      <c r="D91" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E91" s="10" t="s">
         <v>705</v>
-      </c>
-      <c r="D91" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E91" s="10" t="s">
-        <v>706</v>
       </c>
       <c r="F91" s="10"/>
     </row>
@@ -14338,13 +14337,13 @@
         <v>101</v>
       </c>
       <c r="C92" s="23" t="s">
+        <v>706</v>
+      </c>
+      <c r="D92" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E92" s="10" t="s">
         <v>707</v>
-      </c>
-      <c r="D92" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E92" s="10" t="s">
-        <v>708</v>
       </c>
       <c r="F92" s="10"/>
     </row>
@@ -14353,16 +14352,16 @@
         <v>91</v>
       </c>
       <c r="B93" s="10" t="s">
+        <v>708</v>
+      </c>
+      <c r="C93" s="23" t="s">
         <v>709</v>
       </c>
-      <c r="C93" s="23" t="s">
+      <c r="D93" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E93" s="10" t="s">
         <v>710</v>
-      </c>
-      <c r="D93" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E93" s="10" t="s">
-        <v>711</v>
       </c>
       <c r="F93" s="10"/>
     </row>
@@ -14371,16 +14370,16 @@
         <v>92</v>
       </c>
       <c r="B94" s="10" t="s">
+        <v>711</v>
+      </c>
+      <c r="C94" s="23" t="s">
         <v>712</v>
       </c>
-      <c r="C94" s="23" t="s">
+      <c r="D94" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E94" s="10" t="s">
         <v>713</v>
-      </c>
-      <c r="D94" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E94" s="10" t="s">
-        <v>714</v>
       </c>
       <c r="F94" s="10"/>
     </row>
@@ -14389,16 +14388,16 @@
         <v>93</v>
       </c>
       <c r="B95" s="10" t="s">
+        <v>714</v>
+      </c>
+      <c r="C95" s="23" t="s">
         <v>715</v>
       </c>
-      <c r="C95" s="23" t="s">
+      <c r="D95" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E95" s="10" t="s">
         <v>716</v>
-      </c>
-      <c r="D95" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E95" s="10" t="s">
-        <v>717</v>
       </c>
       <c r="F95" s="10"/>
     </row>
@@ -14407,16 +14406,16 @@
         <v>94</v>
       </c>
       <c r="B96" s="10" t="s">
+        <v>717</v>
+      </c>
+      <c r="C96" s="23" t="s">
         <v>718</v>
       </c>
-      <c r="C96" s="23" t="s">
+      <c r="D96" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E96" s="10" t="s">
         <v>719</v>
-      </c>
-      <c r="D96" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E96" s="10" t="s">
-        <v>720</v>
       </c>
       <c r="F96" s="10"/>
     </row>
@@ -14425,16 +14424,16 @@
         <v>95</v>
       </c>
       <c r="B97" s="10" t="s">
+        <v>720</v>
+      </c>
+      <c r="C97" s="23" t="s">
         <v>721</v>
       </c>
-      <c r="C97" s="23" t="s">
+      <c r="D97" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E97" s="10" t="s">
         <v>722</v>
-      </c>
-      <c r="D97" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E97" s="10" t="s">
-        <v>723</v>
       </c>
       <c r="F97" s="10"/>
     </row>
@@ -14443,16 +14442,16 @@
         <v>96</v>
       </c>
       <c r="B98" s="10" t="s">
+        <v>723</v>
+      </c>
+      <c r="C98" s="23" t="s">
         <v>724</v>
       </c>
-      <c r="C98" s="23" t="s">
+      <c r="D98" s="10" t="s">
+        <v>461</v>
+      </c>
+      <c r="E98" s="10" t="s">
         <v>725</v>
-      </c>
-      <c r="D98" s="10" t="s">
-        <v>462</v>
-      </c>
-      <c r="E98" s="10" t="s">
-        <v>726</v>
       </c>
       <c r="F98" s="10"/>
     </row>
@@ -14585,7 +14584,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -14595,10 +14594,10 @@
         <v>44</v>
       </c>
       <c r="B2" s="7" t="s">
+        <v>727</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>728</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>729</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -14606,10 +14605,10 @@
         <v>47</v>
       </c>
       <c r="B3" s="8" t="s">
+        <v>729</v>
+      </c>
+      <c r="C3" s="8" t="s">
         <v>730</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>731</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -14617,10 +14616,10 @@
         <v>49</v>
       </c>
       <c r="B4" s="8" t="s">
+        <v>731</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>732</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>733</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -14628,10 +14627,10 @@
         <v>51</v>
       </c>
       <c r="B5" s="8" t="s">
+        <v>733</v>
+      </c>
+      <c r="C5" s="8" t="s">
         <v>734</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>735</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -14639,10 +14638,10 @@
         <v>53</v>
       </c>
       <c r="B6" s="8" t="s">
+        <v>735</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>736</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>737</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -14650,10 +14649,10 @@
         <v>55</v>
       </c>
       <c r="B7" s="8" t="s">
+        <v>737</v>
+      </c>
+      <c r="C7" s="8" t="s">
         <v>738</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>739</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -14661,10 +14660,10 @@
         <v>56</v>
       </c>
       <c r="B8" s="8" t="s">
+        <v>739</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>740</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>741</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -14672,10 +14671,10 @@
         <v>57</v>
       </c>
       <c r="B9" s="8" t="s">
+        <v>741</v>
+      </c>
+      <c r="C9" s="8" t="s">
         <v>742</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>743</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -14683,10 +14682,10 @@
         <v>58</v>
       </c>
       <c r="B10" s="8" t="s">
+        <v>743</v>
+      </c>
+      <c r="C10" s="8" t="s">
         <v>744</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>745</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -14694,10 +14693,10 @@
         <v>59</v>
       </c>
       <c r="B11" s="8" t="s">
+        <v>745</v>
+      </c>
+      <c r="C11" s="8" t="s">
         <v>746</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>747</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add application link for Tether KYC row in Applications sheet
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -1164,7 +1164,6 @@
     <mergeCell ref="A27:D27"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A32:D32"/>
     <mergeCell ref="A20:D20"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="A26:D26"/>
@@ -1176,6 +1175,7 @@
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A28:D28"/>
     <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A32:D32"/>
     <mergeCell ref="B7:D7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8857,7 +8857,11 @@
           <t>Yes — included in application</t>
         </is>
       </c>
-      <c r="L5" s="1" t="n"/>
+      <c r="L5" s="1" t="inlineStr">
+        <is>
+          <t>https://careers.tether.io/o/senior-frontend-developer-kyc-worldwide/c/new</t>
+        </is>
+      </c>
       <c r="M5" s="1" t="n"/>
       <c r="N5" s="1" t="n"/>
       <c r="O5" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Fix stale Wishlist references: rename to Jobs in Dashboard and Status Legend
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -1240,11 +1240,11 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>Wishlist</t>
+          <t>Jobs</t>
         </is>
       </c>
       <c r="B4" s="10">
-        <f>COUNTA(Wishlist!C2:C1000)</f>
+        <f>COUNTA(Jobs!C2:C1000)</f>
         <v/>
       </c>
       <c r="C4" s="1" t="n"/>
@@ -15941,12 +15941,12 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>Wishlist</t>
+          <t>Jobs</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Saved on Wishlist sheet, not yet applied</t>
+          <t>Saved on Jobs sheet, not yet applied</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Clean up Applications notes: remove row numbers from Preparations references
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -8798,7 +8798,7 @@
       </c>
       <c r="Q4" s="1" t="inlineStr">
         <is>
-          <t>Promoted from Preparations row 2</t>
+          <t>Promoted from Preparations</t>
         </is>
       </c>
     </row>
@@ -8876,7 +8876,7 @@
       </c>
       <c r="Q5" s="1" t="inlineStr">
         <is>
-          <t>Promoted from Preparations row 3</t>
+          <t>Promoted from Preparations</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Hide column to Preparations and Applications; generalize hide toggle
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -1164,7 +1164,6 @@
     <mergeCell ref="A27:D27"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A32:D32"/>
     <mergeCell ref="A20:D20"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="A26:D26"/>
@@ -1176,6 +1175,7 @@
     <mergeCell ref="A10:D10"/>
     <mergeCell ref="A28:D28"/>
     <mergeCell ref="B6:D6"/>
+    <mergeCell ref="A32:D32"/>
     <mergeCell ref="B7:D7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8031,7 +8031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="1" min="1" max="1"/>
@@ -8045,7 +8045,7 @@
     <col width="35" customWidth="1" style="1" min="12" max="12"/>
     <col width="25" customWidth="1" style="1" min="13" max="13"/>
     <col width="18" customWidth="1" style="1" min="14" max="14"/>
-    <col width="55" customWidth="1" style="1" min="15" max="15"/>
+    <col width="10" customWidth="1" style="1" min="15" max="15"/>
     <col width="14" customWidth="1" style="1" min="16" max="16"/>
     <col width="18" customWidth="1" style="1" min="17" max="18"/>
     <col width="55" customWidth="1" style="1" min="19" max="19"/>
@@ -8120,6 +8120,11 @@
       <c r="N1" s="21" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="O1" s="21" t="inlineStr">
+        <is>
+          <t>Hide</t>
         </is>
       </c>
     </row>
@@ -8459,7 +8464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q201"/>
+  <dimension ref="A1:R201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="1" min="1" max="1"/>
@@ -8475,6 +8480,7 @@
     <col width="26" customWidth="1" style="1" min="14" max="15"/>
     <col width="13" customWidth="1" style="1" min="16" max="16"/>
     <col width="40" customWidth="1" style="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8561,6 +8567,11 @@
       <c r="Q1" s="7" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="R1" s="7" t="inlineStr">
+        <is>
+          <t>Hide</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Sumsub L3 Support Engineer: Jobs + Applications rows, cover letter
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -1419,7 +1419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M126"/>
+  <dimension ref="A1:M127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="1" min="1" max="1"/>
@@ -7903,6 +7903,66 @@
       <c r="M126" s="20" t="inlineStr">
         <is>
           <t>Originally LinkedIn 4401055938 (Taipei entry-level); swapped to Jakarta Mid via Greenhouse</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="20">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B127" s="20" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="C127" s="20" t="inlineStr">
+        <is>
+          <t>Sumsub</t>
+        </is>
+      </c>
+      <c r="D127" s="20" t="inlineStr">
+        <is>
+          <t>Technical Support Engineer (L3)</t>
+        </is>
+      </c>
+      <c r="E127" s="20" t="inlineStr">
+        <is>
+          <t>https://careers.sumsub.com/jobs/7232843-technical-support-engineer-l3</t>
+        </is>
+      </c>
+      <c r="F127" s="20" t="inlineStr">
+        <is>
+          <t>Sumsub Careers (direct)</t>
+        </is>
+      </c>
+      <c r="G127" s="20" t="inlineStr">
+        <is>
+          <t>✓ Eligible (APAC Remote — Indonesia GMT+7)</t>
+        </is>
+      </c>
+      <c r="H127" s="20" t="inlineStr">
+        <is>
+          <t>Sumsub SDK integrated at Nespay; REST API/SQL/scripting match; learning Mandarin for APAC team</t>
+        </is>
+      </c>
+      <c r="I127" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="J127" s="20" t="n"/>
+      <c r="K127" s="20" t="inlineStr">
+        <is>
+          <t>2. Easy Apply</t>
+        </is>
+      </c>
+      <c r="L127" s="20" t="inlineStr">
+        <is>
+          <t>Hidden</t>
+        </is>
+      </c>
+      <c r="M127" s="20" t="inlineStr">
+        <is>
+          <t>Mandarin required (hard gap — currently learning). cv-default used. 45 wpm typing speed.</t>
         </is>
       </c>
     </row>
@@ -8892,26 +8952,87 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B6" s="1" t="n"/>
-      <c r="C6" s="1" t="n"/>
-      <c r="D6" s="1" t="n"/>
-      <c r="E6" s="1" t="n"/>
-      <c r="F6" s="1" t="n"/>
-      <c r="G6" s="1" t="n"/>
-      <c r="H6" s="1" t="n"/>
-      <c r="I6" s="1" t="n"/>
-      <c r="J6" s="1" t="n"/>
-      <c r="K6" s="1" t="n"/>
-      <c r="L6" s="1" t="n"/>
-      <c r="M6" s="1" t="n"/>
-      <c r="N6" s="1" t="n"/>
-      <c r="O6" s="1" t="n"/>
-      <c r="P6" s="1" t="n"/>
-      <c r="Q6" s="1" t="n"/>
+      <c r="A6" s="20">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>Sumsub</t>
+        </is>
+      </c>
+      <c r="D6" s="22" t="inlineStr">
+        <is>
+          <t>Technical Support Engineer (L3)</t>
+        </is>
+      </c>
+      <c r="E6" s="22" t="inlineStr">
+        <is>
+          <t>100% Remote (APAC)</t>
+        </is>
+      </c>
+      <c r="F6" s="22" t="inlineStr">
+        <is>
+          <t>Sumsub Careers (direct)</t>
+        </is>
+      </c>
+      <c r="G6" s="22" t="inlineStr">
+        <is>
+          <t>https://careers.sumsub.com/jobs/7232843-technical-support-engineer-l3</t>
+        </is>
+      </c>
+      <c r="H6" s="22" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="I6" s="22" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="J6" s="22" t="inlineStr">
+        <is>
+          <t>cv-default.pdf</t>
+        </is>
+      </c>
+      <c r="K6" s="22" t="inlineStr">
+        <is>
+          <t>Yes — cover letter included</t>
+        </is>
+      </c>
+      <c r="L6" s="22" t="n"/>
+      <c r="M6" s="22" t="inlineStr">
+        <is>
+          <t>Not listed</t>
+        </is>
+      </c>
+      <c r="N6" s="22" t="inlineStr">
+        <is>
+          <t>Sumsub Recruiting (via careers portal)</t>
+        </is>
+      </c>
+      <c r="O6" s="22" t="inlineStr">
+        <is>
+          <t>Wait for recruiter response</t>
+        </is>
+      </c>
+      <c r="P6" s="22" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="Q6" s="22" t="inlineStr">
+        <is>
+          <t>cv-default used. 45 wpm typing speed noted. Screenshot uploaded on application page. Promoted from Preparations</t>
+        </is>
+      </c>
+      <c r="R6" s="20" t="n"/>
     </row>
     <row r="7">
       <c r="A7">

</xml_diff>

<commit_message>
chore: remove Aleph Alpha and n8n from Jobs list
Both roles excluded — Aleph Alpha (model evaluation, PyTorch-heavy) and
n8n (Sr AI Engineer) removed from Jobs sheet.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -1428,7 +1428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M128"/>
+  <dimension ref="A1:M126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="1" min="1" max="1"/>
@@ -1896,12 +1896,12 @@
       </c>
       <c r="D9" s="15" t="inlineStr">
         <is>
-          <t>Sr AI Engineer</t>
+          <t>Sr Cloud Engineer</t>
         </is>
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/n8n/d195a389-6af5-4b95-82e5-2258953c7297</t>
+          <t>https://jobs.ashbyhq.com/n8n/640d55b3-3603-42f4-a05b-90962768fd16</t>
         </is>
       </c>
       <c r="F9" s="15" t="inlineStr">
@@ -1926,58 +1926,58 @@
       </c>
       <c r="M9" s="15" t="inlineStr">
         <is>
-          <t>Loc: Remote - Europe | TS/Vue/NodeJS | verify: unclear</t>
+          <t>Loc: NodeJS + TS/JS | Europe remote | verify: unclear</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="15">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="A10">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="C10" s="15" t="inlineStr">
-        <is>
-          <t>n8n</t>
-        </is>
-      </c>
-      <c r="D10" s="15" t="inlineStr">
-        <is>
-          <t>Sr Cloud Engineer</t>
-        </is>
-      </c>
-      <c r="E10" s="16" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/n8n/640d55b3-3603-42f4-a05b-90962768fd16</t>
-        </is>
-      </c>
-      <c r="F10" s="15" t="inlineStr">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Boomi</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>https://boomi.com/boomi-jobs/?gh_jid=5776784004</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
       <c r="G10" s="1" t="n"/>
-      <c r="H10" s="15" t="inlineStr">
-        <is>
-          <t>REMOTE-unverified • Tier A</t>
-        </is>
-      </c>
-      <c r="I10" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="J10" s="17" t="n"/>
-      <c r="K10" s="15" t="inlineStr">
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Tier A</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>3</v>
+      </c>
+      <c r="J10" s="1" t="n"/>
+      <c r="K10" t="inlineStr">
         <is>
           <t>5. Pending</t>
         </is>
       </c>
-      <c r="M10" s="15" t="inlineStr">
-        <is>
-          <t>Loc: NodeJS + TS/JS | Europe remote | verify: unclear</t>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Loc:  | verify: unclear</t>
         </is>
       </c>
     </row>
@@ -1993,17 +1993,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Aleph Alpha</t>
+          <t>Boomi</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Senior AI Software Engineer - Model Evaluation (f/m/d)</t>
+          <t>Senior Software Engineer (Vancouver Hybrid)</t>
         </is>
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/AlephAlpha/1963147c-dc27-416e-b432-065295733bef</t>
+          <t>https://boomi.com/boomi-jobs/?gh_jid=5789784004</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -2044,17 +2044,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Boomi</t>
+          <t>Celonis</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Senior Software Engineer</t>
+          <t>Salesforce Software Engineer</t>
         </is>
       </c>
       <c r="E12" s="13" t="inlineStr">
         <is>
-          <t>https://boomi.com/boomi-jobs/?gh_jid=5776784004</t>
+          <t>https://job-boards.greenhouse.io/celonis/jobs/7681601003?gh_jid=7681601003</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -2095,17 +2095,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Boomi</t>
+          <t>Celonis</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Vancouver Hybrid)</t>
+          <t>Senior Software Engineer - Java</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>https://boomi.com/boomi-jobs/?gh_jid=5789784004</t>
+          <t>https://job-boards.greenhouse.io/celonis/jobs/7559335003?gh_jid=7559335003</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -2151,12 +2151,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Salesforce Software Engineer</t>
+          <t>Senior Software Engineer - Orchestration and Automation</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/celonis/jobs/7681601003?gh_jid=7681601003</t>
+          <t>https://job-boards.greenhouse.io/celonis/jobs/7678804003?gh_jid=7678804003</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -2202,12 +2202,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Java</t>
+          <t>Senior Software Engineer - Provisioning and Licensing</t>
         </is>
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/celonis/jobs/7559335003?gh_jid=7559335003</t>
+          <t>https://job-boards.greenhouse.io/celonis/jobs/7712675003?gh_jid=7712675003</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2248,17 +2248,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Celonis</t>
+          <t>Contentful</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Orchestration and Automation</t>
+          <t>Full Stack Software Engineer III</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/celonis/jobs/7678804003?gh_jid=7678804003</t>
+          <t>https://job-boards.greenhouse.io/contentful/jobs/7875509</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2299,17 +2299,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Celonis</t>
+          <t>Contentful</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Provisioning and Licensing</t>
+          <t>Fullstack Software Engineer (f/m/d)</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/celonis/jobs/7712675003?gh_jid=7712675003</t>
+          <t>https://job-boards.greenhouse.io/contentful/jobs/7557597</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2355,12 +2355,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Full Stack Software Engineer III</t>
+          <t>Senior Backend Engineer - AI Platform (f/m/d)</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/contentful/jobs/7875509</t>
+          <t>https://job-boards.greenhouse.io/contentful/jobs/7753183</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2406,12 +2406,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer (f/m/d)</t>
+          <t>Senior Software Engineer - Backend &amp; Infrastructure (f/m/d)</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/contentful/jobs/7557597</t>
+          <t>https://job-boards.greenhouse.io/contentful/jobs/7760962</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2452,17 +2452,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Contentful</t>
+          <t>Cradle</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Senior Backend Engineer - AI Platform (f/m/d)</t>
+          <t>Backend Software Engineer, Python</t>
         </is>
       </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/contentful/jobs/7753183</t>
+          <t>https://jobs.ashbyhq.com/cradlebio/ae6e6352-28e5-4b2f-b1d9-da7da078f011</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2503,17 +2503,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Contentful</t>
+          <t>Deepgram</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Backend &amp; Infrastructure (f/m/d)</t>
+          <t>Backend Engineer- Inference Services</t>
         </is>
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/contentful/jobs/7760962</t>
+          <t>https://jobs.ashbyhq.com/deepgram/1ab00006-f525-4e2d-a1a9-5cab4264637b</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2554,17 +2554,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Cradle</t>
+          <t>Deepgram</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Backend Software Engineer, Python</t>
+          <t>Backend Software Engineer - Active Learning Team</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/cradlebio/ae6e6352-28e5-4b2f-b1d9-da7da078f011</t>
+          <t>https://jobs.ashbyhq.com/deepgram/0796cc37-96a7-4158-8a00-155962da275a</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2610,12 +2610,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Backend Engineer- Inference Services</t>
+          <t>Backend Software Engineer - Engine Team (Voice Agent)</t>
         </is>
       </c>
       <c r="E23" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/deepgram/1ab00006-f525-4e2d-a1a9-5cab4264637b</t>
+          <t>https://jobs.ashbyhq.com/deepgram/7c7064bb-2bf0-4f64-81cc-14afe79a15c1</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2661,12 +2661,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Backend Software Engineer - Active Learning Team</t>
+          <t>Billing &amp; Analytics Software Engineer</t>
         </is>
       </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/deepgram/0796cc37-96a7-4158-8a00-155962da275a</t>
+          <t>https://jobs.ashbyhq.com/deepgram/378e83b4-28c0-4b4e-8cf0-9355712bd06d</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2712,12 +2712,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Backend Software Engineer - Engine Team (Voice Agent)</t>
+          <t>Software Engineer - Deepgram for Restaurants</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/deepgram/7c7064bb-2bf0-4f64-81cc-14afe79a15c1</t>
+          <t>https://jobs.ashbyhq.com/deepgram/68372d7d-b7a9-439e-a0a7-76690576aba4</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2763,12 +2763,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Billing &amp; Analytics Software Engineer</t>
+          <t>Software Engineer, Voice Agents / AI - Deepgram for Restaurants</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/deepgram/378e83b4-28c0-4b4e-8cf0-9355712bd06d</t>
+          <t>https://jobs.ashbyhq.com/deepgram/4a873ede-8555-42ae-9ddc-ac89afdd7278</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2809,17 +2809,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Deepgram</t>
+          <t>GetYourGuide</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Software Engineer - Deepgram for Restaurants</t>
+          <t>Associate Software Engineer</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/deepgram/68372d7d-b7a9-439e-a0a7-76690576aba4</t>
+          <t>https://getyourguide.careers/jobs/7738914?gh_jid=7738914</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2849,204 +2849,204 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B28" t="inlineStr">
+      <c r="A28" s="18">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
         <is>
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Deepgram</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Software Engineer, Voice Agents / AI - Deepgram for Restaurants</t>
+      <c r="C28" s="18" t="inlineStr">
+        <is>
+          <t>GetYourGuide</t>
+        </is>
+      </c>
+      <c r="D28" s="18" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer (Backend focused)</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/deepgram/4a873ede-8555-42ae-9ddc-ac89afdd7278</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
+          <t>https://getyourguide.careers/jobs/7526177?gh_jid=7526177</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
       <c r="G28" s="1" t="n"/>
-      <c r="H28" t="inlineStr">
+      <c r="H28" s="18" t="inlineStr">
         <is>
           <t>Tier A</t>
         </is>
       </c>
-      <c r="I28" t="n">
+      <c r="I28" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="J28" s="1" t="n"/>
+      <c r="K28" s="18" t="inlineStr">
+        <is>
+          <t>3. Recommended</t>
+        </is>
+      </c>
+      <c r="M28" s="18" t="inlineStr">
+        <is>
+          <t>Loc:  | verify: unclear</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="18">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B29" s="18" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="C29" s="18" t="inlineStr">
+        <is>
+          <t>GetYourGuide</t>
+        </is>
+      </c>
+      <c r="D29" s="18" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer (Backend focused) - Supply</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>https://getyourguide.careers/jobs/7518806?gh_jid=7518806</t>
+        </is>
+      </c>
+      <c r="F29" s="18" t="inlineStr">
+        <is>
+          <t>career-ops scan</t>
+        </is>
+      </c>
+      <c r="G29" s="1" t="n"/>
+      <c r="H29" s="18" t="inlineStr">
+        <is>
+          <t>Tier A</t>
+        </is>
+      </c>
+      <c r="I29" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="J29" s="1" t="n"/>
+      <c r="K29" s="18" t="inlineStr">
+        <is>
+          <t>3. Recommended</t>
+        </is>
+      </c>
+      <c r="M29" s="18" t="inlineStr">
+        <is>
+          <t>Loc:  | verify: unclear</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>GetYourGuide</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer - (Frontend)</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>https://getyourguide.careers/jobs/7728364?gh_jid=7728364</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>career-ops scan</t>
+        </is>
+      </c>
+      <c r="G30" s="1" t="n"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Tier A</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>3</v>
       </c>
-      <c r="J28" s="1" t="n"/>
-      <c r="K28" t="inlineStr">
+      <c r="J30" s="1" t="n"/>
+      <c r="K30" t="inlineStr">
         <is>
           <t>5. Pending</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr">
+      <c r="M30" t="inlineStr">
         <is>
           <t>Loc:  | verify: unclear</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B29" t="inlineStr">
+    <row r="31">
+      <c r="A31">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B31" t="inlineStr">
         <is>
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>GetYourGuide</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Associate Software Engineer</t>
-        </is>
-      </c>
-      <c r="E29" s="13" t="inlineStr">
-        <is>
-          <t>https://getyourguide.careers/jobs/7738914?gh_jid=7738914</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer,  Developer Enablement</t>
+        </is>
+      </c>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>https://getyourguide.careers/jobs/7234277?gh_jid=7234277</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="G29" s="1" t="n"/>
-      <c r="H29" t="inlineStr">
+      <c r="G31" s="1" t="n"/>
+      <c r="H31" t="inlineStr">
         <is>
           <t>Tier A</t>
         </is>
       </c>
-      <c r="I29" t="n">
+      <c r="I31" t="n">
         <v>3</v>
       </c>
-      <c r="J29" s="1" t="n"/>
-      <c r="K29" t="inlineStr">
+      <c r="J31" s="1" t="n"/>
+      <c r="K31" t="inlineStr">
         <is>
           <t>5. Pending</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unclear</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="18">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B30" s="18" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C30" s="18" t="inlineStr">
-        <is>
-          <t>GetYourGuide</t>
-        </is>
-      </c>
-      <c r="D30" s="18" t="inlineStr">
-        <is>
-          <t>Senior Software Engineer (Backend focused)</t>
-        </is>
-      </c>
-      <c r="E30" s="13" t="inlineStr">
-        <is>
-          <t>https://getyourguide.careers/jobs/7526177?gh_jid=7526177</t>
-        </is>
-      </c>
-      <c r="F30" s="18" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G30" s="1" t="n"/>
-      <c r="H30" s="18" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I30" s="18" t="n">
-        <v>5</v>
-      </c>
-      <c r="J30" s="1" t="n"/>
-      <c r="K30" s="18" t="inlineStr">
-        <is>
-          <t>3. Recommended</t>
-        </is>
-      </c>
-      <c r="M30" s="18" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unclear</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="18">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B31" s="18" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C31" s="18" t="inlineStr">
-        <is>
-          <t>GetYourGuide</t>
-        </is>
-      </c>
-      <c r="D31" s="18" t="inlineStr">
-        <is>
-          <t>Senior Software Engineer (Backend focused) - Supply</t>
-        </is>
-      </c>
-      <c r="E31" s="13" t="inlineStr">
-        <is>
-          <t>https://getyourguide.careers/jobs/7518806?gh_jid=7518806</t>
-        </is>
-      </c>
-      <c r="F31" s="18" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G31" s="1" t="n"/>
-      <c r="H31" s="18" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I31" s="18" t="n">
-        <v>5</v>
-      </c>
-      <c r="J31" s="1" t="n"/>
-      <c r="K31" s="18" t="inlineStr">
-        <is>
-          <t>3. Recommended</t>
-        </is>
-      </c>
-      <c r="M31" s="18" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>Loc:  | verify: unclear</t>
         </is>
@@ -3069,12 +3069,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - (Frontend)</t>
+          <t>Senior Software Engineer, Revenue Platform (Backend Focused)</t>
         </is>
       </c>
       <c r="E32" s="13" t="inlineStr">
         <is>
-          <t>https://getyourguide.careers/jobs/7728364?gh_jid=7728364</t>
+          <t>https://getyourguide.careers/jobs/7641281?gh_jid=7641281</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -3120,12 +3120,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Senior Software Engineer,  Developer Enablement</t>
+          <t>Senior Software Engineer, Search Platform</t>
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr">
         <is>
-          <t>https://getyourguide.careers/jobs/7234277?gh_jid=7234277</t>
+          <t>https://getyourguide.careers/jobs/7581804?gh_jid=7581804</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -3171,12 +3171,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Revenue Platform (Backend Focused)</t>
+          <t>Senior Software Engineer, User Profiles (Backend Focused)</t>
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr">
         <is>
-          <t>https://getyourguide.careers/jobs/7641281?gh_jid=7641281</t>
+          <t>https://getyourguide.careers/jobs/7607497?gh_jid=7607497</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -3222,12 +3222,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Search Platform</t>
+          <t>Software Engineer,  Developer Enablement</t>
         </is>
       </c>
       <c r="E35" s="13" t="inlineStr">
         <is>
-          <t>https://getyourguide.careers/jobs/7581804?gh_jid=7581804</t>
+          <t>https://getyourguide.careers/jobs/7768438?gh_jid=7768438</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -3268,17 +3268,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>GetYourGuide</t>
+          <t>Glacis AI</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, User Profiles (Backend Focused)</t>
+          <t>Founding Software Engineer - Agentic AI (On-site)</t>
         </is>
       </c>
       <c r="E36" s="13" t="inlineStr">
         <is>
-          <t>https://getyourguide.careers/jobs/7607497?gh_jid=7607497</t>
+          <t>https://jobs.ashbyhq.com/glacis-ai/796efc69-0c03-45d9-9f54-f3de7bbccde9</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -3319,17 +3319,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>GetYourGuide</t>
+          <t>Glacis AI</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Software Engineer,  Developer Enablement</t>
+          <t>Founding Software Engineer - Agentic AI (Remote)</t>
         </is>
       </c>
       <c r="E37" s="13" t="inlineStr">
         <is>
-          <t>https://getyourguide.careers/jobs/7768438?gh_jid=7768438</t>
+          <t>https://jobs.ashbyhq.com/glacis-ai/feea2cb6-60db-4afa-8358-ba17d05d1cd5</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -3370,17 +3370,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Glacis AI</t>
+          <t>Glean</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Founding Software Engineer - Agentic AI (On-site)</t>
+          <t>Lead Software Engineer, Product Backend</t>
         </is>
       </c>
       <c r="E38" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/glacis-ai/796efc69-0c03-45d9-9f54-f3de7bbccde9</t>
+          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4598386005</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -3421,17 +3421,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Glacis AI</t>
+          <t>Glean</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Founding Software Engineer - Agentic AI (Remote)</t>
+          <t>Software Engineer, AI &amp; Security</t>
         </is>
       </c>
       <c r="E39" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/glacis-ai/feea2cb6-60db-4afa-8358-ba17d05d1cd5</t>
+          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4605446005</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3477,12 +3477,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Lead Software Engineer, Product Backend</t>
+          <t>Software Engineer, AI Infrastructure</t>
         </is>
       </c>
       <c r="E40" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4598386005</t>
+          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4501783005</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3528,12 +3528,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Software Engineer, AI &amp; Security</t>
+          <t>Software Engineer, Agentic Runtime</t>
         </is>
       </c>
       <c r="E41" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4605446005</t>
+          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4616929005</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3579,12 +3579,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Software Engineer, AI Infrastructure</t>
+          <t>Software Engineer, Backend</t>
         </is>
       </c>
       <c r="E42" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4501783005</t>
+          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4006731005</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3630,12 +3630,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Software Engineer, Agentic Runtime</t>
+          <t>Software Engineer, Billing &amp; Revenue Platform</t>
         </is>
       </c>
       <c r="E43" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4616929005</t>
+          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4675862005</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -3681,12 +3681,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Software Engineer, Backend</t>
+          <t>Software Engineer, Context Platform</t>
         </is>
       </c>
       <c r="E44" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4006731005</t>
+          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4638008005</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3732,12 +3732,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Software Engineer, Billing &amp; Revenue Platform</t>
+          <t>Software Engineer, Data Foundations</t>
         </is>
       </c>
       <c r="E45" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4675862005</t>
+          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4637208005</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -3783,12 +3783,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Software Engineer, Context Platform</t>
+          <t>Software Engineer, Developer Productivity</t>
         </is>
       </c>
       <c r="E46" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4638008005</t>
+          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4614706005</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -3834,12 +3834,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Software Engineer, Data Foundations</t>
+          <t>Software Engineer, Frontend</t>
         </is>
       </c>
       <c r="E47" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4637208005</t>
+          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4006733005</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -3885,12 +3885,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Software Engineer, Developer Productivity</t>
+          <t>Software Engineer, Fullstack</t>
         </is>
       </c>
       <c r="E48" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4614706005</t>
+          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4006734005</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -3936,12 +3936,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Software Engineer, Frontend</t>
+          <t>Software Engineer, Insights</t>
         </is>
       </c>
       <c r="E49" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4006733005</t>
+          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4659229005</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -3987,12 +3987,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Software Engineer, Fullstack</t>
+          <t>Software Engineer, Machine Learning</t>
         </is>
       </c>
       <c r="E50" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4006734005</t>
+          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4012745005</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -4038,12 +4038,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Software Engineer, Insights</t>
+          <t>Software Engineer, Platform</t>
         </is>
       </c>
       <c r="E51" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4659229005</t>
+          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4636739005</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -4089,12 +4089,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Software Engineer, Machine Learning</t>
+          <t>Software Engineer, Platform Security</t>
         </is>
       </c>
       <c r="E52" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4012745005</t>
+          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4436194005</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -4140,12 +4140,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Software Engineer, Platform</t>
+          <t>Software Engineer, Product Backend</t>
         </is>
       </c>
       <c r="E53" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4636739005</t>
+          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4428090005</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -4186,17 +4186,17 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Glean</t>
+          <t>Helsing</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Software Engineer, Platform Security</t>
+          <t>Software Engineer</t>
         </is>
       </c>
       <c r="E54" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4436194005</t>
+          <t>https://helsing.ai/jobs/4737931101?gh_jid=4737931101</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -4237,17 +4237,17 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Glean</t>
+          <t>Helsing</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Software Engineer, Product Backend</t>
+          <t>Software Engineer - Airborne Mission Systems</t>
         </is>
       </c>
       <c r="E55" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/gleanwork/jobs/4428090005</t>
+          <t>https://helsing.ai/jobs/4741565101?gh_jid=4741565101</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -4293,12 +4293,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Software Engineer</t>
+          <t>Software Engineer - Autonomous Air System V&amp;V</t>
         </is>
       </c>
       <c r="E56" s="13" t="inlineStr">
         <is>
-          <t>https://helsing.ai/jobs/4737931101?gh_jid=4737931101</t>
+          <t>https://helsing.ai/jobs/4741219101?gh_jid=4741219101</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -4344,12 +4344,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Software Engineer - Airborne Mission Systems</t>
+          <t>Software Engineer - Autonomous Air Systems</t>
         </is>
       </c>
       <c r="E57" s="13" t="inlineStr">
         <is>
-          <t>https://helsing.ai/jobs/4741565101?gh_jid=4741565101</t>
+          <t>https://helsing.ai/jobs/4741571101?gh_jid=4741571101</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -4395,12 +4395,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Software Engineer - Autonomous Air System V&amp;V</t>
+          <t>Software Engineer - Backend</t>
         </is>
       </c>
       <c r="E58" s="13" t="inlineStr">
         <is>
-          <t>https://helsing.ai/jobs/4741219101?gh_jid=4741219101</t>
+          <t>https://helsing.ai/jobs/4125061101?gh_jid=4125061101</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -4446,12 +4446,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Software Engineer - Autonomous Air Systems</t>
+          <t>Software Engineer - Frontend</t>
         </is>
       </c>
       <c r="E59" s="13" t="inlineStr">
         <is>
-          <t>https://helsing.ai/jobs/4741571101?gh_jid=4741571101</t>
+          <t>https://helsing.ai/jobs/4126378101?gh_jid=4126378101</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -4497,12 +4497,12 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Software Engineer - Backend</t>
+          <t>Software Engineer - Frontend Autonomous Air System V&amp;V</t>
         </is>
       </c>
       <c r="E60" s="13" t="inlineStr">
         <is>
-          <t>https://helsing.ai/jobs/4125061101?gh_jid=4125061101</t>
+          <t>https://helsing.ai/jobs/4741224101?gh_jid=4741224101</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -4548,12 +4548,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Software Engineer - Frontend</t>
+          <t>Software Engineer - Ground to Air HMI</t>
         </is>
       </c>
       <c r="E61" s="13" t="inlineStr">
         <is>
-          <t>https://helsing.ai/jobs/4126378101?gh_jid=4126378101</t>
+          <t>https://helsing.ai/jobs/4741242101?gh_jid=4741242101</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -4599,12 +4599,12 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Software Engineer - Frontend Autonomous Air System V&amp;V</t>
+          <t>Software Engineer - Infrastructure</t>
         </is>
       </c>
       <c r="E62" s="13" t="inlineStr">
         <is>
-          <t>https://helsing.ai/jobs/4741224101?gh_jid=4741224101</t>
+          <t>https://helsing.ai/jobs/4729613101?gh_jid=4729613101</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -4645,17 +4645,17 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Helsing</t>
+          <t>Hootsuite</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Software Engineer - Ground to Air HMI</t>
+          <t>Intermediate Software Developer, DevOps</t>
         </is>
       </c>
       <c r="E63" s="13" t="inlineStr">
         <is>
-          <t>https://helsing.ai/jobs/4741242101?gh_jid=4741242101</t>
+          <t>https://careers.hootsuite.com/job/?gh_jid=7582752</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -4696,17 +4696,17 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Helsing</t>
+          <t>Hootsuite</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Software Engineer - Infrastructure</t>
+          <t>Junior Software Developer, Backend</t>
         </is>
       </c>
       <c r="E64" s="13" t="inlineStr">
         <is>
-          <t>https://helsing.ai/jobs/4729613101?gh_jid=4729613101</t>
+          <t>https://careers.hootsuite.com/job/?gh_jid=7851293</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -4752,12 +4752,12 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Intermediate Software Developer, DevOps</t>
+          <t>Junior Software Developer, Frontend</t>
         </is>
       </c>
       <c r="E65" s="13" t="inlineStr">
         <is>
-          <t>https://careers.hootsuite.com/job/?gh_jid=7582752</t>
+          <t>https://careers.hootsuite.com/job/?gh_jid=7821814</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -4803,12 +4803,12 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Junior Software Developer, Backend</t>
+          <t>Senior Software Developer, DevOps</t>
         </is>
       </c>
       <c r="E66" s="13" t="inlineStr">
         <is>
-          <t>https://careers.hootsuite.com/job/?gh_jid=7851293</t>
+          <t>https://careers.hootsuite.com/job/?gh_jid=7741151</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -4849,17 +4849,17 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Hootsuite</t>
+          <t>Intercom</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Junior Software Developer, Frontend</t>
+          <t>Forward Deployed Software Engineer</t>
         </is>
       </c>
       <c r="E67" s="13" t="inlineStr">
         <is>
-          <t>https://careers.hootsuite.com/job/?gh_jid=7821814</t>
+          <t>https://job-boards.greenhouse.io/intercom/jobs/7556413</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -4900,17 +4900,17 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Hootsuite</t>
+          <t>Intercom</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Senior Software Developer, DevOps</t>
+          <t>Full-Stack Marketer, Customer Advocacy</t>
         </is>
       </c>
       <c r="E68" s="13" t="inlineStr">
         <is>
-          <t>https://careers.hootsuite.com/job/?gh_jid=7741151</t>
+          <t>https://job-boards.greenhouse.io/intercom/jobs/7774295</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -4956,12 +4956,12 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Forward Deployed Software Engineer</t>
+          <t>Senior Full Stack Engineer - Team Web</t>
         </is>
       </c>
       <c r="E69" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/intercom/jobs/7556413</t>
+          <t>https://job-boards.greenhouse.io/intercom/jobs/7274831</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -5007,12 +5007,12 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Full-Stack Marketer, Customer Advocacy</t>
+          <t>Senior Software Engineer</t>
         </is>
       </c>
       <c r="E70" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/intercom/jobs/7774295</t>
+          <t>https://job-boards.greenhouse.io/intercom/jobs/5082494</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -5058,12 +5058,12 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - Team Web</t>
+          <t>Software Engineer</t>
         </is>
       </c>
       <c r="E71" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/intercom/jobs/7274831</t>
+          <t>https://job-boards.greenhouse.io/intercom/jobs/7371989</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -5104,17 +5104,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Intercom</t>
+          <t>Legora</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Senior Software Engineer</t>
+          <t>React Native Engineer</t>
         </is>
       </c>
       <c r="E72" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/intercom/jobs/5082494</t>
+          <t>https://jobs.ashbyhq.com/legora/98e93c0a-b4c9-4083-8037-9c83a22e5bec</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -5155,17 +5155,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Intercom</t>
+          <t>Legora</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Software Engineer</t>
+          <t>Senior Backend Engineer</t>
         </is>
       </c>
       <c r="E73" s="13" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/intercom/jobs/7371989</t>
+          <t>https://jobs.ashbyhq.com/legora/e1b04e64-3eff-4583-b083-dcebc754f80a</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -5211,12 +5211,12 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>React Native Engineer</t>
+          <t>Senior Software Engineer</t>
         </is>
       </c>
       <c r="E74" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/legora/98e93c0a-b4c9-4083-8037-9c83a22e5bec</t>
+          <t>https://jobs.ashbyhq.com/legora/056d9fc6-431c-40b6-b6ff-3a147b23b5c8</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -5262,12 +5262,12 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Senior Backend Engineer</t>
+          <t>Software Engineer</t>
         </is>
       </c>
       <c r="E75" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/legora/e1b04e64-3eff-4583-b083-dcebc754f80a</t>
+          <t>https://jobs.ashbyhq.com/legora/9a04bbd8-0583-48de-9606-431c01079b8b</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -5313,12 +5313,12 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Senior Software Engineer</t>
+          <t>Software Engineer (AI Focus)</t>
         </is>
       </c>
       <c r="E76" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/legora/056d9fc6-431c-40b6-b6ff-3a147b23b5c8</t>
+          <t>https://jobs.ashbyhq.com/legora/f81a4b5e-7ef3-4946-a147-f6c0645e98ca</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -5364,12 +5364,12 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Software Engineer</t>
+          <t>Software Engineer - AI Enablement &amp; Workplace Technology</t>
         </is>
       </c>
       <c r="E77" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/legora/9a04bbd8-0583-48de-9606-431c01079b8b</t>
+          <t>https://jobs.ashbyhq.com/legora/e4ce19dc-e800-42cd-835f-dcc43b96d004</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -5410,17 +5410,17 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Legora</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Software Engineer (AI Focus)</t>
+          <t>Backend Product Engineer</t>
         </is>
       </c>
       <c r="E78" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/legora/f81a4b5e-7ef3-4946-a147-f6c0645e98ca</t>
+          <t>https://jobs.ashbyhq.com/lovable/e54d33ea-5f02-48b6-b75e-76ae704af693</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -5461,17 +5461,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Legora</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Software Engineer - AI Enablement &amp; Workplace Technology</t>
+          <t>FullStack Engineer - Product Security</t>
         </is>
       </c>
       <c r="E79" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/legora/e4ce19dc-e800-42cd-835f-dcc43b96d004</t>
+          <t>https://jobs.ashbyhq.com/lovable/1f86955c-2748-4cd6-bd69-7e5c2c3fe465</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -5517,12 +5517,12 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Backend Product Engineer</t>
+          <t>Fullstack Engineer - AI Code Security</t>
         </is>
       </c>
       <c r="E80" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/lovable/e54d33ea-5f02-48b6-b75e-76ae704af693</t>
+          <t>https://jobs.ashbyhq.com/lovable/e27e931e-79f3-483a-b543-57e42633ac5c</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -5568,12 +5568,12 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>FullStack Engineer - Product Security</t>
+          <t>Fullstack Engineer - Lovable Apps Platform Team</t>
         </is>
       </c>
       <c r="E81" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/lovable/1f86955c-2748-4cd6-bd69-7e5c2c3fe465</t>
+          <t>https://jobs.ashbyhq.com/lovable/0d76fa8d-4aaa-41e2-b5d8-d316648bdff8</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -5619,12 +5619,12 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Fullstack Engineer - AI Code Security</t>
+          <t>Fullstack Growth Engineer</t>
         </is>
       </c>
       <c r="E82" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/lovable/e27e931e-79f3-483a-b543-57e42633ac5c</t>
+          <t>https://jobs.ashbyhq.com/lovable/581951b9-537e-49d5-89fb-dd74cdf3256c</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -5670,12 +5670,12 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Fullstack Engineer - Lovable Apps Platform Team</t>
+          <t>Fullstack Product Engineer</t>
         </is>
       </c>
       <c r="E83" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/lovable/0d76fa8d-4aaa-41e2-b5d8-d316648bdff8</t>
+          <t>https://jobs.ashbyhq.com/lovable/b9894757-c26b-4c5e-9ee8-3e18d9947fd6</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -5721,12 +5721,12 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Fullstack Growth Engineer</t>
+          <t>Software Engineer - Infrastructure</t>
         </is>
       </c>
       <c r="E84" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/lovable/581951b9-537e-49d5-89fb-dd74cdf3256c</t>
+          <t>https://jobs.ashbyhq.com/lovable/920b4099-00bc-4d5e-9469-2c955ef3a662</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -5767,17 +5767,17 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Mistral AI</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Fullstack Product Engineer</t>
+          <t>Applied AI Engineer, Fullstack Software Engineer - EMEA</t>
         </is>
       </c>
       <c r="E85" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/lovable/b9894757-c26b-4c5e-9ee8-3e18d9947fd6</t>
+          <t>https://jobs.lever.co/mistral/aceffeba-c4e9-4b3b-adff-e7e78b986c5c</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -5818,17 +5818,17 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Mistral AI</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Software Engineer - Infrastructure</t>
+          <t>Applied AI, Fullstack Software Engineer, Critical and Sovereign Institutions, Paris</t>
         </is>
       </c>
       <c r="E86" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/lovable/920b4099-00bc-4d5e-9469-2c955ef3a662</t>
+          <t>https://jobs.lever.co/mistral/de237900-114c-4e39-aa19-671bb3201eee</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -5874,12 +5874,12 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Applied AI Engineer, Fullstack Software Engineer - EMEA</t>
+          <t>Mistral Cloud - Software Engineer, Backend (Golang)</t>
         </is>
       </c>
       <c r="E87" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/mistral/aceffeba-c4e9-4b3b-adff-e7e78b986c5c</t>
+          <t>https://jobs.lever.co/mistral/64c9a48e-6d23-4090-bf0f-5a979830fbaf</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -5925,12 +5925,12 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Applied AI, Fullstack Software Engineer, Critical and Sovereign Institutions, Paris</t>
+          <t>Research Software Engineer - Paris/London</t>
         </is>
       </c>
       <c r="E88" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/mistral/de237900-114c-4e39-aa19-671bb3201eee</t>
+          <t>https://jobs.lever.co/mistral/df0d75c1-97ef-4e50-85e6-0ffd8f5b7d7c</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -5976,12 +5976,12 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Mistral Cloud - Software Engineer, Backend (Golang)</t>
+          <t>Software Engineer,  Frontend</t>
         </is>
       </c>
       <c r="E89" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/mistral/64c9a48e-6d23-4090-bf0f-5a979830fbaf</t>
+          <t>https://jobs.lever.co/mistral/305432ef-27ac-4012-a893-a662813ac6e9</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -6027,12 +6027,12 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Research Software Engineer - Paris/London</t>
+          <t>Software Engineer, Backend (London)</t>
         </is>
       </c>
       <c r="E90" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/mistral/df0d75c1-97ef-4e50-85e6-0ffd8f5b7d7c</t>
+          <t>https://jobs.lever.co/mistral/77b8339f-da37-4f38-b554-1d154f72ca8f</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -6078,12 +6078,12 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Software Engineer,  Frontend</t>
+          <t>Software Engineer, Backend (New-York)</t>
         </is>
       </c>
       <c r="E91" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/mistral/305432ef-27ac-4012-a893-a662813ac6e9</t>
+          <t>https://jobs.lever.co/mistral/f2e8ba75-bf5a-4976-bb96-c5d3e0f99366</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -6129,12 +6129,12 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Software Engineer, Backend (London)</t>
+          <t>Software Engineer, Backend (Paris)</t>
         </is>
       </c>
       <c r="E92" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/mistral/77b8339f-da37-4f38-b554-1d154f72ca8f</t>
+          <t>https://jobs.lever.co/mistral/e76d2957-2bf6-4d8f-90a2-29bf9a927823</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -6180,12 +6180,12 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Software Engineer, Backend (New-York)</t>
+          <t>Software Engineer, Deployment Infrastructure</t>
         </is>
       </c>
       <c r="E93" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/mistral/f2e8ba75-bf5a-4976-bb96-c5d3e0f99366</t>
+          <t>https://jobs.lever.co/mistral/31364497-4081-454a-b50c-12d15daf6876</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -6231,12 +6231,12 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Software Engineer, Backend (Paris)</t>
+          <t>Software Engineer, DevEx</t>
         </is>
       </c>
       <c r="E94" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/mistral/e76d2957-2bf6-4d8f-90a2-29bf9a927823</t>
+          <t>https://jobs.lever.co/mistral/c9e16eb0-0cb9-423d-8495-a96d10782622</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -6282,12 +6282,12 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Software Engineer, Deployment Infrastructure</t>
+          <t>Software Engineer, Enterprise Agents</t>
         </is>
       </c>
       <c r="E95" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/mistral/31364497-4081-454a-b50c-12d15daf6876</t>
+          <t>https://jobs.lever.co/mistral/3eef7a1f-cd9d-430e-ac67-9d52534c346a</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -6333,12 +6333,12 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Software Engineer, DevEx</t>
+          <t>Software Engineer, Knowledge and Search</t>
         </is>
       </c>
       <c r="E96" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/mistral/c9e16eb0-0cb9-423d-8495-a96d10782622</t>
+          <t>https://jobs.lever.co/mistral/70d5293a-9183-40d9-874a-cc08a14d5de6</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -6384,12 +6384,12 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Software Engineer, Enterprise Agents</t>
+          <t>Software Engineer, QA</t>
         </is>
       </c>
       <c r="E97" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/mistral/3eef7a1f-cd9d-430e-ac67-9d52534c346a</t>
+          <t>https://jobs.lever.co/mistral/03918386-cb56-4e4d-afa8-1f8b7676a4a6</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -6430,17 +6430,17 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Mistral AI</t>
+          <t>N26</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Software Engineer, Knowledge and Search</t>
+          <t>Lead Backend Engineer - Assistance</t>
         </is>
       </c>
       <c r="E98" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/mistral/70d5293a-9183-40d9-874a-cc08a14d5de6</t>
+          <t>https://n26.com/en-eu/careers/positions/7686804?gh_jid=7686804</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -6481,17 +6481,17 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Mistral AI</t>
+          <t>N26</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Software Engineer, QA</t>
+          <t>Senior Backend Engineer</t>
         </is>
       </c>
       <c r="E99" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/mistral/03918386-cb56-4e4d-afa8-1f8b7676a4a6</t>
+          <t>https://n26.com/en-eu/careers/positions/7811482?gh_jid=7811482</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -6537,12 +6537,12 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Lead Backend Engineer - Assistance</t>
+          <t>Senior Full-Stack Security Automation Engineer</t>
         </is>
       </c>
       <c r="E100" s="13" t="inlineStr">
         <is>
-          <t>https://n26.com/en-eu/careers/positions/7686804?gh_jid=7686804</t>
+          <t>https://n26.com/en-eu/careers/positions/7577884?gh_jid=7577884</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -6588,12 +6588,12 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Senior Backend Engineer</t>
+          <t>Senior Product Manager - Payments Platform (Backend)</t>
         </is>
       </c>
       <c r="E101" s="13" t="inlineStr">
         <is>
-          <t>https://n26.com/en-eu/careers/positions/7811482?gh_jid=7811482</t>
+          <t>https://n26.com/en-eu/careers/positions/7140058?gh_jid=7140058</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -6634,17 +6634,17 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>N26</t>
+          <t>n8n</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Security Automation Engineer</t>
+          <t>Senior Product Engineer (TS/NodeJS/Vue)</t>
         </is>
       </c>
       <c r="E102" s="13" t="inlineStr">
         <is>
-          <t>https://n26.com/en-eu/careers/positions/7577884?gh_jid=7577884</t>
+          <t>https://jobs.ashbyhq.com/n8n/896c58a8-0388-4037-b265-82b15633a568</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -6685,17 +6685,17 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>N26</t>
+          <t>Pigment</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Senior Product Manager - Payments Platform (Backend)</t>
+          <t>Engineering Manager - Front-end background</t>
         </is>
       </c>
       <c r="E103" s="13" t="inlineStr">
         <is>
-          <t>https://n26.com/en-eu/careers/positions/7140058?gh_jid=7140058</t>
+          <t>https://jobs.lever.co/pigment/4c49978c-2aff-45cb-add9-921c8fc41b2b</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -6736,17 +6736,17 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>n8n</t>
+          <t>Pigment</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Senior Product Engineer (TS/NodeJS/Vue)</t>
+          <t>Front-end Engineer</t>
         </is>
       </c>
       <c r="E104" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/n8n/896c58a8-0388-4037-b265-82b15633a568</t>
+          <t>https://jobs.lever.co/pigment/bbb9ea1a-fbb2-44ca-9195-770199323725</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -6792,12 +6792,12 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Engineering Manager - Front-end background</t>
+          <t>Fullstack Software Engineer</t>
         </is>
       </c>
       <c r="E105" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/pigment/4c49978c-2aff-45cb-add9-921c8fc41b2b</t>
+          <t>https://jobs.lever.co/pigment/d41c13a1-9fa5-4d4e-8f50-d3c10852c8e0</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -6843,12 +6843,12 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Front-end Engineer</t>
+          <t>Senior Backend Software Engineer</t>
         </is>
       </c>
       <c r="E106" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/pigment/bbb9ea1a-fbb2-44ca-9195-770199323725</t>
+          <t>https://jobs.lever.co/pigment/5afbde72-ff75-4841-9ab5-2a95decbc6f2</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -6894,12 +6894,12 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer</t>
+          <t>Senior Backend Software Engineer (UK)</t>
         </is>
       </c>
       <c r="E107" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/pigment/d41c13a1-9fa5-4d4e-8f50-d3c10852c8e0</t>
+          <t>https://jobs.lever.co/pigment/068f30f5-4343-4a85-ba52-a35ca2e2581f</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -6945,12 +6945,12 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Senior Backend Software Engineer</t>
+          <t>Senior Frontend Engineer (UK)</t>
         </is>
       </c>
       <c r="E108" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/pigment/5afbde72-ff75-4841-9ab5-2a95decbc6f2</t>
+          <t>https://jobs.lever.co/pigment/cb04a184-0756-461c-b4b3-58f779a82b09</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -6996,12 +6996,12 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Senior Backend Software Engineer (UK)</t>
+          <t>Senior Frontend Software Engineer</t>
         </is>
       </c>
       <c r="E109" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/pigment/068f30f5-4343-4a85-ba52-a35ca2e2581f</t>
+          <t>https://jobs.lever.co/pigment/24e3e6d8-56a3-4917-acbe-ec85d0c8cf13</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -7031,51 +7031,51 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B110" t="inlineStr">
+      <c r="A110" s="18">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B110" s="18" t="inlineStr">
         <is>
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr">
+      <c r="C110" s="18" t="inlineStr">
         <is>
           <t>Pigment</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>Senior Frontend Engineer (UK)</t>
+      <c r="D110" s="18" t="inlineStr">
+        <is>
+          <t>Senior Fullstack Software Engineer</t>
         </is>
       </c>
       <c r="E110" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/pigment/cb04a184-0756-461c-b4b3-58f779a82b09</t>
-        </is>
-      </c>
-      <c r="F110" t="inlineStr">
+          <t>https://jobs.lever.co/pigment/d4f42533-dabb-49c5-9846-24abbb3f61d8</t>
+        </is>
+      </c>
+      <c r="F110" s="18" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
       <c r="G110" s="1" t="n"/>
-      <c r="H110" t="inlineStr">
+      <c r="H110" s="18" t="inlineStr">
         <is>
           <t>Tier A</t>
         </is>
       </c>
-      <c r="I110" t="n">
-        <v>3</v>
+      <c r="I110" s="18" t="n">
+        <v>5</v>
       </c>
       <c r="J110" s="1" t="n"/>
-      <c r="K110" t="inlineStr">
-        <is>
-          <t>5. Pending</t>
-        </is>
-      </c>
-      <c r="M110" t="inlineStr">
+      <c r="K110" s="18" t="inlineStr">
+        <is>
+          <t>3. Recommended</t>
+        </is>
+      </c>
+      <c r="M110" s="18" t="inlineStr">
         <is>
           <t>Loc:  | verify: unclear</t>
         </is>
@@ -7093,17 +7093,17 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Pigment</t>
+          <t>Qonto</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Senior Frontend Software Engineer</t>
+          <t>Full-Stack Engineer - People Products (Freelance)</t>
         </is>
       </c>
       <c r="E111" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/pigment/24e3e6d8-56a3-4917-acbe-ec85d0c8cf13</t>
+          <t>https://jobs.lever.co/qonto/21bf0ae1-b5b1-428a-b1e6-2cdb9476987e</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -7133,51 +7133,51 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="18">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B112" s="18" t="inlineStr">
+      <c r="A112">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B112" t="inlineStr">
         <is>
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="C112" s="18" t="inlineStr">
-        <is>
-          <t>Pigment</t>
-        </is>
-      </c>
-      <c r="D112" s="18" t="inlineStr">
-        <is>
-          <t>Senior Fullstack Software Engineer</t>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Qonto</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Product Engineer - Accounting Domain (Frontend: React)</t>
         </is>
       </c>
       <c r="E112" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/pigment/d4f42533-dabb-49c5-9846-24abbb3f61d8</t>
-        </is>
-      </c>
-      <c r="F112" s="18" t="inlineStr">
+          <t>https://jobs.lever.co/qonto/5e9f184e-0785-41d3-9a41-28b4dc317c87</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
       <c r="G112" s="1" t="n"/>
-      <c r="H112" s="18" t="inlineStr">
+      <c r="H112" t="inlineStr">
         <is>
           <t>Tier A</t>
         </is>
       </c>
-      <c r="I112" s="18" t="n">
-        <v>5</v>
+      <c r="I112" t="n">
+        <v>3</v>
       </c>
       <c r="J112" s="1" t="n"/>
-      <c r="K112" s="18" t="inlineStr">
-        <is>
-          <t>3. Recommended</t>
-        </is>
-      </c>
-      <c r="M112" s="18" t="inlineStr">
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>5. Pending</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
         <is>
           <t>Loc:  | verify: unclear</t>
         </is>
@@ -7200,12 +7200,12 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Full-Stack Engineer - People Products (Freelance)</t>
+          <t>Software Engineer (Engineering Efficiency) - remote friendly</t>
         </is>
       </c>
       <c r="E113" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/qonto/21bf0ae1-b5b1-428a-b1e6-2cdb9476987e</t>
+          <t>https://jobs.lever.co/qonto/1f945bad-2c45-4ac1-be06-a219dc9e1a93</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -7246,17 +7246,17 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Qonto</t>
+          <t>Synthesia</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Product Engineer - Accounting Domain (Frontend: React)</t>
+          <t>Software Engineer, Back End Leaning (Tech Lead Level)</t>
         </is>
       </c>
       <c r="E114" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/qonto/5e9f184e-0785-41d3-9a41-28b4dc317c87</t>
+          <t>https://jobs.ashbyhq.com/synthesia/bf515974-3bab-46cb-85fd-5bacafcc1a91</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -7297,17 +7297,17 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Qonto</t>
+          <t>Synthesia</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Software Engineer (Engineering Efficiency) - remote friendly</t>
+          <t>Software Engineer, Front End Leaning (Accessibility)</t>
         </is>
       </c>
       <c r="E115" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/qonto/1f945bad-2c45-4ac1-be06-a219dc9e1a93</t>
+          <t>https://jobs.ashbyhq.com/synthesia/e1fedec8-ea12-4e7f-95e1-475b95dbd517</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -7353,12 +7353,12 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Software Engineer, Back End Leaning (Tech Lead Level)</t>
+          <t>Software Engineer, Front End Leaning (Tech Lead level)</t>
         </is>
       </c>
       <c r="E116" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/synthesia/bf515974-3bab-46cb-85fd-5bacafcc1a91</t>
+          <t>https://jobs.ashbyhq.com/synthesia/22a00ec6-ac40-4b87-97bc-a0f7bf724be7</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -7404,12 +7404,12 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Software Engineer, Front End Leaning (Accessibility)</t>
+          <t>Webflow Developer / Front-End Engineer</t>
         </is>
       </c>
       <c r="E117" s="13" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/synthesia/e1fedec8-ea12-4e7f-95e1-475b95dbd517</t>
+          <t>https://jobs.ashbyhq.com/synthesia/dcc970b0-9043-4fc6-b628-3b8dad021c84</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -7450,17 +7450,17 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Synthesia</t>
+          <t>Zapier</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Software Engineer, Front End Leaning (Tech Lead level)</t>
-        </is>
-      </c>
-      <c r="E118" s="13" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/synthesia/22a00ec6-ac40-4b87-97bc-a0f7bf724be7</t>
+          <t>Software Engineer — Release Engineering</t>
+        </is>
+      </c>
+      <c r="E118" s="19" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/zapier/6948a0e6-a580-4e9d-b109-20652d9a1507</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -7480,116 +7480,112 @@
       <c r="J118" s="1" t="n"/>
       <c r="K118" t="inlineStr">
         <is>
+          <t>1. Apply</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>Loc:  | verify: unclear</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="20">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B119" s="20" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C119" s="20" t="inlineStr">
+        <is>
+          <t>N26</t>
+        </is>
+      </c>
+      <c r="D119" s="20" t="inlineStr">
+        <is>
+          <t>Backend Engineer - Acquire</t>
+        </is>
+      </c>
+      <c r="E119" s="20" t="inlineStr">
+        <is>
+          <t>https://n26.com/en-eu/careers/positions/7742395?gh_jid=7742395</t>
+        </is>
+      </c>
+      <c r="F119" s="20" t="inlineStr">
+        <is>
+          <t>career-ops scan</t>
+        </is>
+      </c>
+      <c r="G119" s="20" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H119" s="20" t="inlineStr">
+        <is>
+          <t>Loc: Berlin</t>
+        </is>
+      </c>
+      <c r="I119" s="20" t="n"/>
+      <c r="J119" s="20" t="n"/>
+      <c r="K119" s="20" t="inlineStr">
+        <is>
           <t>5. Pending</t>
         </is>
       </c>
-      <c r="M118" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unclear</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>Synthesia</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>Webflow Developer / Front-End Engineer</t>
-        </is>
-      </c>
-      <c r="E119" s="13" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/synthesia/dcc970b0-9043-4fc6-b628-3b8dad021c84</t>
-        </is>
-      </c>
-      <c r="F119" t="inlineStr">
+      <c r="M119" s="20" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="20">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B120" s="20" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C120" s="20" t="inlineStr">
+        <is>
+          <t>N26</t>
+        </is>
+      </c>
+      <c r="D120" s="20" t="inlineStr">
+        <is>
+          <t>Backend Engineer - Engagement</t>
+        </is>
+      </c>
+      <c r="E120" s="20" t="inlineStr">
+        <is>
+          <t>https://n26.com/en-eu/careers/positions/7640893?gh_jid=7640893</t>
+        </is>
+      </c>
+      <c r="F120" s="20" t="inlineStr">
         <is>
           <t>career-ops scan</t>
         </is>
       </c>
-      <c r="G119" s="1" t="n"/>
-      <c r="H119" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I119" t="n">
-        <v>3</v>
-      </c>
-      <c r="J119" s="1" t="n"/>
-      <c r="K119" t="inlineStr">
+      <c r="G120" s="20" t="inlineStr">
+        <is>
+          <t>Visa sponsorship needed</t>
+        </is>
+      </c>
+      <c r="H120" s="20" t="inlineStr">
+        <is>
+          <t>Loc: Berlin / Barcelona</t>
+        </is>
+      </c>
+      <c r="I120" s="20" t="n"/>
+      <c r="J120" s="20" t="n"/>
+      <c r="K120" s="20" t="inlineStr">
         <is>
           <t>5. Pending</t>
         </is>
       </c>
-      <c r="M119" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unclear</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>Zapier</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>Software Engineer — Release Engineering</t>
-        </is>
-      </c>
-      <c r="E120" s="19" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/zapier/6948a0e6-a580-4e9d-b109-20652d9a1507</t>
-        </is>
-      </c>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t>career-ops scan</t>
-        </is>
-      </c>
-      <c r="G120" s="1" t="n"/>
-      <c r="H120" t="inlineStr">
-        <is>
-          <t>Tier A</t>
-        </is>
-      </c>
-      <c r="I120" t="n">
-        <v>3</v>
-      </c>
-      <c r="J120" s="1" t="n"/>
-      <c r="K120" t="inlineStr">
-        <is>
-          <t>1. Apply</t>
-        </is>
-      </c>
-      <c r="M120" t="inlineStr">
-        <is>
-          <t>Loc:  | verify: unclear</t>
-        </is>
-      </c>
+      <c r="M120" s="20" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="20">
@@ -7603,22 +7599,22 @@
       </c>
       <c r="C121" s="20" t="inlineStr">
         <is>
-          <t>N26</t>
+          <t>Shippio</t>
         </is>
       </c>
       <c r="D121" s="20" t="inlineStr">
         <is>
-          <t>Backend Engineer - Acquire</t>
+          <t>Senior Front-End Engineer</t>
         </is>
       </c>
       <c r="E121" s="20" t="inlineStr">
         <is>
-          <t>https://n26.com/en-eu/careers/positions/7742395?gh_jid=7742395</t>
+          <t>https://cs.gittap.jp/jobs/1719</t>
         </is>
       </c>
       <c r="F121" s="20" t="inlineStr">
         <is>
-          <t>career-ops scan</t>
+          <t>career-ops scan / gittap.jp</t>
         </is>
       </c>
       <c r="G121" s="20" t="inlineStr">
@@ -7628,17 +7624,21 @@
       </c>
       <c r="H121" s="20" t="inlineStr">
         <is>
-          <t>Loc: Berlin</t>
+          <t>React/Vue/JS, front-end lead, digital logistics, Japan relocation</t>
         </is>
       </c>
       <c r="I121" s="20" t="n"/>
       <c r="J121" s="20" t="n"/>
       <c r="K121" s="20" t="inlineStr">
         <is>
-          <t>5. Pending</t>
-        </is>
-      </c>
-      <c r="M121" s="20" t="n"/>
+          <t>2. Easy Apply</t>
+        </is>
+      </c>
+      <c r="M121" s="20" t="inlineStr">
+        <is>
+          <t>(via GitTap)</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="20">
@@ -7652,22 +7652,22 @@
       </c>
       <c r="C122" s="20" t="inlineStr">
         <is>
-          <t>N26</t>
+          <t>ReNK CHANNEL</t>
         </is>
       </c>
       <c r="D122" s="20" t="inlineStr">
         <is>
-          <t>Backend Engineer - Engagement</t>
+          <t>Front End Engineer (Visa Support)</t>
         </is>
       </c>
       <c r="E122" s="20" t="inlineStr">
         <is>
-          <t>https://n26.com/en-eu/careers/positions/7640893?gh_jid=7640893</t>
+          <t>https://www.gittap.jp/jobs/5214</t>
         </is>
       </c>
       <c r="F122" s="20" t="inlineStr">
         <is>
-          <t>career-ops scan</t>
+          <t>career-ops scan / gittap.jp</t>
         </is>
       </c>
       <c r="G122" s="20" t="inlineStr">
@@ -7677,7 +7677,7 @@
       </c>
       <c r="H122" s="20" t="inlineStr">
         <is>
-          <t>Loc: Berlin / Barcelona</t>
+          <t>In-house dev, listed-company subsidiary, visa support stated</t>
         </is>
       </c>
       <c r="I122" s="20" t="n"/>
@@ -7687,7 +7687,11 @@
           <t>5. Pending</t>
         </is>
       </c>
-      <c r="M122" s="20" t="n"/>
+      <c r="M122" s="20" t="inlineStr">
+        <is>
+          <t>(via GitTap)</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="20">
@@ -7701,44 +7705,51 @@
       </c>
       <c r="C123" s="20" t="inlineStr">
         <is>
-          <t>Shippio</t>
+          <t>stakefish</t>
         </is>
       </c>
       <c r="D123" s="20" t="inlineStr">
         <is>
-          <t>Senior Front-End Engineer</t>
+          <t>Web3 / Full-stack Software Engineer</t>
         </is>
       </c>
       <c r="E123" s="20" t="inlineStr">
         <is>
-          <t>https://cs.gittap.jp/jobs/1719</t>
+          <t>https://www.linkedin.com/jobs/view/4354681451/</t>
         </is>
       </c>
       <c r="F123" s="20" t="inlineStr">
         <is>
-          <t>career-ops scan / gittap.jp</t>
+          <t>user-submitted (LinkedIn)</t>
         </is>
       </c>
       <c r="G123" s="20" t="inlineStr">
         <is>
-          <t>Visa sponsorship needed</t>
+          <t>Remote — worldwide (Singapore HQ, GMT+8)</t>
         </is>
       </c>
       <c r="H123" s="20" t="inlineStr">
         <is>
-          <t>React/Vue/JS, front-end lead, digital logistics, Japan relocation</t>
-        </is>
-      </c>
-      <c r="I123" s="20" t="n"/>
+          <t>React+TS+Python+web3.js, mid-senior IC, distributed culture, $140-180K</t>
+        </is>
+      </c>
+      <c r="I123" s="20" t="n">
+        <v>5</v>
+      </c>
       <c r="J123" s="20" t="n"/>
       <c r="K123" s="20" t="inlineStr">
         <is>
           <t>2. Easy Apply</t>
         </is>
       </c>
+      <c r="L123" s="20" t="inlineStr">
+        <is>
+          <t>Hidden</t>
+        </is>
+      </c>
       <c r="M123" s="20" t="inlineStr">
         <is>
-          <t>(via GitTap)</t>
+          <t>Applied via LinkedIn Easy Apply 2026-05-07. User-flagged as ideal fit shape (2026-05-07)</t>
         </is>
       </c>
     </row>
@@ -7754,44 +7765,51 @@
       </c>
       <c r="C124" s="20" t="inlineStr">
         <is>
-          <t>ReNK CHANNEL</t>
+          <t>StraitsX</t>
         </is>
       </c>
       <c r="D124" s="20" t="inlineStr">
         <is>
-          <t>Front End Engineer (Visa Support)</t>
+          <t>Mid Software Engineer - Blockchain</t>
         </is>
       </c>
       <c r="E124" s="20" t="inlineStr">
         <is>
-          <t>https://www.gittap.jp/jobs/5214</t>
+          <t>https://job-boards.eu.greenhouse.io/straitsx/jobs/4839243101</t>
         </is>
       </c>
       <c r="F124" s="20" t="inlineStr">
         <is>
-          <t>career-ops scan / gittap.jp</t>
+          <t>user-submitted (LinkedIn -&gt; Greenhouse)</t>
         </is>
       </c>
       <c r="G124" s="20" t="inlineStr">
         <is>
-          <t>Visa sponsorship needed</t>
+          <t>Eligible (Jakarta, Indonesia — home country)</t>
         </is>
       </c>
       <c r="H124" s="20" t="inlineStr">
         <is>
-          <t>In-house dev, listed-company subsidiary, visa support stated</t>
-        </is>
-      </c>
-      <c r="I124" s="20" t="n"/>
+          <t>Stablecoin Web3 infra; mid-IC; Go preferred not required; fintech/regulated</t>
+        </is>
+      </c>
+      <c r="I124" s="20" t="n">
+        <v>4</v>
+      </c>
       <c r="J124" s="20" t="n"/>
       <c r="K124" s="20" t="inlineStr">
         <is>
-          <t>5. Pending</t>
+          <t>2. Easy Apply</t>
+        </is>
+      </c>
+      <c r="L124" s="20" t="inlineStr">
+        <is>
+          <t>Hidden</t>
         </is>
       </c>
       <c r="M124" s="20" t="inlineStr">
         <is>
-          <t>(via GitTap)</t>
+          <t>Originally LinkedIn 4401055938 (Taipei entry-level); swapped to Jakarta Mid via Greenhouse</t>
         </is>
       </c>
     </row>
@@ -7802,41 +7820,41 @@
       </c>
       <c r="B125" s="20" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C125" s="20" t="inlineStr">
         <is>
-          <t>stakefish</t>
+          <t>Sumsub</t>
         </is>
       </c>
       <c r="D125" s="20" t="inlineStr">
         <is>
-          <t>Web3 / Full-stack Software Engineer</t>
+          <t>Technical Support Engineer (L3)</t>
         </is>
       </c>
       <c r="E125" s="20" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/jobs/view/4354681451/</t>
+          <t>https://careers.sumsub.com/jobs/7232843-technical-support-engineer-l3</t>
         </is>
       </c>
       <c r="F125" s="20" t="inlineStr">
         <is>
-          <t>user-submitted (LinkedIn)</t>
+          <t>Sumsub Careers (direct)</t>
         </is>
       </c>
       <c r="G125" s="20" t="inlineStr">
         <is>
-          <t>Remote — worldwide (Singapore HQ, GMT+8)</t>
+          <t>✓ Eligible (APAC Remote — Indonesia GMT+7)</t>
         </is>
       </c>
       <c r="H125" s="20" t="inlineStr">
         <is>
-          <t>React+TS+Python+web3.js, mid-senior IC, distributed culture, $140-180K</t>
+          <t>Sumsub SDK integrated at Nespay; REST API/SQL/scripting match; learning Mandarin for APAC team</t>
         </is>
       </c>
       <c r="I125" s="20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J125" s="20" t="n"/>
       <c r="K125" s="20" t="inlineStr">
@@ -7851,179 +7869,59 @@
       </c>
       <c r="M125" s="20" t="inlineStr">
         <is>
-          <t>Applied via LinkedIn Easy Apply 2026-05-07. User-flagged as ideal fit shape (2026-05-07)</t>
+          <t>Mandarin required (hard gap — currently learning). cv-default used. 45 wpm typing speed.</t>
         </is>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="20">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B126" s="20" t="inlineStr">
-        <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="C126" s="20" t="inlineStr">
-        <is>
-          <t>StraitsX</t>
-        </is>
-      </c>
-      <c r="D126" s="20" t="inlineStr">
-        <is>
-          <t>Mid Software Engineer - Blockchain</t>
-        </is>
-      </c>
-      <c r="E126" s="20" t="inlineStr">
-        <is>
-          <t>https://job-boards.eu.greenhouse.io/straitsx/jobs/4839243101</t>
-        </is>
-      </c>
-      <c r="F126" s="20" t="inlineStr">
-        <is>
-          <t>user-submitted (LinkedIn -&gt; Greenhouse)</t>
-        </is>
-      </c>
-      <c r="G126" s="20" t="inlineStr">
-        <is>
-          <t>Eligible (Jakarta, Indonesia — home country)</t>
-        </is>
-      </c>
-      <c r="H126" s="20" t="inlineStr">
-        <is>
-          <t>Stablecoin Web3 infra; mid-IC; Go preferred not required; fintech/regulated</t>
-        </is>
-      </c>
-      <c r="I126" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="J126" s="20" t="n"/>
-      <c r="K126" s="20" t="inlineStr">
-        <is>
-          <t>2. Easy Apply</t>
-        </is>
-      </c>
-      <c r="L126" s="20" t="inlineStr">
-        <is>
-          <t>Hidden</t>
-        </is>
-      </c>
-      <c r="M126" s="20" t="inlineStr">
-        <is>
-          <t>Originally LinkedIn 4401055938 (Taipei entry-level); swapped to Jakarta Mid via Greenhouse</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="20">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B127" s="20" t="inlineStr">
-        <is>
-          <t>2026-05-08</t>
-        </is>
-      </c>
-      <c r="C127" s="20" t="inlineStr">
-        <is>
-          <t>Sumsub</t>
-        </is>
-      </c>
-      <c r="D127" s="20" t="inlineStr">
-        <is>
-          <t>Technical Support Engineer (L3)</t>
-        </is>
-      </c>
-      <c r="E127" s="20" t="inlineStr">
-        <is>
-          <t>https://careers.sumsub.com/jobs/7232843-technical-support-engineer-l3</t>
-        </is>
-      </c>
-      <c r="F127" s="20" t="inlineStr">
-        <is>
-          <t>Sumsub Careers (direct)</t>
-        </is>
-      </c>
-      <c r="G127" s="20" t="inlineStr">
-        <is>
-          <t>✓ Eligible (APAC Remote — Indonesia GMT+7)</t>
-        </is>
-      </c>
-      <c r="H127" s="20" t="inlineStr">
-        <is>
-          <t>Sumsub SDK integrated at Nespay; REST API/SQL/scripting match; learning Mandarin for APAC team</t>
-        </is>
-      </c>
-      <c r="I127" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="J127" s="20" t="n"/>
-      <c r="K127" s="20" t="inlineStr">
-        <is>
-          <t>2. Easy Apply</t>
-        </is>
-      </c>
-      <c r="L127" s="20" t="inlineStr">
-        <is>
-          <t>Hidden</t>
-        </is>
-      </c>
-      <c r="M127" s="20" t="inlineStr">
-        <is>
-          <t>Mandarin required (hard gap — currently learning). cv-default used. 45 wpm typing speed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="27">
-        <f>ROW()-1</f>
-        <v/>
-      </c>
-      <c r="B128" s="27" t="inlineStr">
+      <c r="A126" s="27">
+        <f>ROW()-1</f>
+        <v/>
+      </c>
+      <c r="B126" s="27" t="inlineStr">
         <is>
           <t>2026-05-10</t>
         </is>
       </c>
-      <c r="C128" s="27" t="inlineStr">
+      <c r="C126" s="27" t="inlineStr">
         <is>
           <t>Sharefull</t>
         </is>
       </c>
-      <c r="D128" s="27" t="inlineStr">
+      <c r="D126" s="27" t="inlineStr">
         <is>
           <t>Software Engineer — Fullstack</t>
         </is>
       </c>
-      <c r="E128" s="27" t="inlineStr">
+      <c r="E126" s="27" t="inlineStr">
         <is>
           <t>https://cs.gittap.jp/jobs/4877</t>
         </is>
       </c>
-      <c r="F128" s="27" t="inlineStr">
+      <c r="F126" s="27" t="inlineStr">
         <is>
           <t>career-ops / gittap.jp</t>
         </is>
       </c>
-      <c r="G128" s="27" t="inlineStr">
+      <c r="G126" s="27" t="inlineStr">
         <is>
           <t>⚠️ Requires Japan residence (no visa sponsorship mentioned)</t>
         </is>
       </c>
-      <c r="H128" s="27" t="inlineStr">
+      <c r="H126" s="27" t="inlineStr">
         <is>
           <t>SaaS shift mgmt; XP/TDD; TypeScript/AWS Lambda; pair programming; English-first team</t>
         </is>
       </c>
-      <c r="I128" s="27" t="n"/>
-      <c r="J128" s="27" t="n"/>
-      <c r="K128" s="27" t="inlineStr">
+      <c r="I126" s="27" t="n"/>
+      <c r="J126" s="27" t="n"/>
+      <c r="K126" s="27" t="inlineStr">
         <is>
           <t>5. Pending</t>
         </is>
       </c>
-      <c r="L128" s="27" t="inlineStr"/>
-      <c r="M128" s="27" t="inlineStr">
+      <c r="L126" s="27" t="inlineStr"/>
+      <c r="M126" s="27" t="inlineStr">
         <is>
           <t>Angular (not React); Lambda (not EC2); Japan residency must-have — visa unknown</t>
         </is>
@@ -8087,62 +7985,61 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E85" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E87" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E93" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E94" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E95" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E96" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E97" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E98" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E99" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E100" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E101" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E102" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E103" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E104" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E105" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E106" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E107" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E108" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E109" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E110" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E111" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E112" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E113" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E114" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E115" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E116" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E117" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E118" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E119" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E120" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E121" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E122" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E123" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E85" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E86" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E87" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E93" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E94" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E95" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E96" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E97" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E98" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E99" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E100" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E101" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E102" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E103" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E104" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E105" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E106" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E107" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E108" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E109" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E110" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E111" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E112" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E113" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E114" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E115" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E116" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E117" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E118" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E119" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E120" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E121" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E122" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E123" r:id="rId60"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
tracker: add Hercules Full-Stack + Frontend to Jobs & Preparations
SF in-office roles (US TZ + travel gate); core stack TS/React/Postgres/
Redis matches. Added prep docs with honest gap framing.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1710" uniqueCount="786">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1750" uniqueCount="805">
   <si>
     <t>Hana Aliyah Mufidah</t>
   </si>
@@ -1207,6 +1207,45 @@
     <t>Angular (not React); Lambda (not EC2); Japan residency must-have — visa unknown</t>
   </si>
   <si>
+    <t>2026-07-13</t>
+  </si>
+  <si>
+    <t>Hercules</t>
+  </si>
+  <si>
+    <t>Full-Stack Engineer</t>
+  </si>
+  <si>
+    <t>https://hercules.app/careers/full-stack-engineer</t>
+  </si>
+  <si>
+    <t>User pick (hercules.app/careers)</t>
+  </si>
+  <si>
+    <t>⚠️ SF in-office; remote only for exceptional (US TZ + travel); no visa mentioned</t>
+  </si>
+  <si>
+    <t>AI-native app builder; core stack TS/React/Postgres/Redis is hers; senior/staff level</t>
+  </si>
+  <si>
+    <t>Prep</t>
+  </si>
+  <si>
+    <t>SF Kearny/Bush in-office, strong preference; remote only for exceptional candidates on US TZ + regular travel. Stack TS/React/Postgres/Redis/Temporal. Gaps: SaaS billing/SSO-SAML, Temporal, US timezone. Prep: prep/hercules-full-stack-engineer-2026-07-13.md</t>
+  </si>
+  <si>
+    <t>Frontend Engineer</t>
+  </si>
+  <si>
+    <t>https://hercules.app/careers/frontend-engineer</t>
+  </si>
+  <si>
+    <t>React/Next/Tailwind front-end + AI-native product; senior/staff level</t>
+  </si>
+  <si>
+    <t>SF Kearny/Bush in-office, strong preference; remote only for exceptional candidates on US TZ + regular travel. Stack TS/React/Tailwind/Clickhouse/Hono/Drizzle/Temporal. Gaps: high-end design/UX bar, newer stack pieces, US timezone. Full-Stack is the closer match. Prep: prep/hercules-frontend-engineer-2026-07-13.md</t>
+  </si>
+  <si>
     <t>Date</t>
   </si>
   <si>
@@ -1321,6 +1360,27 @@
     <t>Not required</t>
   </si>
   <si>
+    <t>(pending tailoring)</t>
+  </si>
+  <si>
+    <t>Pending tailoring</t>
+  </si>
+  <si>
+    <t>prep/hercules-full-stack-engineer-2026-07-13.md</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
+    <t>Not started</t>
+  </si>
+  <si>
+    <t>SF in-office gate; confirm remote/US-TZ acceptance before investing in tailored CV</t>
+  </si>
+  <si>
+    <t>prep/hercules-frontend-engineer-2026-07-13.md</t>
+  </si>
+  <si>
     <t>Date Applied</t>
   </si>
   <si>
@@ -1427,9 +1487,6 @@
   </si>
   <si>
     <t>cv-default used. 45 wpm typing speed noted. Screenshot uploaded on application page. Promoted from Preparations</t>
-  </si>
-  <si>
-    <t>2026-07-13</t>
   </si>
   <si>
     <t>Backend Engineer, Card Issuing</t>
@@ -3635,7 +3692,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:M126"/>
+  <dimension ref="A1:M128"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="5" style="1" customWidth="1"/>
@@ -7959,6 +8016,80 @@
       <c r="L126" s="20"/>
       <c r="M126" s="20" t="s">
         <v>395</v>
+      </c>
+    </row>
+    <row r="127" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A127" s="20">
+        <f>ROW()-1</f>
+      </c>
+      <c r="B127" s="20" t="s">
+        <v>396</v>
+      </c>
+      <c r="C127" s="20" t="s">
+        <v>397</v>
+      </c>
+      <c r="D127" s="20" t="s">
+        <v>398</v>
+      </c>
+      <c r="E127" s="20" t="s">
+        <v>399</v>
+      </c>
+      <c r="F127" s="20" t="s">
+        <v>400</v>
+      </c>
+      <c r="G127" s="20" t="s">
+        <v>401</v>
+      </c>
+      <c r="H127" s="20" t="s">
+        <v>402</v>
+      </c>
+      <c r="I127" s="20">
+        <v>3.5</v>
+      </c>
+      <c r="J127" s="20"/>
+      <c r="K127" s="20" t="s">
+        <v>403</v>
+      </c>
+      <c r="L127" s="20"/>
+      <c r="M127" s="20" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="128" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A128" s="20">
+        <f>ROW()-1</f>
+      </c>
+      <c r="B128" s="20" t="s">
+        <v>396</v>
+      </c>
+      <c r="C128" s="20" t="s">
+        <v>397</v>
+      </c>
+      <c r="D128" s="20" t="s">
+        <v>405</v>
+      </c>
+      <c r="E128" s="20" t="s">
+        <v>406</v>
+      </c>
+      <c r="F128" s="20" t="s">
+        <v>400</v>
+      </c>
+      <c r="G128" s="20" t="s">
+        <v>401</v>
+      </c>
+      <c r="H128" s="20" t="s">
+        <v>407</v>
+      </c>
+      <c r="I128" s="20">
+        <v>3.5</v>
+      </c>
+      <c r="J128" s="20"/>
+      <c r="K128" s="20" t="s">
+        <v>403</v>
+      </c>
+      <c r="L128" s="20"/>
+      <c r="M128" s="20" t="s">
+        <v>408</v>
       </c>
     </row>
   </sheetData>
@@ -8084,7 +8215,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="5" style="1" customWidth="1"/>
@@ -8109,7 +8240,7 @@
         <v>61</v>
       </c>
       <c r="B1" s="21" t="s">
-        <v>396</v>
+        <v>409</v>
       </c>
       <c r="C1" s="21" t="s">
         <v>14</v>
@@ -8121,28 +8252,28 @@
         <v>63</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>397</v>
+        <v>410</v>
       </c>
       <c r="G1" s="21" t="s">
-        <v>398</v>
+        <v>411</v>
       </c>
       <c r="H1" s="21" t="s">
-        <v>399</v>
+        <v>412</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>400</v>
+        <v>413</v>
       </c>
       <c r="J1" s="21" t="s">
-        <v>401</v>
+        <v>414</v>
       </c>
       <c r="K1" s="21" t="s">
-        <v>402</v>
+        <v>415</v>
       </c>
       <c r="L1" s="21" t="s">
-        <v>403</v>
+        <v>416</v>
       </c>
       <c r="M1" s="21" t="s">
-        <v>404</v>
+        <v>417</v>
       </c>
       <c r="N1" s="21" t="s">
         <v>71</v>
@@ -8162,37 +8293,37 @@
         <v>80</v>
       </c>
       <c r="D2" s="22" t="s">
-        <v>405</v>
+        <v>418</v>
       </c>
       <c r="E2" s="22" t="s">
         <v>82</v>
       </c>
       <c r="F2" s="22" t="s">
-        <v>406</v>
+        <v>419</v>
       </c>
       <c r="G2" s="22" t="s">
-        <v>407</v>
+        <v>420</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>408</v>
+        <v>421</v>
       </c>
       <c r="I2" s="22" t="s">
-        <v>409</v>
+        <v>422</v>
       </c>
       <c r="J2" s="22" t="s">
-        <v>410</v>
+        <v>423</v>
       </c>
       <c r="K2" s="22" t="s">
-        <v>411</v>
+        <v>424</v>
       </c>
       <c r="L2" s="22" t="s">
-        <v>412</v>
+        <v>425</v>
       </c>
       <c r="M2" s="22" t="s">
-        <v>413</v>
+        <v>426</v>
       </c>
       <c r="N2" s="22" t="s">
-        <v>414</v>
+        <v>427</v>
       </c>
       <c r="O2" s="1"/>
     </row>
@@ -8207,37 +8338,37 @@
         <v>80</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>415</v>
+        <v>428</v>
       </c>
       <c r="E3" s="22" t="s">
         <v>88</v>
       </c>
       <c r="F3" s="22" t="s">
-        <v>416</v>
+        <v>429</v>
       </c>
       <c r="G3" s="22" t="s">
-        <v>417</v>
+        <v>430</v>
       </c>
       <c r="H3" s="20" t="s">
-        <v>418</v>
+        <v>431</v>
       </c>
       <c r="I3" s="22" t="s">
-        <v>409</v>
+        <v>422</v>
       </c>
       <c r="J3" s="22" t="s">
-        <v>419</v>
+        <v>432</v>
       </c>
       <c r="K3" s="22" t="s">
-        <v>411</v>
+        <v>424</v>
       </c>
       <c r="L3" s="22" t="s">
-        <v>412</v>
+        <v>425</v>
       </c>
       <c r="M3" s="22" t="s">
-        <v>413</v>
+        <v>426</v>
       </c>
       <c r="N3" s="22" t="s">
-        <v>420</v>
+        <v>433</v>
       </c>
       <c r="O3" s="1"/>
     </row>
@@ -8252,37 +8383,37 @@
         <v>80</v>
       </c>
       <c r="D4" s="22" t="s">
-        <v>421</v>
+        <v>434</v>
       </c>
       <c r="E4" s="22" t="s">
         <v>91</v>
       </c>
       <c r="F4" s="22" t="s">
-        <v>422</v>
+        <v>435</v>
       </c>
       <c r="G4" s="22" t="s">
-        <v>423</v>
+        <v>436</v>
       </c>
       <c r="H4" s="20" t="s">
-        <v>424</v>
+        <v>437</v>
       </c>
       <c r="I4" s="22" t="s">
+        <v>438</v>
+      </c>
+      <c r="J4" s="22" t="s">
+        <v>439</v>
+      </c>
+      <c r="K4" s="22" t="s">
+        <v>440</v>
+      </c>
+      <c r="L4" s="22" t="s">
         <v>425</v>
       </c>
-      <c r="J4" s="22" t="s">
-        <v>426</v>
-      </c>
-      <c r="K4" s="22" t="s">
-        <v>427</v>
-      </c>
-      <c r="L4" s="22" t="s">
-        <v>412</v>
-      </c>
       <c r="M4" s="22" t="s">
-        <v>428</v>
+        <v>441</v>
       </c>
       <c r="N4" s="22" t="s">
-        <v>429</v>
+        <v>442</v>
       </c>
       <c r="O4" s="1"/>
     </row>
@@ -8303,25 +8434,107 @@
         <v>346</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>430</v>
+        <v>443</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>431</v>
+        <v>444</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>432</v>
+        <v>445</v>
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1" t="s">
-        <v>433</v>
+        <v>446</v>
       </c>
       <c r="L5" s="1"/>
       <c r="M5" s="1" t="s">
-        <v>428</v>
+        <v>441</v>
       </c>
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <f>ROW()-1</f>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>447</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="H6" s="20" t="s">
+        <v>449</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="O6" s="1"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <f>ROW()-1</f>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>447</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="H7" s="20" t="s">
+        <v>453</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="O7" s="1"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="P2:P1000">
@@ -8414,7 +8627,7 @@
         <v>61</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>434</v>
+        <v>454</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>14</v>
@@ -8423,10 +8636,10 @@
         <v>13</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>435</v>
+        <v>455</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>436</v>
+        <v>456</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>63</v>
@@ -8435,28 +8648,28 @@
         <v>44</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>437</v>
+        <v>457</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>438</v>
+        <v>458</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>439</v>
+        <v>459</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>440</v>
+        <v>460</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>441</v>
+        <v>461</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>442</v>
+        <v>462</v>
       </c>
       <c r="O1" s="7" t="s">
-        <v>443</v>
+        <v>463</v>
       </c>
       <c r="P1" s="7" t="s">
-        <v>444</v>
+        <v>464</v>
       </c>
       <c r="Q1" s="7" t="s">
         <v>71</v>
@@ -8479,10 +8692,10 @@
         <v>367</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>445</v>
+        <v>465</v>
       </c>
       <c r="F2" s="22" t="s">
-        <v>446</v>
+        <v>466</v>
       </c>
       <c r="G2" s="22" t="s">
         <v>368</v>
@@ -8494,24 +8707,24 @@
         <v>347</v>
       </c>
       <c r="J2" s="22" t="s">
-        <v>430</v>
+        <v>443</v>
       </c>
       <c r="K2" s="22" t="s">
-        <v>447</v>
+        <v>467</v>
       </c>
       <c r="L2" s="1"/>
       <c r="M2" s="22" t="s">
-        <v>448</v>
+        <v>468</v>
       </c>
       <c r="N2" s="1"/>
       <c r="O2" s="22" t="s">
-        <v>449</v>
+        <v>469</v>
       </c>
       <c r="P2" s="22" t="s">
-        <v>450</v>
+        <v>470</v>
       </c>
       <c r="Q2" s="22" t="s">
-        <v>451</v>
+        <v>471</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
@@ -8528,10 +8741,10 @@
         <v>374</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>452</v>
+        <v>472</v>
       </c>
       <c r="F3" s="22" t="s">
-        <v>453</v>
+        <v>473</v>
       </c>
       <c r="G3" s="22" t="s">
         <v>375</v>
@@ -8543,22 +8756,22 @@
         <v>347</v>
       </c>
       <c r="J3" s="22" t="s">
-        <v>430</v>
+        <v>443</v>
       </c>
       <c r="K3" s="22" t="s">
-        <v>454</v>
+        <v>474</v>
       </c>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
       <c r="O3" s="22" t="s">
-        <v>449</v>
+        <v>469</v>
       </c>
       <c r="P3" s="22" t="s">
-        <v>450</v>
+        <v>470</v>
       </c>
       <c r="Q3" s="22" t="s">
-        <v>455</v>
+        <v>475</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
@@ -8572,13 +8785,13 @@
         <v>80</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>405</v>
+        <v>418</v>
       </c>
       <c r="E4" s="22" t="s">
-        <v>456</v>
+        <v>476</v>
       </c>
       <c r="F4" s="22" t="s">
-        <v>457</v>
+        <v>477</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>82</v>
@@ -8590,28 +8803,28 @@
         <v>380</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>406</v>
+        <v>419</v>
       </c>
       <c r="K4" s="22" t="s">
-        <v>458</v>
+        <v>478</v>
       </c>
       <c r="L4" s="22" t="s">
-        <v>459</v>
+        <v>479</v>
       </c>
       <c r="M4" s="22" t="s">
-        <v>460</v>
+        <v>480</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>461</v>
+        <v>481</v>
       </c>
       <c r="O4" s="22" t="s">
-        <v>449</v>
+        <v>469</v>
       </c>
       <c r="P4" s="22" t="s">
-        <v>462</v>
+        <v>482</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>463</v>
+        <v>483</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
@@ -8625,13 +8838,13 @@
         <v>80</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>415</v>
+        <v>428</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>456</v>
+        <v>476</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>457</v>
+        <v>477</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>88</v>
@@ -8643,24 +8856,24 @@
         <v>380</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>416</v>
+        <v>429</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>458</v>
+        <v>478</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>464</v>
+        <v>484</v>
       </c>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
       <c r="O5" s="1" t="s">
-        <v>449</v>
+        <v>469</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>462</v>
+        <v>482</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>463</v>
+        <v>483</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
@@ -8677,7 +8890,7 @@
         <v>382</v>
       </c>
       <c r="E6" s="22" t="s">
-        <v>465</v>
+        <v>485</v>
       </c>
       <c r="F6" s="22" t="s">
         <v>384</v>
@@ -8692,26 +8905,26 @@
         <v>380</v>
       </c>
       <c r="J6" s="22" t="s">
-        <v>430</v>
+        <v>443</v>
       </c>
       <c r="K6" s="22" t="s">
-        <v>466</v>
+        <v>486</v>
       </c>
       <c r="L6" s="22"/>
       <c r="M6" s="22" t="s">
-        <v>467</v>
+        <v>487</v>
       </c>
       <c r="N6" s="22" t="s">
-        <v>468</v>
+        <v>488</v>
       </c>
       <c r="O6" s="22" t="s">
-        <v>449</v>
+        <v>469</v>
       </c>
       <c r="P6" s="22" t="s">
-        <v>462</v>
+        <v>482</v>
       </c>
       <c r="Q6" s="22" t="s">
-        <v>469</v>
+        <v>489</v>
       </c>
       <c r="R6" s="20"/>
     </row>
@@ -8720,44 +8933,44 @@
         <f>ROW()-1</f>
       </c>
       <c r="B7" s="22" t="s">
-        <v>470</v>
+        <v>396</v>
       </c>
       <c r="C7" s="22" t="s">
         <v>373</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>471</v>
+        <v>490</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>472</v>
+        <v>491</v>
       </c>
       <c r="F7" s="22" t="s">
-        <v>473</v>
+        <v>492</v>
       </c>
       <c r="G7" s="22" t="s">
-        <v>474</v>
+        <v>493</v>
       </c>
       <c r="H7" s="22" t="s">
         <v>51</v>
       </c>
       <c r="I7" s="22" t="s">
-        <v>470</v>
+        <v>396</v>
       </c>
       <c r="J7" s="22"/>
       <c r="K7" s="22"/>
       <c r="L7" s="22" t="s">
-        <v>475</v>
+        <v>494</v>
       </c>
       <c r="M7" s="22"/>
       <c r="N7" s="22"/>
       <c r="O7" s="22" t="s">
-        <v>449</v>
+        <v>469</v>
       </c>
       <c r="P7" s="22" t="s">
-        <v>476</v>
+        <v>495</v>
       </c>
       <c r="Q7" s="22" t="s">
-        <v>477</v>
+        <v>496</v>
       </c>
       <c r="R7" s="20"/>
     </row>
@@ -12849,7 +13062,7 @@
         <v>356</v>
       </c>
       <c r="E202" s="20" t="s">
-        <v>478</v>
+        <v>497</v>
       </c>
       <c r="F202" s="20" t="s">
         <v>358</v>
@@ -12858,13 +13071,13 @@
         <v>357</v>
       </c>
       <c r="H202" s="20" t="s">
-        <v>479</v>
+        <v>498</v>
       </c>
       <c r="I202" s="20" t="s">
         <v>388</v>
       </c>
       <c r="J202" s="20" t="s">
-        <v>430</v>
+        <v>443</v>
       </c>
       <c r="K202" s="20"/>
       <c r="L202" s="20"/>
@@ -12935,7 +13148,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>480</v>
+        <v>499</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -12951,16 +13164,16 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>481</v>
+        <v>500</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>482</v>
+        <v>501</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>71</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>483</v>
+        <v>502</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -12968,13 +13181,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>484</v>
+        <v>503</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>485</v>
+        <v>504</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E3" s="10"/>
       <c r="F3" s="10"/>
@@ -12984,13 +13197,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>487</v>
+        <v>506</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>488</v>
+        <v>507</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E4" s="10"/>
       <c r="F4" s="10"/>
@@ -13000,16 +13213,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>489</v>
+        <v>508</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>490</v>
+        <v>509</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>491</v>
+        <v>510</v>
       </c>
       <c r="F5" s="10"/>
     </row>
@@ -13018,16 +13231,16 @@
         <v>4</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>492</v>
+        <v>511</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>493</v>
+        <v>512</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>494</v>
+        <v>513</v>
       </c>
       <c r="F6" s="10"/>
     </row>
@@ -13039,13 +13252,13 @@
         <v>240</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>495</v>
+        <v>514</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>496</v>
+        <v>515</v>
       </c>
       <c r="F7" s="10"/>
     </row>
@@ -13054,16 +13267,16 @@
         <v>6</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>497</v>
+        <v>516</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>498</v>
+        <v>517</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>499</v>
+        <v>518</v>
       </c>
       <c r="F8" s="10"/>
     </row>
@@ -13072,16 +13285,16 @@
         <v>7</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>500</v>
+        <v>519</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>501</v>
+        <v>520</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="F9" s="10"/>
     </row>
@@ -13093,13 +13306,13 @@
         <v>141</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>503</v>
+        <v>522</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>504</v>
+        <v>523</v>
       </c>
       <c r="F10" s="10"/>
     </row>
@@ -13108,16 +13321,16 @@
         <v>9</v>
       </c>
       <c r="B11" s="10" t="s">
+        <v>524</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>525</v>
+      </c>
+      <c r="D11" s="10" t="s">
         <v>505</v>
       </c>
-      <c r="C11" s="23" t="s">
-        <v>506</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>486</v>
-      </c>
       <c r="E11" s="10" t="s">
-        <v>507</v>
+        <v>526</v>
       </c>
       <c r="F11" s="10"/>
     </row>
@@ -13126,16 +13339,16 @@
         <v>10</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>508</v>
+        <v>527</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>509</v>
+        <v>528</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>510</v>
+        <v>529</v>
       </c>
       <c r="F12" s="10"/>
     </row>
@@ -13144,16 +13357,16 @@
         <v>11</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>511</v>
+        <v>530</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>512</v>
+        <v>531</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>513</v>
+        <v>532</v>
       </c>
       <c r="F13" s="10"/>
     </row>
@@ -13162,16 +13375,16 @@
         <v>12</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>514</v>
+        <v>533</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>515</v>
+        <v>534</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>516</v>
+        <v>535</v>
       </c>
       <c r="F14" s="10"/>
     </row>
@@ -13180,16 +13393,16 @@
         <v>13</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>517</v>
+        <v>536</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>518</v>
+        <v>537</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>519</v>
+        <v>538</v>
       </c>
       <c r="F15" s="10"/>
     </row>
@@ -13198,16 +13411,16 @@
         <v>14</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>520</v>
+        <v>539</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>521</v>
+        <v>540</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>522</v>
+        <v>541</v>
       </c>
       <c r="F16" s="10"/>
     </row>
@@ -13216,16 +13429,16 @@
         <v>15</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>523</v>
+        <v>542</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>524</v>
+        <v>543</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>525</v>
+        <v>544</v>
       </c>
       <c r="F17" s="10"/>
     </row>
@@ -13234,16 +13447,16 @@
         <v>16</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>526</v>
+        <v>545</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>527</v>
+        <v>546</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>528</v>
+        <v>547</v>
       </c>
       <c r="F18" s="10"/>
     </row>
@@ -13255,13 +13468,13 @@
         <v>179</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>529</v>
+        <v>548</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>530</v>
+        <v>549</v>
       </c>
       <c r="F19" s="10"/>
     </row>
@@ -13270,16 +13483,16 @@
         <v>18</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>531</v>
+        <v>550</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>532</v>
+        <v>551</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>533</v>
+        <v>552</v>
       </c>
       <c r="F20" s="10"/>
     </row>
@@ -13288,16 +13501,16 @@
         <v>19</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>534</v>
+        <v>553</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>535</v>
+        <v>554</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>536</v>
+        <v>555</v>
       </c>
       <c r="F21" s="10"/>
     </row>
@@ -13306,16 +13519,16 @@
         <v>20</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>537</v>
+        <v>556</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>538</v>
+        <v>557</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>539</v>
+        <v>558</v>
       </c>
       <c r="F22" s="10"/>
     </row>
@@ -13324,16 +13537,16 @@
         <v>21</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>540</v>
+        <v>559</v>
       </c>
       <c r="C23" s="23" t="s">
-        <v>541</v>
+        <v>560</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>542</v>
+        <v>561</v>
       </c>
       <c r="F23" s="10"/>
     </row>
@@ -13342,16 +13555,16 @@
         <v>22</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>543</v>
+        <v>562</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>544</v>
+        <v>563</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>545</v>
+        <v>564</v>
       </c>
       <c r="F24" s="10"/>
     </row>
@@ -13360,16 +13573,16 @@
         <v>23</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>546</v>
+        <v>565</v>
       </c>
       <c r="C25" s="23" t="s">
-        <v>547</v>
+        <v>566</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>548</v>
+        <v>567</v>
       </c>
       <c r="F25" s="10"/>
     </row>
@@ -13378,16 +13591,16 @@
         <v>24</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>549</v>
+        <v>568</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>550</v>
+        <v>569</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>551</v>
+        <v>570</v>
       </c>
       <c r="F26" s="10"/>
     </row>
@@ -13396,16 +13609,16 @@
         <v>25</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>552</v>
+        <v>571</v>
       </c>
       <c r="C27" s="23" t="s">
-        <v>553</v>
+        <v>572</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>554</v>
+        <v>573</v>
       </c>
       <c r="F27" s="10"/>
     </row>
@@ -13414,16 +13627,16 @@
         <v>26</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>555</v>
+        <v>574</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>556</v>
+        <v>575</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>557</v>
+        <v>576</v>
       </c>
       <c r="F28" s="10"/>
     </row>
@@ -13432,16 +13645,16 @@
         <v>27</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>558</v>
+        <v>577</v>
       </c>
       <c r="C29" s="23" t="s">
-        <v>559</v>
+        <v>578</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>560</v>
+        <v>579</v>
       </c>
       <c r="F29" s="10"/>
     </row>
@@ -13450,16 +13663,16 @@
         <v>28</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>561</v>
+        <v>580</v>
       </c>
       <c r="C30" s="23" t="s">
-        <v>562</v>
+        <v>581</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>563</v>
+        <v>582</v>
       </c>
       <c r="F30" s="10"/>
     </row>
@@ -13468,16 +13681,16 @@
         <v>29</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>564</v>
+        <v>583</v>
       </c>
       <c r="C31" s="23" t="s">
-        <v>565</v>
+        <v>584</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>566</v>
+        <v>585</v>
       </c>
       <c r="F31" s="10"/>
     </row>
@@ -13486,16 +13699,16 @@
         <v>30</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>567</v>
+        <v>586</v>
       </c>
       <c r="C32" s="23" t="s">
-        <v>568</v>
+        <v>587</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>569</v>
+        <v>588</v>
       </c>
       <c r="F32" s="10"/>
     </row>
@@ -13504,16 +13717,16 @@
         <v>31</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>570</v>
+        <v>589</v>
       </c>
       <c r="C33" s="23" t="s">
-        <v>571</v>
+        <v>590</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>572</v>
+        <v>591</v>
       </c>
       <c r="F33" s="10"/>
     </row>
@@ -13525,13 +13738,13 @@
         <v>108</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>573</v>
+        <v>592</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>574</v>
+        <v>593</v>
       </c>
       <c r="F34" s="10"/>
     </row>
@@ -13543,13 +13756,13 @@
         <v>344</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>575</v>
+        <v>594</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>576</v>
+        <v>595</v>
       </c>
       <c r="F35" s="10"/>
     </row>
@@ -13558,16 +13771,16 @@
         <v>34</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>577</v>
+        <v>596</v>
       </c>
       <c r="C36" s="23" t="s">
-        <v>578</v>
+        <v>597</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>579</v>
+        <v>598</v>
       </c>
       <c r="F36" s="10"/>
     </row>
@@ -13579,13 +13792,13 @@
         <v>113</v>
       </c>
       <c r="C37" s="23" t="s">
-        <v>580</v>
+        <v>599</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>581</v>
+        <v>600</v>
       </c>
       <c r="F37" s="10"/>
     </row>
@@ -13594,16 +13807,16 @@
         <v>36</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>582</v>
+        <v>601</v>
       </c>
       <c r="C38" s="23" t="s">
-        <v>583</v>
+        <v>602</v>
       </c>
       <c r="D38" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>584</v>
+        <v>603</v>
       </c>
       <c r="F38" s="10"/>
     </row>
@@ -13612,16 +13825,16 @@
         <v>37</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>585</v>
+        <v>604</v>
       </c>
       <c r="C39" s="23" t="s">
-        <v>586</v>
+        <v>605</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>587</v>
+        <v>606</v>
       </c>
       <c r="F39" s="10"/>
     </row>
@@ -13630,16 +13843,16 @@
         <v>38</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>588</v>
+        <v>607</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>589</v>
+        <v>608</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>590</v>
+        <v>609</v>
       </c>
       <c r="F40" s="10"/>
     </row>
@@ -13651,13 +13864,13 @@
         <v>274</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>591</v>
+        <v>610</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>592</v>
+        <v>611</v>
       </c>
       <c r="F41" s="10"/>
     </row>
@@ -13666,16 +13879,16 @@
         <v>40</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>593</v>
+        <v>612</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>594</v>
+        <v>613</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>595</v>
+        <v>614</v>
       </c>
       <c r="F42" s="10"/>
     </row>
@@ -13684,16 +13897,16 @@
         <v>41</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>596</v>
+        <v>615</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>597</v>
+        <v>616</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>598</v>
+        <v>617</v>
       </c>
       <c r="F43" s="10"/>
     </row>
@@ -13702,16 +13915,16 @@
         <v>42</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>599</v>
+        <v>618</v>
       </c>
       <c r="C44" s="23" t="s">
-        <v>600</v>
+        <v>619</v>
       </c>
       <c r="D44" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>601</v>
+        <v>620</v>
       </c>
       <c r="F44" s="10"/>
     </row>
@@ -13720,16 +13933,16 @@
         <v>43</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>602</v>
+        <v>621</v>
       </c>
       <c r="C45" s="23" t="s">
-        <v>603</v>
+        <v>622</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>604</v>
+        <v>623</v>
       </c>
       <c r="F45" s="10"/>
     </row>
@@ -13741,13 +13954,13 @@
         <v>231</v>
       </c>
       <c r="C46" s="23" t="s">
-        <v>605</v>
+        <v>624</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>606</v>
+        <v>625</v>
       </c>
       <c r="F46" s="10"/>
     </row>
@@ -13756,16 +13969,16 @@
         <v>45</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>607</v>
+        <v>626</v>
       </c>
       <c r="C47" s="23" t="s">
-        <v>608</v>
+        <v>627</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>609</v>
+        <v>628</v>
       </c>
       <c r="F47" s="10"/>
     </row>
@@ -13777,13 +13990,13 @@
         <v>174</v>
       </c>
       <c r="C48" s="23" t="s">
-        <v>610</v>
+        <v>629</v>
       </c>
       <c r="D48" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>611</v>
+        <v>630</v>
       </c>
       <c r="F48" s="10"/>
     </row>
@@ -13792,16 +14005,16 @@
         <v>47</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>612</v>
+        <v>631</v>
       </c>
       <c r="C49" s="23" t="s">
-        <v>613</v>
+        <v>632</v>
       </c>
       <c r="D49" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E49" s="10" t="s">
-        <v>614</v>
+        <v>633</v>
       </c>
       <c r="F49" s="10"/>
     </row>
@@ -13810,16 +14023,16 @@
         <v>48</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>615</v>
+        <v>634</v>
       </c>
       <c r="C50" s="23" t="s">
-        <v>616</v>
+        <v>635</v>
       </c>
       <c r="D50" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>617</v>
+        <v>636</v>
       </c>
       <c r="F50" s="10"/>
     </row>
@@ -13828,16 +14041,16 @@
         <v>49</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>618</v>
+        <v>637</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>619</v>
+        <v>638</v>
       </c>
       <c r="D51" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>620</v>
+        <v>639</v>
       </c>
       <c r="F51" s="10"/>
     </row>
@@ -13846,16 +14059,16 @@
         <v>50</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>621</v>
+        <v>640</v>
       </c>
       <c r="C52" s="23" t="s">
-        <v>622</v>
+        <v>641</v>
       </c>
       <c r="D52" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>623</v>
+        <v>642</v>
       </c>
       <c r="F52" s="10"/>
     </row>
@@ -13864,16 +14077,16 @@
         <v>51</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>624</v>
+        <v>643</v>
       </c>
       <c r="C53" s="23" t="s">
-        <v>625</v>
+        <v>644</v>
       </c>
       <c r="D53" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>626</v>
+        <v>645</v>
       </c>
       <c r="F53" s="10"/>
     </row>
@@ -13882,16 +14095,16 @@
         <v>52</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>627</v>
+        <v>646</v>
       </c>
       <c r="C54" s="23" t="s">
-        <v>628</v>
+        <v>647</v>
       </c>
       <c r="D54" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>629</v>
+        <v>648</v>
       </c>
       <c r="F54" s="10"/>
     </row>
@@ -13900,16 +14113,16 @@
         <v>53</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>630</v>
+        <v>649</v>
       </c>
       <c r="C55" s="23" t="s">
-        <v>631</v>
+        <v>650</v>
       </c>
       <c r="D55" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>632</v>
+        <v>651</v>
       </c>
       <c r="F55" s="10"/>
     </row>
@@ -13918,16 +14131,16 @@
         <v>54</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>633</v>
+        <v>652</v>
       </c>
       <c r="C56" s="23" t="s">
-        <v>634</v>
+        <v>653</v>
       </c>
       <c r="D56" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E56" s="10" t="s">
-        <v>635</v>
+        <v>654</v>
       </c>
       <c r="F56" s="10"/>
     </row>
@@ -13936,16 +14149,16 @@
         <v>55</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>636</v>
+        <v>655</v>
       </c>
       <c r="C57" s="23" t="s">
-        <v>637</v>
+        <v>656</v>
       </c>
       <c r="D57" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>638</v>
+        <v>657</v>
       </c>
       <c r="F57" s="10"/>
     </row>
@@ -13954,16 +14167,16 @@
         <v>56</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>639</v>
+        <v>658</v>
       </c>
       <c r="C58" s="23" t="s">
-        <v>640</v>
+        <v>659</v>
       </c>
       <c r="D58" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E58" s="10" t="s">
-        <v>641</v>
+        <v>660</v>
       </c>
       <c r="F58" s="10"/>
     </row>
@@ -13975,13 +14188,13 @@
         <v>212</v>
       </c>
       <c r="C59" s="23" t="s">
-        <v>642</v>
+        <v>661</v>
       </c>
       <c r="D59" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>643</v>
+        <v>662</v>
       </c>
       <c r="F59" s="10"/>
     </row>
@@ -13993,13 +14206,13 @@
         <v>120</v>
       </c>
       <c r="C60" s="23" t="s">
-        <v>644</v>
+        <v>663</v>
       </c>
       <c r="D60" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E60" s="10" t="s">
-        <v>645</v>
+        <v>664</v>
       </c>
       <c r="F60" s="10"/>
     </row>
@@ -14011,13 +14224,13 @@
         <v>129</v>
       </c>
       <c r="C61" s="23" t="s">
-        <v>646</v>
+        <v>665</v>
       </c>
       <c r="D61" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E61" s="10" t="s">
-        <v>647</v>
+        <v>666</v>
       </c>
       <c r="F61" s="10"/>
     </row>
@@ -14029,13 +14242,13 @@
         <v>154</v>
       </c>
       <c r="C62" s="23" t="s">
-        <v>648</v>
+        <v>667</v>
       </c>
       <c r="D62" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E62" s="10" t="s">
-        <v>649</v>
+        <v>668</v>
       </c>
       <c r="F62" s="10"/>
     </row>
@@ -14044,16 +14257,16 @@
         <v>61</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>650</v>
+        <v>669</v>
       </c>
       <c r="C63" s="23" t="s">
-        <v>651</v>
+        <v>670</v>
       </c>
       <c r="D63" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E63" s="10" t="s">
-        <v>652</v>
+        <v>671</v>
       </c>
       <c r="F63" s="10"/>
     </row>
@@ -14065,13 +14278,13 @@
         <v>301</v>
       </c>
       <c r="C64" s="23" t="s">
-        <v>653</v>
+        <v>672</v>
       </c>
       <c r="D64" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E64" s="10" t="s">
-        <v>654</v>
+        <v>673</v>
       </c>
       <c r="F64" s="10"/>
     </row>
@@ -14080,16 +14293,16 @@
         <v>63</v>
       </c>
       <c r="B65" s="10" t="s">
-        <v>655</v>
+        <v>674</v>
       </c>
       <c r="C65" s="23" t="s">
-        <v>656</v>
+        <v>675</v>
       </c>
       <c r="D65" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E65" s="10" t="s">
-        <v>657</v>
+        <v>676</v>
       </c>
       <c r="F65" s="10"/>
     </row>
@@ -14098,19 +14311,19 @@
         <v>64</v>
       </c>
       <c r="B66" s="10" t="s">
-        <v>658</v>
+        <v>677</v>
       </c>
       <c r="C66" s="23" t="s">
-        <v>659</v>
+        <v>678</v>
       </c>
       <c r="D66" s="10" t="s">
-        <v>660</v>
+        <v>679</v>
       </c>
       <c r="E66" s="24" t="s">
-        <v>661</v>
+        <v>680</v>
       </c>
       <c r="F66" s="10" t="s">
-        <v>662</v>
+        <v>681</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
@@ -14121,13 +14334,13 @@
         <v>328</v>
       </c>
       <c r="C67" s="23" t="s">
-        <v>663</v>
+        <v>682</v>
       </c>
       <c r="D67" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>664</v>
+        <v>683</v>
       </c>
       <c r="F67" s="10"/>
     </row>
@@ -14136,16 +14349,16 @@
         <v>66</v>
       </c>
       <c r="B68" s="10" t="s">
-        <v>665</v>
+        <v>684</v>
       </c>
       <c r="C68" s="23" t="s">
-        <v>666</v>
+        <v>685</v>
       </c>
       <c r="D68" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E68" s="10" t="s">
-        <v>667</v>
+        <v>686</v>
       </c>
       <c r="F68" s="10"/>
     </row>
@@ -14154,16 +14367,16 @@
         <v>67</v>
       </c>
       <c r="B69" s="10" t="s">
-        <v>668</v>
+        <v>687</v>
       </c>
       <c r="C69" s="23" t="s">
-        <v>669</v>
+        <v>688</v>
       </c>
       <c r="D69" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E69" s="10" t="s">
-        <v>670</v>
+        <v>689</v>
       </c>
       <c r="F69" s="10"/>
     </row>
@@ -14172,16 +14385,16 @@
         <v>68</v>
       </c>
       <c r="B70" s="10" t="s">
-        <v>671</v>
+        <v>690</v>
       </c>
       <c r="C70" s="23" t="s">
-        <v>672</v>
+        <v>691</v>
       </c>
       <c r="D70" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E70" s="10" t="s">
-        <v>673</v>
+        <v>692</v>
       </c>
       <c r="F70" s="10"/>
     </row>
@@ -14193,13 +14406,13 @@
         <v>138</v>
       </c>
       <c r="C71" s="23" t="s">
-        <v>674</v>
+        <v>693</v>
       </c>
       <c r="D71" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E71" s="10" t="s">
-        <v>675</v>
+        <v>694</v>
       </c>
       <c r="F71" s="10"/>
     </row>
@@ -14208,16 +14421,16 @@
         <v>70</v>
       </c>
       <c r="B72" s="10" t="s">
-        <v>676</v>
+        <v>695</v>
       </c>
       <c r="C72" s="23" t="s">
-        <v>677</v>
+        <v>696</v>
       </c>
       <c r="D72" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E72" s="10" t="s">
-        <v>678</v>
+        <v>697</v>
       </c>
       <c r="F72" s="10"/>
     </row>
@@ -14226,16 +14439,16 @@
         <v>71</v>
       </c>
       <c r="B73" s="10" t="s">
-        <v>679</v>
+        <v>698</v>
       </c>
       <c r="C73" s="23" t="s">
-        <v>680</v>
+        <v>699</v>
       </c>
       <c r="D73" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E73" s="10" t="s">
-        <v>681</v>
+        <v>700</v>
       </c>
       <c r="F73" s="10"/>
     </row>
@@ -14247,13 +14460,13 @@
         <v>311</v>
       </c>
       <c r="C74" s="23" t="s">
-        <v>682</v>
+        <v>701</v>
       </c>
       <c r="D74" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E74" s="10" t="s">
-        <v>683</v>
+        <v>702</v>
       </c>
       <c r="F74" s="10"/>
     </row>
@@ -14262,19 +14475,19 @@
         <v>73</v>
       </c>
       <c r="B75" s="10" t="s">
-        <v>684</v>
+        <v>703</v>
       </c>
       <c r="C75" s="23" t="s">
-        <v>685</v>
+        <v>704</v>
       </c>
       <c r="D75" s="10" t="s">
-        <v>660</v>
+        <v>679</v>
       </c>
       <c r="E75" s="24" t="s">
-        <v>686</v>
+        <v>705</v>
       </c>
       <c r="F75" s="10" t="s">
-        <v>662</v>
+        <v>681</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
@@ -14282,16 +14495,16 @@
         <v>74</v>
       </c>
       <c r="B76" s="10" t="s">
-        <v>687</v>
+        <v>706</v>
       </c>
       <c r="C76" s="23" t="s">
-        <v>688</v>
+        <v>707</v>
       </c>
       <c r="D76" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E76" s="10" t="s">
-        <v>689</v>
+        <v>708</v>
       </c>
       <c r="F76" s="10"/>
     </row>
@@ -14300,16 +14513,16 @@
         <v>75</v>
       </c>
       <c r="B77" s="10" t="s">
-        <v>690</v>
+        <v>709</v>
       </c>
       <c r="C77" s="23" t="s">
-        <v>691</v>
+        <v>710</v>
       </c>
       <c r="D77" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>692</v>
+        <v>711</v>
       </c>
       <c r="F77" s="10"/>
     </row>
@@ -14318,16 +14531,16 @@
         <v>76</v>
       </c>
       <c r="B78" s="10" t="s">
-        <v>693</v>
+        <v>712</v>
       </c>
       <c r="C78" s="23" t="s">
-        <v>694</v>
+        <v>713</v>
       </c>
       <c r="D78" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E78" s="10" t="s">
-        <v>695</v>
+        <v>714</v>
       </c>
       <c r="F78" s="10"/>
     </row>
@@ -14339,13 +14552,13 @@
         <v>335</v>
       </c>
       <c r="C79" s="23" t="s">
-        <v>696</v>
+        <v>715</v>
       </c>
       <c r="D79" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E79" s="10" t="s">
-        <v>697</v>
+        <v>716</v>
       </c>
       <c r="F79" s="10"/>
     </row>
@@ -14354,16 +14567,16 @@
         <v>78</v>
       </c>
       <c r="B80" s="10" t="s">
-        <v>698</v>
+        <v>717</v>
       </c>
       <c r="C80" s="23" t="s">
-        <v>699</v>
+        <v>718</v>
       </c>
       <c r="D80" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E80" s="10" t="s">
-        <v>700</v>
+        <v>719</v>
       </c>
       <c r="F80" s="10"/>
     </row>
@@ -14372,16 +14585,16 @@
         <v>79</v>
       </c>
       <c r="B81" s="10" t="s">
-        <v>701</v>
+        <v>720</v>
       </c>
       <c r="C81" s="23" t="s">
-        <v>702</v>
+        <v>721</v>
       </c>
       <c r="D81" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>703</v>
+        <v>722</v>
       </c>
       <c r="F81" s="10"/>
     </row>
@@ -14393,13 +14606,13 @@
         <v>260</v>
       </c>
       <c r="C82" s="23" t="s">
-        <v>704</v>
+        <v>723</v>
       </c>
       <c r="D82" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E82" s="10" t="s">
-        <v>705</v>
+        <v>724</v>
       </c>
       <c r="F82" s="10"/>
     </row>
@@ -14411,13 +14624,13 @@
         <v>249</v>
       </c>
       <c r="C83" s="23" t="s">
-        <v>706</v>
+        <v>725</v>
       </c>
       <c r="D83" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>707</v>
+        <v>726</v>
       </c>
       <c r="F83" s="10"/>
     </row>
@@ -14426,16 +14639,16 @@
         <v>82</v>
       </c>
       <c r="B84" s="10" t="s">
-        <v>708</v>
+        <v>727</v>
       </c>
       <c r="C84" s="23" t="s">
-        <v>709</v>
+        <v>728</v>
       </c>
       <c r="D84" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E84" s="10" t="s">
-        <v>710</v>
+        <v>729</v>
       </c>
       <c r="F84" s="10"/>
     </row>
@@ -14444,16 +14657,16 @@
         <v>83</v>
       </c>
       <c r="B85" s="10" t="s">
-        <v>711</v>
+        <v>730</v>
       </c>
       <c r="C85" s="23" t="s">
-        <v>712</v>
+        <v>731</v>
       </c>
       <c r="D85" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E85" s="10" t="s">
-        <v>713</v>
+        <v>732</v>
       </c>
       <c r="F85" s="10"/>
     </row>
@@ -14462,16 +14675,16 @@
         <v>84</v>
       </c>
       <c r="B86" s="10" t="s">
-        <v>714</v>
+        <v>733</v>
       </c>
       <c r="C86" s="23" t="s">
-        <v>715</v>
+        <v>734</v>
       </c>
       <c r="D86" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E86" s="10" t="s">
-        <v>716</v>
+        <v>735</v>
       </c>
       <c r="F86" s="10"/>
     </row>
@@ -14480,16 +14693,16 @@
         <v>85</v>
       </c>
       <c r="B87" s="10" t="s">
-        <v>717</v>
+        <v>736</v>
       </c>
       <c r="C87" s="23" t="s">
-        <v>718</v>
+        <v>737</v>
       </c>
       <c r="D87" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E87" s="10" t="s">
-        <v>719</v>
+        <v>738</v>
       </c>
       <c r="F87" s="10"/>
     </row>
@@ -14498,16 +14711,16 @@
         <v>86</v>
       </c>
       <c r="B88" s="10" t="s">
-        <v>720</v>
+        <v>739</v>
       </c>
       <c r="C88" s="23" t="s">
-        <v>721</v>
+        <v>740</v>
       </c>
       <c r="D88" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E88" s="10" t="s">
-        <v>722</v>
+        <v>741</v>
       </c>
       <c r="F88" s="10"/>
     </row>
@@ -14516,16 +14729,16 @@
         <v>87</v>
       </c>
       <c r="B89" s="10" t="s">
-        <v>723</v>
+        <v>742</v>
       </c>
       <c r="C89" s="23" t="s">
-        <v>724</v>
+        <v>743</v>
       </c>
       <c r="D89" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E89" s="10" t="s">
-        <v>725</v>
+        <v>744</v>
       </c>
       <c r="F89" s="10"/>
     </row>
@@ -14534,16 +14747,16 @@
         <v>88</v>
       </c>
       <c r="B90" s="10" t="s">
-        <v>726</v>
+        <v>745</v>
       </c>
       <c r="C90" s="23" t="s">
-        <v>727</v>
+        <v>746</v>
       </c>
       <c r="D90" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E90" s="10" t="s">
-        <v>728</v>
+        <v>747</v>
       </c>
       <c r="F90" s="10"/>
     </row>
@@ -14552,16 +14765,16 @@
         <v>89</v>
       </c>
       <c r="B91" s="10" t="s">
-        <v>729</v>
+        <v>748</v>
       </c>
       <c r="C91" s="23" t="s">
-        <v>730</v>
+        <v>749</v>
       </c>
       <c r="D91" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E91" s="10" t="s">
-        <v>731</v>
+        <v>750</v>
       </c>
       <c r="F91" s="10"/>
     </row>
@@ -14573,13 +14786,13 @@
         <v>101</v>
       </c>
       <c r="C92" s="23" t="s">
-        <v>732</v>
+        <v>751</v>
       </c>
       <c r="D92" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E92" s="10" t="s">
-        <v>733</v>
+        <v>752</v>
       </c>
       <c r="F92" s="10"/>
     </row>
@@ -14588,16 +14801,16 @@
         <v>91</v>
       </c>
       <c r="B93" s="10" t="s">
-        <v>734</v>
+        <v>753</v>
       </c>
       <c r="C93" s="23" t="s">
-        <v>735</v>
+        <v>754</v>
       </c>
       <c r="D93" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E93" s="10" t="s">
-        <v>736</v>
+        <v>755</v>
       </c>
       <c r="F93" s="10"/>
     </row>
@@ -14606,16 +14819,16 @@
         <v>92</v>
       </c>
       <c r="B94" s="10" t="s">
-        <v>737</v>
+        <v>756</v>
       </c>
       <c r="C94" s="23" t="s">
-        <v>738</v>
+        <v>757</v>
       </c>
       <c r="D94" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E94" s="10" t="s">
-        <v>739</v>
+        <v>758</v>
       </c>
       <c r="F94" s="10"/>
     </row>
@@ -14624,16 +14837,16 @@
         <v>93</v>
       </c>
       <c r="B95" s="10" t="s">
-        <v>740</v>
+        <v>759</v>
       </c>
       <c r="C95" s="23" t="s">
-        <v>741</v>
+        <v>760</v>
       </c>
       <c r="D95" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E95" s="10" t="s">
-        <v>742</v>
+        <v>761</v>
       </c>
       <c r="F95" s="10"/>
     </row>
@@ -14642,16 +14855,16 @@
         <v>94</v>
       </c>
       <c r="B96" s="10" t="s">
-        <v>743</v>
+        <v>762</v>
       </c>
       <c r="C96" s="23" t="s">
-        <v>744</v>
+        <v>763</v>
       </c>
       <c r="D96" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E96" s="10" t="s">
-        <v>745</v>
+        <v>764</v>
       </c>
       <c r="F96" s="10"/>
     </row>
@@ -14660,16 +14873,16 @@
         <v>95</v>
       </c>
       <c r="B97" s="10" t="s">
-        <v>746</v>
+        <v>765</v>
       </c>
       <c r="C97" s="23" t="s">
-        <v>747</v>
+        <v>766</v>
       </c>
       <c r="D97" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E97" s="10" t="s">
-        <v>748</v>
+        <v>767</v>
       </c>
       <c r="F97" s="10"/>
     </row>
@@ -14678,16 +14891,16 @@
         <v>96</v>
       </c>
       <c r="B98" s="10" t="s">
-        <v>749</v>
+        <v>768</v>
       </c>
       <c r="C98" s="23" t="s">
-        <v>750</v>
+        <v>769</v>
       </c>
       <c r="D98" s="10" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E98" s="10" t="s">
-        <v>751</v>
+        <v>770</v>
       </c>
       <c r="F98" s="10"/>
     </row>
@@ -14699,13 +14912,13 @@
         <v>73</v>
       </c>
       <c r="C99" s="25" t="s">
-        <v>752</v>
+        <v>771</v>
       </c>
       <c r="D99" s="24" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E99" s="24" t="s">
-        <v>753</v>
+        <v>772</v>
       </c>
       <c r="F99" s="24"/>
     </row>
@@ -14717,13 +14930,13 @@
         <v>362</v>
       </c>
       <c r="C100" s="25" t="s">
-        <v>754</v>
+        <v>773</v>
       </c>
       <c r="D100" s="24" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E100" s="24" t="s">
-        <v>755</v>
+        <v>774</v>
       </c>
       <c r="F100" s="24"/>
     </row>
@@ -14735,13 +14948,13 @@
         <v>355</v>
       </c>
       <c r="C101" s="25" t="s">
-        <v>754</v>
+        <v>773</v>
       </c>
       <c r="D101" s="24" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E101" s="24" t="s">
-        <v>756</v>
+        <v>775</v>
       </c>
       <c r="F101" s="24"/>
     </row>
@@ -14753,13 +14966,13 @@
         <v>373</v>
       </c>
       <c r="C102" s="25" t="s">
-        <v>757</v>
+        <v>776</v>
       </c>
       <c r="D102" s="24" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E102" s="24" t="s">
-        <v>758</v>
+        <v>777</v>
       </c>
       <c r="F102" s="24"/>
     </row>
@@ -14771,13 +14984,13 @@
         <v>381</v>
       </c>
       <c r="C103" s="25" t="s">
-        <v>759</v>
+        <v>778</v>
       </c>
       <c r="D103" s="24" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E103" s="24" t="s">
-        <v>760</v>
+        <v>779</v>
       </c>
       <c r="F103" s="24"/>
     </row>
@@ -14789,13 +15002,13 @@
         <v>80</v>
       </c>
       <c r="C104" s="25" t="s">
-        <v>761</v>
+        <v>780</v>
       </c>
       <c r="D104" s="24" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E104" s="24" t="s">
-        <v>762</v>
+        <v>781</v>
       </c>
       <c r="F104" s="24"/>
     </row>
@@ -14807,13 +15020,13 @@
         <v>366</v>
       </c>
       <c r="C105" s="25" t="s">
-        <v>763</v>
+        <v>782</v>
       </c>
       <c r="D105" s="24" t="s">
-        <v>486</v>
+        <v>505</v>
       </c>
       <c r="E105" s="24" t="s">
-        <v>764</v>
+        <v>783</v>
       </c>
       <c r="F105" s="24"/>
     </row>
@@ -14946,7 +15159,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>765</v>
+        <v>784</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -14956,10 +15169,10 @@
         <v>44</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>766</v>
+        <v>785</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>767</v>
+        <v>786</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -14967,10 +15180,10 @@
         <v>47</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>768</v>
+        <v>787</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>769</v>
+        <v>788</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -14978,10 +15191,10 @@
         <v>49</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>770</v>
+        <v>789</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>771</v>
+        <v>790</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -14989,10 +15202,10 @@
         <v>51</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>772</v>
+        <v>791</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>773</v>
+        <v>792</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -15000,10 +15213,10 @@
         <v>53</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>774</v>
+        <v>793</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>775</v>
+        <v>794</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -15011,10 +15224,10 @@
         <v>55</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>776</v>
+        <v>795</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>777</v>
+        <v>796</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -15022,10 +15235,10 @@
         <v>56</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>778</v>
+        <v>797</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>779</v>
+        <v>798</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -15033,10 +15246,10 @@
         <v>57</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>780</v>
+        <v>799</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>781</v>
+        <v>800</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -15044,10 +15257,10 @@
         <v>58</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>782</v>
+        <v>801</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>783</v>
+        <v>802</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -15055,10 +15268,10 @@
         <v>59</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>784</v>
+        <v>803</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>785</v>
+        <v>804</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
prep: add Hercules Technical Customer Support (Upwork worldwide path)
Third Hercules role. Careers page is region-locked (NA/WEU/E-Australia,
Indonesia excluded) but Upwork listing is Worldwide = viable, no visa gate.
Automation/AI-forward angle matches her AI pipeline edge; client rated a
past hire down for not being AI-forward. Prep doc has answers to all 3
Upwork screening questions + honest CS-experience gap.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1750" uniqueCount="805">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1770" uniqueCount="815">
   <si>
     <t>Hana Aliyah Mufidah</t>
   </si>
@@ -1246,6 +1246,27 @@
     <t>SF Kearny/Bush in-office, strong preference; remote only for exceptional candidates on US TZ + regular travel. Stack TS/React/Tailwind/Clickhouse/Hono/Drizzle/Temporal. Gaps: high-end design/UX bar, newer stack pieces, US timezone. Full-Stack is the closer match. Prep: prep/hercules-frontend-engineer-2026-07-13.md</t>
   </si>
   <si>
+    <t>Technical Customer Support Engineer</t>
+  </si>
+  <si>
+    <t>https://www.upwork.com/jobs/Technical-Customer-Success-Specialist_~022074252517164606512/</t>
+  </si>
+  <si>
+    <t>User pick (Upwork + hercules.app/careers)</t>
+  </si>
+  <si>
+    <t>✅ Upwork listing = Worldwide (no visa gate). NOTE: careers page is region-locked NA/WEU/E-Australia, Indonesia excluded — apply via Upwork</t>
+  </si>
+  <si>
+    <t>AI-native support; automation to auto-resolve tickets = her AI-pipeline edge; TS/web/auth/payments core match; URGENT, hourly expert pay</t>
+  </si>
+  <si>
+    <t>Prep (urgent)</t>
+  </si>
+  <si>
+    <t>CS pivot off her SWE archetype but worldwide-remote + urgent + well-paid. Client rated a past hire down for not being AI-forward = her differentiator. Gaps: no formal customer-facing title, DNS depth. Prep: prep/hercules-technical-customer-support-engineer-2026-07-13.md</t>
+  </si>
+  <si>
     <t>Date</t>
   </si>
   <si>
@@ -1381,6 +1402,18 @@
     <t>prep/hercules-frontend-engineer-2026-07-13.md</t>
   </si>
   <si>
+    <t>Default CV (Upwork proposal matters more)</t>
+  </si>
+  <si>
+    <t>prep/hercules-technical-customer-support-engineer-2026-07-13.md</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>URGENT — apply via Upwork (Worldwide). 3 screening-question answers drafted. Lead with AI-forward automation.</t>
+  </si>
+  <si>
     <t>Date Applied</t>
   </si>
   <si>
@@ -2054,9 +2087,6 @@
   </si>
   <si>
     <t>https://job-boards.greenhouse.io/sumup</t>
-  </si>
-  <si>
-    <t>No</t>
   </si>
   <si>
     <t>Berlin / London. Payments fintech, EU + LATAM hiring. OFFICE-FIRST — not remote. Flexible work case-by-case via interview. Excluded from scans (relocation friction + many duplicates).</t>
@@ -3692,7 +3722,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:M128"/>
+  <dimension ref="A1:M129"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="5" style="1" customWidth="1"/>
@@ -8090,6 +8120,43 @@
       <c r="L128" s="20"/>
       <c r="M128" s="20" t="s">
         <v>408</v>
+      </c>
+    </row>
+    <row r="129" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A129" s="20">
+        <f>ROW()-1</f>
+      </c>
+      <c r="B129" s="20" t="s">
+        <v>396</v>
+      </c>
+      <c r="C129" s="20" t="s">
+        <v>397</v>
+      </c>
+      <c r="D129" s="20" t="s">
+        <v>409</v>
+      </c>
+      <c r="E129" s="20" t="s">
+        <v>410</v>
+      </c>
+      <c r="F129" s="20" t="s">
+        <v>411</v>
+      </c>
+      <c r="G129" s="20" t="s">
+        <v>412</v>
+      </c>
+      <c r="H129" s="20" t="s">
+        <v>413</v>
+      </c>
+      <c r="I129" s="20">
+        <v>4</v>
+      </c>
+      <c r="J129" s="20"/>
+      <c r="K129" s="20" t="s">
+        <v>414</v>
+      </c>
+      <c r="L129" s="20"/>
+      <c r="M129" s="20" t="s">
+        <v>415</v>
       </c>
     </row>
   </sheetData>
@@ -8215,7 +8282,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="5" style="1" customWidth="1"/>
@@ -8240,7 +8307,7 @@
         <v>61</v>
       </c>
       <c r="B1" s="21" t="s">
-        <v>409</v>
+        <v>416</v>
       </c>
       <c r="C1" s="21" t="s">
         <v>14</v>
@@ -8252,28 +8319,28 @@
         <v>63</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>410</v>
+        <v>417</v>
       </c>
       <c r="G1" s="21" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
       <c r="H1" s="21" t="s">
-        <v>412</v>
+        <v>419</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>413</v>
+        <v>420</v>
       </c>
       <c r="J1" s="21" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="K1" s="21" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="L1" s="21" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
       <c r="M1" s="21" t="s">
-        <v>417</v>
+        <v>424</v>
       </c>
       <c r="N1" s="21" t="s">
         <v>71</v>
@@ -8293,37 +8360,37 @@
         <v>80</v>
       </c>
       <c r="D2" s="22" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
       <c r="E2" s="22" t="s">
         <v>82</v>
       </c>
       <c r="F2" s="22" t="s">
-        <v>419</v>
+        <v>426</v>
       </c>
       <c r="G2" s="22" t="s">
-        <v>420</v>
+        <v>427</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>421</v>
+        <v>428</v>
       </c>
       <c r="I2" s="22" t="s">
-        <v>422</v>
+        <v>429</v>
       </c>
       <c r="J2" s="22" t="s">
-        <v>423</v>
+        <v>430</v>
       </c>
       <c r="K2" s="22" t="s">
-        <v>424</v>
+        <v>431</v>
       </c>
       <c r="L2" s="22" t="s">
-        <v>425</v>
+        <v>432</v>
       </c>
       <c r="M2" s="22" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
       <c r="N2" s="22" t="s">
-        <v>427</v>
+        <v>434</v>
       </c>
       <c r="O2" s="1"/>
     </row>
@@ -8338,37 +8405,37 @@
         <v>80</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>428</v>
+        <v>435</v>
       </c>
       <c r="E3" s="22" t="s">
         <v>88</v>
       </c>
       <c r="F3" s="22" t="s">
+        <v>436</v>
+      </c>
+      <c r="G3" s="22" t="s">
+        <v>437</v>
+      </c>
+      <c r="H3" s="20" t="s">
+        <v>438</v>
+      </c>
+      <c r="I3" s="22" t="s">
         <v>429</v>
       </c>
-      <c r="G3" s="22" t="s">
-        <v>430</v>
-      </c>
-      <c r="H3" s="20" t="s">
+      <c r="J3" s="22" t="s">
+        <v>439</v>
+      </c>
+      <c r="K3" s="22" t="s">
         <v>431</v>
       </c>
-      <c r="I3" s="22" t="s">
-        <v>422</v>
-      </c>
-      <c r="J3" s="22" t="s">
+      <c r="L3" s="22" t="s">
         <v>432</v>
       </c>
-      <c r="K3" s="22" t="s">
-        <v>424</v>
-      </c>
-      <c r="L3" s="22" t="s">
-        <v>425</v>
-      </c>
       <c r="M3" s="22" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
       <c r="N3" s="22" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="O3" s="1"/>
     </row>
@@ -8383,37 +8450,37 @@
         <v>80</v>
       </c>
       <c r="D4" s="22" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="E4" s="22" t="s">
         <v>91</v>
       </c>
       <c r="F4" s="22" t="s">
-        <v>435</v>
+        <v>442</v>
       </c>
       <c r="G4" s="22" t="s">
-        <v>436</v>
+        <v>443</v>
       </c>
       <c r="H4" s="20" t="s">
-        <v>437</v>
+        <v>444</v>
       </c>
       <c r="I4" s="22" t="s">
-        <v>438</v>
+        <v>445</v>
       </c>
       <c r="J4" s="22" t="s">
-        <v>439</v>
+        <v>446</v>
       </c>
       <c r="K4" s="22" t="s">
-        <v>440</v>
+        <v>447</v>
       </c>
       <c r="L4" s="22" t="s">
-        <v>425</v>
+        <v>432</v>
       </c>
       <c r="M4" s="22" t="s">
-        <v>441</v>
+        <v>448</v>
       </c>
       <c r="N4" s="22" t="s">
-        <v>442</v>
+        <v>449</v>
       </c>
       <c r="O4" s="1"/>
     </row>
@@ -8434,22 +8501,22 @@
         <v>346</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>443</v>
+        <v>450</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>444</v>
+        <v>451</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>445</v>
+        <v>452</v>
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1" t="s">
-        <v>446</v>
+        <v>453</v>
       </c>
       <c r="L5" s="1"/>
       <c r="M5" s="1" t="s">
-        <v>441</v>
+        <v>448</v>
       </c>
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
@@ -8471,27 +8538,27 @@
         <v>399</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>447</v>
+        <v>454</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="H6" s="20" t="s">
-        <v>449</v>
+        <v>456</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>450</v>
+        <v>457</v>
       </c>
       <c r="J6" s="1"/>
       <c r="K6" s="1" t="s">
-        <v>451</v>
+        <v>458</v>
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1" t="s">
-        <v>441</v>
+        <v>448</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>452</v>
+        <v>459</v>
       </c>
       <c r="O6" s="1"/>
     </row>
@@ -8512,29 +8579,70 @@
         <v>406</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>447</v>
+        <v>454</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="H7" s="20" t="s">
-        <v>453</v>
+        <v>460</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>450</v>
+        <v>457</v>
       </c>
       <c r="J7" s="1"/>
       <c r="K7" s="1" t="s">
-        <v>451</v>
+        <v>458</v>
       </c>
       <c r="L7" s="1"/>
       <c r="M7" s="1" t="s">
-        <v>441</v>
+        <v>448</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>452</v>
+        <v>459</v>
       </c>
       <c r="O7" s="1"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <f>ROW()-1</f>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>461</v>
+      </c>
+      <c r="H8" s="20" t="s">
+        <v>462</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="O8" s="1"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="P2:P1000">
@@ -8627,7 +8735,7 @@
         <v>61</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>454</v>
+        <v>465</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>14</v>
@@ -8636,10 +8744,10 @@
         <v>13</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>455</v>
+        <v>466</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>456</v>
+        <v>467</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>63</v>
@@ -8648,28 +8756,28 @@
         <v>44</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>457</v>
+        <v>468</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>458</v>
+        <v>469</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>459</v>
+        <v>470</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>460</v>
+        <v>471</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>461</v>
+        <v>472</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>462</v>
+        <v>473</v>
       </c>
       <c r="O1" s="7" t="s">
-        <v>463</v>
+        <v>474</v>
       </c>
       <c r="P1" s="7" t="s">
-        <v>464</v>
+        <v>475</v>
       </c>
       <c r="Q1" s="7" t="s">
         <v>71</v>
@@ -8692,10 +8800,10 @@
         <v>367</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>465</v>
+        <v>476</v>
       </c>
       <c r="F2" s="22" t="s">
-        <v>466</v>
+        <v>477</v>
       </c>
       <c r="G2" s="22" t="s">
         <v>368</v>
@@ -8707,24 +8815,24 @@
         <v>347</v>
       </c>
       <c r="J2" s="22" t="s">
-        <v>443</v>
+        <v>450</v>
       </c>
       <c r="K2" s="22" t="s">
-        <v>467</v>
+        <v>478</v>
       </c>
       <c r="L2" s="1"/>
       <c r="M2" s="22" t="s">
-        <v>468</v>
+        <v>479</v>
       </c>
       <c r="N2" s="1"/>
       <c r="O2" s="22" t="s">
-        <v>469</v>
+        <v>480</v>
       </c>
       <c r="P2" s="22" t="s">
-        <v>470</v>
+        <v>481</v>
       </c>
       <c r="Q2" s="22" t="s">
-        <v>471</v>
+        <v>482</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
@@ -8741,10 +8849,10 @@
         <v>374</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>472</v>
+        <v>483</v>
       </c>
       <c r="F3" s="22" t="s">
-        <v>473</v>
+        <v>484</v>
       </c>
       <c r="G3" s="22" t="s">
         <v>375</v>
@@ -8756,22 +8864,22 @@
         <v>347</v>
       </c>
       <c r="J3" s="22" t="s">
-        <v>443</v>
+        <v>450</v>
       </c>
       <c r="K3" s="22" t="s">
-        <v>474</v>
+        <v>485</v>
       </c>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
       <c r="O3" s="22" t="s">
-        <v>469</v>
+        <v>480</v>
       </c>
       <c r="P3" s="22" t="s">
-        <v>470</v>
+        <v>481</v>
       </c>
       <c r="Q3" s="22" t="s">
-        <v>475</v>
+        <v>486</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
@@ -8785,13 +8893,13 @@
         <v>80</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
       <c r="E4" s="22" t="s">
-        <v>476</v>
+        <v>487</v>
       </c>
       <c r="F4" s="22" t="s">
-        <v>477</v>
+        <v>488</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>82</v>
@@ -8803,28 +8911,28 @@
         <v>380</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>419</v>
+        <v>426</v>
       </c>
       <c r="K4" s="22" t="s">
-        <v>478</v>
+        <v>489</v>
       </c>
       <c r="L4" s="22" t="s">
-        <v>479</v>
+        <v>490</v>
       </c>
       <c r="M4" s="22" t="s">
+        <v>491</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="O4" s="22" t="s">
         <v>480</v>
       </c>
-      <c r="N4" s="1" t="s">
-        <v>481</v>
-      </c>
-      <c r="O4" s="22" t="s">
-        <v>469</v>
-      </c>
       <c r="P4" s="22" t="s">
-        <v>482</v>
+        <v>493</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>483</v>
+        <v>494</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
@@ -8838,13 +8946,13 @@
         <v>80</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>428</v>
+        <v>435</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>476</v>
+        <v>487</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>477</v>
+        <v>488</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>88</v>
@@ -8856,24 +8964,24 @@
         <v>380</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>429</v>
+        <v>436</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>478</v>
+        <v>489</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>484</v>
+        <v>495</v>
       </c>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
       <c r="O5" s="1" t="s">
-        <v>469</v>
+        <v>480</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>482</v>
+        <v>493</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>483</v>
+        <v>494</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
@@ -8890,7 +8998,7 @@
         <v>382</v>
       </c>
       <c r="E6" s="22" t="s">
-        <v>485</v>
+        <v>496</v>
       </c>
       <c r="F6" s="22" t="s">
         <v>384</v>
@@ -8905,26 +9013,26 @@
         <v>380</v>
       </c>
       <c r="J6" s="22" t="s">
-        <v>443</v>
+        <v>450</v>
       </c>
       <c r="K6" s="22" t="s">
-        <v>486</v>
+        <v>497</v>
       </c>
       <c r="L6" s="22"/>
       <c r="M6" s="22" t="s">
-        <v>487</v>
+        <v>498</v>
       </c>
       <c r="N6" s="22" t="s">
-        <v>488</v>
+        <v>499</v>
       </c>
       <c r="O6" s="22" t="s">
-        <v>469</v>
+        <v>480</v>
       </c>
       <c r="P6" s="22" t="s">
-        <v>482</v>
+        <v>493</v>
       </c>
       <c r="Q6" s="22" t="s">
-        <v>489</v>
+        <v>500</v>
       </c>
       <c r="R6" s="20"/>
     </row>
@@ -8939,16 +9047,16 @@
         <v>373</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>490</v>
+        <v>501</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>491</v>
+        <v>502</v>
       </c>
       <c r="F7" s="22" t="s">
-        <v>492</v>
+        <v>503</v>
       </c>
       <c r="G7" s="22" t="s">
-        <v>493</v>
+        <v>504</v>
       </c>
       <c r="H7" s="22" t="s">
         <v>51</v>
@@ -8959,18 +9067,18 @@
       <c r="J7" s="22"/>
       <c r="K7" s="22"/>
       <c r="L7" s="22" t="s">
-        <v>494</v>
+        <v>505</v>
       </c>
       <c r="M7" s="22"/>
       <c r="N7" s="22"/>
       <c r="O7" s="22" t="s">
-        <v>469</v>
+        <v>480</v>
       </c>
       <c r="P7" s="22" t="s">
-        <v>495</v>
+        <v>506</v>
       </c>
       <c r="Q7" s="22" t="s">
-        <v>496</v>
+        <v>507</v>
       </c>
       <c r="R7" s="20"/>
     </row>
@@ -13062,7 +13170,7 @@
         <v>356</v>
       </c>
       <c r="E202" s="20" t="s">
-        <v>497</v>
+        <v>508</v>
       </c>
       <c r="F202" s="20" t="s">
         <v>358</v>
@@ -13071,13 +13179,13 @@
         <v>357</v>
       </c>
       <c r="H202" s="20" t="s">
-        <v>498</v>
+        <v>509</v>
       </c>
       <c r="I202" s="20" t="s">
         <v>388</v>
       </c>
       <c r="J202" s="20" t="s">
-        <v>443</v>
+        <v>450</v>
       </c>
       <c r="K202" s="20"/>
       <c r="L202" s="20"/>
@@ -13148,7 +13256,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>499</v>
+        <v>510</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -13164,16 +13272,16 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>500</v>
+        <v>511</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>501</v>
+        <v>512</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>71</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>502</v>
+        <v>513</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -13181,13 +13289,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>503</v>
+        <v>514</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>504</v>
+        <v>515</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E3" s="10"/>
       <c r="F3" s="10"/>
@@ -13197,13 +13305,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>506</v>
+        <v>517</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>507</v>
+        <v>518</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E4" s="10"/>
       <c r="F4" s="10"/>
@@ -13213,16 +13321,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>508</v>
+        <v>519</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>509</v>
+        <v>520</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>510</v>
+        <v>521</v>
       </c>
       <c r="F5" s="10"/>
     </row>
@@ -13231,16 +13339,16 @@
         <v>4</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>511</v>
+        <v>522</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>512</v>
+        <v>523</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>513</v>
+        <v>524</v>
       </c>
       <c r="F6" s="10"/>
     </row>
@@ -13252,13 +13360,13 @@
         <v>240</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>514</v>
+        <v>525</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>515</v>
+        <v>526</v>
       </c>
       <c r="F7" s="10"/>
     </row>
@@ -13267,16 +13375,16 @@
         <v>6</v>
       </c>
       <c r="B8" s="10" t="s">
+        <v>527</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>528</v>
+      </c>
+      <c r="D8" s="10" t="s">
         <v>516</v>
       </c>
-      <c r="C8" s="23" t="s">
-        <v>517</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>505</v>
-      </c>
       <c r="E8" s="10" t="s">
-        <v>518</v>
+        <v>529</v>
       </c>
       <c r="F8" s="10"/>
     </row>
@@ -13285,16 +13393,16 @@
         <v>7</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>519</v>
+        <v>530</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>520</v>
+        <v>531</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>521</v>
+        <v>532</v>
       </c>
       <c r="F9" s="10"/>
     </row>
@@ -13306,13 +13414,13 @@
         <v>141</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>522</v>
+        <v>533</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>523</v>
+        <v>534</v>
       </c>
       <c r="F10" s="10"/>
     </row>
@@ -13321,16 +13429,16 @@
         <v>9</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>524</v>
+        <v>535</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>525</v>
+        <v>536</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>526</v>
+        <v>537</v>
       </c>
       <c r="F11" s="10"/>
     </row>
@@ -13339,16 +13447,16 @@
         <v>10</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>527</v>
+        <v>538</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>528</v>
+        <v>539</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>529</v>
+        <v>540</v>
       </c>
       <c r="F12" s="10"/>
     </row>
@@ -13357,16 +13465,16 @@
         <v>11</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>531</v>
+        <v>542</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>532</v>
+        <v>543</v>
       </c>
       <c r="F13" s="10"/>
     </row>
@@ -13375,16 +13483,16 @@
         <v>12</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>533</v>
+        <v>544</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>534</v>
+        <v>545</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>535</v>
+        <v>546</v>
       </c>
       <c r="F14" s="10"/>
     </row>
@@ -13393,16 +13501,16 @@
         <v>13</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>536</v>
+        <v>547</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>537</v>
+        <v>548</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>538</v>
+        <v>549</v>
       </c>
       <c r="F15" s="10"/>
     </row>
@@ -13411,16 +13519,16 @@
         <v>14</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>540</v>
+        <v>551</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>541</v>
+        <v>552</v>
       </c>
       <c r="F16" s="10"/>
     </row>
@@ -13429,16 +13537,16 @@
         <v>15</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>542</v>
+        <v>553</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>543</v>
+        <v>554</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>544</v>
+        <v>555</v>
       </c>
       <c r="F17" s="10"/>
     </row>
@@ -13447,16 +13555,16 @@
         <v>16</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>545</v>
+        <v>556</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>546</v>
+        <v>557</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>547</v>
+        <v>558</v>
       </c>
       <c r="F18" s="10"/>
     </row>
@@ -13468,13 +13576,13 @@
         <v>179</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>548</v>
+        <v>559</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>549</v>
+        <v>560</v>
       </c>
       <c r="F19" s="10"/>
     </row>
@@ -13483,16 +13591,16 @@
         <v>18</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>550</v>
+        <v>561</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>551</v>
+        <v>562</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>552</v>
+        <v>563</v>
       </c>
       <c r="F20" s="10"/>
     </row>
@@ -13501,16 +13609,16 @@
         <v>19</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>553</v>
+        <v>564</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>554</v>
+        <v>565</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>555</v>
+        <v>566</v>
       </c>
       <c r="F21" s="10"/>
     </row>
@@ -13519,16 +13627,16 @@
         <v>20</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>556</v>
+        <v>567</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>557</v>
+        <v>568</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>558</v>
+        <v>569</v>
       </c>
       <c r="F22" s="10"/>
     </row>
@@ -13537,16 +13645,16 @@
         <v>21</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>559</v>
+        <v>570</v>
       </c>
       <c r="C23" s="23" t="s">
-        <v>560</v>
+        <v>571</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>561</v>
+        <v>572</v>
       </c>
       <c r="F23" s="10"/>
     </row>
@@ -13555,16 +13663,16 @@
         <v>22</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>562</v>
+        <v>573</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>563</v>
+        <v>574</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>564</v>
+        <v>575</v>
       </c>
       <c r="F24" s="10"/>
     </row>
@@ -13573,16 +13681,16 @@
         <v>23</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>565</v>
+        <v>576</v>
       </c>
       <c r="C25" s="23" t="s">
-        <v>566</v>
+        <v>577</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>567</v>
+        <v>578</v>
       </c>
       <c r="F25" s="10"/>
     </row>
@@ -13591,16 +13699,16 @@
         <v>24</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>568</v>
+        <v>579</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>569</v>
+        <v>580</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>570</v>
+        <v>581</v>
       </c>
       <c r="F26" s="10"/>
     </row>
@@ -13609,16 +13717,16 @@
         <v>25</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>571</v>
+        <v>582</v>
       </c>
       <c r="C27" s="23" t="s">
-        <v>572</v>
+        <v>583</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>573</v>
+        <v>584</v>
       </c>
       <c r="F27" s="10"/>
     </row>
@@ -13627,16 +13735,16 @@
         <v>26</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>574</v>
+        <v>585</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>575</v>
+        <v>586</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>576</v>
+        <v>587</v>
       </c>
       <c r="F28" s="10"/>
     </row>
@@ -13645,16 +13753,16 @@
         <v>27</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>577</v>
+        <v>588</v>
       </c>
       <c r="C29" s="23" t="s">
-        <v>578</v>
+        <v>589</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>579</v>
+        <v>590</v>
       </c>
       <c r="F29" s="10"/>
     </row>
@@ -13663,16 +13771,16 @@
         <v>28</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>580</v>
+        <v>591</v>
       </c>
       <c r="C30" s="23" t="s">
-        <v>581</v>
+        <v>592</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>582</v>
+        <v>593</v>
       </c>
       <c r="F30" s="10"/>
     </row>
@@ -13681,16 +13789,16 @@
         <v>29</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="C31" s="23" t="s">
-        <v>584</v>
+        <v>595</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>585</v>
+        <v>596</v>
       </c>
       <c r="F31" s="10"/>
     </row>
@@ -13699,16 +13807,16 @@
         <v>30</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>586</v>
+        <v>597</v>
       </c>
       <c r="C32" s="23" t="s">
-        <v>587</v>
+        <v>598</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>588</v>
+        <v>599</v>
       </c>
       <c r="F32" s="10"/>
     </row>
@@ -13717,16 +13825,16 @@
         <v>31</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>589</v>
+        <v>600</v>
       </c>
       <c r="C33" s="23" t="s">
-        <v>590</v>
+        <v>601</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>591</v>
+        <v>602</v>
       </c>
       <c r="F33" s="10"/>
     </row>
@@ -13738,13 +13846,13 @@
         <v>108</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>592</v>
+        <v>603</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>593</v>
+        <v>604</v>
       </c>
       <c r="F34" s="10"/>
     </row>
@@ -13756,13 +13864,13 @@
         <v>344</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>594</v>
+        <v>605</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>595</v>
+        <v>606</v>
       </c>
       <c r="F35" s="10"/>
     </row>
@@ -13771,16 +13879,16 @@
         <v>34</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>596</v>
+        <v>607</v>
       </c>
       <c r="C36" s="23" t="s">
-        <v>597</v>
+        <v>608</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>598</v>
+        <v>609</v>
       </c>
       <c r="F36" s="10"/>
     </row>
@@ -13792,13 +13900,13 @@
         <v>113</v>
       </c>
       <c r="C37" s="23" t="s">
-        <v>599</v>
+        <v>610</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>600</v>
+        <v>611</v>
       </c>
       <c r="F37" s="10"/>
     </row>
@@ -13807,16 +13915,16 @@
         <v>36</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>601</v>
+        <v>612</v>
       </c>
       <c r="C38" s="23" t="s">
-        <v>602</v>
+        <v>613</v>
       </c>
       <c r="D38" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>603</v>
+        <v>614</v>
       </c>
       <c r="F38" s="10"/>
     </row>
@@ -13825,16 +13933,16 @@
         <v>37</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>604</v>
+        <v>615</v>
       </c>
       <c r="C39" s="23" t="s">
-        <v>605</v>
+        <v>616</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>606</v>
+        <v>617</v>
       </c>
       <c r="F39" s="10"/>
     </row>
@@ -13843,16 +13951,16 @@
         <v>38</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>607</v>
+        <v>618</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>608</v>
+        <v>619</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>609</v>
+        <v>620</v>
       </c>
       <c r="F40" s="10"/>
     </row>
@@ -13864,13 +13972,13 @@
         <v>274</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>610</v>
+        <v>621</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>611</v>
+        <v>622</v>
       </c>
       <c r="F41" s="10"/>
     </row>
@@ -13879,16 +13987,16 @@
         <v>40</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>612</v>
+        <v>623</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>613</v>
+        <v>624</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>614</v>
+        <v>625</v>
       </c>
       <c r="F42" s="10"/>
     </row>
@@ -13897,16 +14005,16 @@
         <v>41</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>615</v>
+        <v>626</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>616</v>
+        <v>627</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>617</v>
+        <v>628</v>
       </c>
       <c r="F43" s="10"/>
     </row>
@@ -13915,16 +14023,16 @@
         <v>42</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>618</v>
+        <v>629</v>
       </c>
       <c r="C44" s="23" t="s">
-        <v>619</v>
+        <v>630</v>
       </c>
       <c r="D44" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>620</v>
+        <v>631</v>
       </c>
       <c r="F44" s="10"/>
     </row>
@@ -13933,16 +14041,16 @@
         <v>43</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>621</v>
+        <v>632</v>
       </c>
       <c r="C45" s="23" t="s">
-        <v>622</v>
+        <v>633</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>623</v>
+        <v>634</v>
       </c>
       <c r="F45" s="10"/>
     </row>
@@ -13954,13 +14062,13 @@
         <v>231</v>
       </c>
       <c r="C46" s="23" t="s">
-        <v>624</v>
+        <v>635</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>625</v>
+        <v>636</v>
       </c>
       <c r="F46" s="10"/>
     </row>
@@ -13969,16 +14077,16 @@
         <v>45</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>626</v>
+        <v>637</v>
       </c>
       <c r="C47" s="23" t="s">
-        <v>627</v>
+        <v>638</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>628</v>
+        <v>639</v>
       </c>
       <c r="F47" s="10"/>
     </row>
@@ -13990,13 +14098,13 @@
         <v>174</v>
       </c>
       <c r="C48" s="23" t="s">
-        <v>629</v>
+        <v>640</v>
       </c>
       <c r="D48" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>630</v>
+        <v>641</v>
       </c>
       <c r="F48" s="10"/>
     </row>
@@ -14005,16 +14113,16 @@
         <v>47</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>631</v>
+        <v>642</v>
       </c>
       <c r="C49" s="23" t="s">
-        <v>632</v>
+        <v>643</v>
       </c>
       <c r="D49" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E49" s="10" t="s">
-        <v>633</v>
+        <v>644</v>
       </c>
       <c r="F49" s="10"/>
     </row>
@@ -14023,16 +14131,16 @@
         <v>48</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>634</v>
+        <v>645</v>
       </c>
       <c r="C50" s="23" t="s">
-        <v>635</v>
+        <v>646</v>
       </c>
       <c r="D50" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>636</v>
+        <v>647</v>
       </c>
       <c r="F50" s="10"/>
     </row>
@@ -14041,16 +14149,16 @@
         <v>49</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>637</v>
+        <v>648</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>638</v>
+        <v>649</v>
       </c>
       <c r="D51" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>639</v>
+        <v>650</v>
       </c>
       <c r="F51" s="10"/>
     </row>
@@ -14059,16 +14167,16 @@
         <v>50</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>640</v>
+        <v>651</v>
       </c>
       <c r="C52" s="23" t="s">
-        <v>641</v>
+        <v>652</v>
       </c>
       <c r="D52" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>642</v>
+        <v>653</v>
       </c>
       <c r="F52" s="10"/>
     </row>
@@ -14077,16 +14185,16 @@
         <v>51</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>643</v>
+        <v>654</v>
       </c>
       <c r="C53" s="23" t="s">
-        <v>644</v>
+        <v>655</v>
       </c>
       <c r="D53" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>645</v>
+        <v>656</v>
       </c>
       <c r="F53" s="10"/>
     </row>
@@ -14095,16 +14203,16 @@
         <v>52</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>646</v>
+        <v>657</v>
       </c>
       <c r="C54" s="23" t="s">
-        <v>647</v>
+        <v>658</v>
       </c>
       <c r="D54" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>648</v>
+        <v>659</v>
       </c>
       <c r="F54" s="10"/>
     </row>
@@ -14113,16 +14221,16 @@
         <v>53</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>649</v>
+        <v>660</v>
       </c>
       <c r="C55" s="23" t="s">
-        <v>650</v>
+        <v>661</v>
       </c>
       <c r="D55" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>651</v>
+        <v>662</v>
       </c>
       <c r="F55" s="10"/>
     </row>
@@ -14131,16 +14239,16 @@
         <v>54</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>652</v>
+        <v>663</v>
       </c>
       <c r="C56" s="23" t="s">
-        <v>653</v>
+        <v>664</v>
       </c>
       <c r="D56" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E56" s="10" t="s">
-        <v>654</v>
+        <v>665</v>
       </c>
       <c r="F56" s="10"/>
     </row>
@@ -14149,16 +14257,16 @@
         <v>55</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>655</v>
+        <v>666</v>
       </c>
       <c r="C57" s="23" t="s">
-        <v>656</v>
+        <v>667</v>
       </c>
       <c r="D57" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>657</v>
+        <v>668</v>
       </c>
       <c r="F57" s="10"/>
     </row>
@@ -14167,16 +14275,16 @@
         <v>56</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>658</v>
+        <v>669</v>
       </c>
       <c r="C58" s="23" t="s">
-        <v>659</v>
+        <v>670</v>
       </c>
       <c r="D58" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E58" s="10" t="s">
-        <v>660</v>
+        <v>671</v>
       </c>
       <c r="F58" s="10"/>
     </row>
@@ -14188,13 +14296,13 @@
         <v>212</v>
       </c>
       <c r="C59" s="23" t="s">
-        <v>661</v>
+        <v>672</v>
       </c>
       <c r="D59" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>662</v>
+        <v>673</v>
       </c>
       <c r="F59" s="10"/>
     </row>
@@ -14206,13 +14314,13 @@
         <v>120</v>
       </c>
       <c r="C60" s="23" t="s">
-        <v>663</v>
+        <v>674</v>
       </c>
       <c r="D60" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E60" s="10" t="s">
-        <v>664</v>
+        <v>675</v>
       </c>
       <c r="F60" s="10"/>
     </row>
@@ -14224,13 +14332,13 @@
         <v>129</v>
       </c>
       <c r="C61" s="23" t="s">
-        <v>665</v>
+        <v>676</v>
       </c>
       <c r="D61" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E61" s="10" t="s">
-        <v>666</v>
+        <v>677</v>
       </c>
       <c r="F61" s="10"/>
     </row>
@@ -14242,13 +14350,13 @@
         <v>154</v>
       </c>
       <c r="C62" s="23" t="s">
-        <v>667</v>
+        <v>678</v>
       </c>
       <c r="D62" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E62" s="10" t="s">
-        <v>668</v>
+        <v>679</v>
       </c>
       <c r="F62" s="10"/>
     </row>
@@ -14257,16 +14365,16 @@
         <v>61</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>669</v>
+        <v>680</v>
       </c>
       <c r="C63" s="23" t="s">
-        <v>670</v>
+        <v>681</v>
       </c>
       <c r="D63" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E63" s="10" t="s">
-        <v>671</v>
+        <v>682</v>
       </c>
       <c r="F63" s="10"/>
     </row>
@@ -14278,13 +14386,13 @@
         <v>301</v>
       </c>
       <c r="C64" s="23" t="s">
-        <v>672</v>
+        <v>683</v>
       </c>
       <c r="D64" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E64" s="10" t="s">
-        <v>673</v>
+        <v>684</v>
       </c>
       <c r="F64" s="10"/>
     </row>
@@ -14293,16 +14401,16 @@
         <v>63</v>
       </c>
       <c r="B65" s="10" t="s">
-        <v>674</v>
+        <v>685</v>
       </c>
       <c r="C65" s="23" t="s">
-        <v>675</v>
+        <v>686</v>
       </c>
       <c r="D65" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E65" s="10" t="s">
-        <v>676</v>
+        <v>687</v>
       </c>
       <c r="F65" s="10"/>
     </row>
@@ -14311,19 +14419,19 @@
         <v>64</v>
       </c>
       <c r="B66" s="10" t="s">
-        <v>677</v>
+        <v>688</v>
       </c>
       <c r="C66" s="23" t="s">
-        <v>678</v>
+        <v>689</v>
       </c>
       <c r="D66" s="10" t="s">
-        <v>679</v>
+        <v>463</v>
       </c>
       <c r="E66" s="24" t="s">
-        <v>680</v>
+        <v>690</v>
       </c>
       <c r="F66" s="10" t="s">
-        <v>681</v>
+        <v>691</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
@@ -14334,13 +14442,13 @@
         <v>328</v>
       </c>
       <c r="C67" s="23" t="s">
-        <v>682</v>
+        <v>692</v>
       </c>
       <c r="D67" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>683</v>
+        <v>693</v>
       </c>
       <c r="F67" s="10"/>
     </row>
@@ -14349,16 +14457,16 @@
         <v>66</v>
       </c>
       <c r="B68" s="10" t="s">
-        <v>684</v>
+        <v>694</v>
       </c>
       <c r="C68" s="23" t="s">
-        <v>685</v>
+        <v>695</v>
       </c>
       <c r="D68" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E68" s="10" t="s">
-        <v>686</v>
+        <v>696</v>
       </c>
       <c r="F68" s="10"/>
     </row>
@@ -14367,16 +14475,16 @@
         <v>67</v>
       </c>
       <c r="B69" s="10" t="s">
-        <v>687</v>
+        <v>697</v>
       </c>
       <c r="C69" s="23" t="s">
-        <v>688</v>
+        <v>698</v>
       </c>
       <c r="D69" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E69" s="10" t="s">
-        <v>689</v>
+        <v>699</v>
       </c>
       <c r="F69" s="10"/>
     </row>
@@ -14385,16 +14493,16 @@
         <v>68</v>
       </c>
       <c r="B70" s="10" t="s">
-        <v>690</v>
+        <v>700</v>
       </c>
       <c r="C70" s="23" t="s">
-        <v>691</v>
+        <v>701</v>
       </c>
       <c r="D70" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E70" s="10" t="s">
-        <v>692</v>
+        <v>702</v>
       </c>
       <c r="F70" s="10"/>
     </row>
@@ -14406,13 +14514,13 @@
         <v>138</v>
       </c>
       <c r="C71" s="23" t="s">
-        <v>693</v>
+        <v>703</v>
       </c>
       <c r="D71" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E71" s="10" t="s">
-        <v>694</v>
+        <v>704</v>
       </c>
       <c r="F71" s="10"/>
     </row>
@@ -14421,16 +14529,16 @@
         <v>70</v>
       </c>
       <c r="B72" s="10" t="s">
-        <v>695</v>
+        <v>705</v>
       </c>
       <c r="C72" s="23" t="s">
-        <v>696</v>
+        <v>706</v>
       </c>
       <c r="D72" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E72" s="10" t="s">
-        <v>697</v>
+        <v>707</v>
       </c>
       <c r="F72" s="10"/>
     </row>
@@ -14439,16 +14547,16 @@
         <v>71</v>
       </c>
       <c r="B73" s="10" t="s">
-        <v>698</v>
+        <v>708</v>
       </c>
       <c r="C73" s="23" t="s">
-        <v>699</v>
+        <v>709</v>
       </c>
       <c r="D73" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E73" s="10" t="s">
-        <v>700</v>
+        <v>710</v>
       </c>
       <c r="F73" s="10"/>
     </row>
@@ -14460,13 +14568,13 @@
         <v>311</v>
       </c>
       <c r="C74" s="23" t="s">
-        <v>701</v>
+        <v>711</v>
       </c>
       <c r="D74" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E74" s="10" t="s">
-        <v>702</v>
+        <v>712</v>
       </c>
       <c r="F74" s="10"/>
     </row>
@@ -14475,19 +14583,19 @@
         <v>73</v>
       </c>
       <c r="B75" s="10" t="s">
-        <v>703</v>
+        <v>713</v>
       </c>
       <c r="C75" s="23" t="s">
-        <v>704</v>
+        <v>714</v>
       </c>
       <c r="D75" s="10" t="s">
-        <v>679</v>
+        <v>463</v>
       </c>
       <c r="E75" s="24" t="s">
-        <v>705</v>
+        <v>715</v>
       </c>
       <c r="F75" s="10" t="s">
-        <v>681</v>
+        <v>691</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
@@ -14495,16 +14603,16 @@
         <v>74</v>
       </c>
       <c r="B76" s="10" t="s">
-        <v>706</v>
+        <v>716</v>
       </c>
       <c r="C76" s="23" t="s">
-        <v>707</v>
+        <v>717</v>
       </c>
       <c r="D76" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E76" s="10" t="s">
-        <v>708</v>
+        <v>718</v>
       </c>
       <c r="F76" s="10"/>
     </row>
@@ -14513,16 +14621,16 @@
         <v>75</v>
       </c>
       <c r="B77" s="10" t="s">
-        <v>709</v>
+        <v>719</v>
       </c>
       <c r="C77" s="23" t="s">
-        <v>710</v>
+        <v>720</v>
       </c>
       <c r="D77" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>711</v>
+        <v>721</v>
       </c>
       <c r="F77" s="10"/>
     </row>
@@ -14531,16 +14639,16 @@
         <v>76</v>
       </c>
       <c r="B78" s="10" t="s">
-        <v>712</v>
+        <v>722</v>
       </c>
       <c r="C78" s="23" t="s">
-        <v>713</v>
+        <v>723</v>
       </c>
       <c r="D78" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E78" s="10" t="s">
-        <v>714</v>
+        <v>724</v>
       </c>
       <c r="F78" s="10"/>
     </row>
@@ -14552,13 +14660,13 @@
         <v>335</v>
       </c>
       <c r="C79" s="23" t="s">
-        <v>715</v>
+        <v>725</v>
       </c>
       <c r="D79" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E79" s="10" t="s">
-        <v>716</v>
+        <v>726</v>
       </c>
       <c r="F79" s="10"/>
     </row>
@@ -14567,16 +14675,16 @@
         <v>78</v>
       </c>
       <c r="B80" s="10" t="s">
-        <v>717</v>
+        <v>727</v>
       </c>
       <c r="C80" s="23" t="s">
-        <v>718</v>
+        <v>728</v>
       </c>
       <c r="D80" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E80" s="10" t="s">
-        <v>719</v>
+        <v>729</v>
       </c>
       <c r="F80" s="10"/>
     </row>
@@ -14585,16 +14693,16 @@
         <v>79</v>
       </c>
       <c r="B81" s="10" t="s">
-        <v>720</v>
+        <v>730</v>
       </c>
       <c r="C81" s="23" t="s">
-        <v>721</v>
+        <v>731</v>
       </c>
       <c r="D81" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>722</v>
+        <v>732</v>
       </c>
       <c r="F81" s="10"/>
     </row>
@@ -14606,13 +14714,13 @@
         <v>260</v>
       </c>
       <c r="C82" s="23" t="s">
-        <v>723</v>
+        <v>733</v>
       </c>
       <c r="D82" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E82" s="10" t="s">
-        <v>724</v>
+        <v>734</v>
       </c>
       <c r="F82" s="10"/>
     </row>
@@ -14624,13 +14732,13 @@
         <v>249</v>
       </c>
       <c r="C83" s="23" t="s">
-        <v>725</v>
+        <v>735</v>
       </c>
       <c r="D83" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>726</v>
+        <v>736</v>
       </c>
       <c r="F83" s="10"/>
     </row>
@@ -14639,16 +14747,16 @@
         <v>82</v>
       </c>
       <c r="B84" s="10" t="s">
-        <v>727</v>
+        <v>737</v>
       </c>
       <c r="C84" s="23" t="s">
-        <v>728</v>
+        <v>738</v>
       </c>
       <c r="D84" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E84" s="10" t="s">
-        <v>729</v>
+        <v>739</v>
       </c>
       <c r="F84" s="10"/>
     </row>
@@ -14657,16 +14765,16 @@
         <v>83</v>
       </c>
       <c r="B85" s="10" t="s">
-        <v>730</v>
+        <v>740</v>
       </c>
       <c r="C85" s="23" t="s">
-        <v>731</v>
+        <v>741</v>
       </c>
       <c r="D85" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E85" s="10" t="s">
-        <v>732</v>
+        <v>742</v>
       </c>
       <c r="F85" s="10"/>
     </row>
@@ -14675,16 +14783,16 @@
         <v>84</v>
       </c>
       <c r="B86" s="10" t="s">
-        <v>733</v>
+        <v>743</v>
       </c>
       <c r="C86" s="23" t="s">
-        <v>734</v>
+        <v>744</v>
       </c>
       <c r="D86" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E86" s="10" t="s">
-        <v>735</v>
+        <v>745</v>
       </c>
       <c r="F86" s="10"/>
     </row>
@@ -14693,16 +14801,16 @@
         <v>85</v>
       </c>
       <c r="B87" s="10" t="s">
-        <v>736</v>
+        <v>746</v>
       </c>
       <c r="C87" s="23" t="s">
-        <v>737</v>
+        <v>747</v>
       </c>
       <c r="D87" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E87" s="10" t="s">
-        <v>738</v>
+        <v>748</v>
       </c>
       <c r="F87" s="10"/>
     </row>
@@ -14711,16 +14819,16 @@
         <v>86</v>
       </c>
       <c r="B88" s="10" t="s">
-        <v>739</v>
+        <v>749</v>
       </c>
       <c r="C88" s="23" t="s">
-        <v>740</v>
+        <v>750</v>
       </c>
       <c r="D88" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E88" s="10" t="s">
-        <v>741</v>
+        <v>751</v>
       </c>
       <c r="F88" s="10"/>
     </row>
@@ -14729,16 +14837,16 @@
         <v>87</v>
       </c>
       <c r="B89" s="10" t="s">
-        <v>742</v>
+        <v>752</v>
       </c>
       <c r="C89" s="23" t="s">
-        <v>743</v>
+        <v>753</v>
       </c>
       <c r="D89" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E89" s="10" t="s">
-        <v>744</v>
+        <v>754</v>
       </c>
       <c r="F89" s="10"/>
     </row>
@@ -14747,16 +14855,16 @@
         <v>88</v>
       </c>
       <c r="B90" s="10" t="s">
-        <v>745</v>
+        <v>755</v>
       </c>
       <c r="C90" s="23" t="s">
-        <v>746</v>
+        <v>756</v>
       </c>
       <c r="D90" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E90" s="10" t="s">
-        <v>747</v>
+        <v>757</v>
       </c>
       <c r="F90" s="10"/>
     </row>
@@ -14765,16 +14873,16 @@
         <v>89</v>
       </c>
       <c r="B91" s="10" t="s">
-        <v>748</v>
+        <v>758</v>
       </c>
       <c r="C91" s="23" t="s">
-        <v>749</v>
+        <v>759</v>
       </c>
       <c r="D91" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E91" s="10" t="s">
-        <v>750</v>
+        <v>760</v>
       </c>
       <c r="F91" s="10"/>
     </row>
@@ -14786,13 +14894,13 @@
         <v>101</v>
       </c>
       <c r="C92" s="23" t="s">
-        <v>751</v>
+        <v>761</v>
       </c>
       <c r="D92" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E92" s="10" t="s">
-        <v>752</v>
+        <v>762</v>
       </c>
       <c r="F92" s="10"/>
     </row>
@@ -14801,16 +14909,16 @@
         <v>91</v>
       </c>
       <c r="B93" s="10" t="s">
-        <v>753</v>
+        <v>763</v>
       </c>
       <c r="C93" s="23" t="s">
-        <v>754</v>
+        <v>764</v>
       </c>
       <c r="D93" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E93" s="10" t="s">
-        <v>755</v>
+        <v>765</v>
       </c>
       <c r="F93" s="10"/>
     </row>
@@ -14819,16 +14927,16 @@
         <v>92</v>
       </c>
       <c r="B94" s="10" t="s">
-        <v>756</v>
+        <v>766</v>
       </c>
       <c r="C94" s="23" t="s">
-        <v>757</v>
+        <v>767</v>
       </c>
       <c r="D94" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E94" s="10" t="s">
-        <v>758</v>
+        <v>768</v>
       </c>
       <c r="F94" s="10"/>
     </row>
@@ -14837,16 +14945,16 @@
         <v>93</v>
       </c>
       <c r="B95" s="10" t="s">
-        <v>759</v>
+        <v>769</v>
       </c>
       <c r="C95" s="23" t="s">
-        <v>760</v>
+        <v>770</v>
       </c>
       <c r="D95" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E95" s="10" t="s">
-        <v>761</v>
+        <v>771</v>
       </c>
       <c r="F95" s="10"/>
     </row>
@@ -14855,16 +14963,16 @@
         <v>94</v>
       </c>
       <c r="B96" s="10" t="s">
-        <v>762</v>
+        <v>772</v>
       </c>
       <c r="C96" s="23" t="s">
-        <v>763</v>
+        <v>773</v>
       </c>
       <c r="D96" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E96" s="10" t="s">
-        <v>764</v>
+        <v>774</v>
       </c>
       <c r="F96" s="10"/>
     </row>
@@ -14873,16 +14981,16 @@
         <v>95</v>
       </c>
       <c r="B97" s="10" t="s">
-        <v>765</v>
+        <v>775</v>
       </c>
       <c r="C97" s="23" t="s">
-        <v>766</v>
+        <v>776</v>
       </c>
       <c r="D97" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E97" s="10" t="s">
-        <v>767</v>
+        <v>777</v>
       </c>
       <c r="F97" s="10"/>
     </row>
@@ -14891,16 +14999,16 @@
         <v>96</v>
       </c>
       <c r="B98" s="10" t="s">
-        <v>768</v>
+        <v>778</v>
       </c>
       <c r="C98" s="23" t="s">
-        <v>769</v>
+        <v>779</v>
       </c>
       <c r="D98" s="10" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E98" s="10" t="s">
-        <v>770</v>
+        <v>780</v>
       </c>
       <c r="F98" s="10"/>
     </row>
@@ -14912,13 +15020,13 @@
         <v>73</v>
       </c>
       <c r="C99" s="25" t="s">
-        <v>771</v>
+        <v>781</v>
       </c>
       <c r="D99" s="24" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E99" s="24" t="s">
-        <v>772</v>
+        <v>782</v>
       </c>
       <c r="F99" s="24"/>
     </row>
@@ -14930,13 +15038,13 @@
         <v>362</v>
       </c>
       <c r="C100" s="25" t="s">
-        <v>773</v>
+        <v>783</v>
       </c>
       <c r="D100" s="24" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E100" s="24" t="s">
-        <v>774</v>
+        <v>784</v>
       </c>
       <c r="F100" s="24"/>
     </row>
@@ -14948,13 +15056,13 @@
         <v>355</v>
       </c>
       <c r="C101" s="25" t="s">
-        <v>773</v>
+        <v>783</v>
       </c>
       <c r="D101" s="24" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E101" s="24" t="s">
-        <v>775</v>
+        <v>785</v>
       </c>
       <c r="F101" s="24"/>
     </row>
@@ -14966,13 +15074,13 @@
         <v>373</v>
       </c>
       <c r="C102" s="25" t="s">
-        <v>776</v>
+        <v>786</v>
       </c>
       <c r="D102" s="24" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E102" s="24" t="s">
-        <v>777</v>
+        <v>787</v>
       </c>
       <c r="F102" s="24"/>
     </row>
@@ -14984,13 +15092,13 @@
         <v>381</v>
       </c>
       <c r="C103" s="25" t="s">
-        <v>778</v>
+        <v>788</v>
       </c>
       <c r="D103" s="24" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E103" s="24" t="s">
-        <v>779</v>
+        <v>789</v>
       </c>
       <c r="F103" s="24"/>
     </row>
@@ -15002,13 +15110,13 @@
         <v>80</v>
       </c>
       <c r="C104" s="25" t="s">
-        <v>780</v>
+        <v>790</v>
       </c>
       <c r="D104" s="24" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E104" s="24" t="s">
-        <v>781</v>
+        <v>791</v>
       </c>
       <c r="F104" s="24"/>
     </row>
@@ -15020,13 +15128,13 @@
         <v>366</v>
       </c>
       <c r="C105" s="25" t="s">
-        <v>782</v>
+        <v>792</v>
       </c>
       <c r="D105" s="24" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="E105" s="24" t="s">
-        <v>783</v>
+        <v>793</v>
       </c>
       <c r="F105" s="24"/>
     </row>
@@ -15159,7 +15267,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>784</v>
+        <v>794</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -15169,10 +15277,10 @@
         <v>44</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>785</v>
+        <v>795</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>786</v>
+        <v>796</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -15180,10 +15288,10 @@
         <v>47</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>787</v>
+        <v>797</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>788</v>
+        <v>798</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -15191,10 +15299,10 @@
         <v>49</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>789</v>
+        <v>799</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>790</v>
+        <v>800</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -15202,10 +15310,10 @@
         <v>51</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>791</v>
+        <v>801</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>792</v>
+        <v>802</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -15213,10 +15321,10 @@
         <v>53</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>793</v>
+        <v>803</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>794</v>
+        <v>804</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -15224,10 +15332,10 @@
         <v>55</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>795</v>
+        <v>805</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>796</v>
+        <v>806</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -15235,10 +15343,10 @@
         <v>56</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>797</v>
+        <v>807</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>798</v>
+        <v>808</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -15246,10 +15354,10 @@
         <v>57</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>799</v>
+        <v>809</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>800</v>
+        <v>810</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -15257,10 +15365,10 @@
         <v>58</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>801</v>
+        <v>811</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>802</v>
+        <v>812</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -15268,10 +15376,10 @@
         <v>59</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>803</v>
+        <v>813</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>804</v>
+        <v>814</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
prep: Hercules support role via careers page only (drop Upwork)
Upwork is out of scope for this repo. Repoint Jobs/Preparations rows and
prep doc to the careers URL, keep the honest region flag (NA/WEU/E-Australia),
apply anyway with overlap-hours framing.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1770" uniqueCount="815">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1770" uniqueCount="814">
   <si>
     <t>Hana Aliyah Mufidah</t>
   </si>
@@ -1249,13 +1249,10 @@
     <t>Technical Customer Support Engineer</t>
   </si>
   <si>
-    <t>https://www.upwork.com/jobs/Technical-Customer-Success-Specialist_~022074252517164606512/</t>
-  </si>
-  <si>
-    <t>User pick (Upwork + hercules.app/careers)</t>
-  </si>
-  <si>
-    <t>✅ Upwork listing = Worldwide (no visa gate). NOTE: careers page is region-locked NA/WEU/E-Australia, Indonesia excluded — apply via Upwork</t>
+    <t>https://hercules.app/careers/technical-customer-support-engineer</t>
+  </si>
+  <si>
+    <t>⚠️ Careers page scoped NA/WEU/E-Australia; Indonesia not listed (region flag) — applying anyway, offer overlap hours</t>
   </si>
   <si>
     <t>AI-native support; automation to auto-resolve tickets = her AI-pipeline edge; TS/web/auth/payments core match; URGENT, hourly expert pay</t>
@@ -1264,7 +1261,7 @@
     <t>Prep (urgent)</t>
   </si>
   <si>
-    <t>CS pivot off her SWE archetype but worldwide-remote + urgent + well-paid. Client rated a past hire down for not being AI-forward = her differentiator. Gaps: no formal customer-facing title, DNS depth. Prep: prep/hercules-technical-customer-support-engineer-2026-07-13.md</t>
+    <t>CS pivot off her SWE archetype; region flag. Edge is AI-forward automation (her own AI pipeline). Gaps: no formal customer-facing title, DNS depth. Prep: prep/hercules-technical-customer-support-engineer-2026-07-13.md</t>
   </si>
   <si>
     <t>Date</t>
@@ -1411,7 +1408,7 @@
     <t>No</t>
   </si>
   <si>
-    <t>URGENT — apply via Upwork (Worldwide). 3 screening-question answers drafted. Lead with AI-forward automation.</t>
+    <t>Apply via Hercules careers page. Region flag (NA/WEU/E-Australia) — offer overlap hours. Screening answers drafted; lead with AI-forward automation.</t>
   </si>
   <si>
     <t>Date Applied</t>
@@ -8139,24 +8136,24 @@
         <v>410</v>
       </c>
       <c r="F129" s="20" t="s">
+        <v>400</v>
+      </c>
+      <c r="G129" s="20" t="s">
         <v>411</v>
       </c>
-      <c r="G129" s="20" t="s">
+      <c r="H129" s="20" t="s">
         <v>412</v>
       </c>
-      <c r="H129" s="20" t="s">
-        <v>413</v>
-      </c>
       <c r="I129" s="20">
-        <v>4</v>
+        <v>3.8</v>
       </c>
       <c r="J129" s="20"/>
       <c r="K129" s="20" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="L129" s="20"/>
       <c r="M129" s="20" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
   </sheetData>
@@ -8307,7 +8304,7 @@
         <v>61</v>
       </c>
       <c r="B1" s="21" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C1" s="21" t="s">
         <v>14</v>
@@ -8319,28 +8316,28 @@
         <v>63</v>
       </c>
       <c r="F1" s="21" t="s">
+        <v>416</v>
+      </c>
+      <c r="G1" s="21" t="s">
         <v>417</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="H1" s="21" t="s">
         <v>418</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="I1" s="21" t="s">
         <v>419</v>
       </c>
-      <c r="I1" s="21" t="s">
+      <c r="J1" s="21" t="s">
         <v>420</v>
       </c>
-      <c r="J1" s="21" t="s">
+      <c r="K1" s="21" t="s">
         <v>421</v>
       </c>
-      <c r="K1" s="21" t="s">
+      <c r="L1" s="21" t="s">
         <v>422</v>
       </c>
-      <c r="L1" s="21" t="s">
+      <c r="M1" s="21" t="s">
         <v>423</v>
-      </c>
-      <c r="M1" s="21" t="s">
-        <v>424</v>
       </c>
       <c r="N1" s="21" t="s">
         <v>71</v>
@@ -8360,37 +8357,37 @@
         <v>80</v>
       </c>
       <c r="D2" s="22" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E2" s="22" t="s">
         <v>82</v>
       </c>
       <c r="F2" s="22" t="s">
+        <v>425</v>
+      </c>
+      <c r="G2" s="22" t="s">
         <v>426</v>
       </c>
-      <c r="G2" s="22" t="s">
+      <c r="H2" s="20" t="s">
         <v>427</v>
       </c>
-      <c r="H2" s="20" t="s">
+      <c r="I2" s="22" t="s">
         <v>428</v>
       </c>
-      <c r="I2" s="22" t="s">
+      <c r="J2" s="22" t="s">
         <v>429</v>
       </c>
-      <c r="J2" s="22" t="s">
+      <c r="K2" s="22" t="s">
         <v>430</v>
       </c>
-      <c r="K2" s="22" t="s">
+      <c r="L2" s="22" t="s">
         <v>431</v>
       </c>
-      <c r="L2" s="22" t="s">
+      <c r="M2" s="22" t="s">
         <v>432</v>
       </c>
-      <c r="M2" s="22" t="s">
+      <c r="N2" s="22" t="s">
         <v>433</v>
-      </c>
-      <c r="N2" s="22" t="s">
-        <v>434</v>
       </c>
       <c r="O2" s="1"/>
     </row>
@@ -8405,37 +8402,37 @@
         <v>80</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="E3" s="22" t="s">
         <v>88</v>
       </c>
       <c r="F3" s="22" t="s">
+        <v>435</v>
+      </c>
+      <c r="G3" s="22" t="s">
         <v>436</v>
       </c>
-      <c r="G3" s="22" t="s">
+      <c r="H3" s="20" t="s">
         <v>437</v>
       </c>
-      <c r="H3" s="20" t="s">
+      <c r="I3" s="22" t="s">
+        <v>428</v>
+      </c>
+      <c r="J3" s="22" t="s">
         <v>438</v>
       </c>
-      <c r="I3" s="22" t="s">
-        <v>429</v>
-      </c>
-      <c r="J3" s="22" t="s">
+      <c r="K3" s="22" t="s">
+        <v>430</v>
+      </c>
+      <c r="L3" s="22" t="s">
+        <v>431</v>
+      </c>
+      <c r="M3" s="22" t="s">
+        <v>432</v>
+      </c>
+      <c r="N3" s="22" t="s">
         <v>439</v>
-      </c>
-      <c r="K3" s="22" t="s">
-        <v>431</v>
-      </c>
-      <c r="L3" s="22" t="s">
-        <v>432</v>
-      </c>
-      <c r="M3" s="22" t="s">
-        <v>433</v>
-      </c>
-      <c r="N3" s="22" t="s">
-        <v>440</v>
       </c>
       <c r="O3" s="1"/>
     </row>
@@ -8450,37 +8447,37 @@
         <v>80</v>
       </c>
       <c r="D4" s="22" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="E4" s="22" t="s">
         <v>91</v>
       </c>
       <c r="F4" s="22" t="s">
+        <v>441</v>
+      </c>
+      <c r="G4" s="22" t="s">
         <v>442</v>
       </c>
-      <c r="G4" s="22" t="s">
+      <c r="H4" s="20" t="s">
         <v>443</v>
       </c>
-      <c r="H4" s="20" t="s">
+      <c r="I4" s="22" t="s">
         <v>444</v>
       </c>
-      <c r="I4" s="22" t="s">
+      <c r="J4" s="22" t="s">
         <v>445</v>
       </c>
-      <c r="J4" s="22" t="s">
+      <c r="K4" s="22" t="s">
         <v>446</v>
       </c>
-      <c r="K4" s="22" t="s">
+      <c r="L4" s="22" t="s">
+        <v>431</v>
+      </c>
+      <c r="M4" s="22" t="s">
         <v>447</v>
       </c>
-      <c r="L4" s="22" t="s">
-        <v>432</v>
-      </c>
-      <c r="M4" s="22" t="s">
+      <c r="N4" s="22" t="s">
         <v>448</v>
-      </c>
-      <c r="N4" s="22" t="s">
-        <v>449</v>
       </c>
       <c r="O4" s="1"/>
     </row>
@@ -8501,22 +8498,22 @@
         <v>346</v>
       </c>
       <c r="F5" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>450</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="20" t="s">
         <v>451</v>
-      </c>
-      <c r="H5" s="20" t="s">
-        <v>452</v>
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="L5" s="1"/>
       <c r="M5" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
@@ -8538,27 +8535,27 @@
         <v>399</v>
       </c>
       <c r="F6" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>454</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="20" t="s">
         <v>455</v>
       </c>
-      <c r="H6" s="20" t="s">
+      <c r="I6" s="1" t="s">
         <v>456</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>457</v>
       </c>
       <c r="J6" s="1"/>
       <c r="K6" s="1" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="O6" s="1"/>
     </row>
@@ -8579,27 +8576,27 @@
         <v>406</v>
       </c>
       <c r="F7" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>454</v>
       </c>
-      <c r="G7" s="1" t="s">
-        <v>455</v>
-      </c>
       <c r="H7" s="20" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="J7" s="1"/>
       <c r="K7" s="1" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="L7" s="1"/>
       <c r="M7" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="O7" s="1"/>
     </row>
@@ -8620,27 +8617,27 @@
         <v>410</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="G8" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="H8" s="20" t="s">
         <v>461</v>
       </c>
-      <c r="H8" s="20" t="s">
+      <c r="I8" s="1" t="s">
         <v>462</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>463</v>
       </c>
       <c r="J8" s="1"/>
       <c r="K8" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="L8" s="1"/>
       <c r="M8" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="O8" s="1"/>
     </row>
@@ -8735,7 +8732,7 @@
         <v>61</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>14</v>
@@ -8744,10 +8741,10 @@
         <v>13</v>
       </c>
       <c r="E1" s="7" t="s">
+        <v>465</v>
+      </c>
+      <c r="F1" s="7" t="s">
         <v>466</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>467</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>63</v>
@@ -8756,28 +8753,28 @@
         <v>44</v>
       </c>
       <c r="I1" s="7" t="s">
+        <v>467</v>
+      </c>
+      <c r="J1" s="7" t="s">
         <v>468</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="K1" s="7" t="s">
         <v>469</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="L1" s="7" t="s">
         <v>470</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="M1" s="7" t="s">
         <v>471</v>
       </c>
-      <c r="M1" s="7" t="s">
+      <c r="N1" s="7" t="s">
         <v>472</v>
       </c>
-      <c r="N1" s="7" t="s">
+      <c r="O1" s="7" t="s">
         <v>473</v>
       </c>
-      <c r="O1" s="7" t="s">
+      <c r="P1" s="7" t="s">
         <v>474</v>
-      </c>
-      <c r="P1" s="7" t="s">
-        <v>475</v>
       </c>
       <c r="Q1" s="7" t="s">
         <v>71</v>
@@ -8800,10 +8797,10 @@
         <v>367</v>
       </c>
       <c r="E2" s="22" t="s">
+        <v>475</v>
+      </c>
+      <c r="F2" s="22" t="s">
         <v>476</v>
-      </c>
-      <c r="F2" s="22" t="s">
-        <v>477</v>
       </c>
       <c r="G2" s="22" t="s">
         <v>368</v>
@@ -8815,24 +8812,24 @@
         <v>347</v>
       </c>
       <c r="J2" s="22" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="K2" s="22" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L2" s="1"/>
       <c r="M2" s="22" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="N2" s="1"/>
       <c r="O2" s="22" t="s">
+        <v>479</v>
+      </c>
+      <c r="P2" s="22" t="s">
         <v>480</v>
       </c>
-      <c r="P2" s="22" t="s">
+      <c r="Q2" s="22" t="s">
         <v>481</v>
-      </c>
-      <c r="Q2" s="22" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
@@ -8849,10 +8846,10 @@
         <v>374</v>
       </c>
       <c r="E3" s="22" t="s">
+        <v>482</v>
+      </c>
+      <c r="F3" s="22" t="s">
         <v>483</v>
-      </c>
-      <c r="F3" s="22" t="s">
-        <v>484</v>
       </c>
       <c r="G3" s="22" t="s">
         <v>375</v>
@@ -8864,22 +8861,22 @@
         <v>347</v>
       </c>
       <c r="J3" s="22" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="K3" s="22" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
       <c r="O3" s="22" t="s">
+        <v>479</v>
+      </c>
+      <c r="P3" s="22" t="s">
         <v>480</v>
       </c>
-      <c r="P3" s="22" t="s">
-        <v>481</v>
-      </c>
       <c r="Q3" s="22" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
@@ -8893,13 +8890,13 @@
         <v>80</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E4" s="22" t="s">
+        <v>486</v>
+      </c>
+      <c r="F4" s="22" t="s">
         <v>487</v>
-      </c>
-      <c r="F4" s="22" t="s">
-        <v>488</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>82</v>
@@ -8911,28 +8908,28 @@
         <v>380</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="K4" s="22" t="s">
+        <v>488</v>
+      </c>
+      <c r="L4" s="22" t="s">
         <v>489</v>
       </c>
-      <c r="L4" s="22" t="s">
+      <c r="M4" s="22" t="s">
         <v>490</v>
       </c>
-      <c r="M4" s="22" t="s">
+      <c r="N4" s="1" t="s">
         <v>491</v>
       </c>
-      <c r="N4" s="1" t="s">
+      <c r="O4" s="22" t="s">
+        <v>479</v>
+      </c>
+      <c r="P4" s="22" t="s">
         <v>492</v>
       </c>
-      <c r="O4" s="22" t="s">
-        <v>480</v>
-      </c>
-      <c r="P4" s="22" t="s">
+      <c r="Q4" s="1" t="s">
         <v>493</v>
-      </c>
-      <c r="Q4" s="1" t="s">
-        <v>494</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
@@ -8946,13 +8943,13 @@
         <v>80</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>487</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>488</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>88</v>
@@ -8964,24 +8961,24 @@
         <v>380</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
       <c r="O5" s="1" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="P5" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="Q5" s="1" t="s">
         <v>493</v>
-      </c>
-      <c r="Q5" s="1" t="s">
-        <v>494</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
@@ -8998,7 +8995,7 @@
         <v>382</v>
       </c>
       <c r="E6" s="22" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="F6" s="22" t="s">
         <v>384</v>
@@ -9013,26 +9010,26 @@
         <v>380</v>
       </c>
       <c r="J6" s="22" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="K6" s="22" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="L6" s="22"/>
       <c r="M6" s="22" t="s">
+        <v>497</v>
+      </c>
+      <c r="N6" s="22" t="s">
         <v>498</v>
       </c>
-      <c r="N6" s="22" t="s">
+      <c r="O6" s="22" t="s">
+        <v>479</v>
+      </c>
+      <c r="P6" s="22" t="s">
+        <v>492</v>
+      </c>
+      <c r="Q6" s="22" t="s">
         <v>499</v>
-      </c>
-      <c r="O6" s="22" t="s">
-        <v>480</v>
-      </c>
-      <c r="P6" s="22" t="s">
-        <v>493</v>
-      </c>
-      <c r="Q6" s="22" t="s">
-        <v>500</v>
       </c>
       <c r="R6" s="20"/>
     </row>
@@ -9047,16 +9044,16 @@
         <v>373</v>
       </c>
       <c r="D7" s="22" t="s">
+        <v>500</v>
+      </c>
+      <c r="E7" s="22" t="s">
         <v>501</v>
       </c>
-      <c r="E7" s="22" t="s">
+      <c r="F7" s="22" t="s">
         <v>502</v>
       </c>
-      <c r="F7" s="22" t="s">
+      <c r="G7" s="22" t="s">
         <v>503</v>
-      </c>
-      <c r="G7" s="22" t="s">
-        <v>504</v>
       </c>
       <c r="H7" s="22" t="s">
         <v>51</v>
@@ -9067,18 +9064,18 @@
       <c r="J7" s="22"/>
       <c r="K7" s="22"/>
       <c r="L7" s="22" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="M7" s="22"/>
       <c r="N7" s="22"/>
       <c r="O7" s="22" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="P7" s="22" t="s">
+        <v>505</v>
+      </c>
+      <c r="Q7" s="22" t="s">
         <v>506</v>
-      </c>
-      <c r="Q7" s="22" t="s">
-        <v>507</v>
       </c>
       <c r="R7" s="20"/>
     </row>
@@ -13170,7 +13167,7 @@
         <v>356</v>
       </c>
       <c r="E202" s="20" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="F202" s="20" t="s">
         <v>358</v>
@@ -13179,13 +13176,13 @@
         <v>357</v>
       </c>
       <c r="H202" s="20" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="I202" s="20" t="s">
         <v>388</v>
       </c>
       <c r="J202" s="20" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="K202" s="20"/>
       <c r="L202" s="20"/>
@@ -13256,7 +13253,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -13272,16 +13269,16 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
+        <v>510</v>
+      </c>
+      <c r="D2" s="7" t="s">
         <v>511</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>512</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>71</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -13289,13 +13286,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="10" t="s">
+        <v>513</v>
+      </c>
+      <c r="C3" s="23" t="s">
         <v>514</v>
       </c>
-      <c r="C3" s="23" t="s">
+      <c r="D3" s="10" t="s">
         <v>515</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>516</v>
       </c>
       <c r="E3" s="10"/>
       <c r="F3" s="10"/>
@@ -13305,13 +13302,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="10" t="s">
+        <v>516</v>
+      </c>
+      <c r="C4" s="23" t="s">
         <v>517</v>
       </c>
-      <c r="C4" s="23" t="s">
-        <v>518</v>
-      </c>
       <c r="D4" s="10" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="E4" s="10"/>
       <c r="F4" s="10"/>
@@ -13321,16 +13318,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="10" t="s">
+        <v>518</v>
+      </c>
+      <c r="C5" s="23" t="s">
         <v>519</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="D5" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E5" s="10" t="s">
         <v>520</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>521</v>
       </c>
       <c r="F5" s="10"/>
     </row>
@@ -13339,16 +13336,16 @@
         <v>4</v>
       </c>
       <c r="B6" s="10" t="s">
+        <v>521</v>
+      </c>
+      <c r="C6" s="23" t="s">
         <v>522</v>
       </c>
-      <c r="C6" s="23" t="s">
+      <c r="D6" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E6" s="10" t="s">
         <v>523</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>524</v>
       </c>
       <c r="F6" s="10"/>
     </row>
@@ -13360,13 +13357,13 @@
         <v>240</v>
       </c>
       <c r="C7" s="23" t="s">
+        <v>524</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E7" s="10" t="s">
         <v>525</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>526</v>
       </c>
       <c r="F7" s="10"/>
     </row>
@@ -13375,16 +13372,16 @@
         <v>6</v>
       </c>
       <c r="B8" s="10" t="s">
+        <v>526</v>
+      </c>
+      <c r="C8" s="23" t="s">
         <v>527</v>
       </c>
-      <c r="C8" s="23" t="s">
+      <c r="D8" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E8" s="10" t="s">
         <v>528</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>529</v>
       </c>
       <c r="F8" s="10"/>
     </row>
@@ -13393,16 +13390,16 @@
         <v>7</v>
       </c>
       <c r="B9" s="10" t="s">
+        <v>529</v>
+      </c>
+      <c r="C9" s="23" t="s">
         <v>530</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="D9" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E9" s="10" t="s">
         <v>531</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>532</v>
       </c>
       <c r="F9" s="10"/>
     </row>
@@ -13414,13 +13411,13 @@
         <v>141</v>
       </c>
       <c r="C10" s="23" t="s">
+        <v>532</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E10" s="10" t="s">
         <v>533</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>534</v>
       </c>
       <c r="F10" s="10"/>
     </row>
@@ -13429,16 +13426,16 @@
         <v>9</v>
       </c>
       <c r="B11" s="10" t="s">
+        <v>534</v>
+      </c>
+      <c r="C11" s="23" t="s">
         <v>535</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="D11" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E11" s="10" t="s">
         <v>536</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>537</v>
       </c>
       <c r="F11" s="10"/>
     </row>
@@ -13447,16 +13444,16 @@
         <v>10</v>
       </c>
       <c r="B12" s="10" t="s">
+        <v>537</v>
+      </c>
+      <c r="C12" s="23" t="s">
         <v>538</v>
       </c>
-      <c r="C12" s="23" t="s">
+      <c r="D12" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E12" s="10" t="s">
         <v>539</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>540</v>
       </c>
       <c r="F12" s="10"/>
     </row>
@@ -13465,16 +13462,16 @@
         <v>11</v>
       </c>
       <c r="B13" s="10" t="s">
+        <v>540</v>
+      </c>
+      <c r="C13" s="23" t="s">
         <v>541</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="D13" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E13" s="10" t="s">
         <v>542</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>543</v>
       </c>
       <c r="F13" s="10"/>
     </row>
@@ -13483,16 +13480,16 @@
         <v>12</v>
       </c>
       <c r="B14" s="10" t="s">
+        <v>543</v>
+      </c>
+      <c r="C14" s="23" t="s">
         <v>544</v>
       </c>
-      <c r="C14" s="23" t="s">
+      <c r="D14" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E14" s="10" t="s">
         <v>545</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>546</v>
       </c>
       <c r="F14" s="10"/>
     </row>
@@ -13501,16 +13498,16 @@
         <v>13</v>
       </c>
       <c r="B15" s="10" t="s">
+        <v>546</v>
+      </c>
+      <c r="C15" s="23" t="s">
         <v>547</v>
       </c>
-      <c r="C15" s="23" t="s">
+      <c r="D15" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E15" s="10" t="s">
         <v>548</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>549</v>
       </c>
       <c r="F15" s="10"/>
     </row>
@@ -13519,16 +13516,16 @@
         <v>14</v>
       </c>
       <c r="B16" s="10" t="s">
+        <v>549</v>
+      </c>
+      <c r="C16" s="23" t="s">
         <v>550</v>
       </c>
-      <c r="C16" s="23" t="s">
+      <c r="D16" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E16" s="10" t="s">
         <v>551</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>552</v>
       </c>
       <c r="F16" s="10"/>
     </row>
@@ -13537,16 +13534,16 @@
         <v>15</v>
       </c>
       <c r="B17" s="10" t="s">
+        <v>552</v>
+      </c>
+      <c r="C17" s="23" t="s">
         <v>553</v>
       </c>
-      <c r="C17" s="23" t="s">
+      <c r="D17" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E17" s="10" t="s">
         <v>554</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>555</v>
       </c>
       <c r="F17" s="10"/>
     </row>
@@ -13555,16 +13552,16 @@
         <v>16</v>
       </c>
       <c r="B18" s="10" t="s">
+        <v>555</v>
+      </c>
+      <c r="C18" s="23" t="s">
         <v>556</v>
       </c>
-      <c r="C18" s="23" t="s">
+      <c r="D18" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E18" s="10" t="s">
         <v>557</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E18" s="10" t="s">
-        <v>558</v>
       </c>
       <c r="F18" s="10"/>
     </row>
@@ -13576,13 +13573,13 @@
         <v>179</v>
       </c>
       <c r="C19" s="23" t="s">
+        <v>558</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E19" s="10" t="s">
         <v>559</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E19" s="10" t="s">
-        <v>560</v>
       </c>
       <c r="F19" s="10"/>
     </row>
@@ -13591,16 +13588,16 @@
         <v>18</v>
       </c>
       <c r="B20" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="C20" s="23" t="s">
         <v>561</v>
       </c>
-      <c r="C20" s="23" t="s">
+      <c r="D20" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E20" s="10" t="s">
         <v>562</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E20" s="10" t="s">
-        <v>563</v>
       </c>
       <c r="F20" s="10"/>
     </row>
@@ -13609,16 +13606,16 @@
         <v>19</v>
       </c>
       <c r="B21" s="10" t="s">
+        <v>563</v>
+      </c>
+      <c r="C21" s="23" t="s">
         <v>564</v>
       </c>
-      <c r="C21" s="23" t="s">
+      <c r="D21" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E21" s="10" t="s">
         <v>565</v>
-      </c>
-      <c r="D21" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E21" s="10" t="s">
-        <v>566</v>
       </c>
       <c r="F21" s="10"/>
     </row>
@@ -13627,16 +13624,16 @@
         <v>20</v>
       </c>
       <c r="B22" s="10" t="s">
+        <v>566</v>
+      </c>
+      <c r="C22" s="23" t="s">
         <v>567</v>
       </c>
-      <c r="C22" s="23" t="s">
+      <c r="D22" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E22" s="10" t="s">
         <v>568</v>
-      </c>
-      <c r="D22" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>569</v>
       </c>
       <c r="F22" s="10"/>
     </row>
@@ -13645,16 +13642,16 @@
         <v>21</v>
       </c>
       <c r="B23" s="10" t="s">
+        <v>569</v>
+      </c>
+      <c r="C23" s="23" t="s">
         <v>570</v>
       </c>
-      <c r="C23" s="23" t="s">
+      <c r="D23" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E23" s="10" t="s">
         <v>571</v>
-      </c>
-      <c r="D23" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E23" s="10" t="s">
-        <v>572</v>
       </c>
       <c r="F23" s="10"/>
     </row>
@@ -13663,16 +13660,16 @@
         <v>22</v>
       </c>
       <c r="B24" s="10" t="s">
+        <v>572</v>
+      </c>
+      <c r="C24" s="23" t="s">
         <v>573</v>
       </c>
-      <c r="C24" s="23" t="s">
+      <c r="D24" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E24" s="10" t="s">
         <v>574</v>
-      </c>
-      <c r="D24" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E24" s="10" t="s">
-        <v>575</v>
       </c>
       <c r="F24" s="10"/>
     </row>
@@ -13681,16 +13678,16 @@
         <v>23</v>
       </c>
       <c r="B25" s="10" t="s">
+        <v>575</v>
+      </c>
+      <c r="C25" s="23" t="s">
         <v>576</v>
       </c>
-      <c r="C25" s="23" t="s">
+      <c r="D25" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E25" s="10" t="s">
         <v>577</v>
-      </c>
-      <c r="D25" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E25" s="10" t="s">
-        <v>578</v>
       </c>
       <c r="F25" s="10"/>
     </row>
@@ -13699,16 +13696,16 @@
         <v>24</v>
       </c>
       <c r="B26" s="10" t="s">
+        <v>578</v>
+      </c>
+      <c r="C26" s="23" t="s">
         <v>579</v>
       </c>
-      <c r="C26" s="23" t="s">
+      <c r="D26" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E26" s="10" t="s">
         <v>580</v>
-      </c>
-      <c r="D26" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E26" s="10" t="s">
-        <v>581</v>
       </c>
       <c r="F26" s="10"/>
     </row>
@@ -13717,16 +13714,16 @@
         <v>25</v>
       </c>
       <c r="B27" s="10" t="s">
+        <v>581</v>
+      </c>
+      <c r="C27" s="23" t="s">
         <v>582</v>
       </c>
-      <c r="C27" s="23" t="s">
+      <c r="D27" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E27" s="10" t="s">
         <v>583</v>
-      </c>
-      <c r="D27" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E27" s="10" t="s">
-        <v>584</v>
       </c>
       <c r="F27" s="10"/>
     </row>
@@ -13735,16 +13732,16 @@
         <v>26</v>
       </c>
       <c r="B28" s="10" t="s">
+        <v>584</v>
+      </c>
+      <c r="C28" s="23" t="s">
         <v>585</v>
       </c>
-      <c r="C28" s="23" t="s">
+      <c r="D28" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E28" s="10" t="s">
         <v>586</v>
-      </c>
-      <c r="D28" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E28" s="10" t="s">
-        <v>587</v>
       </c>
       <c r="F28" s="10"/>
     </row>
@@ -13753,16 +13750,16 @@
         <v>27</v>
       </c>
       <c r="B29" s="10" t="s">
+        <v>587</v>
+      </c>
+      <c r="C29" s="23" t="s">
         <v>588</v>
       </c>
-      <c r="C29" s="23" t="s">
+      <c r="D29" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E29" s="10" t="s">
         <v>589</v>
-      </c>
-      <c r="D29" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E29" s="10" t="s">
-        <v>590</v>
       </c>
       <c r="F29" s="10"/>
     </row>
@@ -13771,16 +13768,16 @@
         <v>28</v>
       </c>
       <c r="B30" s="10" t="s">
+        <v>590</v>
+      </c>
+      <c r="C30" s="23" t="s">
         <v>591</v>
       </c>
-      <c r="C30" s="23" t="s">
+      <c r="D30" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E30" s="10" t="s">
         <v>592</v>
-      </c>
-      <c r="D30" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E30" s="10" t="s">
-        <v>593</v>
       </c>
       <c r="F30" s="10"/>
     </row>
@@ -13789,16 +13786,16 @@
         <v>29</v>
       </c>
       <c r="B31" s="10" t="s">
+        <v>593</v>
+      </c>
+      <c r="C31" s="23" t="s">
         <v>594</v>
       </c>
-      <c r="C31" s="23" t="s">
+      <c r="D31" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E31" s="10" t="s">
         <v>595</v>
-      </c>
-      <c r="D31" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E31" s="10" t="s">
-        <v>596</v>
       </c>
       <c r="F31" s="10"/>
     </row>
@@ -13807,16 +13804,16 @@
         <v>30</v>
       </c>
       <c r="B32" s="10" t="s">
+        <v>596</v>
+      </c>
+      <c r="C32" s="23" t="s">
         <v>597</v>
       </c>
-      <c r="C32" s="23" t="s">
+      <c r="D32" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E32" s="10" t="s">
         <v>598</v>
-      </c>
-      <c r="D32" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E32" s="10" t="s">
-        <v>599</v>
       </c>
       <c r="F32" s="10"/>
     </row>
@@ -13825,16 +13822,16 @@
         <v>31</v>
       </c>
       <c r="B33" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="C33" s="23" t="s">
         <v>600</v>
       </c>
-      <c r="C33" s="23" t="s">
+      <c r="D33" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E33" s="10" t="s">
         <v>601</v>
-      </c>
-      <c r="D33" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E33" s="10" t="s">
-        <v>602</v>
       </c>
       <c r="F33" s="10"/>
     </row>
@@ -13846,13 +13843,13 @@
         <v>108</v>
       </c>
       <c r="C34" s="23" t="s">
+        <v>602</v>
+      </c>
+      <c r="D34" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E34" s="10" t="s">
         <v>603</v>
-      </c>
-      <c r="D34" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E34" s="10" t="s">
-        <v>604</v>
       </c>
       <c r="F34" s="10"/>
     </row>
@@ -13864,13 +13861,13 @@
         <v>344</v>
       </c>
       <c r="C35" s="23" t="s">
+        <v>604</v>
+      </c>
+      <c r="D35" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E35" s="10" t="s">
         <v>605</v>
-      </c>
-      <c r="D35" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E35" s="10" t="s">
-        <v>606</v>
       </c>
       <c r="F35" s="10"/>
     </row>
@@ -13879,16 +13876,16 @@
         <v>34</v>
       </c>
       <c r="B36" s="10" t="s">
+        <v>606</v>
+      </c>
+      <c r="C36" s="23" t="s">
         <v>607</v>
       </c>
-      <c r="C36" s="23" t="s">
+      <c r="D36" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E36" s="10" t="s">
         <v>608</v>
-      </c>
-      <c r="D36" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E36" s="10" t="s">
-        <v>609</v>
       </c>
       <c r="F36" s="10"/>
     </row>
@@ -13900,13 +13897,13 @@
         <v>113</v>
       </c>
       <c r="C37" s="23" t="s">
+        <v>609</v>
+      </c>
+      <c r="D37" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E37" s="10" t="s">
         <v>610</v>
-      </c>
-      <c r="D37" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E37" s="10" t="s">
-        <v>611</v>
       </c>
       <c r="F37" s="10"/>
     </row>
@@ -13915,16 +13912,16 @@
         <v>36</v>
       </c>
       <c r="B38" s="10" t="s">
+        <v>611</v>
+      </c>
+      <c r="C38" s="23" t="s">
         <v>612</v>
       </c>
-      <c r="C38" s="23" t="s">
+      <c r="D38" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E38" s="10" t="s">
         <v>613</v>
-      </c>
-      <c r="D38" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E38" s="10" t="s">
-        <v>614</v>
       </c>
       <c r="F38" s="10"/>
     </row>
@@ -13933,16 +13930,16 @@
         <v>37</v>
       </c>
       <c r="B39" s="10" t="s">
+        <v>614</v>
+      </c>
+      <c r="C39" s="23" t="s">
         <v>615</v>
       </c>
-      <c r="C39" s="23" t="s">
+      <c r="D39" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E39" s="10" t="s">
         <v>616</v>
-      </c>
-      <c r="D39" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E39" s="10" t="s">
-        <v>617</v>
       </c>
       <c r="F39" s="10"/>
     </row>
@@ -13951,16 +13948,16 @@
         <v>38</v>
       </c>
       <c r="B40" s="10" t="s">
+        <v>617</v>
+      </c>
+      <c r="C40" s="23" t="s">
         <v>618</v>
       </c>
-      <c r="C40" s="23" t="s">
+      <c r="D40" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E40" s="10" t="s">
         <v>619</v>
-      </c>
-      <c r="D40" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E40" s="10" t="s">
-        <v>620</v>
       </c>
       <c r="F40" s="10"/>
     </row>
@@ -13972,13 +13969,13 @@
         <v>274</v>
       </c>
       <c r="C41" s="23" t="s">
+        <v>620</v>
+      </c>
+      <c r="D41" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E41" s="10" t="s">
         <v>621</v>
-      </c>
-      <c r="D41" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E41" s="10" t="s">
-        <v>622</v>
       </c>
       <c r="F41" s="10"/>
     </row>
@@ -13987,16 +13984,16 @@
         <v>40</v>
       </c>
       <c r="B42" s="10" t="s">
+        <v>622</v>
+      </c>
+      <c r="C42" s="23" t="s">
         <v>623</v>
       </c>
-      <c r="C42" s="23" t="s">
+      <c r="D42" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E42" s="10" t="s">
         <v>624</v>
-      </c>
-      <c r="D42" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E42" s="10" t="s">
-        <v>625</v>
       </c>
       <c r="F42" s="10"/>
     </row>
@@ -14005,16 +14002,16 @@
         <v>41</v>
       </c>
       <c r="B43" s="10" t="s">
+        <v>625</v>
+      </c>
+      <c r="C43" s="23" t="s">
         <v>626</v>
       </c>
-      <c r="C43" s="23" t="s">
+      <c r="D43" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E43" s="10" t="s">
         <v>627</v>
-      </c>
-      <c r="D43" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E43" s="10" t="s">
-        <v>628</v>
       </c>
       <c r="F43" s="10"/>
     </row>
@@ -14023,16 +14020,16 @@
         <v>42</v>
       </c>
       <c r="B44" s="10" t="s">
+        <v>628</v>
+      </c>
+      <c r="C44" s="23" t="s">
         <v>629</v>
       </c>
-      <c r="C44" s="23" t="s">
+      <c r="D44" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E44" s="10" t="s">
         <v>630</v>
-      </c>
-      <c r="D44" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E44" s="10" t="s">
-        <v>631</v>
       </c>
       <c r="F44" s="10"/>
     </row>
@@ -14041,16 +14038,16 @@
         <v>43</v>
       </c>
       <c r="B45" s="10" t="s">
+        <v>631</v>
+      </c>
+      <c r="C45" s="23" t="s">
         <v>632</v>
       </c>
-      <c r="C45" s="23" t="s">
+      <c r="D45" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E45" s="10" t="s">
         <v>633</v>
-      </c>
-      <c r="D45" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E45" s="10" t="s">
-        <v>634</v>
       </c>
       <c r="F45" s="10"/>
     </row>
@@ -14062,13 +14059,13 @@
         <v>231</v>
       </c>
       <c r="C46" s="23" t="s">
+        <v>634</v>
+      </c>
+      <c r="D46" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E46" s="10" t="s">
         <v>635</v>
-      </c>
-      <c r="D46" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E46" s="10" t="s">
-        <v>636</v>
       </c>
       <c r="F46" s="10"/>
     </row>
@@ -14077,16 +14074,16 @@
         <v>45</v>
       </c>
       <c r="B47" s="10" t="s">
+        <v>636</v>
+      </c>
+      <c r="C47" s="23" t="s">
         <v>637</v>
       </c>
-      <c r="C47" s="23" t="s">
+      <c r="D47" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E47" s="10" t="s">
         <v>638</v>
-      </c>
-      <c r="D47" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E47" s="10" t="s">
-        <v>639</v>
       </c>
       <c r="F47" s="10"/>
     </row>
@@ -14098,13 +14095,13 @@
         <v>174</v>
       </c>
       <c r="C48" s="23" t="s">
+        <v>639</v>
+      </c>
+      <c r="D48" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E48" s="10" t="s">
         <v>640</v>
-      </c>
-      <c r="D48" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E48" s="10" t="s">
-        <v>641</v>
       </c>
       <c r="F48" s="10"/>
     </row>
@@ -14113,16 +14110,16 @@
         <v>47</v>
       </c>
       <c r="B49" s="10" t="s">
+        <v>641</v>
+      </c>
+      <c r="C49" s="23" t="s">
         <v>642</v>
       </c>
-      <c r="C49" s="23" t="s">
+      <c r="D49" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E49" s="10" t="s">
         <v>643</v>
-      </c>
-      <c r="D49" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E49" s="10" t="s">
-        <v>644</v>
       </c>
       <c r="F49" s="10"/>
     </row>
@@ -14131,16 +14128,16 @@
         <v>48</v>
       </c>
       <c r="B50" s="10" t="s">
+        <v>644</v>
+      </c>
+      <c r="C50" s="23" t="s">
         <v>645</v>
       </c>
-      <c r="C50" s="23" t="s">
+      <c r="D50" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E50" s="10" t="s">
         <v>646</v>
-      </c>
-      <c r="D50" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E50" s="10" t="s">
-        <v>647</v>
       </c>
       <c r="F50" s="10"/>
     </row>
@@ -14149,16 +14146,16 @@
         <v>49</v>
       </c>
       <c r="B51" s="10" t="s">
+        <v>647</v>
+      </c>
+      <c r="C51" s="23" t="s">
         <v>648</v>
       </c>
-      <c r="C51" s="23" t="s">
+      <c r="D51" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E51" s="10" t="s">
         <v>649</v>
-      </c>
-      <c r="D51" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E51" s="10" t="s">
-        <v>650</v>
       </c>
       <c r="F51" s="10"/>
     </row>
@@ -14167,16 +14164,16 @@
         <v>50</v>
       </c>
       <c r="B52" s="10" t="s">
+        <v>650</v>
+      </c>
+      <c r="C52" s="23" t="s">
         <v>651</v>
       </c>
-      <c r="C52" s="23" t="s">
+      <c r="D52" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E52" s="10" t="s">
         <v>652</v>
-      </c>
-      <c r="D52" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E52" s="10" t="s">
-        <v>653</v>
       </c>
       <c r="F52" s="10"/>
     </row>
@@ -14185,16 +14182,16 @@
         <v>51</v>
       </c>
       <c r="B53" s="10" t="s">
+        <v>653</v>
+      </c>
+      <c r="C53" s="23" t="s">
         <v>654</v>
       </c>
-      <c r="C53" s="23" t="s">
+      <c r="D53" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E53" s="10" t="s">
         <v>655</v>
-      </c>
-      <c r="D53" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E53" s="10" t="s">
-        <v>656</v>
       </c>
       <c r="F53" s="10"/>
     </row>
@@ -14203,16 +14200,16 @@
         <v>52</v>
       </c>
       <c r="B54" s="10" t="s">
+        <v>656</v>
+      </c>
+      <c r="C54" s="23" t="s">
         <v>657</v>
       </c>
-      <c r="C54" s="23" t="s">
+      <c r="D54" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E54" s="10" t="s">
         <v>658</v>
-      </c>
-      <c r="D54" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E54" s="10" t="s">
-        <v>659</v>
       </c>
       <c r="F54" s="10"/>
     </row>
@@ -14221,16 +14218,16 @@
         <v>53</v>
       </c>
       <c r="B55" s="10" t="s">
+        <v>659</v>
+      </c>
+      <c r="C55" s="23" t="s">
         <v>660</v>
       </c>
-      <c r="C55" s="23" t="s">
+      <c r="D55" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E55" s="10" t="s">
         <v>661</v>
-      </c>
-      <c r="D55" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E55" s="10" t="s">
-        <v>662</v>
       </c>
       <c r="F55" s="10"/>
     </row>
@@ -14239,16 +14236,16 @@
         <v>54</v>
       </c>
       <c r="B56" s="10" t="s">
+        <v>662</v>
+      </c>
+      <c r="C56" s="23" t="s">
         <v>663</v>
       </c>
-      <c r="C56" s="23" t="s">
+      <c r="D56" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E56" s="10" t="s">
         <v>664</v>
-      </c>
-      <c r="D56" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E56" s="10" t="s">
-        <v>665</v>
       </c>
       <c r="F56" s="10"/>
     </row>
@@ -14257,16 +14254,16 @@
         <v>55</v>
       </c>
       <c r="B57" s="10" t="s">
+        <v>665</v>
+      </c>
+      <c r="C57" s="23" t="s">
         <v>666</v>
       </c>
-      <c r="C57" s="23" t="s">
+      <c r="D57" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E57" s="10" t="s">
         <v>667</v>
-      </c>
-      <c r="D57" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E57" s="10" t="s">
-        <v>668</v>
       </c>
       <c r="F57" s="10"/>
     </row>
@@ -14275,16 +14272,16 @@
         <v>56</v>
       </c>
       <c r="B58" s="10" t="s">
+        <v>668</v>
+      </c>
+      <c r="C58" s="23" t="s">
         <v>669</v>
       </c>
-      <c r="C58" s="23" t="s">
+      <c r="D58" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E58" s="10" t="s">
         <v>670</v>
-      </c>
-      <c r="D58" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E58" s="10" t="s">
-        <v>671</v>
       </c>
       <c r="F58" s="10"/>
     </row>
@@ -14296,13 +14293,13 @@
         <v>212</v>
       </c>
       <c r="C59" s="23" t="s">
+        <v>671</v>
+      </c>
+      <c r="D59" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E59" s="10" t="s">
         <v>672</v>
-      </c>
-      <c r="D59" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E59" s="10" t="s">
-        <v>673</v>
       </c>
       <c r="F59" s="10"/>
     </row>
@@ -14314,13 +14311,13 @@
         <v>120</v>
       </c>
       <c r="C60" s="23" t="s">
+        <v>673</v>
+      </c>
+      <c r="D60" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E60" s="10" t="s">
         <v>674</v>
-      </c>
-      <c r="D60" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E60" s="10" t="s">
-        <v>675</v>
       </c>
       <c r="F60" s="10"/>
     </row>
@@ -14332,13 +14329,13 @@
         <v>129</v>
       </c>
       <c r="C61" s="23" t="s">
+        <v>675</v>
+      </c>
+      <c r="D61" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E61" s="10" t="s">
         <v>676</v>
-      </c>
-      <c r="D61" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E61" s="10" t="s">
-        <v>677</v>
       </c>
       <c r="F61" s="10"/>
     </row>
@@ -14350,13 +14347,13 @@
         <v>154</v>
       </c>
       <c r="C62" s="23" t="s">
+        <v>677</v>
+      </c>
+      <c r="D62" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E62" s="10" t="s">
         <v>678</v>
-      </c>
-      <c r="D62" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E62" s="10" t="s">
-        <v>679</v>
       </c>
       <c r="F62" s="10"/>
     </row>
@@ -14365,16 +14362,16 @@
         <v>61</v>
       </c>
       <c r="B63" s="10" t="s">
+        <v>679</v>
+      </c>
+      <c r="C63" s="23" t="s">
         <v>680</v>
       </c>
-      <c r="C63" s="23" t="s">
+      <c r="D63" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E63" s="10" t="s">
         <v>681</v>
-      </c>
-      <c r="D63" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E63" s="10" t="s">
-        <v>682</v>
       </c>
       <c r="F63" s="10"/>
     </row>
@@ -14386,13 +14383,13 @@
         <v>301</v>
       </c>
       <c r="C64" s="23" t="s">
+        <v>682</v>
+      </c>
+      <c r="D64" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E64" s="10" t="s">
         <v>683</v>
-      </c>
-      <c r="D64" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E64" s="10" t="s">
-        <v>684</v>
       </c>
       <c r="F64" s="10"/>
     </row>
@@ -14401,16 +14398,16 @@
         <v>63</v>
       </c>
       <c r="B65" s="10" t="s">
+        <v>684</v>
+      </c>
+      <c r="C65" s="23" t="s">
         <v>685</v>
       </c>
-      <c r="C65" s="23" t="s">
+      <c r="D65" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E65" s="10" t="s">
         <v>686</v>
-      </c>
-      <c r="D65" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E65" s="10" t="s">
-        <v>687</v>
       </c>
       <c r="F65" s="10"/>
     </row>
@@ -14419,19 +14416,19 @@
         <v>64</v>
       </c>
       <c r="B66" s="10" t="s">
+        <v>687</v>
+      </c>
+      <c r="C66" s="23" t="s">
         <v>688</v>
       </c>
-      <c r="C66" s="23" t="s">
+      <c r="D66" s="10" t="s">
+        <v>462</v>
+      </c>
+      <c r="E66" s="24" t="s">
         <v>689</v>
       </c>
-      <c r="D66" s="10" t="s">
-        <v>463</v>
-      </c>
-      <c r="E66" s="24" t="s">
+      <c r="F66" s="10" t="s">
         <v>690</v>
-      </c>
-      <c r="F66" s="10" t="s">
-        <v>691</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
@@ -14442,13 +14439,13 @@
         <v>328</v>
       </c>
       <c r="C67" s="23" t="s">
+        <v>691</v>
+      </c>
+      <c r="D67" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E67" s="10" t="s">
         <v>692</v>
-      </c>
-      <c r="D67" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E67" s="10" t="s">
-        <v>693</v>
       </c>
       <c r="F67" s="10"/>
     </row>
@@ -14457,16 +14454,16 @@
         <v>66</v>
       </c>
       <c r="B68" s="10" t="s">
+        <v>693</v>
+      </c>
+      <c r="C68" s="23" t="s">
         <v>694</v>
       </c>
-      <c r="C68" s="23" t="s">
+      <c r="D68" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E68" s="10" t="s">
         <v>695</v>
-      </c>
-      <c r="D68" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E68" s="10" t="s">
-        <v>696</v>
       </c>
       <c r="F68" s="10"/>
     </row>
@@ -14475,16 +14472,16 @@
         <v>67</v>
       </c>
       <c r="B69" s="10" t="s">
+        <v>696</v>
+      </c>
+      <c r="C69" s="23" t="s">
         <v>697</v>
       </c>
-      <c r="C69" s="23" t="s">
+      <c r="D69" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E69" s="10" t="s">
         <v>698</v>
-      </c>
-      <c r="D69" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E69" s="10" t="s">
-        <v>699</v>
       </c>
       <c r="F69" s="10"/>
     </row>
@@ -14493,16 +14490,16 @@
         <v>68</v>
       </c>
       <c r="B70" s="10" t="s">
+        <v>699</v>
+      </c>
+      <c r="C70" s="23" t="s">
         <v>700</v>
       </c>
-      <c r="C70" s="23" t="s">
+      <c r="D70" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E70" s="10" t="s">
         <v>701</v>
-      </c>
-      <c r="D70" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E70" s="10" t="s">
-        <v>702</v>
       </c>
       <c r="F70" s="10"/>
     </row>
@@ -14514,13 +14511,13 @@
         <v>138</v>
       </c>
       <c r="C71" s="23" t="s">
+        <v>702</v>
+      </c>
+      <c r="D71" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E71" s="10" t="s">
         <v>703</v>
-      </c>
-      <c r="D71" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E71" s="10" t="s">
-        <v>704</v>
       </c>
       <c r="F71" s="10"/>
     </row>
@@ -14529,16 +14526,16 @@
         <v>70</v>
       </c>
       <c r="B72" s="10" t="s">
+        <v>704</v>
+      </c>
+      <c r="C72" s="23" t="s">
         <v>705</v>
       </c>
-      <c r="C72" s="23" t="s">
+      <c r="D72" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E72" s="10" t="s">
         <v>706</v>
-      </c>
-      <c r="D72" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E72" s="10" t="s">
-        <v>707</v>
       </c>
       <c r="F72" s="10"/>
     </row>
@@ -14547,16 +14544,16 @@
         <v>71</v>
       </c>
       <c r="B73" s="10" t="s">
+        <v>707</v>
+      </c>
+      <c r="C73" s="23" t="s">
         <v>708</v>
       </c>
-      <c r="C73" s="23" t="s">
+      <c r="D73" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E73" s="10" t="s">
         <v>709</v>
-      </c>
-      <c r="D73" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E73" s="10" t="s">
-        <v>710</v>
       </c>
       <c r="F73" s="10"/>
     </row>
@@ -14568,13 +14565,13 @@
         <v>311</v>
       </c>
       <c r="C74" s="23" t="s">
+        <v>710</v>
+      </c>
+      <c r="D74" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E74" s="10" t="s">
         <v>711</v>
-      </c>
-      <c r="D74" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E74" s="10" t="s">
-        <v>712</v>
       </c>
       <c r="F74" s="10"/>
     </row>
@@ -14583,19 +14580,19 @@
         <v>73</v>
       </c>
       <c r="B75" s="10" t="s">
+        <v>712</v>
+      </c>
+      <c r="C75" s="23" t="s">
         <v>713</v>
       </c>
-      <c r="C75" s="23" t="s">
+      <c r="D75" s="10" t="s">
+        <v>462</v>
+      </c>
+      <c r="E75" s="24" t="s">
         <v>714</v>
       </c>
-      <c r="D75" s="10" t="s">
-        <v>463</v>
-      </c>
-      <c r="E75" s="24" t="s">
-        <v>715</v>
-      </c>
       <c r="F75" s="10" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
@@ -14603,16 +14600,16 @@
         <v>74</v>
       </c>
       <c r="B76" s="10" t="s">
+        <v>715</v>
+      </c>
+      <c r="C76" s="23" t="s">
         <v>716</v>
       </c>
-      <c r="C76" s="23" t="s">
+      <c r="D76" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E76" s="10" t="s">
         <v>717</v>
-      </c>
-      <c r="D76" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E76" s="10" t="s">
-        <v>718</v>
       </c>
       <c r="F76" s="10"/>
     </row>
@@ -14621,16 +14618,16 @@
         <v>75</v>
       </c>
       <c r="B77" s="10" t="s">
+        <v>718</v>
+      </c>
+      <c r="C77" s="23" t="s">
         <v>719</v>
       </c>
-      <c r="C77" s="23" t="s">
+      <c r="D77" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E77" s="10" t="s">
         <v>720</v>
-      </c>
-      <c r="D77" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E77" s="10" t="s">
-        <v>721</v>
       </c>
       <c r="F77" s="10"/>
     </row>
@@ -14639,16 +14636,16 @@
         <v>76</v>
       </c>
       <c r="B78" s="10" t="s">
+        <v>721</v>
+      </c>
+      <c r="C78" s="23" t="s">
         <v>722</v>
       </c>
-      <c r="C78" s="23" t="s">
+      <c r="D78" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E78" s="10" t="s">
         <v>723</v>
-      </c>
-      <c r="D78" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E78" s="10" t="s">
-        <v>724</v>
       </c>
       <c r="F78" s="10"/>
     </row>
@@ -14660,13 +14657,13 @@
         <v>335</v>
       </c>
       <c r="C79" s="23" t="s">
+        <v>724</v>
+      </c>
+      <c r="D79" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E79" s="10" t="s">
         <v>725</v>
-      </c>
-      <c r="D79" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E79" s="10" t="s">
-        <v>726</v>
       </c>
       <c r="F79" s="10"/>
     </row>
@@ -14675,16 +14672,16 @@
         <v>78</v>
       </c>
       <c r="B80" s="10" t="s">
+        <v>726</v>
+      </c>
+      <c r="C80" s="23" t="s">
         <v>727</v>
       </c>
-      <c r="C80" s="23" t="s">
+      <c r="D80" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E80" s="10" t="s">
         <v>728</v>
-      </c>
-      <c r="D80" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E80" s="10" t="s">
-        <v>729</v>
       </c>
       <c r="F80" s="10"/>
     </row>
@@ -14693,16 +14690,16 @@
         <v>79</v>
       </c>
       <c r="B81" s="10" t="s">
+        <v>729</v>
+      </c>
+      <c r="C81" s="23" t="s">
         <v>730</v>
       </c>
-      <c r="C81" s="23" t="s">
+      <c r="D81" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E81" s="10" t="s">
         <v>731</v>
-      </c>
-      <c r="D81" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E81" s="10" t="s">
-        <v>732</v>
       </c>
       <c r="F81" s="10"/>
     </row>
@@ -14714,13 +14711,13 @@
         <v>260</v>
       </c>
       <c r="C82" s="23" t="s">
+        <v>732</v>
+      </c>
+      <c r="D82" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E82" s="10" t="s">
         <v>733</v>
-      </c>
-      <c r="D82" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E82" s="10" t="s">
-        <v>734</v>
       </c>
       <c r="F82" s="10"/>
     </row>
@@ -14732,13 +14729,13 @@
         <v>249</v>
       </c>
       <c r="C83" s="23" t="s">
+        <v>734</v>
+      </c>
+      <c r="D83" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E83" s="10" t="s">
         <v>735</v>
-      </c>
-      <c r="D83" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E83" s="10" t="s">
-        <v>736</v>
       </c>
       <c r="F83" s="10"/>
     </row>
@@ -14747,16 +14744,16 @@
         <v>82</v>
       </c>
       <c r="B84" s="10" t="s">
+        <v>736</v>
+      </c>
+      <c r="C84" s="23" t="s">
         <v>737</v>
       </c>
-      <c r="C84" s="23" t="s">
+      <c r="D84" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E84" s="10" t="s">
         <v>738</v>
-      </c>
-      <c r="D84" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E84" s="10" t="s">
-        <v>739</v>
       </c>
       <c r="F84" s="10"/>
     </row>
@@ -14765,16 +14762,16 @@
         <v>83</v>
       </c>
       <c r="B85" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="C85" s="23" t="s">
         <v>740</v>
       </c>
-      <c r="C85" s="23" t="s">
+      <c r="D85" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E85" s="10" t="s">
         <v>741</v>
-      </c>
-      <c r="D85" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E85" s="10" t="s">
-        <v>742</v>
       </c>
       <c r="F85" s="10"/>
     </row>
@@ -14783,16 +14780,16 @@
         <v>84</v>
       </c>
       <c r="B86" s="10" t="s">
+        <v>742</v>
+      </c>
+      <c r="C86" s="23" t="s">
         <v>743</v>
       </c>
-      <c r="C86" s="23" t="s">
+      <c r="D86" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E86" s="10" t="s">
         <v>744</v>
-      </c>
-      <c r="D86" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E86" s="10" t="s">
-        <v>745</v>
       </c>
       <c r="F86" s="10"/>
     </row>
@@ -14801,16 +14798,16 @@
         <v>85</v>
       </c>
       <c r="B87" s="10" t="s">
+        <v>745</v>
+      </c>
+      <c r="C87" s="23" t="s">
         <v>746</v>
       </c>
-      <c r="C87" s="23" t="s">
+      <c r="D87" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E87" s="10" t="s">
         <v>747</v>
-      </c>
-      <c r="D87" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E87" s="10" t="s">
-        <v>748</v>
       </c>
       <c r="F87" s="10"/>
     </row>
@@ -14819,16 +14816,16 @@
         <v>86</v>
       </c>
       <c r="B88" s="10" t="s">
+        <v>748</v>
+      </c>
+      <c r="C88" s="23" t="s">
         <v>749</v>
       </c>
-      <c r="C88" s="23" t="s">
+      <c r="D88" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E88" s="10" t="s">
         <v>750</v>
-      </c>
-      <c r="D88" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E88" s="10" t="s">
-        <v>751</v>
       </c>
       <c r="F88" s="10"/>
     </row>
@@ -14837,16 +14834,16 @@
         <v>87</v>
       </c>
       <c r="B89" s="10" t="s">
+        <v>751</v>
+      </c>
+      <c r="C89" s="23" t="s">
         <v>752</v>
       </c>
-      <c r="C89" s="23" t="s">
+      <c r="D89" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E89" s="10" t="s">
         <v>753</v>
-      </c>
-      <c r="D89" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E89" s="10" t="s">
-        <v>754</v>
       </c>
       <c r="F89" s="10"/>
     </row>
@@ -14855,16 +14852,16 @@
         <v>88</v>
       </c>
       <c r="B90" s="10" t="s">
+        <v>754</v>
+      </c>
+      <c r="C90" s="23" t="s">
         <v>755</v>
       </c>
-      <c r="C90" s="23" t="s">
+      <c r="D90" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E90" s="10" t="s">
         <v>756</v>
-      </c>
-      <c r="D90" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E90" s="10" t="s">
-        <v>757</v>
       </c>
       <c r="F90" s="10"/>
     </row>
@@ -14873,16 +14870,16 @@
         <v>89</v>
       </c>
       <c r="B91" s="10" t="s">
+        <v>757</v>
+      </c>
+      <c r="C91" s="23" t="s">
         <v>758</v>
       </c>
-      <c r="C91" s="23" t="s">
+      <c r="D91" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E91" s="10" t="s">
         <v>759</v>
-      </c>
-      <c r="D91" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E91" s="10" t="s">
-        <v>760</v>
       </c>
       <c r="F91" s="10"/>
     </row>
@@ -14894,13 +14891,13 @@
         <v>101</v>
       </c>
       <c r="C92" s="23" t="s">
+        <v>760</v>
+      </c>
+      <c r="D92" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E92" s="10" t="s">
         <v>761</v>
-      </c>
-      <c r="D92" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E92" s="10" t="s">
-        <v>762</v>
       </c>
       <c r="F92" s="10"/>
     </row>
@@ -14909,16 +14906,16 @@
         <v>91</v>
       </c>
       <c r="B93" s="10" t="s">
+        <v>762</v>
+      </c>
+      <c r="C93" s="23" t="s">
         <v>763</v>
       </c>
-      <c r="C93" s="23" t="s">
+      <c r="D93" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E93" s="10" t="s">
         <v>764</v>
-      </c>
-      <c r="D93" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E93" s="10" t="s">
-        <v>765</v>
       </c>
       <c r="F93" s="10"/>
     </row>
@@ -14927,16 +14924,16 @@
         <v>92</v>
       </c>
       <c r="B94" s="10" t="s">
+        <v>765</v>
+      </c>
+      <c r="C94" s="23" t="s">
         <v>766</v>
       </c>
-      <c r="C94" s="23" t="s">
+      <c r="D94" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E94" s="10" t="s">
         <v>767</v>
-      </c>
-      <c r="D94" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E94" s="10" t="s">
-        <v>768</v>
       </c>
       <c r="F94" s="10"/>
     </row>
@@ -14945,16 +14942,16 @@
         <v>93</v>
       </c>
       <c r="B95" s="10" t="s">
+        <v>768</v>
+      </c>
+      <c r="C95" s="23" t="s">
         <v>769</v>
       </c>
-      <c r="C95" s="23" t="s">
+      <c r="D95" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E95" s="10" t="s">
         <v>770</v>
-      </c>
-      <c r="D95" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E95" s="10" t="s">
-        <v>771</v>
       </c>
       <c r="F95" s="10"/>
     </row>
@@ -14963,16 +14960,16 @@
         <v>94</v>
       </c>
       <c r="B96" s="10" t="s">
+        <v>771</v>
+      </c>
+      <c r="C96" s="23" t="s">
         <v>772</v>
       </c>
-      <c r="C96" s="23" t="s">
+      <c r="D96" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E96" s="10" t="s">
         <v>773</v>
-      </c>
-      <c r="D96" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E96" s="10" t="s">
-        <v>774</v>
       </c>
       <c r="F96" s="10"/>
     </row>
@@ -14981,16 +14978,16 @@
         <v>95</v>
       </c>
       <c r="B97" s="10" t="s">
+        <v>774</v>
+      </c>
+      <c r="C97" s="23" t="s">
         <v>775</v>
       </c>
-      <c r="C97" s="23" t="s">
+      <c r="D97" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E97" s="10" t="s">
         <v>776</v>
-      </c>
-      <c r="D97" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E97" s="10" t="s">
-        <v>777</v>
       </c>
       <c r="F97" s="10"/>
     </row>
@@ -14999,16 +14996,16 @@
         <v>96</v>
       </c>
       <c r="B98" s="10" t="s">
+        <v>777</v>
+      </c>
+      <c r="C98" s="23" t="s">
         <v>778</v>
       </c>
-      <c r="C98" s="23" t="s">
+      <c r="D98" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="E98" s="10" t="s">
         <v>779</v>
-      </c>
-      <c r="D98" s="10" t="s">
-        <v>516</v>
-      </c>
-      <c r="E98" s="10" t="s">
-        <v>780</v>
       </c>
       <c r="F98" s="10"/>
     </row>
@@ -15020,13 +15017,13 @@
         <v>73</v>
       </c>
       <c r="C99" s="25" t="s">
+        <v>780</v>
+      </c>
+      <c r="D99" s="24" t="s">
+        <v>515</v>
+      </c>
+      <c r="E99" s="24" t="s">
         <v>781</v>
-      </c>
-      <c r="D99" s="24" t="s">
-        <v>516</v>
-      </c>
-      <c r="E99" s="24" t="s">
-        <v>782</v>
       </c>
       <c r="F99" s="24"/>
     </row>
@@ -15038,13 +15035,13 @@
         <v>362</v>
       </c>
       <c r="C100" s="25" t="s">
+        <v>782</v>
+      </c>
+      <c r="D100" s="24" t="s">
+        <v>515</v>
+      </c>
+      <c r="E100" s="24" t="s">
         <v>783</v>
-      </c>
-      <c r="D100" s="24" t="s">
-        <v>516</v>
-      </c>
-      <c r="E100" s="24" t="s">
-        <v>784</v>
       </c>
       <c r="F100" s="24"/>
     </row>
@@ -15056,13 +15053,13 @@
         <v>355</v>
       </c>
       <c r="C101" s="25" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="D101" s="24" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="E101" s="24" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="F101" s="24"/>
     </row>
@@ -15074,13 +15071,13 @@
         <v>373</v>
       </c>
       <c r="C102" s="25" t="s">
+        <v>785</v>
+      </c>
+      <c r="D102" s="24" t="s">
+        <v>515</v>
+      </c>
+      <c r="E102" s="24" t="s">
         <v>786</v>
-      </c>
-      <c r="D102" s="24" t="s">
-        <v>516</v>
-      </c>
-      <c r="E102" s="24" t="s">
-        <v>787</v>
       </c>
       <c r="F102" s="24"/>
     </row>
@@ -15092,13 +15089,13 @@
         <v>381</v>
       </c>
       <c r="C103" s="25" t="s">
+        <v>787</v>
+      </c>
+      <c r="D103" s="24" t="s">
+        <v>515</v>
+      </c>
+      <c r="E103" s="24" t="s">
         <v>788</v>
-      </c>
-      <c r="D103" s="24" t="s">
-        <v>516</v>
-      </c>
-      <c r="E103" s="24" t="s">
-        <v>789</v>
       </c>
       <c r="F103" s="24"/>
     </row>
@@ -15110,13 +15107,13 @@
         <v>80</v>
       </c>
       <c r="C104" s="25" t="s">
+        <v>789</v>
+      </c>
+      <c r="D104" s="24" t="s">
+        <v>515</v>
+      </c>
+      <c r="E104" s="24" t="s">
         <v>790</v>
-      </c>
-      <c r="D104" s="24" t="s">
-        <v>516</v>
-      </c>
-      <c r="E104" s="24" t="s">
-        <v>791</v>
       </c>
       <c r="F104" s="24"/>
     </row>
@@ -15128,13 +15125,13 @@
         <v>366</v>
       </c>
       <c r="C105" s="25" t="s">
+        <v>791</v>
+      </c>
+      <c r="D105" s="24" t="s">
+        <v>515</v>
+      </c>
+      <c r="E105" s="24" t="s">
         <v>792</v>
-      </c>
-      <c r="D105" s="24" t="s">
-        <v>516</v>
-      </c>
-      <c r="E105" s="24" t="s">
-        <v>793</v>
       </c>
       <c r="F105" s="24"/>
     </row>
@@ -15267,7 +15264,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -15277,10 +15274,10 @@
         <v>44</v>
       </c>
       <c r="B2" s="7" t="s">
+        <v>794</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>795</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>796</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -15288,10 +15285,10 @@
         <v>47</v>
       </c>
       <c r="B3" s="8" t="s">
+        <v>796</v>
+      </c>
+      <c r="C3" s="8" t="s">
         <v>797</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>798</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -15299,10 +15296,10 @@
         <v>49</v>
       </c>
       <c r="B4" s="8" t="s">
+        <v>798</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>799</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>800</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -15310,10 +15307,10 @@
         <v>51</v>
       </c>
       <c r="B5" s="8" t="s">
+        <v>800</v>
+      </c>
+      <c r="C5" s="8" t="s">
         <v>801</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>802</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -15321,10 +15318,10 @@
         <v>53</v>
       </c>
       <c r="B6" s="8" t="s">
+        <v>802</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>803</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>804</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -15332,10 +15329,10 @@
         <v>55</v>
       </c>
       <c r="B7" s="8" t="s">
+        <v>804</v>
+      </c>
+      <c r="C7" s="8" t="s">
         <v>805</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>806</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -15343,10 +15340,10 @@
         <v>56</v>
       </c>
       <c r="B8" s="8" t="s">
+        <v>806</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>807</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -15354,10 +15351,10 @@
         <v>57</v>
       </c>
       <c r="B9" s="8" t="s">
+        <v>808</v>
+      </c>
+      <c r="C9" s="8" t="s">
         <v>809</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>810</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -15365,10 +15362,10 @@
         <v>58</v>
       </c>
       <c r="B10" s="8" t="s">
+        <v>810</v>
+      </c>
+      <c r="C10" s="8" t="s">
         <v>811</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>812</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -15376,10 +15373,10 @@
         <v>59</v>
       </c>
       <c r="B11" s="8" t="s">
+        <v>812</v>
+      </c>
+      <c r="C11" s="8" t="s">
         <v>813</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>814</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
tracker: reconcile hides+jobs into xlsx; capture JSON-backed dashboard brainstorm
Reconcile step (xlsx is current SoT): apply 39 liveness/on-site hides that
had only landed in derived jobs.json, and promote 14 viable scanner jobs
into the Jobs sheet (98 visible / 44 hidden). This xlsx is the migration
seed for the JSON-backed dashboard brainstorm.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Job_Hunting_Progress.xlsx
+++ b/Job_Hunting_Progress.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1770" uniqueCount="814">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1935" uniqueCount="857">
   <si>
     <t>Hana Aliyah Mufidah</t>
   </si>
@@ -1264,6 +1264,138 @@
     <t>CS pivot off her SWE archetype; region flag. Edge is AI-forward automation (her own AI pipeline). Gaps: no formal customer-facing title, DNS depth. Prep: prep/hercules-technical-customer-support-engineer-2026-07-13.md</t>
   </si>
   <si>
+    <t>The Flex</t>
+  </si>
+  <si>
+    <t>Full-Stack Product Engineer</t>
+  </si>
+  <si>
+    <t>https://jobs.ashbyhq.com/The-Flex/82eafc9b-c4c0-4310-8b9d-9f5410ff0d53</t>
+  </si>
+  <si>
+    <t>career-ops scan (pipeline)</t>
+  </si>
+  <si>
+    <t>✅ Local/remote SE-Asia, no visa</t>
+  </si>
+  <si>
+    <t>From portal scan; viable location (no visa gate)</t>
+  </si>
+  <si>
+    <t>pending</t>
+  </si>
+  <si>
+    <t>Pending evaluation</t>
+  </si>
+  <si>
+    <t>Founding Software Engineer</t>
+  </si>
+  <si>
+    <t>https://jobs.ashbyhq.com/The-Flex/806abd84-e07a-4ffc-9823-39fa097896a4</t>
+  </si>
+  <si>
+    <t>Full-Stack Engineering Lead</t>
+  </si>
+  <si>
+    <t>https://jobs.ashbyhq.com/The-Flex/e8178837-0319-460c-8a51-6f9d5a6f36fa</t>
+  </si>
+  <si>
+    <t>https://jobs.ashbyhq.com/The-Flex/51693fcc-7a24-4a4c-9c87-84130b72c751</t>
+  </si>
+  <si>
+    <t>Software Engineer, Treasury</t>
+  </si>
+  <si>
+    <t>https://job-boards.eu.greenhouse.io/straitsx/jobs/4919950101</t>
+  </si>
+  <si>
+    <t>✅ Jakarta, Indonesia (local, no visa)</t>
+  </si>
+  <si>
+    <t>Evaluated 3.6/5 — see reports/</t>
+  </si>
+  <si>
+    <t>Backend Engineer - Card Issuing Team</t>
+  </si>
+  <si>
+    <t>https://job-boards.eu.greenhouse.io/straitsx/jobs/4925745101</t>
+  </si>
+  <si>
+    <t>apply</t>
+  </si>
+  <si>
+    <t>Evaluated 4.3/5 — see reports/</t>
+  </si>
+  <si>
+    <t>Software Engineer, Engineering Excellence</t>
+  </si>
+  <si>
+    <t>https://job-boards.eu.greenhouse.io/straitsx/jobs/4905659101</t>
+  </si>
+  <si>
+    <t>✅ Singapore (confirm Jakarta seat)</t>
+  </si>
+  <si>
+    <t>Evaluated 3.9/5 — see reports/</t>
+  </si>
+  <si>
+    <t>Startale Group</t>
+  </si>
+  <si>
+    <t>TypeScript Backend Engineer</t>
+  </si>
+  <si>
+    <t>https://job-boards.greenhouse.io/startale/jobs/5291409008</t>
+  </si>
+  <si>
+    <t>✅ Japan / Remote / Singapore (APAC)</t>
+  </si>
+  <si>
+    <t>Evaluated 4.4/5 — see reports/</t>
+  </si>
+  <si>
+    <t>OKX</t>
+  </si>
+  <si>
+    <t>Senior/Staff Software Engineer, Liquidity Platform</t>
+  </si>
+  <si>
+    <t>https://job-boards.greenhouse.io/okx/jobs/7774179003</t>
+  </si>
+  <si>
+    <t>✅ APAC-remote / global-remote, no visa</t>
+  </si>
+  <si>
+    <t>https://job-boards.greenhouse.io/okx/jobs/7774178003</t>
+  </si>
+  <si>
+    <t>Staff/Senior Staff Web3 Big Data Engineer</t>
+  </si>
+  <si>
+    <t>https://job-boards.greenhouse.io/okx/jobs/7795773003</t>
+  </si>
+  <si>
+    <t>Senior Software Engineer, AI Trading</t>
+  </si>
+  <si>
+    <t>https://job-boards.greenhouse.io/okx/jobs/7786389003</t>
+  </si>
+  <si>
+    <t>Senior/Staff Java Engineer - Web3 Wallet Defi Earn</t>
+  </si>
+  <si>
+    <t>https://job-boards.greenhouse.io/okx/jobs/7802448003</t>
+  </si>
+  <si>
+    <t>Alchemy</t>
+  </si>
+  <si>
+    <t>Backend Software Engineer</t>
+  </si>
+  <si>
+    <t>https://jobs.ashbyhq.com/alchemy/e9114029-c645-44f8-8f7e-9b718c10ad94</t>
+  </si>
+  <si>
     <t>Date</t>
   </si>
   <si>
@@ -1526,9 +1658,6 @@
   </si>
   <si>
     <t>career-ops scan / Greenhouse</t>
-  </si>
-  <si>
-    <t>https://job-boards.eu.greenhouse.io/straitsx/jobs/4925745101</t>
   </si>
   <si>
     <t>https://my.greenhouse.io/applications/63920375</t>
@@ -3719,7 +3848,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:M129"/>
+  <dimension ref="A1:M143"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="5" style="1" customWidth="1"/>
@@ -4017,6 +4146,9 @@
       <c r="K8" s="14" t="s">
         <v>106</v>
       </c>
+      <c r="L8" t="s">
+        <v>96</v>
+      </c>
       <c r="M8" s="14" t="s">
         <v>107</v>
       </c>
@@ -4051,6 +4183,9 @@
       <c r="K9" s="15" t="s">
         <v>106</v>
       </c>
+      <c r="L9" t="s">
+        <v>96</v>
+      </c>
       <c r="M9" s="15" t="s">
         <v>112</v>
       </c>
@@ -4119,6 +4254,9 @@
       <c r="K11" t="s">
         <v>106</v>
       </c>
+      <c r="L11" t="s">
+        <v>96</v>
+      </c>
       <c r="M11" t="s">
         <v>117</v>
       </c>
@@ -4289,6 +4427,9 @@
       <c r="K16" t="s">
         <v>106</v>
       </c>
+      <c r="L16" t="s">
+        <v>96</v>
+      </c>
       <c r="M16" t="s">
         <v>117</v>
       </c>
@@ -4323,6 +4464,9 @@
       <c r="K17" t="s">
         <v>106</v>
       </c>
+      <c r="L17" t="s">
+        <v>96</v>
+      </c>
       <c r="M17" t="s">
         <v>117</v>
       </c>
@@ -4357,6 +4501,9 @@
       <c r="K18" t="s">
         <v>106</v>
       </c>
+      <c r="L18" t="s">
+        <v>96</v>
+      </c>
       <c r="M18" t="s">
         <v>117</v>
       </c>
@@ -4391,6 +4538,9 @@
       <c r="K19" t="s">
         <v>106</v>
       </c>
+      <c r="L19" t="s">
+        <v>96</v>
+      </c>
       <c r="M19" t="s">
         <v>117</v>
       </c>
@@ -4425,6 +4575,9 @@
       <c r="K20" t="s">
         <v>106</v>
       </c>
+      <c r="L20" t="s">
+        <v>96</v>
+      </c>
       <c r="M20" t="s">
         <v>117</v>
       </c>
@@ -4459,6 +4612,9 @@
       <c r="K21" t="s">
         <v>106</v>
       </c>
+      <c r="L21" t="s">
+        <v>96</v>
+      </c>
       <c r="M21" t="s">
         <v>117</v>
       </c>
@@ -4493,6 +4649,9 @@
       <c r="K22" t="s">
         <v>106</v>
       </c>
+      <c r="L22" t="s">
+        <v>96</v>
+      </c>
       <c r="M22" t="s">
         <v>117</v>
       </c>
@@ -4527,6 +4686,9 @@
       <c r="K23" t="s">
         <v>106</v>
       </c>
+      <c r="L23" t="s">
+        <v>96</v>
+      </c>
       <c r="M23" t="s">
         <v>117</v>
       </c>
@@ -4561,6 +4723,9 @@
       <c r="K24" t="s">
         <v>106</v>
       </c>
+      <c r="L24" t="s">
+        <v>96</v>
+      </c>
       <c r="M24" t="s">
         <v>117</v>
       </c>
@@ -4595,6 +4760,9 @@
       <c r="K25" t="s">
         <v>106</v>
       </c>
+      <c r="L25" t="s">
+        <v>96</v>
+      </c>
       <c r="M25" t="s">
         <v>117</v>
       </c>
@@ -4629,6 +4797,9 @@
       <c r="K26" t="s">
         <v>106</v>
       </c>
+      <c r="L26" t="s">
+        <v>96</v>
+      </c>
       <c r="M26" t="s">
         <v>117</v>
       </c>
@@ -4969,6 +5140,9 @@
       <c r="K36" t="s">
         <v>106</v>
       </c>
+      <c r="L36" t="s">
+        <v>96</v>
+      </c>
       <c r="M36" t="s">
         <v>117</v>
       </c>
@@ -5003,6 +5177,9 @@
       <c r="K37" t="s">
         <v>106</v>
       </c>
+      <c r="L37" t="s">
+        <v>96</v>
+      </c>
       <c r="M37" t="s">
         <v>117</v>
       </c>
@@ -5717,6 +5894,9 @@
       <c r="K58" t="s">
         <v>106</v>
       </c>
+      <c r="L58" t="s">
+        <v>96</v>
+      </c>
       <c r="M58" t="s">
         <v>117</v>
       </c>
@@ -5751,6 +5931,9 @@
       <c r="K59" t="s">
         <v>106</v>
       </c>
+      <c r="L59" t="s">
+        <v>96</v>
+      </c>
       <c r="M59" t="s">
         <v>117</v>
       </c>
@@ -5785,6 +5968,9 @@
       <c r="K60" t="s">
         <v>106</v>
       </c>
+      <c r="L60" t="s">
+        <v>96</v>
+      </c>
       <c r="M60" t="s">
         <v>117</v>
       </c>
@@ -5819,6 +6005,9 @@
       <c r="K61" t="s">
         <v>106</v>
       </c>
+      <c r="L61" t="s">
+        <v>96</v>
+      </c>
       <c r="M61" t="s">
         <v>117</v>
       </c>
@@ -5853,6 +6042,9 @@
       <c r="K62" t="s">
         <v>106</v>
       </c>
+      <c r="L62" t="s">
+        <v>96</v>
+      </c>
       <c r="M62" t="s">
         <v>117</v>
       </c>
@@ -5887,6 +6079,9 @@
       <c r="K63" t="s">
         <v>106</v>
       </c>
+      <c r="L63" t="s">
+        <v>96</v>
+      </c>
       <c r="M63" t="s">
         <v>117</v>
       </c>
@@ -5921,6 +6116,9 @@
       <c r="K64" t="s">
         <v>106</v>
       </c>
+      <c r="L64" t="s">
+        <v>96</v>
+      </c>
       <c r="M64" t="s">
         <v>117</v>
       </c>
@@ -5955,6 +6153,9 @@
       <c r="K65" t="s">
         <v>106</v>
       </c>
+      <c r="L65" t="s">
+        <v>96</v>
+      </c>
       <c r="M65" t="s">
         <v>117</v>
       </c>
@@ -5989,6 +6190,9 @@
       <c r="K66" t="s">
         <v>106</v>
       </c>
+      <c r="L66" t="s">
+        <v>96</v>
+      </c>
       <c r="M66" t="s">
         <v>117</v>
       </c>
@@ -6023,6 +6227,9 @@
       <c r="K67" t="s">
         <v>106</v>
       </c>
+      <c r="L67" t="s">
+        <v>96</v>
+      </c>
       <c r="M67" t="s">
         <v>117</v>
       </c>
@@ -6057,6 +6264,9 @@
       <c r="K68" t="s">
         <v>106</v>
       </c>
+      <c r="L68" t="s">
+        <v>96</v>
+      </c>
       <c r="M68" t="s">
         <v>117</v>
       </c>
@@ -6091,6 +6301,9 @@
       <c r="K69" t="s">
         <v>106</v>
       </c>
+      <c r="L69" t="s">
+        <v>96</v>
+      </c>
       <c r="M69" t="s">
         <v>117</v>
       </c>
@@ -6125,6 +6338,9 @@
       <c r="K70" t="s">
         <v>106</v>
       </c>
+      <c r="L70" t="s">
+        <v>96</v>
+      </c>
       <c r="M70" t="s">
         <v>117</v>
       </c>
@@ -6159,6 +6375,9 @@
       <c r="K71" t="s">
         <v>106</v>
       </c>
+      <c r="L71" t="s">
+        <v>96</v>
+      </c>
       <c r="M71" t="s">
         <v>117</v>
       </c>
@@ -6193,6 +6412,9 @@
       <c r="K72" t="s">
         <v>106</v>
       </c>
+      <c r="L72" t="s">
+        <v>96</v>
+      </c>
       <c r="M72" t="s">
         <v>117</v>
       </c>
@@ -6227,6 +6449,9 @@
       <c r="K73" t="s">
         <v>106</v>
       </c>
+      <c r="L73" t="s">
+        <v>96</v>
+      </c>
       <c r="M73" t="s">
         <v>117</v>
       </c>
@@ -6261,6 +6486,9 @@
       <c r="K74" t="s">
         <v>106</v>
       </c>
+      <c r="L74" t="s">
+        <v>96</v>
+      </c>
       <c r="M74" t="s">
         <v>117</v>
       </c>
@@ -6295,6 +6523,9 @@
       <c r="K75" t="s">
         <v>106</v>
       </c>
+      <c r="L75" t="s">
+        <v>96</v>
+      </c>
       <c r="M75" t="s">
         <v>117</v>
       </c>
@@ -6329,6 +6560,9 @@
       <c r="K76" t="s">
         <v>106</v>
       </c>
+      <c r="L76" t="s">
+        <v>96</v>
+      </c>
       <c r="M76" t="s">
         <v>117</v>
       </c>
@@ -6363,6 +6597,9 @@
       <c r="K77" t="s">
         <v>106</v>
       </c>
+      <c r="L77" t="s">
+        <v>96</v>
+      </c>
       <c r="M77" t="s">
         <v>117</v>
       </c>
@@ -6397,6 +6634,9 @@
       <c r="K78" t="s">
         <v>106</v>
       </c>
+      <c r="L78" t="s">
+        <v>96</v>
+      </c>
       <c r="M78" t="s">
         <v>117</v>
       </c>
@@ -6464,6 +6704,9 @@
       <c r="J80" s="1"/>
       <c r="K80" t="s">
         <v>106</v>
+      </c>
+      <c r="L80" t="s">
+        <v>96</v>
       </c>
       <c r="M80" t="s">
         <v>117</v>
@@ -8040,7 +8283,9 @@
       <c r="K126" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="L126" s="20"/>
+      <c r="L126" s="20" t="s">
+        <v>96</v>
+      </c>
       <c r="M126" s="20" t="s">
         <v>395</v>
       </c>
@@ -8154,6 +8399,504 @@
       <c r="L129" s="20"/>
       <c r="M129" s="20" t="s">
         <v>414</v>
+      </c>
+    </row>
+    <row r="130" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A130" s="20">
+        <f>ROW()-1</f>
+      </c>
+      <c r="B130" s="20" t="s">
+        <v>396</v>
+      </c>
+      <c r="C130" s="20" t="s">
+        <v>415</v>
+      </c>
+      <c r="D130" s="20" t="s">
+        <v>416</v>
+      </c>
+      <c r="E130" s="20" t="s">
+        <v>417</v>
+      </c>
+      <c r="F130" s="20" t="s">
+        <v>418</v>
+      </c>
+      <c r="G130" s="20" t="s">
+        <v>419</v>
+      </c>
+      <c r="H130" s="20" t="s">
+        <v>420</v>
+      </c>
+      <c r="I130" s="20"/>
+      <c r="J130" s="20"/>
+      <c r="K130" s="20" t="s">
+        <v>421</v>
+      </c>
+      <c r="L130" s="20"/>
+      <c r="M130" s="20" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="131" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A131" s="20">
+        <f>ROW()-1</f>
+      </c>
+      <c r="B131" s="20" t="s">
+        <v>396</v>
+      </c>
+      <c r="C131" s="20" t="s">
+        <v>415</v>
+      </c>
+      <c r="D131" s="20" t="s">
+        <v>423</v>
+      </c>
+      <c r="E131" s="20" t="s">
+        <v>424</v>
+      </c>
+      <c r="F131" s="20" t="s">
+        <v>418</v>
+      </c>
+      <c r="G131" s="20" t="s">
+        <v>419</v>
+      </c>
+      <c r="H131" s="20" t="s">
+        <v>420</v>
+      </c>
+      <c r="I131" s="20"/>
+      <c r="J131" s="20"/>
+      <c r="K131" s="20" t="s">
+        <v>421</v>
+      </c>
+      <c r="L131" s="20"/>
+      <c r="M131" s="20" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="132" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A132" s="20">
+        <f>ROW()-1</f>
+      </c>
+      <c r="B132" s="20" t="s">
+        <v>396</v>
+      </c>
+      <c r="C132" s="20" t="s">
+        <v>415</v>
+      </c>
+      <c r="D132" s="20" t="s">
+        <v>425</v>
+      </c>
+      <c r="E132" s="20" t="s">
+        <v>426</v>
+      </c>
+      <c r="F132" s="20" t="s">
+        <v>418</v>
+      </c>
+      <c r="G132" s="20" t="s">
+        <v>419</v>
+      </c>
+      <c r="H132" s="20" t="s">
+        <v>420</v>
+      </c>
+      <c r="I132" s="20"/>
+      <c r="J132" s="20"/>
+      <c r="K132" s="20" t="s">
+        <v>421</v>
+      </c>
+      <c r="L132" s="20"/>
+      <c r="M132" s="20" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="133" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A133" s="20">
+        <f>ROW()-1</f>
+      </c>
+      <c r="B133" s="20" t="s">
+        <v>396</v>
+      </c>
+      <c r="C133" s="20" t="s">
+        <v>415</v>
+      </c>
+      <c r="D133" s="20" t="s">
+        <v>213</v>
+      </c>
+      <c r="E133" s="20" t="s">
+        <v>427</v>
+      </c>
+      <c r="F133" s="20" t="s">
+        <v>418</v>
+      </c>
+      <c r="G133" s="20" t="s">
+        <v>419</v>
+      </c>
+      <c r="H133" s="20" t="s">
+        <v>420</v>
+      </c>
+      <c r="I133" s="20"/>
+      <c r="J133" s="20"/>
+      <c r="K133" s="20" t="s">
+        <v>421</v>
+      </c>
+      <c r="L133" s="20"/>
+      <c r="M133" s="20" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="134" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A134" s="20">
+        <f>ROW()-1</f>
+      </c>
+      <c r="B134" s="20" t="s">
+        <v>396</v>
+      </c>
+      <c r="C134" s="20" t="s">
+        <v>373</v>
+      </c>
+      <c r="D134" s="20" t="s">
+        <v>428</v>
+      </c>
+      <c r="E134" s="20" t="s">
+        <v>429</v>
+      </c>
+      <c r="F134" s="20" t="s">
+        <v>418</v>
+      </c>
+      <c r="G134" s="20" t="s">
+        <v>430</v>
+      </c>
+      <c r="H134" s="20" t="s">
+        <v>420</v>
+      </c>
+      <c r="I134" s="20">
+        <v>3.6</v>
+      </c>
+      <c r="J134" s="20"/>
+      <c r="K134" s="20" t="s">
+        <v>421</v>
+      </c>
+      <c r="L134" s="20"/>
+      <c r="M134" s="20" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="135" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A135" s="20">
+        <f>ROW()-1</f>
+      </c>
+      <c r="B135" s="20" t="s">
+        <v>396</v>
+      </c>
+      <c r="C135" s="20" t="s">
+        <v>373</v>
+      </c>
+      <c r="D135" s="20" t="s">
+        <v>432</v>
+      </c>
+      <c r="E135" s="20" t="s">
+        <v>433</v>
+      </c>
+      <c r="F135" s="20" t="s">
+        <v>418</v>
+      </c>
+      <c r="G135" s="20" t="s">
+        <v>430</v>
+      </c>
+      <c r="H135" s="20" t="s">
+        <v>420</v>
+      </c>
+      <c r="I135" s="20">
+        <v>4.3</v>
+      </c>
+      <c r="J135" s="20"/>
+      <c r="K135" s="20" t="s">
+        <v>434</v>
+      </c>
+      <c r="L135" s="20"/>
+      <c r="M135" s="20" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="136" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A136" s="20">
+        <f>ROW()-1</f>
+      </c>
+      <c r="B136" s="20" t="s">
+        <v>396</v>
+      </c>
+      <c r="C136" s="20" t="s">
+        <v>373</v>
+      </c>
+      <c r="D136" s="20" t="s">
+        <v>436</v>
+      </c>
+      <c r="E136" s="20" t="s">
+        <v>437</v>
+      </c>
+      <c r="F136" s="20" t="s">
+        <v>418</v>
+      </c>
+      <c r="G136" s="20" t="s">
+        <v>438</v>
+      </c>
+      <c r="H136" s="20" t="s">
+        <v>420</v>
+      </c>
+      <c r="I136" s="20">
+        <v>3.9</v>
+      </c>
+      <c r="J136" s="20"/>
+      <c r="K136" s="20" t="s">
+        <v>421</v>
+      </c>
+      <c r="L136" s="20"/>
+      <c r="M136" s="20" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="137" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A137" s="20">
+        <f>ROW()-1</f>
+      </c>
+      <c r="B137" s="20" t="s">
+        <v>396</v>
+      </c>
+      <c r="C137" s="20" t="s">
+        <v>440</v>
+      </c>
+      <c r="D137" s="20" t="s">
+        <v>441</v>
+      </c>
+      <c r="E137" s="20" t="s">
+        <v>442</v>
+      </c>
+      <c r="F137" s="20" t="s">
+        <v>418</v>
+      </c>
+      <c r="G137" s="20" t="s">
+        <v>443</v>
+      </c>
+      <c r="H137" s="20" t="s">
+        <v>420</v>
+      </c>
+      <c r="I137" s="20">
+        <v>4.4</v>
+      </c>
+      <c r="J137" s="20"/>
+      <c r="K137" s="20" t="s">
+        <v>434</v>
+      </c>
+      <c r="L137" s="20"/>
+      <c r="M137" s="20" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="138" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A138" s="20">
+        <f>ROW()-1</f>
+      </c>
+      <c r="B138" s="20" t="s">
+        <v>396</v>
+      </c>
+      <c r="C138" s="20" t="s">
+        <v>445</v>
+      </c>
+      <c r="D138" s="20" t="s">
+        <v>446</v>
+      </c>
+      <c r="E138" s="20" t="s">
+        <v>447</v>
+      </c>
+      <c r="F138" s="20" t="s">
+        <v>418</v>
+      </c>
+      <c r="G138" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="H138" s="20" t="s">
+        <v>420</v>
+      </c>
+      <c r="I138" s="20"/>
+      <c r="J138" s="20"/>
+      <c r="K138" s="20" t="s">
+        <v>421</v>
+      </c>
+      <c r="L138" s="20"/>
+      <c r="M138" s="20" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="139" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A139" s="20">
+        <f>ROW()-1</f>
+      </c>
+      <c r="B139" s="20" t="s">
+        <v>396</v>
+      </c>
+      <c r="C139" s="20" t="s">
+        <v>445</v>
+      </c>
+      <c r="D139" s="20" t="s">
+        <v>446</v>
+      </c>
+      <c r="E139" s="20" t="s">
+        <v>449</v>
+      </c>
+      <c r="F139" s="20" t="s">
+        <v>418</v>
+      </c>
+      <c r="G139" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="H139" s="20" t="s">
+        <v>420</v>
+      </c>
+      <c r="I139" s="20"/>
+      <c r="J139" s="20"/>
+      <c r="K139" s="20" t="s">
+        <v>421</v>
+      </c>
+      <c r="L139" s="20"/>
+      <c r="M139" s="20" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="140" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A140" s="20">
+        <f>ROW()-1</f>
+      </c>
+      <c r="B140" s="20" t="s">
+        <v>396</v>
+      </c>
+      <c r="C140" s="20" t="s">
+        <v>445</v>
+      </c>
+      <c r="D140" s="20" t="s">
+        <v>450</v>
+      </c>
+      <c r="E140" s="20" t="s">
+        <v>451</v>
+      </c>
+      <c r="F140" s="20" t="s">
+        <v>418</v>
+      </c>
+      <c r="G140" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="H140" s="20" t="s">
+        <v>420</v>
+      </c>
+      <c r="I140" s="20"/>
+      <c r="J140" s="20"/>
+      <c r="K140" s="20" t="s">
+        <v>421</v>
+      </c>
+      <c r="L140" s="20"/>
+      <c r="M140" s="20" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="141" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A141" s="20">
+        <f>ROW()-1</f>
+      </c>
+      <c r="B141" s="20" t="s">
+        <v>396</v>
+      </c>
+      <c r="C141" s="20" t="s">
+        <v>445</v>
+      </c>
+      <c r="D141" s="20" t="s">
+        <v>452</v>
+      </c>
+      <c r="E141" s="20" t="s">
+        <v>453</v>
+      </c>
+      <c r="F141" s="20" t="s">
+        <v>418</v>
+      </c>
+      <c r="G141" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="H141" s="20" t="s">
+        <v>420</v>
+      </c>
+      <c r="I141" s="20"/>
+      <c r="J141" s="20"/>
+      <c r="K141" s="20" t="s">
+        <v>421</v>
+      </c>
+      <c r="L141" s="20"/>
+      <c r="M141" s="20" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="142" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A142" s="20">
+        <f>ROW()-1</f>
+      </c>
+      <c r="B142" s="20" t="s">
+        <v>396</v>
+      </c>
+      <c r="C142" s="20" t="s">
+        <v>445</v>
+      </c>
+      <c r="D142" s="20" t="s">
+        <v>454</v>
+      </c>
+      <c r="E142" s="20" t="s">
+        <v>455</v>
+      </c>
+      <c r="F142" s="20" t="s">
+        <v>418</v>
+      </c>
+      <c r="G142" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="H142" s="20" t="s">
+        <v>420</v>
+      </c>
+      <c r="I142" s="20"/>
+      <c r="J142" s="20"/>
+      <c r="K142" s="20" t="s">
+        <v>421</v>
+      </c>
+      <c r="L142" s="20"/>
+      <c r="M142" s="20" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="143" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A143" s="20">
+        <f>ROW()-1</f>
+      </c>
+      <c r="B143" s="20" t="s">
+        <v>396</v>
+      </c>
+      <c r="C143" s="20" t="s">
+        <v>456</v>
+      </c>
+      <c r="D143" s="20" t="s">
+        <v>457</v>
+      </c>
+      <c r="E143" s="20" t="s">
+        <v>458</v>
+      </c>
+      <c r="F143" s="20" t="s">
+        <v>418</v>
+      </c>
+      <c r="G143" s="20" t="s">
+        <v>448</v>
+      </c>
+      <c r="H143" s="20" t="s">
+        <v>420</v>
+      </c>
+      <c r="I143" s="20"/>
+      <c r="J143" s="20"/>
+      <c r="K143" s="20" t="s">
+        <v>421</v>
+      </c>
+      <c r="L143" s="20"/>
+      <c r="M143" s="20" t="s">
+        <v>422</v>
       </c>
     </row>
   </sheetData>
@@ -8304,7 +9047,7 @@
         <v>61</v>
       </c>
       <c r="B1" s="21" t="s">
-        <v>415</v>
+        <v>459</v>
       </c>
       <c r="C1" s="21" t="s">
         <v>14</v>
@@ -8316,28 +9059,28 @@
         <v>63</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>416</v>
+        <v>460</v>
       </c>
       <c r="G1" s="21" t="s">
-        <v>417</v>
+        <v>461</v>
       </c>
       <c r="H1" s="21" t="s">
-        <v>418</v>
+        <v>462</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>419</v>
+        <v>463</v>
       </c>
       <c r="J1" s="21" t="s">
-        <v>420</v>
+        <v>464</v>
       </c>
       <c r="K1" s="21" t="s">
-        <v>421</v>
+        <v>465</v>
       </c>
       <c r="L1" s="21" t="s">
-        <v>422</v>
+        <v>466</v>
       </c>
       <c r="M1" s="21" t="s">
-        <v>423</v>
+        <v>467</v>
       </c>
       <c r="N1" s="21" t="s">
         <v>71</v>
@@ -8357,37 +9100,37 @@
         <v>80</v>
       </c>
       <c r="D2" s="22" t="s">
-        <v>424</v>
+        <v>468</v>
       </c>
       <c r="E2" s="22" t="s">
         <v>82</v>
       </c>
       <c r="F2" s="22" t="s">
-        <v>425</v>
+        <v>469</v>
       </c>
       <c r="G2" s="22" t="s">
-        <v>426</v>
+        <v>470</v>
       </c>
       <c r="H2" s="20" t="s">
-        <v>427</v>
+        <v>471</v>
       </c>
       <c r="I2" s="22" t="s">
-        <v>428</v>
+        <v>472</v>
       </c>
       <c r="J2" s="22" t="s">
-        <v>429</v>
+        <v>473</v>
       </c>
       <c r="K2" s="22" t="s">
-        <v>430</v>
+        <v>474</v>
       </c>
       <c r="L2" s="22" t="s">
-        <v>431</v>
+        <v>475</v>
       </c>
       <c r="M2" s="22" t="s">
-        <v>432</v>
+        <v>476</v>
       </c>
       <c r="N2" s="22" t="s">
-        <v>433</v>
+        <v>477</v>
       </c>
       <c r="O2" s="1"/>
     </row>
@@ -8402,37 +9145,37 @@
         <v>80</v>
       </c>
       <c r="D3" s="22" t="s">
-        <v>434</v>
+        <v>478</v>
       </c>
       <c r="E3" s="22" t="s">
         <v>88</v>
       </c>
       <c r="F3" s="22" t="s">
-        <v>435</v>
+        <v>479</v>
       </c>
       <c r="G3" s="22" t="s">
-        <v>436</v>
+        <v>480</v>
       </c>
       <c r="H3" s="20" t="s">
-        <v>437</v>
+        <v>481</v>
       </c>
       <c r="I3" s="22" t="s">
-        <v>428</v>
+        <v>472</v>
       </c>
       <c r="J3" s="22" t="s">
-        <v>438</v>
+        <v>482</v>
       </c>
       <c r="K3" s="22" t="s">
-        <v>430</v>
+        <v>474</v>
       </c>
       <c r="L3" s="22" t="s">
-        <v>431</v>
+        <v>475</v>
       </c>
       <c r="M3" s="22" t="s">
-        <v>432</v>
+        <v>476</v>
       </c>
       <c r="N3" s="22" t="s">
-        <v>439</v>
+        <v>483</v>
       </c>
       <c r="O3" s="1"/>
     </row>
@@ -8447,37 +9190,37 @@
         <v>80</v>
       </c>
       <c r="D4" s="22" t="s">
-        <v>440</v>
+        <v>484</v>
       </c>
       <c r="E4" s="22" t="s">
         <v>91</v>
       </c>
       <c r="F4" s="22" t="s">
-        <v>441</v>
+        <v>485</v>
       </c>
       <c r="G4" s="22" t="s">
-        <v>442</v>
+        <v>486</v>
       </c>
       <c r="H4" s="20" t="s">
-        <v>443</v>
+        <v>487</v>
       </c>
       <c r="I4" s="22" t="s">
-        <v>444</v>
+        <v>488</v>
       </c>
       <c r="J4" s="22" t="s">
-        <v>445</v>
+        <v>489</v>
       </c>
       <c r="K4" s="22" t="s">
-        <v>446</v>
+        <v>490</v>
       </c>
       <c r="L4" s="22" t="s">
-        <v>431</v>
+        <v>475</v>
       </c>
       <c r="M4" s="22" t="s">
-        <v>447</v>
+        <v>491</v>
       </c>
       <c r="N4" s="22" t="s">
-        <v>448</v>
+        <v>492</v>
       </c>
       <c r="O4" s="1"/>
     </row>
@@ -8498,22 +9241,22 @@
         <v>346</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>449</v>
+        <v>493</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>450</v>
+        <v>494</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>451</v>
+        <v>495</v>
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1" t="s">
-        <v>452</v>
+        <v>496</v>
       </c>
       <c r="L5" s="1"/>
       <c r="M5" s="1" t="s">
-        <v>447</v>
+        <v>491</v>
       </c>
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
@@ -8535,27 +9278,27 @@
         <v>399</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>453</v>
+        <v>497</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>454</v>
+        <v>498</v>
       </c>
       <c r="H6" s="20" t="s">
-        <v>455</v>
+        <v>499</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>456</v>
+        <v>500</v>
       </c>
       <c r="J6" s="1"/>
       <c r="K6" s="1" t="s">
-        <v>457</v>
+        <v>501</v>
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1" t="s">
-        <v>447</v>
+        <v>491</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>458</v>
+        <v>502</v>
       </c>
       <c r="O6" s="1"/>
     </row>
@@ -8576,27 +9319,27 @@
         <v>406</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>453</v>
+        <v>497</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>454</v>
+        <v>498</v>
       </c>
       <c r="H7" s="20" t="s">
-        <v>459</v>
+        <v>503</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>456</v>
+        <v>500</v>
       </c>
       <c r="J7" s="1"/>
       <c r="K7" s="1" t="s">
-        <v>457</v>
+        <v>501</v>
       </c>
       <c r="L7" s="1"/>
       <c r="M7" s="1" t="s">
-        <v>447</v>
+        <v>491</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>458</v>
+        <v>502</v>
       </c>
       <c r="O7" s="1"/>
     </row>
@@ -8617,27 +9360,27 @@
         <v>410</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>449</v>
+        <v>493</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>460</v>
+        <v>504</v>
       </c>
       <c r="H8" s="20" t="s">
-        <v>461</v>
+        <v>505</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>462</v>
+        <v>506</v>
       </c>
       <c r="J8" s="1"/>
       <c r="K8" s="1" t="s">
-        <v>452</v>
+        <v>496</v>
       </c>
       <c r="L8" s="1"/>
       <c r="M8" s="1" t="s">
-        <v>447</v>
+        <v>491</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>463</v>
+        <v>507</v>
       </c>
       <c r="O8" s="1"/>
     </row>
@@ -8732,7 +9475,7 @@
         <v>61</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>464</v>
+        <v>508</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>14</v>
@@ -8741,10 +9484,10 @@
         <v>13</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>465</v>
+        <v>509</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>466</v>
+        <v>510</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>63</v>
@@ -8753,28 +9496,28 @@
         <v>44</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>467</v>
+        <v>511</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>468</v>
+        <v>512</v>
       </c>
       <c r="K1" s="7" t="s">
-        <v>469</v>
+        <v>513</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>470</v>
+        <v>514</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>471</v>
+        <v>515</v>
       </c>
       <c r="N1" s="7" t="s">
-        <v>472</v>
+        <v>516</v>
       </c>
       <c r="O1" s="7" t="s">
-        <v>473</v>
+        <v>517</v>
       </c>
       <c r="P1" s="7" t="s">
-        <v>474</v>
+        <v>518</v>
       </c>
       <c r="Q1" s="7" t="s">
         <v>71</v>
@@ -8797,10 +9540,10 @@
         <v>367</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>475</v>
+        <v>519</v>
       </c>
       <c r="F2" s="22" t="s">
-        <v>476</v>
+        <v>520</v>
       </c>
       <c r="G2" s="22" t="s">
         <v>368</v>
@@ -8812,24 +9555,24 @@
         <v>347</v>
       </c>
       <c r="J2" s="22" t="s">
-        <v>449</v>
+        <v>493</v>
       </c>
       <c r="K2" s="22" t="s">
-        <v>477</v>
+        <v>521</v>
       </c>
       <c r="L2" s="1"/>
       <c r="M2" s="22" t="s">
-        <v>478</v>
+        <v>522</v>
       </c>
       <c r="N2" s="1"/>
       <c r="O2" s="22" t="s">
-        <v>479</v>
+        <v>523</v>
       </c>
       <c r="P2" s="22" t="s">
-        <v>480</v>
+        <v>524</v>
       </c>
       <c r="Q2" s="22" t="s">
-        <v>481</v>
+        <v>525</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
@@ -8846,10 +9589,10 @@
         <v>374</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>482</v>
+        <v>526</v>
       </c>
       <c r="F3" s="22" t="s">
-        <v>483</v>
+        <v>527</v>
       </c>
       <c r="G3" s="22" t="s">
         <v>375</v>
@@ -8861,22 +9604,22 @@
         <v>347</v>
       </c>
       <c r="J3" s="22" t="s">
-        <v>449</v>
+        <v>493</v>
       </c>
       <c r="K3" s="22" t="s">
-        <v>484</v>
+        <v>528</v>
       </c>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
       <c r="O3" s="22" t="s">
-        <v>479</v>
+        <v>523</v>
       </c>
       <c r="P3" s="22" t="s">
-        <v>480</v>
+        <v>524</v>
       </c>
       <c r="Q3" s="22" t="s">
-        <v>485</v>
+        <v>529</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
@@ -8890,13 +9633,13 @@
         <v>80</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>424</v>
+        <v>468</v>
       </c>
       <c r="E4" s="22" t="s">
-        <v>486</v>
+        <v>530</v>
       </c>
       <c r="F4" s="22" t="s">
-        <v>487</v>
+        <v>531</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>82</v>
@@ -8908,28 +9651,28 @@
         <v>380</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>425</v>
+        <v>469</v>
       </c>
       <c r="K4" s="22" t="s">
-        <v>488</v>
+        <v>532</v>
       </c>
       <c r="L4" s="22" t="s">
-        <v>489</v>
+        <v>533</v>
       </c>
       <c r="M4" s="22" t="s">
-        <v>490</v>
+        <v>534</v>
       </c>
       <c r="N4" s="1" t="s">
-        <v>491</v>
+        <v>535</v>
       </c>
       <c r="O4" s="22" t="s">
-        <v>479</v>
+        <v>523</v>
       </c>
       <c r="P4" s="22" t="s">
-        <v>492</v>
+        <v>536</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>493</v>
+        <v>537</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
@@ -8943,13 +9686,13 @@
         <v>80</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>434</v>
+        <v>478</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>486</v>
+        <v>530</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>487</v>
+        <v>531</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>88</v>
@@ -8961,24 +9704,24 @@
         <v>380</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>435</v>
+        <v>479</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>488</v>
+        <v>532</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>494</v>
+        <v>538</v>
       </c>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
       <c r="O5" s="1" t="s">
-        <v>479</v>
+        <v>523</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>492</v>
+        <v>536</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>493</v>
+        <v>537</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
@@ -8995,7 +9738,7 @@
         <v>382</v>
       </c>
       <c r="E6" s="22" t="s">
-        <v>495</v>
+        <v>539</v>
       </c>
       <c r="F6" s="22" t="s">
         <v>384</v>
@@ -9010,26 +9753,26 @@
         <v>380</v>
       </c>
       <c r="J6" s="22" t="s">
-        <v>449</v>
+        <v>493</v>
       </c>
       <c r="K6" s="22" t="s">
-        <v>496</v>
+        <v>540</v>
       </c>
       <c r="L6" s="22"/>
       <c r="M6" s="22" t="s">
-        <v>497</v>
+        <v>541</v>
       </c>
       <c r="N6" s="22" t="s">
-        <v>498</v>
+        <v>542</v>
       </c>
       <c r="O6" s="22" t="s">
-        <v>479</v>
+        <v>523</v>
       </c>
       <c r="P6" s="22" t="s">
-        <v>492</v>
+        <v>536</v>
       </c>
       <c r="Q6" s="22" t="s">
-        <v>499</v>
+        <v>543</v>
       </c>
       <c r="R6" s="20"/>
     </row>
@@ -9044,16 +9787,16 @@
         <v>373</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>500</v>
+        <v>544</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>501</v>
+        <v>545</v>
       </c>
       <c r="F7" s="22" t="s">
-        <v>502</v>
+        <v>546</v>
       </c>
       <c r="G7" s="22" t="s">
-        <v>503</v>
+        <v>433</v>
       </c>
       <c r="H7" s="22" t="s">
         <v>51</v>
@@ -9064,18 +9807,18 @@
       <c r="J7" s="22"/>
       <c r="K7" s="22"/>
       <c r="L7" s="22" t="s">
-        <v>504</v>
+        <v>547</v>
       </c>
       <c r="M7" s="22"/>
       <c r="N7" s="22"/>
       <c r="O7" s="22" t="s">
-        <v>479</v>
+        <v>523</v>
       </c>
       <c r="P7" s="22" t="s">
-        <v>505</v>
+        <v>548</v>
       </c>
       <c r="Q7" s="22" t="s">
-        <v>506</v>
+        <v>549</v>
       </c>
       <c r="R7" s="20"/>
     </row>
@@ -13167,7 +13910,7 @@
         <v>356</v>
       </c>
       <c r="E202" s="20" t="s">
-        <v>507</v>
+        <v>550</v>
       </c>
       <c r="F202" s="20" t="s">
         <v>358</v>
@@ -13176,13 +13919,13 @@
         <v>357</v>
       </c>
       <c r="H202" s="20" t="s">
-        <v>508</v>
+        <v>551</v>
       </c>
       <c r="I202" s="20" t="s">
         <v>388</v>
       </c>
       <c r="J202" s="20" t="s">
-        <v>449</v>
+        <v>493</v>
       </c>
       <c r="K202" s="20"/>
       <c r="L202" s="20"/>
@@ -13253,7 +13996,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>509</v>
+        <v>552</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -13269,16 +14012,16 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>510</v>
+        <v>553</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>511</v>
+        <v>554</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>71</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>512</v>
+        <v>555</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -13286,13 +14029,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>513</v>
+        <v>556</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>514</v>
+        <v>557</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E3" s="10"/>
       <c r="F3" s="10"/>
@@ -13302,13 +14045,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>516</v>
+        <v>559</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>517</v>
+        <v>560</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E4" s="10"/>
       <c r="F4" s="10"/>
@@ -13318,16 +14061,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>518</v>
+        <v>561</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>519</v>
+        <v>562</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>520</v>
+        <v>563</v>
       </c>
       <c r="F5" s="10"/>
     </row>
@@ -13336,16 +14079,16 @@
         <v>4</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>521</v>
+        <v>564</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>522</v>
+        <v>565</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>523</v>
+        <v>566</v>
       </c>
       <c r="F6" s="10"/>
     </row>
@@ -13357,13 +14100,13 @@
         <v>240</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>524</v>
+        <v>567</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>525</v>
+        <v>568</v>
       </c>
       <c r="F7" s="10"/>
     </row>
@@ -13372,16 +14115,16 @@
         <v>6</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>526</v>
+        <v>569</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>527</v>
+        <v>570</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>528</v>
+        <v>571</v>
       </c>
       <c r="F8" s="10"/>
     </row>
@@ -13390,16 +14133,16 @@
         <v>7</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>529</v>
+        <v>572</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>530</v>
+        <v>573</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>531</v>
+        <v>574</v>
       </c>
       <c r="F9" s="10"/>
     </row>
@@ -13411,13 +14154,13 @@
         <v>141</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>532</v>
+        <v>575</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>533</v>
+        <v>576</v>
       </c>
       <c r="F10" s="10"/>
     </row>
@@ -13426,16 +14169,16 @@
         <v>9</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>534</v>
+        <v>577</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>535</v>
+        <v>578</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>536</v>
+        <v>579</v>
       </c>
       <c r="F11" s="10"/>
     </row>
@@ -13444,16 +14187,16 @@
         <v>10</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>537</v>
+        <v>580</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>538</v>
+        <v>581</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>539</v>
+        <v>582</v>
       </c>
       <c r="F12" s="10"/>
     </row>
@@ -13462,16 +14205,16 @@
         <v>11</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>540</v>
+        <v>583</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>541</v>
+        <v>584</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>542</v>
+        <v>585</v>
       </c>
       <c r="F13" s="10"/>
     </row>
@@ -13480,16 +14223,16 @@
         <v>12</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>543</v>
+        <v>586</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>544</v>
+        <v>587</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>545</v>
+        <v>588</v>
       </c>
       <c r="F14" s="10"/>
     </row>
@@ -13498,16 +14241,16 @@
         <v>13</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>546</v>
+        <v>589</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>547</v>
+        <v>590</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>548</v>
+        <v>591</v>
       </c>
       <c r="F15" s="10"/>
     </row>
@@ -13516,16 +14259,16 @@
         <v>14</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>549</v>
+        <v>592</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>550</v>
+        <v>593</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>551</v>
+        <v>594</v>
       </c>
       <c r="F16" s="10"/>
     </row>
@@ -13534,16 +14277,16 @@
         <v>15</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>552</v>
+        <v>595</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>553</v>
+        <v>596</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>554</v>
+        <v>597</v>
       </c>
       <c r="F17" s="10"/>
     </row>
@@ -13552,16 +14295,16 @@
         <v>16</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>555</v>
+        <v>598</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>556</v>
+        <v>599</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>557</v>
+        <v>600</v>
       </c>
       <c r="F18" s="10"/>
     </row>
@@ -13573,13 +14316,13 @@
         <v>179</v>
       </c>
       <c r="C19" s="23" t="s">
+        <v>601</v>
+      </c>
+      <c r="D19" s="10" t="s">
         <v>558</v>
       </c>
-      <c r="D19" s="10" t="s">
-        <v>515</v>
-      </c>
       <c r="E19" s="10" t="s">
-        <v>559</v>
+        <v>602</v>
       </c>
       <c r="F19" s="10"/>
     </row>
@@ -13588,16 +14331,16 @@
         <v>18</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>560</v>
+        <v>603</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>561</v>
+        <v>604</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>562</v>
+        <v>605</v>
       </c>
       <c r="F20" s="10"/>
     </row>
@@ -13606,16 +14349,16 @@
         <v>19</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>563</v>
+        <v>606</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>564</v>
+        <v>607</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>565</v>
+        <v>608</v>
       </c>
       <c r="F21" s="10"/>
     </row>
@@ -13624,16 +14367,16 @@
         <v>20</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>566</v>
+        <v>609</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>567</v>
+        <v>610</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>568</v>
+        <v>611</v>
       </c>
       <c r="F22" s="10"/>
     </row>
@@ -13642,16 +14385,16 @@
         <v>21</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>569</v>
+        <v>612</v>
       </c>
       <c r="C23" s="23" t="s">
-        <v>570</v>
+        <v>613</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>571</v>
+        <v>614</v>
       </c>
       <c r="F23" s="10"/>
     </row>
@@ -13660,16 +14403,16 @@
         <v>22</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>572</v>
+        <v>615</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>573</v>
+        <v>616</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>574</v>
+        <v>617</v>
       </c>
       <c r="F24" s="10"/>
     </row>
@@ -13678,16 +14421,16 @@
         <v>23</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>575</v>
+        <v>618</v>
       </c>
       <c r="C25" s="23" t="s">
-        <v>576</v>
+        <v>619</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>577</v>
+        <v>620</v>
       </c>
       <c r="F25" s="10"/>
     </row>
@@ -13696,16 +14439,16 @@
         <v>24</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>578</v>
+        <v>621</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>579</v>
+        <v>622</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>580</v>
+        <v>623</v>
       </c>
       <c r="F26" s="10"/>
     </row>
@@ -13714,16 +14457,16 @@
         <v>25</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>581</v>
+        <v>624</v>
       </c>
       <c r="C27" s="23" t="s">
-        <v>582</v>
+        <v>625</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>583</v>
+        <v>626</v>
       </c>
       <c r="F27" s="10"/>
     </row>
@@ -13732,16 +14475,16 @@
         <v>26</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>584</v>
+        <v>627</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>585</v>
+        <v>628</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>586</v>
+        <v>629</v>
       </c>
       <c r="F28" s="10"/>
     </row>
@@ -13750,16 +14493,16 @@
         <v>27</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>587</v>
+        <v>630</v>
       </c>
       <c r="C29" s="23" t="s">
-        <v>588</v>
+        <v>631</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>589</v>
+        <v>632</v>
       </c>
       <c r="F29" s="10"/>
     </row>
@@ -13768,16 +14511,16 @@
         <v>28</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>590</v>
+        <v>633</v>
       </c>
       <c r="C30" s="23" t="s">
-        <v>591</v>
+        <v>634</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>592</v>
+        <v>635</v>
       </c>
       <c r="F30" s="10"/>
     </row>
@@ -13786,16 +14529,16 @@
         <v>29</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>593</v>
+        <v>636</v>
       </c>
       <c r="C31" s="23" t="s">
-        <v>594</v>
+        <v>637</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>595</v>
+        <v>638</v>
       </c>
       <c r="F31" s="10"/>
     </row>
@@ -13804,16 +14547,16 @@
         <v>30</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>596</v>
+        <v>639</v>
       </c>
       <c r="C32" s="23" t="s">
-        <v>597</v>
+        <v>640</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>598</v>
+        <v>641</v>
       </c>
       <c r="F32" s="10"/>
     </row>
@@ -13822,16 +14565,16 @@
         <v>31</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>599</v>
+        <v>642</v>
       </c>
       <c r="C33" s="23" t="s">
-        <v>600</v>
+        <v>643</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>601</v>
+        <v>644</v>
       </c>
       <c r="F33" s="10"/>
     </row>
@@ -13843,13 +14586,13 @@
         <v>108</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>602</v>
+        <v>645</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>603</v>
+        <v>646</v>
       </c>
       <c r="F34" s="10"/>
     </row>
@@ -13861,13 +14604,13 @@
         <v>344</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>604</v>
+        <v>647</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>605</v>
+        <v>648</v>
       </c>
       <c r="F35" s="10"/>
     </row>
@@ -13876,16 +14619,16 @@
         <v>34</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>606</v>
+        <v>649</v>
       </c>
       <c r="C36" s="23" t="s">
-        <v>607</v>
+        <v>650</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>608</v>
+        <v>651</v>
       </c>
       <c r="F36" s="10"/>
     </row>
@@ -13897,13 +14640,13 @@
         <v>113</v>
       </c>
       <c r="C37" s="23" t="s">
-        <v>609</v>
+        <v>652</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>610</v>
+        <v>653</v>
       </c>
       <c r="F37" s="10"/>
     </row>
@@ -13912,16 +14655,16 @@
         <v>36</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>611</v>
+        <v>654</v>
       </c>
       <c r="C38" s="23" t="s">
-        <v>612</v>
+        <v>655</v>
       </c>
       <c r="D38" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>613</v>
+        <v>656</v>
       </c>
       <c r="F38" s="10"/>
     </row>
@@ -13930,16 +14673,16 @@
         <v>37</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>614</v>
+        <v>657</v>
       </c>
       <c r="C39" s="23" t="s">
-        <v>615</v>
+        <v>658</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>616</v>
+        <v>659</v>
       </c>
       <c r="F39" s="10"/>
     </row>
@@ -13948,16 +14691,16 @@
         <v>38</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>617</v>
+        <v>660</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>618</v>
+        <v>661</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>619</v>
+        <v>662</v>
       </c>
       <c r="F40" s="10"/>
     </row>
@@ -13969,13 +14712,13 @@
         <v>274</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>620</v>
+        <v>663</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>621</v>
+        <v>664</v>
       </c>
       <c r="F41" s="10"/>
     </row>
@@ -13984,16 +14727,16 @@
         <v>40</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>622</v>
+        <v>665</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>623</v>
+        <v>666</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>624</v>
+        <v>667</v>
       </c>
       <c r="F42" s="10"/>
     </row>
@@ -14002,16 +14745,16 @@
         <v>41</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>625</v>
+        <v>668</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>626</v>
+        <v>669</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>627</v>
+        <v>670</v>
       </c>
       <c r="F43" s="10"/>
     </row>
@@ -14020,16 +14763,16 @@
         <v>42</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>628</v>
+        <v>671</v>
       </c>
       <c r="C44" s="23" t="s">
-        <v>629</v>
+        <v>672</v>
       </c>
       <c r="D44" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>630</v>
+        <v>673</v>
       </c>
       <c r="F44" s="10"/>
     </row>
@@ -14038,16 +14781,16 @@
         <v>43</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>631</v>
+        <v>674</v>
       </c>
       <c r="C45" s="23" t="s">
-        <v>632</v>
+        <v>675</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>633</v>
+        <v>676</v>
       </c>
       <c r="F45" s="10"/>
     </row>
@@ -14059,13 +14802,13 @@
         <v>231</v>
       </c>
       <c r="C46" s="23" t="s">
-        <v>634</v>
+        <v>677</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>635</v>
+        <v>678</v>
       </c>
       <c r="F46" s="10"/>
     </row>
@@ -14074,16 +14817,16 @@
         <v>45</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>636</v>
+        <v>679</v>
       </c>
       <c r="C47" s="23" t="s">
-        <v>637</v>
+        <v>680</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>638</v>
+        <v>681</v>
       </c>
       <c r="F47" s="10"/>
     </row>
@@ -14095,13 +14838,13 @@
         <v>174</v>
       </c>
       <c r="C48" s="23" t="s">
-        <v>639</v>
+        <v>682</v>
       </c>
       <c r="D48" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>640</v>
+        <v>683</v>
       </c>
       <c r="F48" s="10"/>
     </row>
@@ -14110,16 +14853,16 @@
         <v>47</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>641</v>
+        <v>684</v>
       </c>
       <c r="C49" s="23" t="s">
-        <v>642</v>
+        <v>685</v>
       </c>
       <c r="D49" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E49" s="10" t="s">
-        <v>643</v>
+        <v>686</v>
       </c>
       <c r="F49" s="10"/>
     </row>
@@ -14128,16 +14871,16 @@
         <v>48</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>644</v>
+        <v>687</v>
       </c>
       <c r="C50" s="23" t="s">
-        <v>645</v>
+        <v>688</v>
       </c>
       <c r="D50" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>646</v>
+        <v>689</v>
       </c>
       <c r="F50" s="10"/>
     </row>
@@ -14146,16 +14889,16 @@
         <v>49</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>647</v>
+        <v>690</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>648</v>
+        <v>691</v>
       </c>
       <c r="D51" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>649</v>
+        <v>692</v>
       </c>
       <c r="F51" s="10"/>
     </row>
@@ -14164,16 +14907,16 @@
         <v>50</v>
       </c>
       <c r="B52" s="10" t="s">
-        <v>650</v>
+        <v>693</v>
       </c>
       <c r="C52" s="23" t="s">
-        <v>651</v>
+        <v>694</v>
       </c>
       <c r="D52" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>652</v>
+        <v>695</v>
       </c>
       <c r="F52" s="10"/>
     </row>
@@ -14182,16 +14925,16 @@
         <v>51</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>653</v>
+        <v>696</v>
       </c>
       <c r="C53" s="23" t="s">
-        <v>654</v>
+        <v>697</v>
       </c>
       <c r="D53" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>655</v>
+        <v>698</v>
       </c>
       <c r="F53" s="10"/>
     </row>
@@ -14200,16 +14943,16 @@
         <v>52</v>
       </c>
       <c r="B54" s="10" t="s">
-        <v>656</v>
+        <v>699</v>
       </c>
       <c r="C54" s="23" t="s">
-        <v>657</v>
+        <v>700</v>
       </c>
       <c r="D54" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>658</v>
+        <v>701</v>
       </c>
       <c r="F54" s="10"/>
     </row>
@@ -14218,16 +14961,16 @@
         <v>53</v>
       </c>
       <c r="B55" s="10" t="s">
-        <v>659</v>
+        <v>702</v>
       </c>
       <c r="C55" s="23" t="s">
-        <v>660</v>
+        <v>703</v>
       </c>
       <c r="D55" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>661</v>
+        <v>704</v>
       </c>
       <c r="F55" s="10"/>
     </row>
@@ -14236,16 +14979,16 @@
         <v>54</v>
       </c>
       <c r="B56" s="10" t="s">
-        <v>662</v>
+        <v>705</v>
       </c>
       <c r="C56" s="23" t="s">
-        <v>663</v>
+        <v>706</v>
       </c>
       <c r="D56" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E56" s="10" t="s">
-        <v>664</v>
+        <v>707</v>
       </c>
       <c r="F56" s="10"/>
     </row>
@@ -14254,16 +14997,16 @@
         <v>55</v>
       </c>
       <c r="B57" s="10" t="s">
-        <v>665</v>
+        <v>708</v>
       </c>
       <c r="C57" s="23" t="s">
-        <v>666</v>
+        <v>709</v>
       </c>
       <c r="D57" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>667</v>
+        <v>710</v>
       </c>
       <c r="F57" s="10"/>
     </row>
@@ -14272,16 +15015,16 @@
         <v>56</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>668</v>
+        <v>711</v>
       </c>
       <c r="C58" s="23" t="s">
-        <v>669</v>
+        <v>712</v>
       </c>
       <c r="D58" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E58" s="10" t="s">
-        <v>670</v>
+        <v>713</v>
       </c>
       <c r="F58" s="10"/>
     </row>
@@ -14293,13 +15036,13 @@
         <v>212</v>
       </c>
       <c r="C59" s="23" t="s">
-        <v>671</v>
+        <v>714</v>
       </c>
       <c r="D59" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>672</v>
+        <v>715</v>
       </c>
       <c r="F59" s="10"/>
     </row>
@@ -14311,13 +15054,13 @@
         <v>120</v>
       </c>
       <c r="C60" s="23" t="s">
-        <v>673</v>
+        <v>716</v>
       </c>
       <c r="D60" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E60" s="10" t="s">
-        <v>674</v>
+        <v>717</v>
       </c>
       <c r="F60" s="10"/>
     </row>
@@ -14329,13 +15072,13 @@
         <v>129</v>
       </c>
       <c r="C61" s="23" t="s">
-        <v>675</v>
+        <v>718</v>
       </c>
       <c r="D61" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E61" s="10" t="s">
-        <v>676</v>
+        <v>719</v>
       </c>
       <c r="F61" s="10"/>
     </row>
@@ -14347,13 +15090,13 @@
         <v>154</v>
       </c>
       <c r="C62" s="23" t="s">
-        <v>677</v>
+        <v>720</v>
       </c>
       <c r="D62" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E62" s="10" t="s">
-        <v>678</v>
+        <v>721</v>
       </c>
       <c r="F62" s="10"/>
     </row>
@@ -14362,16 +15105,16 @@
         <v>61</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>679</v>
+        <v>722</v>
       </c>
       <c r="C63" s="23" t="s">
-        <v>680</v>
+        <v>723</v>
       </c>
       <c r="D63" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E63" s="10" t="s">
-        <v>681</v>
+        <v>724</v>
       </c>
       <c r="F63" s="10"/>
     </row>
@@ -14383,13 +15126,13 @@
         <v>301</v>
       </c>
       <c r="C64" s="23" t="s">
-        <v>682</v>
+        <v>725</v>
       </c>
       <c r="D64" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E64" s="10" t="s">
-        <v>683</v>
+        <v>726</v>
       </c>
       <c r="F64" s="10"/>
     </row>
@@ -14398,16 +15141,16 @@
         <v>63</v>
       </c>
       <c r="B65" s="10" t="s">
-        <v>684</v>
+        <v>727</v>
       </c>
       <c r="C65" s="23" t="s">
-        <v>685</v>
+        <v>728</v>
       </c>
       <c r="D65" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E65" s="10" t="s">
-        <v>686</v>
+        <v>729</v>
       </c>
       <c r="F65" s="10"/>
     </row>
@@ -14416,19 +15159,19 @@
         <v>64</v>
       </c>
       <c r="B66" s="10" t="s">
-        <v>687</v>
+        <v>730</v>
       </c>
       <c r="C66" s="23" t="s">
-        <v>688</v>
+        <v>731</v>
       </c>
       <c r="D66" s="10" t="s">
-        <v>462</v>
+        <v>506</v>
       </c>
       <c r="E66" s="24" t="s">
-        <v>689</v>
+        <v>732</v>
       </c>
       <c r="F66" s="10" t="s">
-        <v>690</v>
+        <v>733</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
@@ -14439,13 +15182,13 @@
         <v>328</v>
       </c>
       <c r="C67" s="23" t="s">
-        <v>691</v>
+        <v>734</v>
       </c>
       <c r="D67" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>692</v>
+        <v>735</v>
       </c>
       <c r="F67" s="10"/>
     </row>
@@ -14454,16 +15197,16 @@
         <v>66</v>
       </c>
       <c r="B68" s="10" t="s">
-        <v>693</v>
+        <v>736</v>
       </c>
       <c r="C68" s="23" t="s">
-        <v>694</v>
+        <v>737</v>
       </c>
       <c r="D68" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E68" s="10" t="s">
-        <v>695</v>
+        <v>738</v>
       </c>
       <c r="F68" s="10"/>
     </row>
@@ -14472,16 +15215,16 @@
         <v>67</v>
       </c>
       <c r="B69" s="10" t="s">
-        <v>696</v>
+        <v>739</v>
       </c>
       <c r="C69" s="23" t="s">
-        <v>697</v>
+        <v>740</v>
       </c>
       <c r="D69" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E69" s="10" t="s">
-        <v>698</v>
+        <v>741</v>
       </c>
       <c r="F69" s="10"/>
     </row>
@@ -14490,16 +15233,16 @@
         <v>68</v>
       </c>
       <c r="B70" s="10" t="s">
-        <v>699</v>
+        <v>742</v>
       </c>
       <c r="C70" s="23" t="s">
-        <v>700</v>
+        <v>743</v>
       </c>
       <c r="D70" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E70" s="10" t="s">
-        <v>701</v>
+        <v>744</v>
       </c>
       <c r="F70" s="10"/>
     </row>
@@ -14511,13 +15254,13 @@
         <v>138</v>
       </c>
       <c r="C71" s="23" t="s">
-        <v>702</v>
+        <v>745</v>
       </c>
       <c r="D71" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E71" s="10" t="s">
-        <v>703</v>
+        <v>746</v>
       </c>
       <c r="F71" s="10"/>
     </row>
@@ -14526,16 +15269,16 @@
         <v>70</v>
       </c>
       <c r="B72" s="10" t="s">
-        <v>704</v>
+        <v>747</v>
       </c>
       <c r="C72" s="23" t="s">
-        <v>705</v>
+        <v>748</v>
       </c>
       <c r="D72" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E72" s="10" t="s">
-        <v>706</v>
+        <v>749</v>
       </c>
       <c r="F72" s="10"/>
     </row>
@@ -14544,16 +15287,16 @@
         <v>71</v>
       </c>
       <c r="B73" s="10" t="s">
-        <v>707</v>
+        <v>750</v>
       </c>
       <c r="C73" s="23" t="s">
-        <v>708</v>
+        <v>751</v>
       </c>
       <c r="D73" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E73" s="10" t="s">
-        <v>709</v>
+        <v>752</v>
       </c>
       <c r="F73" s="10"/>
     </row>
@@ -14565,13 +15308,13 @@
         <v>311</v>
       </c>
       <c r="C74" s="23" t="s">
-        <v>710</v>
+        <v>753</v>
       </c>
       <c r="D74" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E74" s="10" t="s">
-        <v>711</v>
+        <v>754</v>
       </c>
       <c r="F74" s="10"/>
     </row>
@@ -14580,19 +15323,19 @@
         <v>73</v>
       </c>
       <c r="B75" s="10" t="s">
-        <v>712</v>
+        <v>755</v>
       </c>
       <c r="C75" s="23" t="s">
-        <v>713</v>
+        <v>756</v>
       </c>
       <c r="D75" s="10" t="s">
-        <v>462</v>
+        <v>506</v>
       </c>
       <c r="E75" s="24" t="s">
-        <v>714</v>
+        <v>757</v>
       </c>
       <c r="F75" s="10" t="s">
-        <v>690</v>
+        <v>733</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
@@ -14600,16 +15343,16 @@
         <v>74</v>
       </c>
       <c r="B76" s="10" t="s">
-        <v>715</v>
+        <v>758</v>
       </c>
       <c r="C76" s="23" t="s">
-        <v>716</v>
+        <v>759</v>
       </c>
       <c r="D76" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E76" s="10" t="s">
-        <v>717</v>
+        <v>760</v>
       </c>
       <c r="F76" s="10"/>
     </row>
@@ -14618,16 +15361,16 @@
         <v>75</v>
       </c>
       <c r="B77" s="10" t="s">
-        <v>718</v>
+        <v>761</v>
       </c>
       <c r="C77" s="23" t="s">
-        <v>719</v>
+        <v>762</v>
       </c>
       <c r="D77" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>720</v>
+        <v>763</v>
       </c>
       <c r="F77" s="10"/>
     </row>
@@ -14636,16 +15379,16 @@
         <v>76</v>
       </c>
       <c r="B78" s="10" t="s">
-        <v>721</v>
+        <v>764</v>
       </c>
       <c r="C78" s="23" t="s">
-        <v>722</v>
+        <v>765</v>
       </c>
       <c r="D78" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E78" s="10" t="s">
-        <v>723</v>
+        <v>766</v>
       </c>
       <c r="F78" s="10"/>
     </row>
@@ -14657,13 +15400,13 @@
         <v>335</v>
       </c>
       <c r="C79" s="23" t="s">
-        <v>724</v>
+        <v>767</v>
       </c>
       <c r="D79" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E79" s="10" t="s">
-        <v>725</v>
+        <v>768</v>
       </c>
       <c r="F79" s="10"/>
     </row>
@@ -14672,16 +15415,16 @@
         <v>78</v>
       </c>
       <c r="B80" s="10" t="s">
-        <v>726</v>
+        <v>769</v>
       </c>
       <c r="C80" s="23" t="s">
-        <v>727</v>
+        <v>770</v>
       </c>
       <c r="D80" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E80" s="10" t="s">
-        <v>728</v>
+        <v>771</v>
       </c>
       <c r="F80" s="10"/>
     </row>
@@ -14690,16 +15433,16 @@
         <v>79</v>
       </c>
       <c r="B81" s="10" t="s">
-        <v>729</v>
+        <v>772</v>
       </c>
       <c r="C81" s="23" t="s">
-        <v>730</v>
+        <v>773</v>
       </c>
       <c r="D81" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>731</v>
+        <v>774</v>
       </c>
       <c r="F81" s="10"/>
     </row>
@@ -14711,13 +15454,13 @@
         <v>260</v>
       </c>
       <c r="C82" s="23" t="s">
-        <v>732</v>
+        <v>775</v>
       </c>
       <c r="D82" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E82" s="10" t="s">
-        <v>733</v>
+        <v>776</v>
       </c>
       <c r="F82" s="10"/>
     </row>
@@ -14729,13 +15472,13 @@
         <v>249</v>
       </c>
       <c r="C83" s="23" t="s">
-        <v>734</v>
+        <v>777</v>
       </c>
       <c r="D83" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>735</v>
+        <v>778</v>
       </c>
       <c r="F83" s="10"/>
     </row>
@@ -14744,16 +15487,16 @@
         <v>82</v>
       </c>
       <c r="B84" s="10" t="s">
-        <v>736</v>
+        <v>779</v>
       </c>
       <c r="C84" s="23" t="s">
-        <v>737</v>
+        <v>780</v>
       </c>
       <c r="D84" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E84" s="10" t="s">
-        <v>738</v>
+        <v>781</v>
       </c>
       <c r="F84" s="10"/>
     </row>
@@ -14762,16 +15505,16 @@
         <v>83</v>
       </c>
       <c r="B85" s="10" t="s">
-        <v>739</v>
+        <v>782</v>
       </c>
       <c r="C85" s="23" t="s">
-        <v>740</v>
+        <v>783</v>
       </c>
       <c r="D85" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E85" s="10" t="s">
-        <v>741</v>
+        <v>784</v>
       </c>
       <c r="F85" s="10"/>
     </row>
@@ -14780,16 +15523,16 @@
         <v>84</v>
       </c>
       <c r="B86" s="10" t="s">
-        <v>742</v>
+        <v>785</v>
       </c>
       <c r="C86" s="23" t="s">
-        <v>743</v>
+        <v>786</v>
       </c>
       <c r="D86" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E86" s="10" t="s">
-        <v>744</v>
+        <v>787</v>
       </c>
       <c r="F86" s="10"/>
     </row>
@@ -14798,16 +15541,16 @@
         <v>85</v>
       </c>
       <c r="B87" s="10" t="s">
-        <v>745</v>
+        <v>788</v>
       </c>
       <c r="C87" s="23" t="s">
-        <v>746</v>
+        <v>789</v>
       </c>
       <c r="D87" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E87" s="10" t="s">
-        <v>747</v>
+        <v>790</v>
       </c>
       <c r="F87" s="10"/>
     </row>
@@ -14816,16 +15559,16 @@
         <v>86</v>
       </c>
       <c r="B88" s="10" t="s">
-        <v>748</v>
+        <v>791</v>
       </c>
       <c r="C88" s="23" t="s">
-        <v>749</v>
+        <v>792</v>
       </c>
       <c r="D88" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E88" s="10" t="s">
-        <v>750</v>
+        <v>793</v>
       </c>
       <c r="F88" s="10"/>
     </row>
@@ -14834,16 +15577,16 @@
         <v>87</v>
       </c>
       <c r="B89" s="10" t="s">
-        <v>751</v>
+        <v>794</v>
       </c>
       <c r="C89" s="23" t="s">
-        <v>752</v>
+        <v>795</v>
       </c>
       <c r="D89" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E89" s="10" t="s">
-        <v>753</v>
+        <v>796</v>
       </c>
       <c r="F89" s="10"/>
     </row>
@@ -14852,16 +15595,16 @@
         <v>88</v>
       </c>
       <c r="B90" s="10" t="s">
-        <v>754</v>
+        <v>797</v>
       </c>
       <c r="C90" s="23" t="s">
-        <v>755</v>
+        <v>798</v>
       </c>
       <c r="D90" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E90" s="10" t="s">
-        <v>756</v>
+        <v>799</v>
       </c>
       <c r="F90" s="10"/>
     </row>
@@ -14870,16 +15613,16 @@
         <v>89</v>
       </c>
       <c r="B91" s="10" t="s">
-        <v>757</v>
+        <v>800</v>
       </c>
       <c r="C91" s="23" t="s">
-        <v>758</v>
+        <v>801</v>
       </c>
       <c r="D91" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E91" s="10" t="s">
-        <v>759</v>
+        <v>802</v>
       </c>
       <c r="F91" s="10"/>
     </row>
@@ -14891,13 +15634,13 @@
         <v>101</v>
       </c>
       <c r="C92" s="23" t="s">
-        <v>760</v>
+        <v>803</v>
       </c>
       <c r="D92" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E92" s="10" t="s">
-        <v>761</v>
+        <v>804</v>
       </c>
       <c r="F92" s="10"/>
     </row>
@@ -14906,16 +15649,16 @@
         <v>91</v>
       </c>
       <c r="B93" s="10" t="s">
-        <v>762</v>
+        <v>805</v>
       </c>
       <c r="C93" s="23" t="s">
-        <v>763</v>
+        <v>806</v>
       </c>
       <c r="D93" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E93" s="10" t="s">
-        <v>764</v>
+        <v>807</v>
       </c>
       <c r="F93" s="10"/>
     </row>
@@ -14924,16 +15667,16 @@
         <v>92</v>
       </c>
       <c r="B94" s="10" t="s">
-        <v>765</v>
+        <v>808</v>
       </c>
       <c r="C94" s="23" t="s">
-        <v>766</v>
+        <v>809</v>
       </c>
       <c r="D94" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E94" s="10" t="s">
-        <v>767</v>
+        <v>810</v>
       </c>
       <c r="F94" s="10"/>
     </row>
@@ -14942,16 +15685,16 @@
         <v>93</v>
       </c>
       <c r="B95" s="10" t="s">
-        <v>768</v>
+        <v>811</v>
       </c>
       <c r="C95" s="23" t="s">
-        <v>769</v>
+        <v>812</v>
       </c>
       <c r="D95" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E95" s="10" t="s">
-        <v>770</v>
+        <v>813</v>
       </c>
       <c r="F95" s="10"/>
     </row>
@@ -14960,16 +15703,16 @@
         <v>94</v>
       </c>
       <c r="B96" s="10" t="s">
-        <v>771</v>
+        <v>814</v>
       </c>
       <c r="C96" s="23" t="s">
-        <v>772</v>
+        <v>815</v>
       </c>
       <c r="D96" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E96" s="10" t="s">
-        <v>773</v>
+        <v>816</v>
       </c>
       <c r="F96" s="10"/>
     </row>
@@ -14978,16 +15721,16 @@
         <v>95</v>
       </c>
       <c r="B97" s="10" t="s">
-        <v>774</v>
+        <v>817</v>
       </c>
       <c r="C97" s="23" t="s">
-        <v>775</v>
+        <v>818</v>
       </c>
       <c r="D97" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E97" s="10" t="s">
-        <v>776</v>
+        <v>819</v>
       </c>
       <c r="F97" s="10"/>
     </row>
@@ -14996,16 +15739,16 @@
         <v>96</v>
       </c>
       <c r="B98" s="10" t="s">
-        <v>777</v>
+        <v>820</v>
       </c>
       <c r="C98" s="23" t="s">
-        <v>778</v>
+        <v>821</v>
       </c>
       <c r="D98" s="10" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E98" s="10" t="s">
-        <v>779</v>
+        <v>822</v>
       </c>
       <c r="F98" s="10"/>
     </row>
@@ -15017,13 +15760,13 @@
         <v>73</v>
       </c>
       <c r="C99" s="25" t="s">
-        <v>780</v>
+        <v>823</v>
       </c>
       <c r="D99" s="24" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E99" s="24" t="s">
-        <v>781</v>
+        <v>824</v>
       </c>
       <c r="F99" s="24"/>
     </row>
@@ -15035,13 +15778,13 @@
         <v>362</v>
       </c>
       <c r="C100" s="25" t="s">
-        <v>782</v>
+        <v>825</v>
       </c>
       <c r="D100" s="24" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E100" s="24" t="s">
-        <v>783</v>
+        <v>826</v>
       </c>
       <c r="F100" s="24"/>
     </row>
@@ -15053,13 +15796,13 @@
         <v>355</v>
       </c>
       <c r="C101" s="25" t="s">
-        <v>782</v>
+        <v>825</v>
       </c>
       <c r="D101" s="24" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E101" s="24" t="s">
-        <v>784</v>
+        <v>827</v>
       </c>
       <c r="F101" s="24"/>
     </row>
@@ -15071,13 +15814,13 @@
         <v>373</v>
       </c>
       <c r="C102" s="25" t="s">
-        <v>785</v>
+        <v>828</v>
       </c>
       <c r="D102" s="24" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E102" s="24" t="s">
-        <v>786</v>
+        <v>829</v>
       </c>
       <c r="F102" s="24"/>
     </row>
@@ -15089,13 +15832,13 @@
         <v>381</v>
       </c>
       <c r="C103" s="25" t="s">
-        <v>787</v>
+        <v>830</v>
       </c>
       <c r="D103" s="24" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E103" s="24" t="s">
-        <v>788</v>
+        <v>831</v>
       </c>
       <c r="F103" s="24"/>
     </row>
@@ -15107,13 +15850,13 @@
         <v>80</v>
       </c>
       <c r="C104" s="25" t="s">
-        <v>789</v>
+        <v>832</v>
       </c>
       <c r="D104" s="24" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E104" s="24" t="s">
-        <v>790</v>
+        <v>833</v>
       </c>
       <c r="F104" s="24"/>
     </row>
@@ -15125,13 +15868,13 @@
         <v>366</v>
       </c>
       <c r="C105" s="25" t="s">
-        <v>791</v>
+        <v>834</v>
       </c>
       <c r="D105" s="24" t="s">
-        <v>515</v>
+        <v>558</v>
       </c>
       <c r="E105" s="24" t="s">
-        <v>792</v>
+        <v>835</v>
       </c>
       <c r="F105" s="24"/>
     </row>
@@ -15264,7 +16007,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>793</v>
+        <v>836</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -15274,10 +16017,10 @@
         <v>44</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>794</v>
+        <v>837</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>795</v>
+        <v>838</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -15285,10 +16028,10 @@
         <v>47</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>796</v>
+        <v>839</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>797</v>
+        <v>840</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -15296,10 +16039,10 @@
         <v>49</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>798</v>
+        <v>841</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>799</v>
+        <v>842</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -15307,10 +16050,10 @@
         <v>51</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>800</v>
+        <v>843</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>801</v>
+        <v>844</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -15318,10 +16061,10 @@
         <v>53</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>802</v>
+        <v>845</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>803</v>
+        <v>846</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -15329,10 +16072,10 @@
         <v>55</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>804</v>
+        <v>847</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>805</v>
+        <v>848</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -15340,10 +16083,10 @@
         <v>56</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>806</v>
+        <v>849</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>807</v>
+        <v>850</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -15351,10 +16094,10 @@
         <v>57</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>808</v>
+        <v>851</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>809</v>
+        <v>852</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -15362,10 +16105,10 @@
         <v>58</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>810</v>
+        <v>853</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>811</v>
+        <v>854</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -15373,10 +16116,10 @@
         <v>59</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>812</v>
+        <v>855</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>813</v>
+        <v>856</v>
       </c>
     </row>
   </sheetData>

</xml_diff>